<commit_message>
Improving the Top sources
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="123">
   <si>
     <t>timestamp</t>
   </si>
@@ -160,6 +160,21 @@
     <t>2025-09-19T14:41:22.557021</t>
   </si>
   <si>
+    <t>2025-09-19T15:45:45.428812</t>
+  </si>
+  <si>
+    <t>2025-09-19T15:48:16.253621</t>
+  </si>
+  <si>
+    <t>2025-09-19T15:50:58.980303</t>
+  </si>
+  <si>
+    <t>2025-09-19T15:57:36.879063</t>
+  </si>
+  <si>
+    <t>2025-09-19T15:59:13.835247</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -173,6 +188,9 @@
   </si>
   <si>
     <t xml:space="preserve"> What evidence architecture and rigor standards underpin the report’s claims? </t>
+  </si>
+  <si>
+    <t>What is the 2025–30 Impact Assessment (IA) strategy addressing, and what will be delivered to funders and managers?</t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -217,6 +235,9 @@
   </si>
   <si>
     <t>pdf:CGIAR_ImpactReport_2022-24.pdf:p67pt1:0.176, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.132, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p1pt2:0.127, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1:0.125, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p17pt3:0.119, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt2:0.119, pdf:Type3_2024Report.pdf:p4pt1:0.119, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4:0.117, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4:0.109, pdf:Portfolio Narrative_2024.pdf:p6pt1:0.106, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.106, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3:0.104, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt1:0.102, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p22pt3:0.102, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p1pt1:0.102, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p24pt3:0.101, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p29pt2:0.099, docx:Submitting evidence.docx:u1-4:0.099, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt4:0.098, pdf:CGIAR_ImpactReport_2022-24.pdf:p66pt2:0.097, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4:0.096, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p17pt2:0.095, pdf:CGIAR_ImpactReport_2022-24.pdf:p66pt4:0.095, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p17pt2:0.095, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p1pt1:0.095, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p28pt3:0.093, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt1:0.092, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt1:0.092, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p8pt4:0.092, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1:0.092, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt1:0.092, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt1:0.091, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt1:0.091, pdf:Climate Action_Inception Report 30-06-2025.pdf:p26pt3:0.091, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p4pt4:0.090, pdf:Type3_2024Report.pdf:p4pt2:0.090, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.090, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.090, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p16pt1:0.089, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p1pt2:0.089, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p27pt3:0.089, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p9pt2:0.089, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p17pt1:0.088, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p6pt3:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p17pt2:0.088, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt4:0.087, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p1pt1:0.087, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p19pt3:0.087, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p9pt1:0.087, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt4:0.087, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p12pt4:0.086, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt1:0.085, docx:Guidance on ensuring quality over quantity.docx:u4-7:0.084, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3:0.084, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt1:0.084, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p6pt4:0.084, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.083, pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt3:0.083, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p19pt2:0.082, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.082, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt3:0.082, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.082, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt3:0.080, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p1pt1:0.080, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p4pt1:0.080, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt1:0.080, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.080, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.079, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt4:0.078, pdf:Climate Action_Inception Report 30-06-2025.pdf:p12pt1:0.078, pdf:Genebanks_Inception Report 30-06-2025.pdf:p1pt1:0.078, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt1:0.078, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt3:0.078, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p4pt4:0.078, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p28pt2:0.077, pdf:Climate Action_Inception Report 30-06-2025.pdf:p7pt3:0.077, pdf:Portfolio Narrative_2024.pdf:p6pt2:0.077, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p29pt1:0.077, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.077, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt2:0.077, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p32pt2:0.076, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p15pt2:0.076, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p30pt2:0.076, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt2:0.076, pdf:Portfolio Narrative_2024.pdf:p6pt4:0.075, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p1pt1:0.075, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p13pt3:0.075, pdf:Type3_2024Report.pdf:p1pt1:0.075, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.075, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p9pt3:0.074, pdf:CGI21_508012_PORB_Genebanks.pdf:p40pt4:0.074, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p1pt2:0.074, pdf:Climate Action_Inception Report 30-06-2025.pdf:p5pt2:0.074, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p15pt3:0.073, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.072, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt3:0.072, pdf:CGI21_508012_PORB_Genebanks.pdf:p49pt4:0.072</t>
+  </si>
+  <si>
+    <t>docx:Engagement Plan 2025 Technical Reporting.docx:u46-49:0.248, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt4:0.241, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.233, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4:0.225, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt3:0.220, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt1:0.215, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3:0.215, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1:0.213, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt1:0.205, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.203, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p2pt2:0.195, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p18pt3:0.194, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p14pt1:0.192, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.191, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt3:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23pt2:0.189, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p2pt2:0.188, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt2:0.185, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3:0.183, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2:0.183, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3:0.183, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p13pt3:0.183, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2:0.182, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2:0.182, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2:0.182, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2:0.182, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.182, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.182, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.182, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.182, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.180, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt2:0.179, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt2:0.179, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p19pt4:0.178, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p2pt4:0.177, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt2:0.177, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p50pt3:0.177, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.176, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt3:0.176, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt3:0.175, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1:0.175, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1:0.174, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.173, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p2pt3:0.171, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt4:0.171, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.170, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3:0.169, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p2pt2:0.167, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p2pt3:0.165, pdf:CGIAR_ImpactReport_2022-24.pdf:p9pt1:0.164, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.164, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.162, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.162, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.161, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.160, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt3:0.160, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p2pt3:0.158, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.157, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p35pt1:0.157, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p18pt2:0.156, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt1:0.156, pdf:Type3_2024Report.pdf:p6pt2:0.156, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.155, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.154, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt1:0.154, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4:0.153, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p34pt4:0.153, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt4:0.152, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p10pt1:0.151, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.151, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p10pt2:0.150, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p16pt3:0.150, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p22pt4:0.149, pdf:Climate Action_Inception Report 30-06-2025.pdf:p16pt3:0.149, pdf:Type3_2024Report.pdf:p11pt1:0.148, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1:0.148, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p9pt1:0.147, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p10pt4:0.147, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.147, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt2:0.147, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p20pt4:0.147, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p6pt3:0.146, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt2:0.146, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3:0.146, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p17pt3:0.146, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.146, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p15pt2:0.146, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p16pt2:0.145, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.145, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p15pt1:0.144, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p22pt4:0.144, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p15pt2:0.144, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.144, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt2:0.143, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p22pt3:0.143, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt4:0.143, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3:0.143, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1:0.142, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.141, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p2pt2:0.141</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -431,6 +452,22 @@
 CGIAR_ImpactReport_2022-24.pdf — page 46 part 3 — pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3</t>
   </si>
   <si>
+    <t>The 2025–30 Impact Assessment (IA) strategy focuses on evaluating the causal effects of research outputs and related activities, aiming to measure the magnitude of impact achieved across various interventions. It emphasizes a bottom-up approach to ensure that the assessments provide sufficient evidence against CGIAR impact indicators. Deliverables to funders and managers will include comprehensive reports on the findings from these assessments, which will be accessible to program managers, researchers, and external stakeholders. This strategy aims to enhance the coherence and quality of information sourced from different funding avenues over time. 
+Sources:
+File — Location — Cited IDs
+pdf:Genebanks_MELIA Plan 30-06-2025.pdf — page 8 part 4 — [ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]
+pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 17 part 1 — [ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1]
+pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf — page 18 part 3 — [ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p18pt3]</t>
+  </si>
+  <si>
+    <t>The 2025–30 Impact Assessment (IA) strategy focuses on evaluating the causal effects of research outputs and related activities, aiming to measure the magnitude of impact achieved across various interventions. It emphasizes a bottom-up approach to ensure that the assessments provide sufficient evidence against CGIAR impact indicators. Deliverables to funders and managers will include comprehensive reports on the impact assessments, which will be informed by both quantitative and qualitative data, and will help in making necessary adjustments to program implementations based on the findings. This strategy is designed to enhance the coherence and quality of information sourced from different funding avenues over time. 
+Sources:
+File — Location — Cited IDs
+pdf:Genebanks_MELIA Plan 30-06-2025.pdf — page 8 part 4 — 4
+pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 17 part 1 — 6
+pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf — page 18 part 3 — 4</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -450,6 +487,9 @@
   </si>
   <si>
     <t>https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9 — page 67 part 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p67pt1, https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9 — page 7 part 3 — pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1 — page 1 part 2 — pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p1pt2</t>
+  </si>
+  <si>
+    <t>Engagement Plan: 2025 Technical Reporting (Full Word document) — section 'Fortnightly update emails' paragraph 80 to section 'Fortnightly update emails' paragraph 83 — docx:Engagement Plan 2025 Technical Reporting.docx:u46-49, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1 — page 29 part 4 — pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt4, https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 2 part 1 — pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -666,6 +706,148 @@
 with other CGIAR reporting products. Section 1: Introduction 1 Un</t>
   </si>
   <si>
+    <t>[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u46-49]
+CGSpace Team Lead KM Managers Curators/Repository Managers PRMS Team
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt4]
+The current funding landscape uncertainty as well as a realistic assessment of resources that can be dedicated to IA led us to prioritize IA activities in 6 countries, where we can easily leverage on human and financial resources for impact assessment: Colombia, Peru, Tunisia, Kenya, India, Vietnam. The site prioritization, as well as prioritization of the key impact indicators that the IA should target (potential indicators are presented in the table below), will be a specific action of the MELIA team at the end of 2025, when future financial capacity will be clearer. Further funding for IA studies will be sought in 2026 and during the implementation of
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]
+Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]
+exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. Impact assessments are conducted after an intervention has been completed and are used to substantiate claims of sustained results. They seek to measure impact at scale, i.e., benefits to a large number of people/large areas of land. It employs both quantitative and qualitative methods, often combined for deeper insights. IA goes beyond monitoring indicators to evidenced attribution of observed changes to CGIAR interventions. IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives.
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt3]
+the learnings and what are other critical areas that require further focused support? (AoW 5) Evaluation collaboration plans Genebanks will seek to collaborate with the Multifunctional Landscapes Program to study in situ and on farm site monitoring of diversity conservation. Genebanks will also collaborate with the Crop Trust and Aarhus University to review the Scientific Impact of the Seed Quality Management and Quality Management System Communities of Practice. Collaborations with W3/bilateral projects will be explored during phase 2 of the mapping exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 10 Thematic Impact 2022-30 Report The Thematic Impact 2022 -30 Report provides a m acro level view of CGIAR’s role in Food, Land and Water System Transformation covering the period 2022 -30. It will be released in 2031. Its format and content will be developed during the period 2025-30. Results Dashboard • The Results Dashboard will be enhanced to better present curated information a gainst Impact Area targets, geographies and key topics. • Headline impacts and outcomes will be more clearly communicated in the Dashboard. • Using AI, users will be able to easily query the results data and underlying sources of evidence data using
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3]
+Impact assessment (IA) .............................................................................................................. 13 Program impact overview .................................................................................................................... 13 IA activities and collaboration plans ..................................................................................................... 14 IA studies ........................................................................................................................................... 15 5. Learning and adaptive management ........................................................................................... 16 Learning ............................................................................................................................................. 16 Annual review and adaptive planning ...................................................................................................
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 17 The amount of quality information sourced from different funding sources, and the coherence between those different information sources will increase over time (specific metrics and targets to be developed) 6. Impact Assessment Strategy/ Approach/ Case studies CGIAR will develop a 2025 -30 Impact Assessment Plan and integrate its design, budgeting and delivery into the 25-30 Portfolio. The bottom-up approach to impact assessment that has been used within CGIAR for the past decades has not produced sufficient quantity or quality of studies to prov ide evidence against CGIAR impact indicators. SPIA fills in some of this gap, but even their new undertaking of country studies will likely not be able to contribute to most of the indicators
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt1]
+• Bilateral/W3-funded projects: to identify embedded impact assessment opportunities and avoid duplication. • CGIAR IA teams : to contribute to portfolio -level meta -evaluation and harmonize data with common CGIAR indicators. Priority will be given to impact in integrative countries, where multiple AoWs operate. These broader IA studies will assess the synergies between interventions and provide system -level insights into the pathways driving impact. Potential integrative countries include Bangladesh, Ethiopia, Nigeria, and Tanzania, based on portfolio density and MELIA feasibility. A senior Impact Specialist will guide study design and implementation, ensure alignment with the CGIAR results framework indicators, and coordinate data quality assurance across IA efforts. Impact assessment studies The Program has identified initial IA study themes for inclusion in the MELIA studies. However , these initial themes are not included in the
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3]
+activities of the CapSha Accelerator, its products and services, contribute to improved capacity development practices, resulting in more equitable partnerships? • Are CGIAR NARES partners, donors and CapSha expert institutions making use of CapSha products and services? • Are CGIAR NARES partners, donors and CapSha expert institutions member of the CapSha Cop? • To what extent are the CapSha Accelerator’s objectives aligned with the needs and priorities of Southern partners? • What elements of the partnership model have the potential to be scaled or replicated in other regions or contexts? What are the enabling and limiting factors affecting scalability? How have Southern partners contributed to or led scaling efforts, and what support mechanisms have been most effective? • What measurable
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p2pt2]
+................................ ................................ ............... 7 Data collection strategy ................................ ................................ ................................ 7 3. Evaluation plan ................................ ................................ ................................ ..................... 7 Evaluation studies ................................ ................................ ................................ ....... 7 Evaluation collaboration plans ................................ ................................ ....................... 8 4. Impact assessment ................................ ................................ ................................ ............... 8 Program/Accelerator impact overview ................................ ................................ ............ 8 IA activities and collaboration
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p18pt3]
+All the knowledge generated by these studies will be available not only to Program managers, but also researchers, the CGIAR community, and external stakeholders. Finally, analyzing monitoring data will be a continuous process, and results, along with recommendations, will be made available to Program managers to make any necessary adjustments to the Program implementation. Annual review and adaptive planning The Climate Action Program will implement an annual review and adaptive planning process, building on the experience and lessons from the 2022–24 CGIAR Portfolio and aligned with evolving guidance on the Reﬂect and Re-Plan processes. Each year, the Program will conduct structured annual performance reviews at both program-wide and AoW levels. These reviews will assess progress toward the intended outputs and outcomes, using both quantitative and qualitative data drawn from the CGIAR Performance and Results Management System
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p14pt1]
+14 5. Impact assessment Impact Assessment (IA) is a key approach for evaluating the effectiveness and impact of innovations, technologies, or practices on target populations and geographies. By systematically measuring outcomes and impacts, IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives. IA goes beyond monitoring indicators, requiring a rigorous approach to attribut ing observed changes to CGIAR interventions (e.g., innovations, policies). It employs both quantitative and qualitative methods, often combined for deeper insights. Program/Accelerator impact overview The AoWs of the Sustainable Framing Program will collectively contribute to the program’s outcomes and expected impacts by co -developing and delivering whole -farm innovation bundles to at least five million farmers, with positive impacts on socially equitable and sustainable agronomic gain across two million ha of land. At least 50 public and private development partners are expected to facilitate the scaling of solutions to farming communities and integrating innovations in their investments.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]
+2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt3]
+the Policy Program is no exception. Recurring assumptions in the ToC revolve around empowering actors and creating improved knowledge and building capacity to empower these actors. This theme is at the heart of the P olicy Program's operations, encompassing concepts such as co -creation and demand-driven research that build capacity and create the right conditions for policy change to occur. IA activities and collaboration plans The Impact Assessment (IA) strategy employs a combination of quantitative (both experimental and non-experimental) and qualitative (outcome evidencing) research methods to substantiate the Program's contributions to CGIAR's Impact Areas. Additionally, rapid impact assessment methods are utilized when necessary to track achievements and support swift policy responses. Aligned with the learning objectives of the Monitoring, Evaluation, and Learning (MEL) component, the IA strategy provides empirical evidence on the Program's effects, aiming to understand the causal mechanisms underlying both expected and unanticipated outcomes. Each of the 2030
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23pt2]
+into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p2pt2]
+Monitoring plan for HLOs and outcomes ........................................................................................ 7 Data collection strategy ...................................................................................................... 7 3. Evaluation plan ................................................................................................................................ 8 Evaluation studies .............................................................................................................. 8 Evaluation collaboration plans ............................................................................................ 8 4. Impact assessment .......................................................................................................................... 8 Program/Accelerator impact overview ................................................................................. 9 IA activities
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt2]
+for high-level outputs (HLOs) and outcomes ........................................................ 7 Data collection strategy ........................................................................................................................ 7 3. Evaluation plan ........................................................................................................................... 9 Evaluation studies .............................................................................................................................. 10 Evaluation collaboration plans ............................................................................................................ 12 4. Impact assessment (IA) .............................................................................................................. 13 Program impact overview ....................................................................................................................
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3]
+and Impact Assessment (MELIA)
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2]
+and Impact Assessment (MELIA)
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3]
+section): • Under what conditions and through which mechanisms agroecological and nature positive approaches, within a multifunctional landscape lens, optimize landscape multifunctionality? • What are the behavioral outcomes of such a multifunctional landscapes approach? For whom? Under what conditions? The following MELIA studies will allow us to answer these questions through multiple analysis angles. System Based Theory of Change: in order to analyze how the changes at the landscape level influenced by the Program will generate changes at the country level and be influenced by changes at the country level, we will implement System Based Theory of Change methodology developed by Worldfish (see references in the Evidence Base section under Impact Assessment). We will engage relevant landscape stakeholders in pilot landscapes (e.g. Peru, Kenya,
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p13pt3]
+is built on the assumption that shifting harmful gender norms and unequal power dynamics is foundational to achieving sustained, system -level transformation in FLWS. Detailed assumptions can be found in the (please refer to the Results Framework attachment ). Strong relationships with Science Programs such as Breeding for Tomorrow, Climate Action, Food Frontiers and Security, Better Diets for Nutrition, and Scaling for Impact, ensuring gender-focused research is integrated across CGIAR’s Portfolio. IA activities and collaboration plans The Gender Accelerator’s approach to impact assessment (IA) relies on the premise that research questions should drive the methodological approach and depending on the decisions that need to be informed, the appropriate type of evidence must be generated. Based on this, the IA activities of the Accelerator use both causal and non -causal impact assessments — recognizing that only causal
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p29pt4]
+on ground results, and if not, why not (AOW2 AB)? RQ14 What additional impact could be achieved with additional investment? (AOW1 MI) RQ15 What is the trajectory of genetic gain for each crop, and what benefits could this mean for smallholder farmers who adopt improved products? (AOW4 BR) RQ16 When is the scale of adoption for recently released varieties and products in the pipeline expected to be sufficient to reduce weighted average variety age (WAVA) in targeted market segments to 10 years or less? (AOW3 ID) Demonstrate impacts achieved by B4T and encourage ongoing investment Identify opportunities to improve uptake and adoption, to maximize impact Guide future target
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt4]
+of environmental conditions controlled and high heritability of targeted traits. Quality of science is required for Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended The first part of RQ15 What is the trajectory of genetic gain for each crop, is relevant here. RQ21 To what extent have market set targets been successfully converted into breeding targets? (AOW2 AB) 1 It would be ideal to question if the level of benefit gained from adoption of improved varieties was sufficient for empowerme nt. However, determining the sufficiency of benefit is likely to be unfeasible in the timeframe and resourcing available. Opportun ities to incorporate data collection at this depth of enquiry should be keep in mind.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4]
+and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt2]
+Reports are shared for integration, Centers will have a role in r eviewing and validating how their information is represented in aggregate Program/Accelerator and Portfolio reporting. 5. A set of Impact Studies responding to the CGIAR Results Framework and key strategic questions from Funders/Partners/Global Leadership will be integrated into the design and delivery of the Programs &amp; Accelerators; W3/bilaterals may contribute to these. 6. Funders and Centers will be able to adopt more/fully aligned monitoring and reporting approaches for their w3 and bilateral projects during development. It will also be possible to increase alignment during the implementation of a w3/bilateral project through e.g. the contribution to Impact Case Studies. 7. Common CGIAR best of class indicators, data collection protocols, tools, and systems will be promoted for use in W3/bilateral project design. The CGIAR Monitoring, Evaluation and Learning Community of
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt2]
+results from other authoritative internal and external databases. The Results Dashboard will provide greater access to evidence of CGIAR’s contribution to impact based on quality-assured data. Triennial reports covering the periods 25-27 and 28-30 will consolidate Portfolio -level contribution to Impact targets. A Thematic Impact report will compile results delivered against the CGIAR Research and Innovation Strategy for the full period 2022-30. Technical Report product Content overview – All content will progressively integrate pooled and non-pooled content Periodicity Annual Program/ Accelerator Report - Annual
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p19pt4]
+IFPRI Kenya Causal impact assessment Q4 2025 Q1 2027 Effectivenes s of STIBs; research question: what are the TBD in WCA, ESA, SA Causal impact assessment
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p2pt4]
+.................................................................. 27 7. Plan of Results and Budget ............................................................................................ 28 8. Cross-Portfolio linkages and geographic coordination .................................................... 30 8.1 Cross-portfolio linkages .......................................................................................... 30 8.2 Geographic coordination ......................................................................................... 30 9. Risk management .......................................................................................................... 31 10. Addressing feedback on select topics .......................................................................... 33 Appendix 1: Addressing specific feedback..........................................................................
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt2]
+outcomes and i mpacts of the whole portfolio through progressive alignment of reporting on w3/bilaterally funded components with a common framework. • Line of sight: The TRA is designed to meet the needs of diverse funders, ensuring transparency and accountability by linking investment to results, both for pooled and non-pooled funds. • Impact focus: Research results will be better linked to CGIAR’s 2030 targets using enhanced impact area indicators. Impact assessments will be integrated into Program/Accelerator design. The use of geographically-bounded targets will be explored for priority locations. A robust approach to project cross-Portfolio benefits by Impact Area for different funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified reporting: Overly complex requirements will be avoided, aiming to
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p50pt3]
+adaptive management and learning. Lessons are used to proactively reflect on and adapt the Theory of Change. Impact assessment strategy outlined. The MELIA approach will be managed by dedicated full-time officers and monitored regularly. Data collection is aligned with the key elements of the Theory of Change, which could be improved with better monitoring for other unintended outcomes, political instability, urban framing, displacement and the integration of generative AI tools for monitoring. One problem is that it is not clear at what stage various people will become involved in the process, and those who are supposed to benefit will be associated. An early assessment should be whether the new varieties are appreciated by the target farmers or not. More information could be given regarding the feedback loops among the various Areas of Work. For example, How MARKET INTELLIGENCE, ACCELERATED BREEDING, INCLUSIVE DELIVERY and BREEDING RESOURCES are related to learning opportunities. A robust framework for MELIA has been
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2]
+has CGIAR-NARES prioritization of products encouraged targeted investment for breeding? (AOW2 AB) RQ9 To what extent has the amount and quality of active collaboration on products increased? (AOW5 E) RQ11 To what extent has B4T influenced more equitable access to improved varieties by marginalized groups? (AOW3 ID) RQ27 To what extent have interoperable tools and services
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt3]
+-30. The list is extracted from the Management Response Actions Tracker. Annex 5: Relevant materials • CGIAR Research and Innovation Strategy 2022-30 • Performance and Results Management Framework
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt3]
+promote agroecological transitions: https://reporting.cgiar.org/reports/result-details/17243 • Feed pellet mechanized production based on locally availably by product s: https://hdl.handle.net/10568/173132 • Capacity strengthening of advisory services: https://reporting.cgiar.org/reports/result- details/18088 IA studies The impact assessment strategy aims to gauge the outcomes of interventions in multifunctional landscapes at different levels, from farmers, to organizations, market systems, policies and global actors. This strategy also seeks a clear understanding of the mechanisms and reasons behind the impacts achieved under the main program assumption, as outlined in the MELIA plan. The current funding landscape uncertainty as well as a realistic assessment of resources that can be dedicated to IA led us to prioritize IA activities in 6
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1]
+Technical Reporting Arrangement (TRA) 2025-30 Approved by the CGIAR Global Leadership Team on 5 June 2025, provides the operational basis to plan, monitor, learn, and report on the 2025-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled and W3/bilateral projects of the 2025-30 portfolio in
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1]
+24 The key impact evaluation questions addressed in this component are: • To what extent do multistakeholder engagement processes and co-design of science-based processes and tools lead to ownership of results by landscape stakeholders and to the sustainable uptake of solutions? • Through which mechanisms does the multidisciplinary and transdisciplinary science promoted by the Multifunctional Landscapes program generate adoption of bundles of solutions and innovations at the landscape level? • Under what conditions and through which mechanisms agroecological and nature positive approaches, within a multifunctional landscape lens, optimize landscape multifunctionality? • What are the behavioral outcomes of such
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4]
+the extent of improvement in the individual product and the number of smallholder farmers that adopt the product. KEQ1 How has B4T’s contribution to the impact areas (return on investment) been maximized? The research questions for relevance also apply here. The research questions on learning and effectiveness will assist contribution analysis. RQ13 Have the expected projections from product concept and design translated into on-farm trial results, and if different why/how has more or less been achieved? (AOW2 AB, AOW3 ID)? RQ14 What additional impact could be achieved with additional investment? (AOW1 MI) RQ15 What is the trajectory of genetic gain for each crop, and what benefits could this mean
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p2pt3]
+................................ ................................ ................................ ..... 23 Program/Accelerator impact overview ................................ ................................ ....... 25 IA activities and collaboration plans ................................ ................................ .......... 26 IA studies ................................ ................................ ................................ ................ 29 Learning and adaptive management ................................ ................................ ......... 33 Reporting
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt4]
+the learning objectives of the Monitoring, Evaluation, and Learning (MEL) component, the IA strategy provides empirical evidence on the Program's effects, aiming to understand the causal mechanisms underlying both expected and unanticipated outcomes. Each of the 2030 outcomes is associated with an impact assessment study designed to evaluate the impact of the Policy Program's Theory of Change (ToC). Several Areas of Work (AoWs) have planned IA studies that explore the impact pathways between intermedia te outcomes and the 2030 outcomes. Additionally, some impact evaluations are planned to test the validity of the research questions underpinning the Policy Program. The specific research questions addressed and the exact nature of each study (quantitative, qualitative, or mixed methods) are currently under consideration. While IA studies assess the achievements of the Policy Program, their objective is not to internally evaluate the Program's work. These studies are conducted in collaboration with other programs and
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3]
+funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified r</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -682,6 +864,9 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question:  What evidence architecture and rigor standards underpin the report’s claims? \n\nContext:\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p67pt1]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 67 part 1\nContent: Figure 31: Methods and rigor of the impact evaluations included in this report. Note: Some studies used multiple methods or received multiple rigor scores for different reported impact estimates. Therefore, the sum of the number of studies reflected in the graph is more than the total number of 62. 4 1 6 4 15 125 4 5 13 62 43210 98765 Rigor score 0 5 10 15 20 4 3 1 43 32 2 3 5 2 2 13 1 2 1 1 1 1 2 1 1 4 6 2 4 4 1 Other ﬁxed eﬀects models Diﬀerence in diﬀerence Propensity score matching and other matching approaches Instrumental variables Endogenous switching regression Randomized control trial Number of publications by rigor score Rigor of the evidence by study design Figure 32: Proportion of impact evaluation analyses which met each of the best-practice rigor score criteria. Included are 125 studies, which contained 488 indicator analyses. 0 100 200 300 400 Spillovers Sensitivity analysis Representativeness Random treatment assignment Random sampling Power Heterogeneous treatment eﬀects Baseline balance Attrition UncertainDid not meet criteriaMet criteria 1%58% 41% 60%40% 56%15% 29% 81%19% 81% 19% 18% 82% 14% 86% 50% 50% 21% 79% B. Impact indicators CGIAR’s Results Framework contains 19 Impact Area indicators it committed to tracking in the 2022 to 2024 period. These indicators are well aligned with the SDG targets and supporting indicators. CGIAR poverty-related indicators are closely linked with SDG targets 1.1 and 1.2 (on reducing poverty) and target 2.3 (on increasing agricultural productivity on small farms). CGIAR nutrition-related indicators are well aligned with SDG targets 2.1 and 2.2 (on reducing hunger and\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 7 part 3\nContent: fully contextualize the results. Are you an implementer? Consider jumping directly to your Impact Area or Continent of interest. But be sure to return and read about the Scope of the Report so that you know what is, and is not, included in this report. Tips on interpretation When interpreting the outcomes reported, be cautious about aggregating across data sources (e.g., as Performance and Results Management System [PRMS] and SPIA country studies), Impact Areas, and continents. Some outcomes are included in more than one of these categories. Pay attention to the specified time period. The report focuses on evidence reported during the 2022 to 2024 period, but outcomes and impacts often developed over much longer periods. Consider the overall weight of the evidence, not individual pieces of evidence. This report presents a body of evidence, drawing on a variety of different epistemological approaches: outcome evidence, impact evaluations, and other types of information, which collectively provide different insights into CGIARs impact. However , only impact evaluations were assessed for the number of best research practices they used, with a composite score of 0 to 9 assigned based on the number of key components of rigor addressed by the study. While weighted equally in this work, these components do not all have equal implications for overall study\n\n---\n\n[ID: pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_Inception Report 30-06-2025.pdf\nLocation: page 1 part 2\nContent: Report Food Frontiers and Security Science Program Inception Report\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 12 part 1\nContent: All impact study submissions were reviewed for potential inclusion into the evidence base of the report. The two primary inclusion considerations were relevance and rigor (see Annex A. Selection of evidence). Studies were determined to be relevant if they considered the outcomes and impacts of CGIAR-supported interventions, regardless of the authorship of the study. Outcomes reported into the CGIAR PRMS are quality assessed for relevance (that is, CGIAR’s role in the outcome is validated); therefore, none of these reported outcomes were excluded on the basis of relevance. Studies with unclear or misleading methods were excluded on the basis of rigor. Studies meeting this threshold of clarity were then classed as “impact assessments” or “impact evaluations.” Impact evaluations were the primary study designs of interest. Impact evaluations are studies that use statistical methods (experimental or quasi-experimental) to quantify the causal change in a condition that was achieved by an intervention. Studies using other study designs were included under the umbrella term of impact assessments (including impact evaluations), if they provided information relevant to understanding impacts, such as cost- benefit analyses, reviews of CGIAR work, and measures of the adoption of CGIAR technology. These included the country studies supported by CGIAR’s SPIA. While impact evaluations are necessary to establish causal change linking intervention and impact, they can be limited in scope due to practical constraints, such as resources and measurement challenges. Other types of impact assessments can provide valuable insights into CGIAR’s contributions to real-world change in a wider spatial or temporal context; however , they do c This can be common for power calculations. Authors may have conducted power calculations but not r eported that they did so in-text. Assessment is based on what is reported in-text, not what may have been done but not reported. d See Annex A. Included studies and rigor of\n\n---\n\n[ID: pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p17pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_Inception Report 30-06-2025.pdf\nLocation: page 17 part 3\nContent: underpin the work being done and provide the solid positioning for holding the CA. This collaboration means the work being done relies on the most capable parts of both the CGIAR and the relevant partner and that this collaboration changes over time. A part of the Program’s objectives\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt2]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 12 part 2\nContent: challenges. Other types of impact assessments can provide valuable insights into CGIAR’s contributions to real-world change in a wider spatial or temporal context; however , they do c This can be common for power calculations. Authors may have conducted power calculations but not r eported that they did so in-text. Assessment is based on what is reported in-text, not what may have been done but not reported. d See Annex A. Included studies and rigor of evidence for details. Criteria related to random sampling and treatment assignment; reporting of power calculation and sensitivity analysis; consideration of attrition, spillovers, and heterogenous treatment effects; and sample representativeness and baseline balance. not establish causality. Impact evaluations were further appraised to determine the number of best practices followed per study. A composite score45 was calculated to reflect the level of confidence in the findings of a study and to help understand the application of best practices in CGIAR impact evaluation. Nine best practices were identified (see Annex A. Included studies and rigor of evidence), resulting in the composite best- practice score ranging from 0 to 9. Not all the criteria were relevant to all studies, and some studies may have met criteria but did not clearly describe them in the publication.c Studies following three or more best practices were featured preferentially in this report (assuming equality in relevance). Details of the method and analysis of the scores are in Annex A. Included studies and rigor of evidence. Included impact studies Approximately 500 studies were reviewed for eligibility and 125 studies were included in the primary dataset. Of these, 62 were impact evaluations and 63 were impact assessments which did not attempt to establish the causal effect of an intervention on an impact. Randomized controlled trials (RCT) were the most common impact evaluation design (n = 21), followed by\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p4pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 4 part 1\nContent: Integration with other outputs The Portfolio Narrative informs the 2024 CGIAR Annual Report – a comprehensive summary of the organization’s collective achievements, impacts, and strategic outlook. Elements of the Type 2 report were integrated into the CGIAR Flagship Report released in April 2025 during the CGIAR Science Week. The Flagship Report synthesizes CGIAR research in an accessible format designed specifically to provide policy- and decisionmakers at national, regional, and global levels with the evidence they require to formulate, develop, and negotiate evidence-based policies and investments. The diagram below illustrates these relationships, emphasizing the interconnectedness of the Type 3 Report with other reporting products. CGIAR Results Dashboard Portfolio Narrative report CGIAR Annual report Type 1 Initiative, Impact Platform, and Science Group Project reports Type 2 CGIAR Contributions to Impact in Agrifood Systems: evidence and learnings from 2022 to 2024 Flagship report Type 3 Portfolio Practice Change report 2024 Technical Reporting Figure 1. CGIAR’s 2024 Technical Reporting components and their integration with other CGIAR reporting products. Section 1: Introduction 1 Under the CGIAR Technical Reporting Arrangement for the next Portfolio (2025-30), relevant aspects of the Type 3 Report will be included in the annual Portfolio Narrative, and a separate Type 3 Report will no longer be produced. The 2024 CGIAR Portfolio Practice Change\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 48 part 4\nContent: against CGIAR’s Results Framework is that, apart from the SPIA country studies, other internal and external studies are designed in an uncoordinated bottom-up way. Because such studies are undertaken to meet specific information needs, opportunities to learn through synthesis or aggregation are missed due to the differences in indicators used and measurement approaches employed. For example, impact assessments are rarely connected with data on innovation use, preventing case study results from being used to extrapolate possible large-scale effects. Thus, moving forward, two areas for improvement are: (1) to collectively undertake strategic impact assessments that will answer high-priority impact assessment questions and (2) to develop and enforce the use of a core set of common indicators and measurement methodsq that should be used in impact assessment studies regardless of who initiates them. In addition, during the 2022 to 2024 period, Initiatives defined targets for outcomes and made commitments to measuring and reporting on those outcomes. They did not have a similar plan or commitment to measuring impacts. As CGIAR evolves to longer-term programs covering the whole of CGIAR, there should be commitments to the consistent measurement of impacts. However , this has been an ongoing challenge within the organization, with similar recommendations from a review of the 2017 to 2021 portfolio.176 Rigor of the evidence All impact evaluations identified were assessed for their rigor based on criteria established by Rao 2025.45 The most common score was a 4 of 9 key elements being present, suggesting moderate overall quality and room for improvement. A high number of impact evaluations used rigorous methods to infer causality between a CGIAR innovation and impacts (see Annex A. Included studies and rigor of evidence). However , many failed to consider heterogeneous treatment effects or report power calculations. Most of the impact evaluations used experimental or quasi-experimental designs with two or more measurement periods. However , a sizeable group of the studies were based on cross-sectional (single measurement) studies. While they are peer-reviewed and employ recommended methods of controlling for unobservable variables to enhance the likelihood of a causal inference, there remain limitations to such designs. In addition to rigor , this study paid attention to the relevance of the studies. Often, studies employing less rigorous, cross-sectional methodologies were able to provide evidence more relevant to policymaking and decision-making Tradititional rice variety in Ilagan, Isabela, the Philippines. Photo credit: Miguel Mamon/CIAT CGIAR Impacts in Agrifood Systems: | Learnings | Page 90 of 130 CGIAR CGIAR CGIAR Impacts in Agrifood Systems: | Learnings| Page 91 of 130\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 4\nContent: four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the \"challenges and megatrends\" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p6pt1]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 6 part 1\nContent: Integration with other outputs The Portfolio Narrative informs the 2024 CGIAR Annual Report – a comprehensive summary of the organization’s collective achievements, impacts, and strategic outlook. Elements of the Type 2 report fed into the CGIAR Flagship Report, released in April 2025 at CGIAR Science Week. The Flagship Report\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 3\nContent: activities of the CapSha Accelerator, its products and services, contribute to improved capacity development practices, resulting in more equitable partnerships? • Are CGIAR NARES partners, donors and CapSha expert institutions making use of CapSha products and services? • Are CGIAR NARES partners, donors and CapSha expert institutions member of the CapSha Cop? • To what extent are the CapSha Accelerator’s objectives aligned with the needs and priorities of Southern partners? • What elements of the partnership model have the potential to be scaled or replicated in other regions or contexts? What are the enabling and limiting factors affecting scalability? How have Southern partners contributed to or led scaling efforts, and what support mechanisms have been most effective? • What measurable\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 46 part 3\nContent: to ensure common terminology across the reporting units. At the impact level, there were 19 indicators across the five Impact Areas. The frequency of reporting against exact indicators is very low (18 percent of indicators assessed match those in the Results Framework; Annex B. Impact indicators). In addition, there is an imbalance across Impact Areas and indicators in the frequency with which 2022 to 2024 studies attempt to measure those indicators. There were many impact assessments that measured yields or income related to the poverty indicators, and relatively few that looked at environmental, climate, or gender indicators. This is consistent with what Templeton (2023)176 found in her review of evidence used to support the impact claims made by the CGIAR Research Programs between 2017 and 2021. Thus, there remains a huge challenge to define feasible indicators for"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: What is the 2025–30 Impact Assessment (IA) strategy addressing, and what will be delivered to funders and managers?\n\nContext:\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u46-49]\nLink: Engagement Plan: 2025 Technical Reporting (Full Word document)\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Fortnightly update emails' paragraph 80 to section 'Fortnightly update emails' paragraph 83\nContent: CGSpace Team Lead KM Managers Curators/Repository Managers PRMS Team\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p29pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 29 part 4\nContent: The current funding landscape uncertainty as well as a realistic assessment of resources that can be dedicated to IA led us to prioritize IA activities in 6 countries, where we can easily leverage on human and financial resources for impact assessment: Colombia, Peru, Tunisia, Kenya, India, Vietnam. The site prioritization, as well as prioritization of the key impact indicators that the IA should target (potential indicators are presented in the table below), will be a specific action of the MELIA team at the end of 2025, when future financial capacity will be clearer. Further funding for IA studies will be sought in 2026 and during the implementation of\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_MELIA Plan 30-06-2025.pdf\nLocation: page 8 part 4\nContent: exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. Impact assessments are conducted after an intervention has been completed and are used to substantiate claims of sustained results. They seek to measure impact at scale, i.e., benefits to a large number of people/large areas of land. It employs both quantitative and qualitative methods, often combined for deeper insights. IA goes beyond monitoring indicators to evidenced attribution of observed changes to CGIAR interventions. IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives.\n\n---\n\n[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_MELIA Plan 30-06-2025.pdf\nLocation: page 8 part 3\nContent: the learnings and what are other critical areas that require further focused support? (AoW 5) Evaluation collaboration plans Genebanks will seek to collaborate with the Multifunctional Landscapes Program to study in situ and on farm site monitoring of diversity conservation. Genebanks will also collaborate with the Crop Trust and Aarhus University to review the Scientific Impact of the Seed Quality Management and Quality Management System Communities of Practice. Collaborations with W3/bilateral projects will be explored during phase 2 of the mapping exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 10 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 10 Thematic Impact 2022-30 Report The Thematic Impact 2022 -30 Report provides a m acro level view of CGIAR’s role in Food, Land and Water System Transformation covering the period 2022 -30. It will be released in 2031. Its format and content will be developed during the period 2025-30. Results Dashboard • The Results Dashboard will be enhanced to better present curated information a gainst Impact Area targets, geographies and key topics. • Headline impacts and outcomes will be more clearly communicated in the Dashboard. • Using AI, users will be able to easily query the results data and underlying sources of evidence data using\n\n---\n\n[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 2 part 3\nContent: Impact assessment (IA) .............................................................................................................. 13 Program impact overview .................................................................................................................... 13 IA activities and collaboration plans ..................................................................................................... 14 IA studies ........................................................................................................................................... 15 5. Learning and adaptive management ........................................................................................... 16 Learning ............................................................................................................................................. 16 Annual review and adaptive planning ...................................................................................................\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 17 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 17 The amount of quality information sourced from different funding sources, and the coherence between those different information sources will increase over time (specific metrics and targets to be developed) 6. Impact Assessment Strategy/ Approach/ Case studies CGIAR will develop a 2025 -30 Impact Assessment Plan and integrate its design, budgeting and delivery into the 25-30 Portfolio. The bottom-up approach to impact assessment that has been used within CGIAR for the past decades has not produced sufficient quantity or quality of studies to prov ide evidence against CGIAR impact indicators. SPIA fills in some of this gap, but even their new undertaking of country studies will likely not be able to contribute to most of the indicators\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 25 part 1\nContent: • Bilateral/W3-funded projects: to identify embedded impact assessment opportunities and avoid duplication. • CGIAR IA teams : to contribute to portfolio -level meta -evaluation and harmonize data with common CGIAR indicators. Priority will be given to impact in integrative countries, where multiple AoWs operate. These broader IA studies will assess the synergies between interventions and provide system -level insights into the pathways driving impact. Potential integrative countries include Bangladesh, Ethiopia, Nigeria, and Tanzania, based on portfolio density and MELIA feasibility. A senior Impact Specialist will guide study design and implementation, ensure alignment with the CGIAR results framework indicators, and coordinate data quality assurance across IA efforts. Impact assessment studies The Program has identified initial IA study themes for inclusion in the MELIA studies. However , these initial themes are not included in the\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 3\nContent: activities of the CapSha Accelerator, its products and services, contribute to improved capacity development practices, resulting in more equitable partnerships? • Are CGIAR NARES partners, donors and CapSha expert institutions making use of CapSha products and services? • Are CGIAR NARES partners, donors and CapSha expert institutions member of the CapSha Cop? • To what extent are the CapSha Accelerator’s objectives aligned with the needs and priorities of Southern partners? • What elements of the partnership model have the potential to be scaled or replicated in other regions or contexts? What are the enabling and limiting factors affecting scalability? How have Southern partners contributed to or led scaling efforts, and what support mechanisms have been most effective? • What measurable\n\n---\n\n[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p2pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP03%20%2D%20Sustainable%20Animal%20and%20Aquatic%20Foods%2FSustainable%20Animal%20and%20Aquatic%20Foods%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP03%20%2D%20Sustainable%20Animal%20and%20Aquatic%20Foods&amp;p=true&amp;ga=1\nFile: Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf\nLocation: page 2 part 2\nContent: ................................ ................................ ............... 7 Data collection strategy ................................ ................................ ................................ 7 3. Evaluation plan ................................ ................................ ................................ ..................... 7 Evaluation studies ................................ ................................ ................................ ....... 7 Evaluation collaboration plans ................................ ................................ ....................... 8 4. Impact assessment ................................ ................................ ................................ ............... 8 Program/Accelerator impact overview ................................ ................................ ............ 8 IA activities and collaboration\n\n---\n\n[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p18pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 18 part 3\nContent: All the knowledge generated by these studies will be available not only to Program managers, but also researchers, the CGIAR community, and external stakeholders. Finally, analyzing monitoring data will be a continuous process, and results, along with recommendations, will be made available to Program managers to make any necessary adjustments to the Program implementation. Annual review and adaptive planning The Climate Action Program will implement an annual review and adaptive planning process, building on the experience and lessons from the 2022–24 CGIAR Portfolio and aligned with evolving guidance on the Reﬂect and Re-Plan processes. Each year, the Program will conduct structured annual performance reviews at both program-wide and AoW levels. These reviews will assess progress toward the intended outputs and outcomes, using both quantitative and qualitative data drawn from the CGIAR Performance and Results Management System"}]</t>
   </si>
 </sst>
 </file>
@@ -1052,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1095,7 +1280,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -1107,16 +1292,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1124,7 +1309,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -1136,16 +1321,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H3" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1153,7 +1338,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -1165,16 +1350,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="G4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H4" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1182,7 +1367,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1194,16 +1379,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="G5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H5" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1211,7 +1396,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -1223,16 +1408,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1240,7 +1425,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -1252,16 +1437,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="I7" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1269,7 +1454,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -1281,16 +1466,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="G8" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H8" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1298,7 +1483,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1310,16 +1495,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H9" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1327,7 +1512,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -1339,16 +1524,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="H10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1356,7 +1541,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -1368,16 +1553,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I11" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1385,7 +1570,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -1397,16 +1582,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="I12" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1414,7 +1599,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -1426,16 +1611,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="I13" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -1443,7 +1628,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -1455,16 +1640,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H14" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="I14" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -1472,7 +1657,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C15">
         <v>100</v>
@@ -1484,16 +1669,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H15" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="I15" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -1501,7 +1686,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -1513,16 +1698,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H16" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I16" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -1530,7 +1715,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -1542,16 +1727,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="I17" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -1559,7 +1744,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -1571,16 +1756,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="I18" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -1588,7 +1773,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -1600,16 +1785,16 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H19" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="I19" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -1617,7 +1802,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -1629,16 +1814,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G20" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H20" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I20" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -1646,7 +1831,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -1658,22 +1843,22 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G21" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H21" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I21" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J21" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K21" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -1681,7 +1866,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -1693,22 +1878,22 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G22" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H22" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J22" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K22" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -1716,7 +1901,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -1728,22 +1913,22 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G23" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H23" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I23" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J23" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K23" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -1751,7 +1936,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C24">
         <v>200</v>
@@ -1763,22 +1948,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G24" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H24" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I24" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J24" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K24" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -1786,7 +1971,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C25">
         <v>200</v>
@@ -1798,22 +1983,22 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G25" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="H25" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I25" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="J25" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="K25" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -1821,7 +2006,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C26">
         <v>200</v>
@@ -1833,22 +2018,22 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G26" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H26" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="I26" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J26" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="K26" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -1856,7 +2041,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C27">
         <v>200</v>
@@ -1868,22 +2053,22 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G27" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H27" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="I27" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J27" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="K27" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -1891,7 +2076,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C28">
         <v>200</v>
@@ -1903,22 +2088,22 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G28" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H28" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="I28" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J28" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="K28" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -1926,7 +2111,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C29">
         <v>200</v>
@@ -1938,22 +2123,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G29" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="H29" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="I29" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J29" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="K29" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -1961,7 +2146,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -1973,22 +2158,22 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G30" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H30" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="I30" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="J30" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="K30" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -1996,7 +2181,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -2008,22 +2193,22 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G31" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="H31" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="I31" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="J31" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="K31" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2031,7 +2216,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -2043,22 +2228,22 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G32" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H32" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="I32" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="J32" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K32" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2066,7 +2251,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -2078,22 +2263,22 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G33" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H33" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J33" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K33" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2101,7 +2286,7 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -2113,22 +2298,22 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G34" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H34" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J34" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K34" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2136,7 +2321,7 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -2148,22 +2333,22 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G35" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H35" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J35" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K35" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2171,7 +2356,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -2183,22 +2368,22 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G36" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H36" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J36" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K36" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2206,7 +2391,7 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -2218,22 +2403,22 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="G37" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="H37" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="J37" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K37" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2241,34 +2426,209 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38">
+        <v>100</v>
+      </c>
+      <c r="D38">
+        <v>100</v>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
+      </c>
+      <c r="F38" t="s">
+        <v>59</v>
+      </c>
+      <c r="G38" t="s">
+        <v>71</v>
+      </c>
+      <c r="H38" t="s">
+        <v>100</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J38" t="s">
+        <v>114</v>
+      </c>
+      <c r="K38" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39">
+        <v>100</v>
+      </c>
+      <c r="D39">
+        <v>100</v>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+      <c r="F39" t="s">
+        <v>59</v>
+      </c>
+      <c r="G39" t="s">
+        <v>72</v>
+      </c>
+      <c r="H39" t="s">
+        <v>101</v>
+      </c>
+      <c r="I39" t="s">
+        <v>110</v>
+      </c>
+      <c r="J39" t="s">
+        <v>115</v>
+      </c>
+      <c r="K39" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11">
+      <c r="A40" t="s">
+        <v>49</v>
+      </c>
+      <c r="B40" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40">
+        <v>100</v>
+      </c>
+      <c r="D40">
+        <v>100</v>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+      <c r="F40" t="s">
+        <v>59</v>
+      </c>
+      <c r="G40" t="s">
+        <v>72</v>
+      </c>
+      <c r="H40" t="s">
+        <v>101</v>
+      </c>
+      <c r="I40" t="s">
+        <v>110</v>
+      </c>
+      <c r="J40" t="s">
+        <v>115</v>
+      </c>
+      <c r="K40" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" t="s">
+        <v>58</v>
+      </c>
+      <c r="C41">
+        <v>100</v>
+      </c>
+      <c r="D41">
+        <v>100</v>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>59</v>
+      </c>
+      <c r="G41" t="s">
+        <v>72</v>
+      </c>
+      <c r="H41" t="s">
+        <v>101</v>
+      </c>
+      <c r="I41" t="s">
+        <v>110</v>
+      </c>
+      <c r="J41" t="s">
+        <v>115</v>
+      </c>
+      <c r="K41" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" t="s">
+        <v>58</v>
+      </c>
+      <c r="C42">
+        <v>100</v>
+      </c>
+      <c r="D42">
+        <v>100</v>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" t="s">
+        <v>59</v>
+      </c>
+      <c r="G42" t="s">
+        <v>72</v>
+      </c>
+      <c r="H42" t="s">
+        <v>101</v>
+      </c>
+      <c r="I42" t="s">
+        <v>110</v>
+      </c>
+      <c r="J42" t="s">
+        <v>115</v>
+      </c>
+      <c r="K42" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" t="s">
         <v>52</v>
       </c>
-      <c r="C38">
-        <v>100</v>
-      </c>
-      <c r="D38">
-        <v>100</v>
-      </c>
-      <c r="E38" t="b">
-        <v>1</v>
-      </c>
-      <c r="F38" t="s">
-        <v>53</v>
-      </c>
-      <c r="G38" t="s">
-        <v>65</v>
-      </c>
-      <c r="H38" t="s">
-        <v>93</v>
-      </c>
-      <c r="I38" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="J38" t="s">
-        <v>104</v>
-      </c>
-      <c r="K38" t="s">
+      <c r="B43" t="s">
+        <v>58</v>
+      </c>
+      <c r="C43">
+        <v>100</v>
+      </c>
+      <c r="D43">
+        <v>100</v>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+      <c r="F43" t="s">
+        <v>59</v>
+      </c>
+      <c r="G43" t="s">
+        <v>72</v>
+      </c>
+      <c r="H43" t="s">
+        <v>102</v>
+      </c>
+      <c r="I43" t="s">
         <v>110</v>
+      </c>
+      <c r="J43" t="s">
+        <v>115</v>
+      </c>
+      <c r="K43" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update max_ctx to 20, and move name_to_link outside render_app
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="176">
   <si>
     <t>timestamp</t>
   </si>
@@ -202,6 +202,18 @@
     <t>2025-09-24T09:25:37.525385</t>
   </si>
   <si>
+    <t>2025-09-24T09:37:22.340959</t>
+  </si>
+  <si>
+    <t>2025-09-24T09:58:46.173297</t>
+  </si>
+  <si>
+    <t>2025-09-24T10:08:10.540962</t>
+  </si>
+  <si>
+    <t>2025-09-24T10:32:33.484279</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -224,6 +236,15 @@
   </si>
   <si>
     <t>¿Quién tiene la responsabilidad fiduciaria y programática?</t>
+  </si>
+  <si>
+    <t>Se reportan desvíos potenciales en su uso. ¿Quién tiene la responsabilidad fiduciaria y programática, qué debe informar el Center y qué facultades de acción tiene la System Organization (SO)?</t>
+  </si>
+  <si>
+    <t>¿Quién gestiona colectivamente los requisitos de M&amp;E de los Funders y cómo se evita la duplicación?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Who coordinates funders’ M&amp;E requirements across the CGIAR Portfolio and how is duplication avoided? </t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -283,6 +304,12 @@
   </si>
   <si>
     <t>pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.396, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.387, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.364, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.361, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.330, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.327, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2:0.319, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.283, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.210, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.204, docx:2025 Technical Reporting Information (Session 2).docx:u52-56:0.204, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.196, docx:2025 Technical Reporting Information (Session 1).docx:u43-45:0.193, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.193, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.157, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.151, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.144, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1:0.144, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1:0.142, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.141, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3:0.137, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4:0.133, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2:0.133, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2:0.129, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2:0.120, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3:0.119, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.113, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3:0.111, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.108, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3:0.102, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1:0.102, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.099, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt2:0.091, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.088, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1:0.084, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt1:0.080, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p53pt4:0.074, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3:0.072, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p40pt4:0.064, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt2:0.062, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.055, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p32pt3:0.047, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p32pt2:0.047</t>
+  </si>
+  <si>
+    <t>pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.403, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.368, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.344, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.316, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.310, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.288, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.238, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.218, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.215, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.211, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.199, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.196, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2:0.190, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p24pt1:0.186, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p30pt1:0.186, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.157, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.154, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p55pt2:0.152, docx:2025 Technical Reporting Information (Session 2).docx:u52-56:0.149, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.136, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p31pt1:0.132, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.130, docx:2025 Technical Reporting Information (Session 1).docx:u43-45:0.129, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.127, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.122, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p57pt2:0.122, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1:0.121, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3:0.121, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p28pt1:0.119, pdf:CGI21-507032-PORB-Climate Action.pdf:p38pt1:0.117, pdf:CGI21_508012_PORB_Genebanks.pdf:p20pt1:0.116, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1:0.114, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.114, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt1:0.114, pdf:CGI21-507032-PORB-Climate Action.pdf:p27pt1:0.114, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p31pt1:0.113, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p49pt2:0.113, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p25pt1:0.113, pdf:CGI21_508012_PORB_Genebanks.pdf:p21pt1:0.113, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p33pt1:0.110, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.110, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt1:0.109, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p81pt2:0.109, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1:0.108, pdf:CGI21-507032-PORB-Climate Action.pdf:p30pt1:0.108, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p42pt1:0.107, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p49pt4:0.107, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2:0.107, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2:0.106, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p29pt1:0.106, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p24pt1:0.106, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1:0.105, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p58pt3:0.105, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.105, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3:0.104, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p22pt1:0.104, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p37pt1:0.102, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p59pt1:0.101, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p21pt1:0.101, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p49pt1:0.099, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p71pt1:0.097, docx:2025 Technical Reporting Information (Session 2).docx:u25-28:0.097, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2:0.096, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3:0.095, docx:Standard Provisions 2026.docx:u7-10:0.095, docx:2025 Technical Reporting Information (Session 2).docx:u22-25:0.095, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4:0.095, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2:0.094, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt2:0.093, pdf:Portfolio Narrative_2024.pdf:p47pt3:0.093, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3:0.092, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p13pt1:0.092, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p11pt1:0.092, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p8pt2:0.091, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p52pt1:0.091, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p37pt1:0.091, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p23pt1:0.090, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p43pt1:0.090, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p21pt1:0.088, docx:Standard Provisions 2026.docx:u142-145:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u7-10:0.088, docx:Standard Provisions 2026.docx:u148-151:0.086, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p51pt1:0.086, pdf:Type3_2024Report.pdf:p2pt1:0.085, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3:0.084, docx:Standard Provisions 2026.docx:u139-142:0.083, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.081, pdf:CGI21_508012_PORB_Genebanks.pdf:p3pt2:0.081, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p23pt1:0.081, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p67pt1:0.081, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.080, docx:2025 Technical Reporting Information (Session 1).docx:u19-22:0.080, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.080, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.079, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p39pt1:0.079, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3:0.079, docx:Standard Provisions 2026.docx:u115-118:0.079, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p41pt1:0.079, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p34pt3:0.078, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p33pt1:0.078, docx:2025 Technical Reporting Information (Session 1).docx:u22-25:0.077, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p32pt1:0.077, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.076, pdf:CGI21_508012_PORB_Genebanks.pdf:p42pt1:0.075, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p53pt4:0.075, docx:Standard Provisions 2026.docx:u40-43:0.075, docx:2025 Technical Reporting Information (Session 1).docx:u37-40:0.074, docx:Standard Provisions 2026.docx:u124-127:0.074, pdf:Portfolio Narrative_2024.pdf:p47pt2:0.074, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.074, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p3pt2:0.073, docx:Standard Provisions 2026.docx:u175-178:0.073, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p62pt1:0.073, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p12pt1:0.073, docx:2025 Technical Reporting Information (Session 1).docx:u34-37:0.072, docx:Standard Provisions 2026.docx:u151-154:0.071, pdf:CGI21_508012_PORB_Genebanks.pdf:p3pt1:0.071, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p70pt1:0.071, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p64pt1:0.070, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p3pt1:0.070, pdf:Quick style guide Feb 2024 (1).pdf:p9pt2:0.070, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.069, docx:2025 Technical Reporting Information (Session 1).docx:u40-43:0.068, docx:2025 Technical Reporting Information (Session 2).docx:u46-49:0.068, docx:Standard Provisions 2026.docx:u52-55:0.068, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p66pt1:0.068, pdf:CGI21-507032-PORB-Climate Action.pdf:p26pt1:0.067, docx:2025 Technical Reporting Information (Session 2).docx:u10-13:0.067, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p3pt1:0.067, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p82pt1:0.066, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p63pt1:0.066, docx:Standard Provisions 2026.docx:u112-115:0.066, docx:Standard Provisions 2026.docx:u73-76:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4:0.065, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p64pt1:0.065, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p28pt2:0.065, docx:Standard Provisions 2026.docx:u88-91:0.065, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p27pt1:0.065, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p8pt3:0.065, docx:Standard Provisions 2026.docx:u127-130:0.065, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p53pt1:0.064, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p3pt2:0.064, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p26pt1:0.064, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p42pt1:0.064, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p63pt1:0.064, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p80pt1:0.064, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt3:0.064, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p48pt1:0.064, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p46pt1:0.064, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p85pt1:0.063, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p58pt2:0.063, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p64pt1:0.063, docx:Standard Provisions 2026.docx:u4-7:0.063, docx:Standard Provisions 2026.docx:u100-103:0.063, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p10pt1:0.062, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt1:0.062, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p3pt1:0.062, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt4:0.062, docx:Standard Provisions 2026.docx:u160-163:0.062, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p52pt1:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p26pt1:0.062, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p3pt1:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p28pt1:0.062, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p36pt1:0.061, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p53pt1:0.061, docx:Standard Provisions 2026.docx:u85-88:0.061, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.061, pdf:CGI21-507032-PORB-Climate Action.pdf:p37pt1:0.061, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p17pt1:0.061, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p3pt1:0.061, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p3pt1:0.061, docx:Standard Provisions 2026.docx:u154-157:0.060, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p14pt1:0.060, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p50pt1:0.060, pdf:CGI21-507032-PORB-Climate Action.pdf:p3pt1:0.060, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p44pt1:0.060, docx:Standard Provisions 2026.docx:u97-100:0.059, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p40pt1:0.059, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p3pt1:0.059, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p51pt1:0.059, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p3pt1:0.059, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p56pt1:0.059, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2:0.059, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.059, docx:2025 Technical Reporting Information (Session 1).docx:u31-34:0.059, docx:Standard Provisions 2026.docx:u16-19:0.058, pdf:CGI21-507032-PORB-Climate Action.pdf:p36pt1:0.058, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p51pt1:0.058, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p18pt1:0.058, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p79pt1:0.058, docx:Standard Provisions 2026.docx:u130-133:0.058, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p38pt1:0.058, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p80pt1:0.057, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p15pt1:0.057, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p70pt1:0.057, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2:0.057, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p3pt1:0.056, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p3pt1:0.056, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p3pt2:0.056, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p25pt1:0.056</t>
+  </si>
+  <si>
+    <t>pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.321, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.276, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.272, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.256, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.252, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.231, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.216, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.198, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.196, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.186, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.184, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3:0.166, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.163, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.157, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.146, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.138, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.137, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1:0.137, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3:0.130, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.124, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2:0.121, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.120, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3:0.118, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4:0.118, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2:0.116, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2:0.112, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2:0.112, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p32pt1:0.106, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt2:0.106, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4:0.104, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2:0.104, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.103, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.103, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2:0.102, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2:0.101, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4:0.100, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1:0.097, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.096, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.096, pdf:CGI21-507032-PORB-Climate Action.pdf:p21pt3:0.094, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt3:0.092, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt3:0.091, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1:0.088, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt4:0.087, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1:0.087, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.083, pdf:Portfolio Narrative_2024.pdf:p47pt3:0.082, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt2:0.082, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4:0.081, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt4:0.081, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2:0.079, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt2:0.078, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt4:0.078, pdf:Portfolio Narrative_2024.pdf:p47pt4:0.075, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p7pt4:0.075, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt1:0.075, pdf:CGIAR_ImpactReport_2022-24.pdf:p56pt2:0.073, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3:0.072, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.072, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p23pt1:0.072, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p53pt4:0.070, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt2:0.070, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3:0.068, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt1:0.067, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p29pt1:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p54pt3:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt3:0.065, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt2:0.064, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt3:0.063, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt2:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3:0.062, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt4:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt3:0.061, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt1:0.060, docx:Standard Provisions 2026.docx:u22-25:0.060, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt1:0.059, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p10pt4:0.059, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt3:0.058, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt4:0.058, docx:Standard Provisions 2026.docx:u115-118:0.057, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p28pt3:0.057, pdf:Climate Action_Inception Report 30-06-2025.pdf:p11pt3:0.057, pdf:Portfolio Narrative_2024.pdf:p47pt2:0.056, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p25pt4:0.056, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt4:0.056, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt2:0.056, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt1:0.054, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.054, docx:2025 Technical Reporting Information (Session 2).docx:u52-56:0.054, docx:Standard Provisions 2026.docx:u127-130:0.053, docx:2025 Technical Reporting Information (Session 1).docx:u43-45:0.051, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt4:0.050, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.049, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt1:0.049, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p30pt1:0.048, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt4:0.048, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt4:0.048, docx:Standard Provisions 2026.docx:u100-103:0.048, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt2:0.047, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt1:0.047, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt1:0.045, pdf:CGIAR_ImpactReport_2022-24.pdf:p34pt1:0.045, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt2:0.045, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt4:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p43pt4:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p44pt4:0.044, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4:0.044, pdf:Type3_2024Report.pdf:p2pt4:0.043, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt3:0.043, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p40pt4:0.042, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt2:0.042, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p18pt2:0.042, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt2:0.041, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p22pt2:0.041, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt2:0.041, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt3:0.041, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt1:0.041, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt1:0.040, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p52pt3:0.040, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt1:0.040, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt3:0.040, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt4:0.040, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt2:0.040, pdf:Portfolio Narrative_2024.pdf:p83pt1:0.040, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt2:0.040, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt1:0.040, pdf:Type3_2024Report.pdf:p8pt4:0.039, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p9pt4:0.038, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt2:0.038, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3:0.038, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.038, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt2:0.038, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt3:0.037, docx:Standard Provisions 2026.docx:u103-106:0.037, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p13pt4:0.037, pdf:Portfolio Narrative_2024.pdf:p28pt4:0.037, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt4:0.036, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt2:0.036, pdf:CGIAR_ImpactReport_2022-24.pdf:p45pt4:0.035, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p22pt1:0.035, pdf:Portfolio Narrative_2024.pdf:p19pt1:0.035, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p26pt1:0.035, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p29pt4:0.034, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt2:0.034, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt1:0.034, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p30pt3:0.033, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p51pt1:0.033, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt2:0.033, docx:Standard Provisions 2026.docx:u85-88:0.033, docx:Standard Provisions 2026.docx:u172-175:0.033, docx:Standard Provisions 2026.docx:u124-127:0.032, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p20pt2:0.032, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt3:0.032, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt3:0.031, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p13pt1:0.031, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt3:0.030, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt4:0.030, pdf:CGIAR_ImpactReport_2022-24.pdf:p23pt4:0.030, pdf:Type3_2024Report.pdf:p10pt4:0.030, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt3:0.030, docx:Standard Provisions 2026.docx:u82-85:0.029, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt3:0.029, docx:Standard Provisions 2026.docx:u97-100:0.029, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p22pt2:0.028, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p39pt2:0.028, pdf:CGIAR_ImpactReport_2022-24.pdf:p41pt4:0.028, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt2:0.028, docx:Standard Provisions 2026.docx:u52-55:0.027, pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt2:0.027, pdf:Portfolio Narrative_2024.pdf:p82pt4:0.026, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p6pt4:0.026, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt3:0.026, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt3:0.026, docx:Standard Provisions 2026.docx:u112-115:0.026, pdf:CGI21-507032-PORB-Climate Action.pdf:p24pt2:0.026, docx:Standard Provisions 2026.docx:u106-109:0.025, pdf:CGI21-507032-PORB-Climate Action.pdf:p24pt3:0.025, pdf:CGIAR_ImpactReport_2022-24.pdf:p40pt1:0.025, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.024, docx:Standard Provisions 2026.docx:u7-10:0.024, docx:Standard Provisions 2026.docx:u130-133:0.024, docx:Standard Provisions 2026.docx:u4-7:0.024, pdf:Type3_2024Report.pdf:p7pt2:0.024, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.024, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p22pt2:0.024, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.024, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt4:0.023, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3:0.023, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt3:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p22pt1:0.023, docx:Standard Provisions 2026.docx:u34-37:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p14pt3:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p22pt2:0.023, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.023, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p18pt1:0.022, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt4:0.022, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt4:0.022, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt2:0.022, pdf:Quick style guide Feb 2024 (1).pdf:p5pt1:0.022, pdf:Climate Action_Inception Report 30-06-2025.pdf:p28pt3:0.022</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -580,6 +607,46 @@
 CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1</t>
   </si>
   <si>
+    <t>I cannot find information in the provided chunks to answer this. The documents do not specify the fiduciary and programmatic responsibilities, the reporting obligations of the Center, or the action powers of the System Organization (SO) regarding potential deviations in usage. For detailed insights on these topics, further context or specific documents may be required. 
+Sources:
+File — Location — Cited IDs
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1
+Climate Action_Inception Report 30-06-2025.pdf — page 4 part 3 — pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1</t>
+  </si>
+  <si>
+    <t>I cannot find information in the provided chunks to answer this. The documents do not specify who collectively manages the M&amp;E requirements of the Funders or the methods used to avoid duplication. Further details on these processes may be found in other sources or documents not included in the provided chunks. 
+Sources:
+File — Location — Cited IDs
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1
+CGIAR_PORB_Breeding_Tomorrow.pdf — page 45 part 3 — pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1</t>
+  </si>
+  <si>
+    <t>I cannot find information in the provided chunks to answer this. The documents do not specify who collectively manages the M&amp;E requirements of the Funders or the methods used to avoid duplication. Further details on these processes may be found in other resources or specific reports related to M&amp;E practices within the relevant organizations. 
+Sources:
+File — Location — Cited IDs
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1
+CGIAR_PORB_Breeding_Tomorrow.pdf — page 45 part 3 — pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3
+CGIAR_PORB_Scaling_4Impact.pdf — page 23 part 3 — pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3</t>
+  </si>
+  <si>
+    <t>The coordination of funders' M&amp;E requirements across the CGIAR Portfolio is primarily managed by the Portfolio Performance Unit, which collaborates with a cross-CGIAR working group that includes Center experts and System functions. To avoid duplication, the Technical Reporting Arrangement (TRA) for 2025-30 aims to promote progressive alignment between reporting requirements for pooled and non-pooled funding components. This structured approach is designed to ensure transparency and accountability while facilitating effective engagement and communication among stakeholders, thereby minimizing overlapping evaluations and activities. 
+Sources:
+File — Location — Cited IDs
+CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 23 part 4 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23pt4
+CGIAR_ImpactReport_2022-24.pdf — page 2 part 4 — pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4
+Type3_2024Report.pdf — page 6 part 1 — pdf:Type3_2024Report.pdf:p6pt1
+Capacity Sharing_Inception Report 30-06-2025.pdf — page 39 part 4 — pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p39pt4
+Standard Provisions 2026.docx — section 'Monitoring and Evaluations' paragraph 115 — docx:Standard Provisions 2026.docx:u103-106</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -611,6 +678,12 @@
   </si>
   <si>
     <t>https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2, https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 24 part 3 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3, https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 22 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1</t>
+  </si>
+  <si>
+    <t>https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1 — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1, https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1</t>
+  </si>
+  <si>
+    <t>https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1 — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1, CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -1214,6 +1287,347 @@
 LLP Kazakh RI of Ag &amp; Plt Grow, Kazakhstan CIMMYT Phenotyping-Int Nurseries The Kyrgyz Research Institute of Livestock and Pasture, Kyrgyzstan CIMMYT Phenotyping-Int Nurseries NAFRI, Laos CIMMYT Phenotyping-Int Nurseries Misurata Agric. Res. Stn., Libya CIMMYT Phenotyping-Int Nurseries Pixus Agriculture Malawi Ltd., Malawi CIMMYT Phenotyping-Int Nurseries INIFAP , Mexico CIMMYT Phenotyping-Int Nurseries ICAMEX, Mexico CIMMYT Phenotyping-Int Nurseries Agroq. y Semillas La Fuerte SA, Mexico CIMMYT Phenotyping-Int Nurseries Fertilizantes Tepeyac, Mexico CIMMYT Phenotyping-Int Nurseries INRA-Morocco, Morocco CIMMYT Phenotyping-Int Nurseries</t>
   </si>
   <si>
+    <t>[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]
+el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]
+Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos
+---
+[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]
+Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]
+- 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness" 411,914 "Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 "Andean Crop Diversity for Climate Change P-1560-DGUL" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 "Youth, Citizen Science and E-commerce:
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]
+nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]
+business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]
+at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]
+2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]
+2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]
+II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p24pt1]
+System Organization and center allocations
+---
+[ID: pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p30pt1]
+System Organization and center allocations
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]
+Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]
+de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 "Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p55pt2]
+budget 2025 | System Organization and center allocations | Page
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u52-56]
+Aryal, Bishal (IFPRI) 44:47 Thank you. Thank you. Nirmal, Rajalakshmi (IFPRI) 44:50 Thank you. Bye, bye. Trifa, Nicoleta (CGIAR System Organization) 44:53 Hi. Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 13 of 86 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) Alliance Bioversity CIAT AoW 3-Markets and Business Models; AoW 5-Gender Equality, Social Inclusion and Fairness Intermediate Outcome - AOW-IOC 3.2. Local producer organizations, national and sub-national public actors and private sector actors co-design or strengthen inclusive business models; 2030 Outcome - 2030 OC-4. Marginalized people participate in implementing innovations; 2030 Outcome - 2030 OC-3 Government, market and finance actors implement
+---
+[ID: pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p31pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 31 of 56 System Organization:
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]
+Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u43-45]
+Colomer, Julien (One CGIAR - France) 48:19 Thanks. Hurt, Chris (ILRI) 48:19 Thank you. Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]
+de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 32 of 90 August 2025 | CGIAR Contracted partner Center Current Status of Partnership Area of Work Title and Number High level output (If Available) Dirección de Coordinación Regional y Extensión Rural (DICORER) CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Fundación para la Innovación Tecnológica Agropecuaria y Forestal
+---
+[ID: pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p57pt2]
+2025 | System Organization and center allocations | Page 57 of
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 25 of 44 Partner Center Area of Work Title and Number High level output (If Available) Local Governments for Sustainability, Nairobi City County, Dhaka North City Corporation, Local Government of Quezon City (Philippines), RUAF Foundation International Potato Center / Centro Internacional de la Papa 3.5.5 Urban food systems governance - Delivering knowledge products, evidence and capacity sharing with policy makers to guide interventions aimed at strengthening
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]
+(INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p28pt1]
+System Organization and center allocations Herder
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p38pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 38
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p20pt1]
+System Organization and center allocations Multispectral
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 55 of 86 External collaborations/partners Center Area of Work Title and Number High level output (If Available) Arab Center for the Studies of Arid Zones and Dry Areas - ACSAD ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de la Recherche Agronomique de Tunisie; National Agricultural Research Institute of Tunisia - INRAT ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de Recherche Agronomique de Tunisie. INRAT. ICARDA AoW2, AoW3 HLO: Accelerate - Stage2 &amp; Stage 3 testing &amp; Deploy Ankara University, Faculty of Agriculture ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]
+to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 51 of 90 System Organization: Scaling for Impact Implementation timelines (2025) Pooled
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p27pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 27 of 50 System Organization: Climate Action Implementation timelines (2025) Pooled
+---
+[ID: pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p31pt1]
+CGIAR | September 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 31 of 84 System Organization: Sustainable Farming Implementation timelines (2025)
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p49pt2]
+2025 | System Organization and center allocations | Page 49 of 86
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p25pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 25 of 86 System Organization: Multifunctional Landscapes Implementation timelines (2025) Pooled
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p21pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 21 of 52 System Organization: Genebanks Implementation timelines (2025) Pooled funding
+---
+[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p33pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 33 of 52 System Organization: Sustainable Animal and Aquatic Foods Implementation timelines (2025)
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4]
+Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations, and evidence-based programs for enhancing inclusive informal food markets that effectively create quality jobs for young women and men and deliver safe and healthy foods in urban environments University of Peradeniya, Wayamba University of Sri Lanka, Asian Development Bank, World Food Programme International Food Policy Research Institute 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents CGI21-507031-PORB-Food Frontiers and Security.indd 24CGI21-507031-PORB-Food Frontiers and Security.indd 24 29/07/2025 19:3929/07/2025 19:39
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 50 of 86 August 2025 | CGIAR External collaborations/partners Center Area of Work Title and Number High level output (If Available) CSIR-CRI - Ghana AfricaRice AB, EN Accelerate, Transform EIAR-Ethiopia AfricaRice AB, EN Accelerate, Transform IER-Mali AfricaRice AB, EN Accelerate, Transform CNRA- Côte d'Ivoire AfricaRice AB, MI, ID, EN Accelerate, Transform, Share, Design, Invest ITRAD-Chad AfricaRice AB Accelerate FOFIFA-Madagascar AfricaRice AB, ID, MI, EN Accelerate, Transform, Share, Design, Invest NARO-Uganda AfricaRice MI Design, Invest NARI - the Gambia AfricaRice ID
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p81pt2]
+2025 | System Organization and center allocations | Page 81 of 86
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1]
+Capacity Sharing Accelerator Inception Report 4 ISNAR International Service for National Agricultural Research ISRA Institut Sénégalais de la Recherche Agricole (Senegalese Agricultural Research Institute) ITU International Telecommunication Union KOICA Korea International Cooperation Agency KPIs Key Performance Indicators. MELIA Monitoring, Evaluation, Learning, and Impact Assessment NARES National Agricultural Research and Extension Systems NARS National Agricultural Research System PCT Program Coordination Team
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p30pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 30 of 50
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p42pt1]
+System Organization and center allocations Taking care of the
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p49pt4]
+Accelerate, Design, Umudike Seed IITA ID, MI Accelerate, Design, INERA-Burkina Faso AfricaRice AB, EN Accelerate, Transform INERA-DRC AfricaRice AB, MI, EN Accelerate, Transform, Share ISRA- Senegal AfricaRice AB, ID, MI, EN Accelerate, Transform, Design, Invest CARI- Liberia AfricaRice AB Accelerate NCRI-Nigeria AfricaRice AB, ID, MI, EN Accelerate, Transform, Share, Design, Invest SLARI-Sierra Leone AfricaRice AB, MI, EN Accelerate, Transform INRAB-Benin AfricaRice AB Accelerate IRAG-Guinea Conakry AfricaRice AB, EN Accelerate, Transform INRAN-Niger AfricaRice AB, EN Accelerate, Transform CGI21-508008-PORB-Breeding for Tomorrow.indd 49CGI21-508008-PORB-Breeding for Tomorrow.indd 49 08/08/2025 16:0208/08/2025 16:02
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2]
+Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The World Bank, German Red Cross (Germany), Dhaka City North Corporation, Nairobi City County, International Water Management Institute, WorldFish International Food Policy Research Institute 1.2.2 Evidence Synthesis and Adaptive Learning - Co-develop knowledge products and action plans, and identify key investment and innovation priorities for stakeholders and partners to guide interventions aimed at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2]
+(SME) Private Ltd CIMMYT ID DEPLOY IFFA Seed Co Ltd CIMMYT ID DEPLOY Indian Institute of Maize Research CIMMYT AB, ID DEPLOY Indo American Hybrid Seeds (India) Pvt. Ltd CIMMYT ID DEPLOY Institut de Recherche Agricole pour le Développement (IRAD) CIMMYT AB, ID DEPLOY Institut des Sciences Agronomiques du Burundi (ISABU) CIMMYT AB, ID DEPLOY Institut National de la Recherche Agronomique du Niger (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p29pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 29 of 44 System Organization: Food Frontiers and Security Implementation timelines (2025) Pooled funding Budget
+---
+[ID: pdf:CGI21-508004-PORB-Digital Transformation.pdf:p24pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 24 of 38
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 36 of 86 August 2025 | CGIAR External collaborations/partners Center Area of Work Title and Number High level output (If Available) L’Institut Tchadien de Recherche Agronomique pour le Développement – ITRAD – Chad CIMMYT AB, ID, MI, Enable l’Institut National de la Recherche Agronomique du Niger – INRAN – Niger CIMMYT AB, ID, MI, Enable Ministry of Agriculture and Food Security – MAFS – Sudan CIMMYT AB, ID, MI, Enable MyAgro – USA CIMMYT ID National Agricultural Research Organization
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p58pt3]
+| System Organization and center allocations | Page 58 of 86 August 2025
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1]
+23 Bilateral Contribution to Multifunctional Landscapes MELIA Studies UK FCDO - Seed to tree: value chains and partnerships for resilient restored forests in Malaysia • Actor engagement and outcome tracking UK – GCBC (UK-Defra) - Deploying Diversity as a Strategic Asset for Scaling of Ethiopia’s Green Legacy Initiative for Climate Change Resilience and Livelihoods • Program learning review • Actor engagement and outcome tracking FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) • Actor engagement and outcome tracking CoIMPACT INDIA • Program learning review Fruitful Lands India Phase II • Actor engagement and outcome tracking Sustainable Investments for Large-scale Rangeland R • Actor engagement and outcome tracking Building Community
+---
+[ID: pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3]
+Lebanese Agriculture Research Institute (LARI), Institut National De La Recherche Agronmique en Tunisie (INRAT) IFPRI, Alliance, ICARDA Area of Work: Accelerating Solutions for Impact 1.4.3: Evidence on effectiveness of solutions for inclusive leadership TBD GENDER Accelerator Area of Work: Accelerating Solutions for Impact 1.5.1: Analysis of constraints and pathways for youth in FLWS n/a n/a Area of Work: Accelerating Solutions for Impact 1.5.2: Co-designed approaches to engaging youth in FLWS n/a n/a Area of Work: Accelerating Solutions for Impact 1.5.3: Evidence on effectiveness of approaches to engaging youth in FLWS AGRA, IFAD, FAO, WFP IFPRI Area of Work: Accelerating Change Through Evidence 2.1.1: Guidance on ethical gender research AGRA, IFAD,
+---
+[ID: pdf:CGI21-508004-PORB-Digital Transformation.pdf:p22pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 22 of 38
+---
+[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p37pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 37
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p59pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 59 of 86 System Organization: Breeding for Tomorrow Implementation timelines (2025) Pooled funding Budget Total Program Q1 Q2
+---
+[ID: pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p21pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 21 of 42 System Organization: Gender Equality and Inclusion Implementation timelines (2025) Pooled funding Budget Total Accelerator Q1 Q2
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p49pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 49
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p71pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 71
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u25-28]
+Trifa, Nicoleta (CGIAR System Organization) 33:46 Yes, the answer is more people beyond Media can access PRMS. We are now actually taking the user role from PRMS reporting from the previous portfolio and. Make sure that they apply to this portfolio as well. So I will share my screen again just to give you a quick insight into that. So the roles we use in the previous portfolio were, you know, lead, what the lead can do, co-lead, coordinator, member and admin and then a guest. And then so these are the roles. I will share this link with you so if you have a better look at the definition who is part of what category. So based on these roles we have asked the program coordinators to. Put a name next to each role for PRMS from their own teams. So they had to, you know, ask in the teams to see, OK, who will play the, who will play, who will be a colleague, a lead, an admin, a guest and so on in PRMS. So I believe that list is still a work in progress. We did not receive. Feedback from old programs and accelerators by now, but based on that list, basically we will give initial access to PRMS reporting and obviously if in the meantime people come and go and so on, if there are requests to add new people to the list. It's never an exhaustive list, so this is a live list throughout the year. So you can request to be added to the list with you know certain a certain role and that will be you know in enabled in the system. Nirmal, Rajalakshmi (IFPRI) 35:30 Right. My, I had another question, Nicoletta, if it's OK on the reporting for the bilateral projects, right. So when we did the TOC, we just mapped it to each area of work and the, you know, and put them under the high level outputs. Trifa, Nicoleta (CGIAR System Organization) 35:34 Go ahead. Sure. Nirmal, Rajalakshmi (IFPRI) 35:48 But we haven't gone to the level of mentioning the targets or indicators for these bilateral projects that were mapped, right. So when we are about to start the reporting process, what's the plan? How are we going to go about this part? Yeah, Mandy Jules.
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2]
+capacity AfriSeed, Zambia CIMMYT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact HLO 5.2: Insights for CGIAR scaling success through impact assessments.HLO 2.2: Co-designed scaling pathways for regional and national agrifood systems through improved stakeholder capacity Secretaría de Agricultura y Desarrollo Rural (SADER) de México CIMMYT Potential AoW1 - Engage and Empower HLO 1.1: A toolbox of methods, data, and dashboards HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Agencia Mexicana de Cooperación Internacional para el Desarrollo (AMEXCID) CIMMYT Potential AoW1 - Engage and Empower HLO
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3]
+Bolivia CIMMYT Phenotyping ZARI - Zambia Agricultural Research Institute, Zambia CIMMYT Phenotyping INIA Chile -Instituto de Investigaciones Agropecuarias, Chile CIMMYT Phenotyping INIA Uruguay -Instituto Ncional de Investigacion Agropecuaria, Uruguay CIMMYT Phenotyping IRESA - Institution de la Recherche et de l’Enseignement Supérieur Agricoles, Tunisia CIMMYT Phenotyping TAGEM - Ministry of Food Agriculture and Livestock, Turkey CIMMYT Phenotyping KALRO- Kenya Agricultural &amp; Livestock Research Organization, Kenya ARIA, Afghanistan CIMMYT Phenotyping-Int Nurseries ITGC, Algeria CIMMYT Phenotyping-Int
+---
+[ID: docx:Standard Provisions 2026.docx:u7-10]
+between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization; between the System Organization and each Center apply to the Financial Framework Agreement between the System Organization and each Center; and between a Funder and a Center apply to each Window 3 Side Agreement or Arrangement between a Funder and a Center. Use and administration of the Contributions
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u22-25]
+Colomer, Julien (One CGIAR - France) 32:14 Mm-hmm. Yeah. Yeah, thanks. No, I I hear You and and that's really the also the the intent was to um. Build a sort of, um, a bridge between outputs and outcomes, right? So to IT wouldn't be either an output or an outcome, and IT would be the sort of category that spanned both and we would use IT to collect evidence of all of the things that Help foment or catalyze. You know, outcomes, right. But yeah, either we Go or we don't. So I I think, You know, we've been sort of umming and ahhing for too Long now an</t>
+  </si>
+  <si>
+    <t>[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]
+el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]
+Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]
+Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]
+Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]
+- 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness" 411,914 "Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 "Andean Crop Diversity for Climate Change P-1560-DGUL" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 "Youth, Citizen Science and E-commerce:
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]
+de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]
+nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]
+2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]
+2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]
+C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L.
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]
+to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4]
+del Bienestar (SEBIEN) de Quintana Roo CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Secretaría de Desarrollo Agropecuario (SEDAGRO) de Morelos CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Ministerio de Agricultura, Ganadería y Alimentación (MAGA) de Guatemala CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio CGI21-508007-PORB-Scaling for Impact.indd 31CGI21-508007-PORB-Scaling for Impact.indd 31
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]
+de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 "Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The
+---
+[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]
+Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 55 of 86 External collaborations/partners Center Area of Work Title and Number High level output (If Available) Arab Center for the Studies of Arid Zones and Dry Areas - ACSAD ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de la Recherche Agronomique de Tunisie; National Agricultural Research Institute of Tunisia - INRAT ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de Recherche Agronomique de Tunisie. INRAT. ICARDA AoW2, AoW3 HLO: Accelerate - Stage2 &amp; Stage 3 testing &amp; Deploy Ankara University, Faculty of Agriculture ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]
+(INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]
+at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]
+II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2]
+(SLARI) Africa Rice Potential AoW 4 - Achieving Impact by Unlocking Finance and Partnerships GrainPro Inc Africa Rice Potential AoW 2 - Pathways to Scale in Agrifood Systems African Development Bank Africa Rice Contracted AoW 4 - Achieving Impact by Unlocking Finance and Partnerships Seed Development and Certification Agency, Liberia Africa Rice Potential AoW 3 - Enabling Environment Lab Central de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3]
+Bolivia CIMMYT Phenotyping ZARI - Zambia Agricultural Research Institute, Zambia CIMMYT Phenotyping INIA Chile -Instituto de Investigaciones Agropecuarias, Chile CIMMYT Phenotyping INIA Uruguay -Instituto Ncional de Investigacion Agropecuaria, Uruguay CIMMYT Phenotyping IRESA - Institution de la Recherche et de l’Enseignement Supérieur Agricoles, Tunisia CIMMYT Phenotyping TAGEM - Ministry of Food Agriculture and Livestock, Turkey CIMMYT Phenotyping KALRO- Kenya Agricultural &amp; Livestock Research Organization, Kenya ARIA, Afghanistan CIMMYT Phenotyping-Int Nurseries ITGC, Algeria CIMMYT Phenotyping-Int
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4]
+Senegalais de Recherches Agricoles – ISRA – Senegal CIMMYT AB, ID, MI, Enable Instituto de Investigacao Agraria de Mocambique – IIAM – Mozambique CIMMYT AB, ID, MI, Enable International Institute of Tropical Agriculture – IITA – Nigeria CIMMYT AB, ID, MI, Enable Kenya Agricultural and Livestock Research Organization – KALRO – Kenya CIMMYT AB, ID, MI, Enable Lake Chad Research Institute – LCRI – Nigeria CIMMYT AB, ID, MI, Enable L’Institut de l’Environnement et de Recherches Agricoles – INERA – Burkina Faso CIMMYT AB, ID, MI, Enable CGI21-508008-PORB-Breeding for Tomorrow.indd 35CGI21-508008-PORB-Breeding for Tomorrow.indd 35 08/08/2025 16:0208/08/2025
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2]
+capacity AfriSeed, Zambia CIMMYT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact HLO 5.2: Insights for CGIAR scaling success through impact assessments.HLO 2.2: Co-designed scaling pathways for regional and national agrifood systems through improved stakeholder capacity Secretaría de Agricultura y Desarrollo Rural (SADER) de México CIMMYT Potential AoW1 - Engage and Empower HLO 1.1: A toolbox of methods, data, and dashboards HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Agencia Mexicana de Cooperación Internacional para el Desarrollo (AMEXCID) CIMMYT Potential AoW1 - Engage and Empower HLO
+---
+[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2]
+system Provincial govt. AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Colombian Roundtable for Sustainable Cattle AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Universidad del Cauca AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Universidad de los Andes AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system EAFIT University Colombia AOW 4 Market Systems, Policy Solutions and
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2]
+Report June 2025 Contact: Nicoline de Haan (n.dehaan@cgiar.org)
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p32pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 32 of 72 July 2025 | CGIAR Contracted partner Center Area of Work Title and Number High level output (If Available) University of Los Andes CIAT Governance and Political Economy (AOW03) 3.3: New communities of practice, political economy and policy process tools are developed and strengthened, bringing together decision makers and diverse stakeholders to strengthen science diplomacy, science policy engagement, design, and implementation. Tegemeo Institute in Kenya IFPRI Governance and Political Economy (AOW03) 3.3: New communities of practice, political economy
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt2]
+Research for Development (IRAD) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems Centre National de Recherche Agronomique (CNRA) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems The Council for Scientific and Industrial Research – Savannah Agricultural Research Institute (CSIR- SARI) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems Centre National de Recherche Appliqué au Développement Rural (FOFIFA/CENRADERU) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems L’Institut Sénégalais de Recherches
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4]
+for delivering SAAF outputs and outcomes. These organizations are either think tanks and consultancy firms (e.g. MacKenzie), governmental extension services (Fisheries Commission Ghana), or NGOs (Heifer International, CARE). In those instances, CGIAR is well-positioned to undertake the work. Still, stakeholder engagement can be pursued with stakeholders to transition toward sustainability and scaling. The remaining 80% have been rated as moderately efficient and impactful in undertaking HLO work. This group encompasses NARES (KALRO, IFReDI), NGOs (Vétérinaires Sans Frontières); private sector organizations (EON Aquaculture Limited, Githunguri Dairy Cooperative); international organizations (FAO, World Bank, AfDB); universities from the Global North (Corwell, Kiel) or targeted countries (Universidad de los Andes, University of Nairobi, Hanoi University of Public Health). While CGIAR is well or moderately positioned in most instances, there are significant opportunities for collaboration, stakeholder engagement, and in some instances, formal partnerships. Sustainable Animal &amp; Aquatic Food Science Program Comparative Advantage analysis
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2]
+(SME) Private Ltd CIMMYT ID DEPLOY IFFA Seed Co Ltd CIMMYT ID DEPLOY Indian Institute of Maize Research CIMMYT AB, ID DEPLOY Indo American Hybrid Seeds (India) Pvt. Ltd CIMMYT ID DEPLOY Institut de Recherche Agricole pour le Développement (IRAD) CIMMYT AB, ID DEPLOY Institut des Sciences Agronomiques du Burundi (ISABU) CIMMYT AB, ID DEPLOY Institut National de la Recherche Agronomique du Niger (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]
+business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 13 of 86 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) Alliance Bioversity CIAT AoW 3-Markets and Business Models; AoW 5-Gender Equality, Social Inclusion and Fairness Intermediate Outcome - AOW-IOC 3.2. Local producer organizations, national and sub-national public actors and private sector actors co-design or strengthen inclusive business models; 2030 Outcome - 2030 OC-4. Marginalized people participate in implementing innovations; 2030 Outcome - 2030 OC-3 Government, market and finance actors implement
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2]
+National Agricultural Research and Extension Systems NARS National Agricultural Research System PCT Program Coordination Team PMU Program Management Unit PORB Plans of Results and Budgets RAB Rwanda Agriculture and Animal Resources Development Board RELASER Red Latinoamericana de Servicios de Extensión Rural (Latin American Network for Rural Extension Services) RUFORUM Regional Universities Forum for Capacity Building in Agriculture SAARC South Asian
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2]
+la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics (Breeding for Tomorrow) ● T-PJ-003670- Long-term funding of Ex Situ collections of germplasm (IITA) (Breeding for Tomorrow and CapSha) ● L-LTG001-Long term funding of ex situ collections of germplasm (ILRI) (Breeding for Tomorrow) ● R-A-2023-9-Genebank-AI (Breeding for Tomorrow) ● T-PJ-003575: Cassava Allele Mining Project: (IITA) Mining useful alleles for climate change adaptation in the cassava from CGIAR Genebanks (Breeding for Tomorrow and Climate Action) ● T-PJ-003576- (IITA) Mining useful alleles for climate change adaptation cowpea (Cowpea Allele mining project: Mining useful alleles for climate change adaptation in cowpea from CGIAR Genebanks (year 2022-26) (Breeding for Tomorrow, CapSha, and Climate Acti on) ● T-PJ-004017-VACS (IITA): Vision for Adapted Crops and Soil: Bambara Groundnut (Breeding for Tomorrow, CapSha and
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4]
+Cooperation TAP Tropical Agriculture Platform ToC Theory of Change ToR Terms of References TPI The Partnering Initiative UM6P Université Mohammed VI Polytechnique UNCTAD United Nations Conference on Trade and Development UNESCO United Nations Educational, Scientific and Cultural Organization. UNICEF United Nations International Children's Emergency Fund UPLB University of the Philippines Los Baños W3 Window 3 WCDI Wageningen Centre for Development
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 36 of 86 August 2025 | CGIAR External collaborations/partners Center Area of Work Title and Number High level output (If Available) L’Institut Tchadien de Recherche Agronomique pour le Développement – ITRAD – Chad CIMMYT AB, ID, MI, Enable l’Institut National de la Recherche Agronomique du Niger – INRAN – Niger CIMMYT AB, ID, MI, Enable Ministry of Agriculture and Food Security – MAFS – Sudan CIMMYT AB, ID, MI, Enable MyAgro – USA CIMMYT ID National Agricultural Research Organization
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3]
+management of research &amp; scaling activities across CGIAR’s portfolio Agencia Mexicana de Cooperación Internacional para el Desarrollo (AMEXCID) CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Secretaría de Fomento Agroalimentario y Desarrollo Rural (SEFADER) Oaxaca CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Secretaría del Bienestar (SEBIEN) de Quintana Roo CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp;
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 32 of 90 August 2025 | CGIAR Contracted partner Center Current Status of Partnership Area of Work Title and Number High level output (If Available) Dirección de Coordinación Regional y Extensión Rural (DICORER) CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Fundación para la Innovación Tecnológica Agropecuaria y Forestal
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p21pt3]
+and Technology (DOST) Philippines IRRI AoW03 Locally led adaptation 3.3, 3.4 and 3.5--- for 3.5 Policies, institutions, and interventions for equitable climate change adaptation Ministry of Agriculture Kenya IRRI AoW03 Locally led adaptation HLO 3.5 Recommendations on policies and institutions for addressing the root causes of inequality University of the Philippines, Los Banos and Xavier University IRRI AoW03 Locally led adaptation 3.3 and 3.4 - for 3.4 Novel framework and methods for avoiding maladaptation Royal University of Agriculture, Cambodia IRRI Aow04 Low-emission transitions 4.2 and 4.4
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt3]
+MI, Enable Ethiopian Institute of Agricultural Research – EIAR – Ethiopia CIMMYT AB, ID, MI, Enable Institut d’Economie Rurale – IER – Mali CIMMYT AB, ID, MI, Enable Institute for Agricultural Research, Samaru – IAR – Nigeria CIMMYT AB, ID, MI, Enable Institute Togolais de Recherche Agronomique – ITRA – Togo CIMMYT AB, ID, MI, Enable Insitute of Agricultural Research for Development – IRAD – Cameroon CIMMYT AB, ID, MI, Enable Institut Senegalais de Recherches Agricoles – ISRA – Senegal CIMMYT AB, ID, MI, Enable Instituto de Investigacao Agraria de Mocambique – IIAM – Mozambique CIMMYT
+---
+[ID: pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt3]
+producer with Felistus Chipungu (right), OFSP breeder and scientist, CIP . Credit: C. de Bode/CGIAR
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 25 of 44 Partner Center Area of Work Title and Number High level output (If Available) Local Governments for Sustainability, Nairobi City County, Dhaka North City Corporation, Local Government of Quezon City (Philippines), RUAF Foundation International Potato Center / Centro Internacional de la Papa 3.5.5 Urban food systems governance - Delivering knowledge products, evidence and capacity sharing with policy makers to guide interventions aimed at strengthening
+---
+[ID: pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt4]
+3.3, 5.2, 5.3, 5.4 or 5.5. Climate adaptation Overall the impact area with third highest prioritized activities. Broad prioritization of AoW2&gt;AoW4&gt;AoW 3&gt;AoW 1&gt;AoW5 Relatively moderate priority. No priority for HLO 1.2, 1.5, 5.1, 5.4 or 5.5. Relatively moderate priority. No priority for HLO 1.5, 5.4 or 5.5. Second Highest ABI priority for IA Relatively moderate priority. No priority for HLO 1.5, 5.1, 5.4 or 5.5. Highest ABI priority for IA Relatively moderate priority. No priority for HLO 1.5, 5.4 or 5.5. Third Highest ABI priority for IA Relatively moderate priority. Relatively moderate priority. Environmental Health Moderate-low prioritization. Third highest prioritization of regions. De- prioritization of HLO 1.2, 1.5, 5.1 and 5.5 Relative low prioritization. Lowest across regions. De- prioritization of HLO 1.2, 1.5, 3.3, 5.1, 5.3 and 5.5 Moderate-low prioritization with additional de- prioritization of HLO 1.5, 5.4 and 5.5 Moderate- low prioritization . De- prioritization of HLO 1.5, 5.1 and 5.5 Moderate-low prioritization. Second highest prioritization of regions. De- prioritization of HLO 1.5, 5.1 and 5.5 Moderate-low prioritization. Highest prioritization of regions. De- prioritization of HLO 1.5, 5.1 and
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1]
+Capacity Sharing Accelerator Inception Report 4 ISNAR International Service for National Agricultural Research ISRA Institut Sénégalais de la Recherche Agricole (Senegalese Agricultural Research Institute) ITU International Telecommunication Union KOICA Korea International Cooperation Agency KPIs Key Performance Indicators. MELIA Monitoring, Evaluation, Learning, and Impact Assessment NARES National Agricultural Research and Extension Systems NARS National Agricultural Research System PCT Program Coordination Team
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1]
+23 Bilateral Contribution to Multifunctional Landscapes MELIA Studies UK FCDO - Seed to tree: value chains and partnerships for resilient restored forests in Malaysia • Actor engagement and outcome tracking UK – GCBC (UK-Defra) - Deploying Diversity as a Strategic Asset for Scaling of Ethiopia’s Green Legacy Initiative for Climate Change Resilience and Livelihoods • Program learning review • Actor engagement and outcome tracking FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) • Actor engagement and outcome tracking CoIMPACT INDIA • Program learning review Fruitful Lands India Phase II • Actor engagement and outcome tracking Sustainable Investments for Large-scale Rangeland R • Actor engagement and outcome tracking Building Community
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p47pt3]
+Research Organization Centre de coopération internationale en recherche agronomique pour le développement Wageningen University and Research Centre Cornell University Zambia Agriculture Research Institute Ethiopian Institute of Agricultural Research Agricultural Research Institute - Tanzania Food and Agriculture Organization of the United Nations Indian Council of Agricultural Research 176 118 135 111 106 87 98 80 79 78 Food and Agriculture Organization of the United Nations Agricultural Research Institute - Tanzania National Agricultural Research Organisation (Uganda) Ministry of Agriculture and Rural Development (Vietnam) Kenya Agricultural and Livestock Research Organization Instituto de Investigacao Agraria de Mozambique Department of Agriculture Extension (Bangladesh) Indian Council of Agricultural Research Zambia Agric</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -1248,6 +1662,15 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria y programática?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]\nLink: https://cgspace.cgiar.org/items/8acc660f-7305-4e4b-ab21-1c192611b017\nFile: CGI21-507032-PORB-Climate Action.pdf\nLocation: page 11 part 2\nContent: II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 4\nContent: Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations, and evidence-based programs for enhancing inclusive informal food markets that effectively create quality jobs for young women and men and deliver safe and healthy foods in urban environments University of Peradeniya, Wayamba University of Sri Lanka, Asian Development Bank, World Food Programme International Food Policy Research Institute 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents CGI21-507031-PORB-Food Frontiers and Security.indd 24CGI21-507031-PORB-Food Frontiers and Security.indd 24 29/07/2025 19:3929/07/2025 19:39\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u52-56]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 52 to paragraph 55\nContent: Aryal, Bishal (IFPRI) 44:47 Thank you. Thank you. Nirmal, Rajalakshmi (IFPRI) 44:50 Thank you. Bye, bye. Trifa, Nicoleta (CGIAR System Organization) 44:53 Hi. Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Se reportan desvíos potenciales en su uso. ¿Quién tiene la responsabilidad fiduciaria y programática, qué debe informar el Center y qué facultades de acción tiene la System Organization (SO)?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_Inception Report 30-06-2025.pdf\nLocation: page 4 part 3\nContent: Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién gestiona colectivamente los requisitos de M&amp;E de los Funders y cómo se evita la duplicación?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 45 part 3\nContent: Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 3\nContent: de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 46 part 3\nContent: C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L."}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who coordinates funders’ M&amp;E requirements across the CGIAR Portfolio and how is duplication avoided? \n\nContext:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23 part 4\nContent: additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 2 part 4\nContent: report is part of the CGIAR System Organisations’ technical reporting arrangement. We would like to thank all funders who supported this work through their contributions to the CGIAR Trust Fund, and those who supported bilaterally: https://www.cgiar .org/funders. The report was led by the Portfolio Performance Unit, with expert technical support from the Food Security Evidence Brokerage. We gratefully acknowledge the contributions and insights from many CGIAR staff who provided access to source materials, selected prominent themes, and reviewed drafts. This included Impact Area Platform Directors, regional leaders, CGIAR Center assessment and monitoring specialists, the Independent Advisory and Evaluation Services, the Donor Relations and Business Development unit, the Communications and Advocacy unit, CGIAR research leaders and senior\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p29pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 29 part 2\nContent: of information on how climate mitigation is covered in the Portfolio. There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. There is a lack of information on how orphan and opportunity crops and pulses are covered in the Portfolio. There is a lack of information on how\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p33pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 33 part 2\nContent: is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. N/A There is a lack of information on how orphan and opportunity crops and pulses are covered in the Portfolio. N/A There is a lack of information on how youth and social inclusion (that does not relate to gender) is covered in the Portfolio. N/A There is a lack of information on how capacity sharing (as it relates to internal learning and decolonization of research) is covered in the Portfolio. Capacity sharing is foundational to\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p39pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 39 part 4\nContent: more details on ToC, Areas of Work, etc. We have significantly reworked and streamlined the research questions. They are now underpinned by the assumptions formulated in the revised ToC these also serve as hypotheses (in terms of fulfilled assumptions) for the research questions. Linkages with other Programs and Accelerators A concern is how the accelerator will effectively work with and build on other capacity sharing activities at CGIAR (with other Programs and Accelerators) without duplication or competition (pp. 85). The Accelerator will include a matrix analysis of Programs and other Accelerator during inception, to map Programs’ AoW and its own AoW, in order to define common interests in research questions or challenges, synergies, alignments, complementarities, and avoid duplication of actions. Section 8 of the inception report details how the accelerator would work with other programs to ensure synergy, and avoid duplication and support complementarity in terms of delivery of its service portfolio.\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 1\nContent: 2.2. Close-out of the 2022-24 Portfolio As the 2022-24 Portfolio closed, close-out guidelines were designed to ensure a smooth transition to the new Portfolio, building on past achievements while maintaining continuity in science and innovation delivery. The close-out process focused on the timely preparation and submission of 2024 technical and financial reports, ensuring all CGIAR teams and partners met Portfolio deliverables, and facilitating effective engagement and continuous communication with stakeholders. Proactive mitigation measures were identified to manage risks associated with the transition to the new research Portfolio. Focus was placed on sustaining partnerships beyond the conclusion of the 2022-24 Portfolio to ensure ongoing collaboration. The guidelines included a section on SGPs to ensure alignment. This structured approach ensures that the achievements and collaborations of the 2022-24 cycle are seamlessly integrated into the new Portfolio. 2.3. Transitioning to the 2025-30 Portfolio Support was provided to the CGIAR Portfolio Transition Team, which included the development of Inception Guidelines that outlined the principles and processes to assist Transition Teams in planning and achieving inception deliverables for the 2025-30 CGIAR Portfolio. In 2024 work began on developing a new Technical Reporting Arrangement for 2025-30 (TRA 25-30) to define the Technical Reporting requirements for the next CGIAR Portfolio. A cross-CGIAR working group – comprising Center experts and System functions – led its development. The TRA 25-30 will promote progressive alignment between reporting requirements for pooled and non-pooled\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p30pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 30 part 4\nContent: S4I will map scaling efforts across Programs to reduce duplication, achieve synergies, and strengthen system-wide coherence.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 3 part 2\nContent: outcomes and i mpacts of the whole portfolio through progressive alignment of reporting on w3/bilaterally funded components with a common framework. • Line of sight: The TRA is designed to meet the needs of diverse funders, ensuring transparency and accountability by linking investment to results, both for pooled and non-pooled funds. • Impact focus: Research results will be better linked to CGIAR’s 2030 targets using enhanced impact area indicators. Impact assessments will be integrated into Program/Accelerator design. The use of geographically-bounded targets will be explored for priority locations. A robust approach to project cross-Portfolio benefits by Impact Area for different funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified reporting: Overly complex requirements will be avoided, aiming to\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p2pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 2 part 4\nContent: reviewed and validated by the authors to ensure accuracy, coherence, and alignment with the original intent. Acknowledgements This work is part of the CGIAR System Organization. We would like to thank all funders who supported this research through their contributions to the CGIAR Trust Fund:\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p32pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 32 part 1\nContent: Genebanks Accelerator Inception Report 31 10. Addressing feedback on selects topics Concise summary of feedback Details on how the Program/ Accelerator has addressed or will address this feedback (in the Inception Phase or beyond) There is a lack of information on how water systems are covered in the Portfolio. N/A There is a lack of information on how climate mitigation is covered in the Portfolio. N/A There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. The Genebanks proposal noted that activities will lead to a stronger overall global system of international and national institutions, policies, and mechanisms contributing\n\n---\n\n[ID: pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p25pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_Inception Report 30-06-2025.pdf\nLocation: page 25 part 1\nContent: Food Frontiers and Security Program | Inception Report 25 operational efficiency, avoid duplication, and generate broader, more context-responsive insights than either program could produce alone, delivering greater value to partners and stakeholders across the CGIAR portfolio. Together with The Climate Action SP,\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 3 part 3\nContent: funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified reporting: Overly complex requirements will be avoided, aiming to reduce the reporting burden on Centers. Technical Report products include the following: • A Results Dashboard including AI functionalities will be updated several times a year (e.g. quarterly) to offer funders and partners closer to real-time data. • Annual Program/Accelerator Technical Reports will be complemented by an Annual Portfolio Report which will convey progress by Impact Area, geographic and thematic priorities and include information on CGIAR’s internal practice change and learning. • Portfolio outcomes and impacts will be consolidated in a specific report every 3 years. Evidence of CGIAR contributions to impact will be synthesized and regularly updated through an\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u103-106]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use of Materials' paragraph 108 to section 'Monitoring and Evaluations' paragraph 115\nContent: Intellectual Property rights. The System Organization and each Center will, respectively, ensure that necessary intellectual property rights are obtained to allow the rights referred to under this paragraph 6 to be granted. If third party copyright restrictions or attribution requirements apply to such documents, this will be indicated on the documents. Monitoring and Evaluations General Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p8pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 8 part 4\nContent: other organizations as well as by funders. “CGIAR’s efforts to mainstream scaling put it at the cutting edge …” compared to other research and innovation organizations, and development organizations generally (Global Scaling Community of Practice). Figure 5: A pile of LEGO pieces that represents CGIAR’s innovation portfolio management pre-2022. What was once a fragmented system is now becoming more structured and strategic. Until 2022, there was no efficient way to manage ‘’CGIAR’s innovation portfolio’’. Innovation data was scattered, not up-to-date and lacked evidence. Furthermore, there was no operational framework to track or support scaling for impact. It led to organizational risks and inefficiencies as leadership, partners and funders could not easily access CGIAR innovations. This changed under the CGIAR 2030 Research and Innovation Strategy that embraced a more systematic and evidence-based innovation management based on principles of the Scaling Readiness approach. Currently, information on more than 1,325 innovations under development or use are now easily accessible on the CGIAR Results Dashboard, which is widely used by partners and funders. The World Bank Group, FAO, Gates Foundation, GIZ, ENABEL, and the African Development Bank are among organizations that have embraced (elements of) the CGIAR innovation management approach. CGIAR is actively sharing its innovation portfolio management journey with other organizations. The Gates Foundation partnered with CGIAR to co-develop a protocol for scaling strategies aimed at high-impact innovations. Internally, CGIAR Centers such as the Alliance of Bioversity and CIAT (ABC) and the International Livestock Research Institute (ILRI) and CGIAR projects such as the Accelerate for Impact Platform (A4IP), Technologies for African Agricultural Transformation (TAAT) and HarvestPlus Solutions have adopted elements of innovation portfolio management. May 2025 1110 CGIAR Portfolio Practice Change (Type 3)\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 2\nContent: 2025-30 CGIAR Portfolio. In 2024 work began on developing a new Technical Reporting Arrangement for 2025-30 (TRA 25-30) to define the Technical Reporting requirements for the next CGIAR Portfolio. A cross-CGIAR working group – comprising Center experts and System functions – led its development. The TRA 25-30 will promote progressive alignment between reporting requirements for pooled and non-pooled funding components, and sets expectations for transparency, performance tracking, and accountability across CGIAR and with funders. It will also operationalize the PRMF , inform decision-making, and provide direction for Portfolio-level monitoring, evaluation, learning and impact assessment (MELIA) and the design of the next version of the PRMS. The TRA 25-30 is expected to be endorsed in the first half of 2025. A durum wheat field at Toluca Station. Credit: Alfonso Cortés/CIMMYT Section 3: Implementation Status: Management Responses to CGIAR Evaluations 5. For more information see the CGIAR Evaluation Policy, the CGIAR Evaluation Guidelines, and the Process Note on Developing, Tracking and Reporting on Management Responses to Evaluations. A Management Response is a formal mechanism through which Evaluation Recommendations are addressed by management. These responses are designed to ensure that Evaluations inform decision-making, enhance organizational effectiveness, promote learning, and strengthen accountability. They include time-bound commitments from management to implement Evaluation Recommendations and are systematically followed up as outlined in the CGIAR Evaluation Policy, which identifies follow-up as a critical component of the evaluative process.5 Since\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p87pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 87 part 2\nContent: 2025–2030 The creation of a Scaling for Impact Program in CGIAR’s Portfolio 2025–2030 creates even more space and resources for innovation and scaling work. The Scaling for Impact Program plays an important role in catalyzing innovation scaling on the ground with CGIAR colleagues and partners while more System-wide innovation portfolio management functions continue to be delivered by CGIAR’s Portfolio Performance Unit. In CGIAR’s 2025–2030 Portfolio (Figure 6.4), innovation management is not just a process or tool — it is the central instrument for driving coherence and collaboration between the Science Programs and the Scaling for Impact Program while also aligning demand with supply and guiding strategic Portfolio priorities. Figure 6.4. Schematic overview of the CGIAR 2025–2030 Portfolio. CGIAR’s Portfolio Performance Unit and Project Coordination Unit work closely with the Scaling for Impact Program to deliver key innovation portfolio management functions for the 2025–2030 Portfolio. These two units continue to mainstream innovation and scaling tracking and performance across the\n\n---\n\n[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations_Inception Report 30-06-2025.pdf\nLocation: page 26 part 2\nContent: to national policy research ecosystems through coordinated capacity sharing activities. A prime example of this effective coordination and the efficiencies it generates is the policy program hub in Kenya. This hub actively coordinates with other CGIAR Programs, Accelerators, and individual CGIAR Centers building on efforts that the CGIAR country convener for Kenya had started. It therefore also provides an integration mechanism with W3/bilateral projects. Coordination is fundamental for avoiding duplication of efforts: They serve as a critical platform to share research plans, identify synergies, and proactively prevent overlapping activities, thereby ensuring a highly efficient deployment of collective resources across various CGIAR programs in Kenya. Beyond internal CGIAR coordination, the Kenya hub takes a leading role in planning joint policy dialogue series, country policy notes, bringing diverse stakeholders together for impactful co- design and co-implementation.\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p33pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 33 part 1\nContent: Capacity Sharing Accelerator Inception Report 33 10. Addressing feedback on select topics Only one feedback (lack of information on how capacity sharing) applies directly to the CapSha Accelerator. Concise summary of feedback Details on how the Program/ Accelerator has addressed or will address this feedback (in the Inception Phase or beyond) There is a lack of information on how water systems are covered in the Portfolio. N/A There is a lack of information on how climate mitigation is covered in the Portfolio. N/A There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome"}]</t>
   </si>
 </sst>
 </file>
@@ -1618,7 +2041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -1661,7 +2084,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -1673,16 +2096,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I2" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1690,7 +2113,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -1702,16 +2125,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H3" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1719,7 +2142,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -1731,16 +2154,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H4" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="I4" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1748,7 +2171,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -1760,16 +2183,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H5" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="I5" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1777,7 +2200,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -1789,16 +2212,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="H6" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="I6" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1806,7 +2229,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -1818,16 +2241,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H7" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="I7" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1835,7 +2258,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -1847,16 +2270,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="G8" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="H8" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="I8" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1864,7 +2287,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -1876,16 +2299,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="H9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="I9" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -1893,7 +2316,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -1905,16 +2328,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="H10" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="I10" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -1922,7 +2345,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -1934,16 +2357,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H11" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I11" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -1951,7 +2374,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -1963,16 +2386,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G12" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H12" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="I12" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -1980,7 +2403,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -1992,16 +2415,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H13" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="I13" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2009,7 +2432,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -2021,16 +2444,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G14" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H14" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="I14" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2038,7 +2461,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C15">
         <v>100</v>
@@ -2050,16 +2473,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G15" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="I15" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2067,7 +2490,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -2079,16 +2502,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G16" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H16" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="I16" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2096,7 +2519,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -2108,16 +2531,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G17" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H17" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="I17" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2125,7 +2548,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -2137,16 +2560,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G18" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H18" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="I18" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2154,7 +2577,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -2166,16 +2589,16 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="G19" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H19" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="I19" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2183,7 +2606,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -2195,16 +2618,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H20" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I20" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2212,7 +2635,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -2224,22 +2647,22 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G21" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H21" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="J21" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K21" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2247,7 +2670,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -2259,22 +2682,22 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G22" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I22" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="J22" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K22" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2282,7 +2705,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -2294,22 +2717,22 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G23" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="H23" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I23" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="J23" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K23" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2317,7 +2740,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C24">
         <v>200</v>
@@ -2329,22 +2752,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G24" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H24" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I24" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="J24" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K24" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2352,7 +2775,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C25">
         <v>200</v>
@@ -2364,22 +2787,22 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G25" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H25" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="J25" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="K25" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2387,7 +2810,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C26">
         <v>200</v>
@@ -2399,22 +2822,22 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G26" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="H26" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="I26" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="J26" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="K26" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2422,7 +2845,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C27">
         <v>200</v>
@@ -2434,22 +2857,22 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G27" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="H27" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="I27" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="J27" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="K27" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2457,7 +2880,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C28">
         <v>200</v>
@@ -2469,22 +2892,22 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G28" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="H28" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I28" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="J28" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="K28" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2492,7 +2915,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C29">
         <v>200</v>
@@ -2504,22 +2927,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G29" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="H29" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="I29" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="J29" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="K29" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2527,7 +2950,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -2539,22 +2962,22 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G30" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="H30" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="I30" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="J30" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="K30" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2562,7 +2985,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -2574,22 +2997,22 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G31" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="H31" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="I31" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="J31" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="K31" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2597,7 +3020,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -2609,22 +3032,22 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G32" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H32" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="I32" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="J32" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K32" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2632,7 +3055,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -2644,22 +3067,22 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G33" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H33" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="J33" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K33" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2667,7 +3090,7 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -2679,22 +3102,22 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G34" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H34" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="J34" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K34" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2702,7 +3125,7 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -2714,22 +3137,22 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G35" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H35" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="J35" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K35" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2737,7 +3160,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -2749,22 +3172,22 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G36" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H36" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="J36" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K36" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2772,7 +3195,7 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -2784,22 +3207,22 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G37" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H37" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="J37" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K37" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2807,7 +3230,7 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -2819,22 +3242,22 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G38" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="H38" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="J38" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="K38" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2842,7 +3265,7 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -2854,22 +3277,22 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G39" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H39" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="I39" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J39" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K39" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2877,7 +3300,7 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -2889,22 +3312,22 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G40" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H40" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="I40" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J40" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K40" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2912,7 +3335,7 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -2924,22 +3347,22 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G41" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H41" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="I41" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J41" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K41" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2947,7 +3370,7 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C42">
         <v>100</v>
@@ -2959,22 +3382,22 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G42" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H42" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="I42" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J42" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K42" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2982,7 +3405,7 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -2994,22 +3417,22 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G43" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H43" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="I43" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J43" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K43" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -3017,7 +3440,7 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -3029,22 +3452,22 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G44" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H44" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="I44" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J44" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K44" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -3061,13 +3484,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="H45" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="K45" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3075,7 +3498,7 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -3087,22 +3510,22 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G46" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H46" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="I46" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J46" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K46" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3110,7 +3533,7 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -3122,22 +3545,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G47" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H47" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="I47" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="J47" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K47" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3145,7 +3568,7 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -3157,22 +3580,22 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="G48" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H48" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
       <c r="J48" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="K48" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3180,7 +3603,7 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C49">
         <v>200</v>
@@ -3192,22 +3615,22 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="G49" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="H49" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="J49" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="K49" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3215,7 +3638,7 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C50">
         <v>200</v>
@@ -3227,22 +3650,22 @@
         <v>1</v>
       </c>
       <c r="F50" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="G50" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H50" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="J50" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="K50" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3250,7 +3673,7 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C51">
         <v>200</v>
@@ -3262,22 +3685,22 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="G51" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H51" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="J51" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="K51" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3285,7 +3708,7 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C52">
         <v>200</v>
@@ -3297,22 +3720,162 @@
         <v>1</v>
       </c>
       <c r="F52" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G52" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="H52" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="I52" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="J52" t="s">
+        <v>158</v>
+      </c>
+      <c r="K52" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11">
+      <c r="A53" t="s">
+        <v>62</v>
+      </c>
+      <c r="B53" t="s">
+        <v>74</v>
+      </c>
+      <c r="C53">
+        <v>200</v>
+      </c>
+      <c r="D53">
+        <v>200</v>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+      <c r="F53" t="s">
+        <v>84</v>
+      </c>
+      <c r="G53" t="s">
+        <v>95</v>
+      </c>
+      <c r="H53" t="s">
+        <v>135</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J53" t="s">
+        <v>159</v>
+      </c>
+      <c r="K53" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11">
+      <c r="A54" t="s">
+        <v>63</v>
+      </c>
+      <c r="B54" t="s">
+        <v>75</v>
+      </c>
+      <c r="C54">
+        <v>200</v>
+      </c>
+      <c r="D54">
+        <v>200</v>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+      <c r="F54" t="s">
+        <v>84</v>
+      </c>
+      <c r="G54" t="s">
+        <v>96</v>
+      </c>
+      <c r="H54" t="s">
         <v>136</v>
       </c>
-      <c r="J52" t="s">
-        <v>143</v>
-      </c>
-      <c r="K52" t="s">
-        <v>155</v>
+      <c r="I54" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J54" t="s">
+        <v>160</v>
+      </c>
+      <c r="K54" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11">
+      <c r="A55" t="s">
+        <v>64</v>
+      </c>
+      <c r="B55" t="s">
+        <v>75</v>
+      </c>
+      <c r="C55">
+        <v>200</v>
+      </c>
+      <c r="D55">
+        <v>200</v>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+      <c r="F55" t="s">
+        <v>84</v>
+      </c>
+      <c r="G55" t="s">
+        <v>96</v>
+      </c>
+      <c r="H55" t="s">
+        <v>137</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J55" t="s">
+        <v>160</v>
+      </c>
+      <c r="K55" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11">
+      <c r="A56" t="s">
+        <v>65</v>
+      </c>
+      <c r="B56" t="s">
+        <v>76</v>
+      </c>
+      <c r="C56">
+        <v>200</v>
+      </c>
+      <c r="D56">
+        <v>200</v>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+      <c r="F56" t="s">
+        <v>84</v>
+      </c>
+      <c r="G56" t="s">
+        <v>93</v>
+      </c>
+      <c r="H56" t="s">
+        <v>138</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="J56" t="s">
+        <v>157</v>
+      </c>
+      <c r="K56" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -3328,6 +3891,10 @@
     <hyperlink ref="I50" r:id="rId9"/>
     <hyperlink ref="I51" r:id="rId10"/>
     <hyperlink ref="I52" r:id="rId11"/>
+    <hyperlink ref="I53" r:id="rId12"/>
+    <hyperlink ref="I54" r:id="rId13"/>
+    <hyperlink ref="I55" r:id="rId14"/>
+    <hyperlink ref="I56" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implementing table indexing, cache/hash optimization, TF-IDF and context adjustments, and adding fallback in answers
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="203">
   <si>
     <t>timestamp</t>
   </si>
@@ -214,6 +214,21 @@
     <t>2025-09-24T10:32:33.484279</t>
   </si>
   <si>
+    <t>2025-09-24T14:07:12.455528</t>
+  </si>
+  <si>
+    <t>2025-09-24T14:07:44.638768</t>
+  </si>
+  <si>
+    <t>2025-09-24T14:09:48.670116</t>
+  </si>
+  <si>
+    <t>2025-09-24T15:17:26.408043</t>
+  </si>
+  <si>
+    <t>2025-09-25T00:45:44.397869</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -245,6 +260,12 @@
   </si>
   <si>
     <t xml:space="preserve">Who coordinates funders’ M&amp;E requirements across the CGIAR Portfolio and how is duplication avoided? </t>
+  </si>
+  <si>
+    <t>¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?</t>
+  </si>
+  <si>
+    <t>Who holds fiduciary responsibility over Window 1 and Window 2 Funds?</t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -276,6 +297,12 @@
     <t>You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.</t>
   </si>
   <si>
+    <t>deeper research</t>
+  </si>
+  <si>
+    <t>You are a RAG assistant for deeper research. Use all the chunks that you receive. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.</t>
+  </si>
+  <si>
     <t>pptx:Information Session on 2025 Technical Reporting.pptx:s9:0.307, docx:Engagement Plan 2025 Technical Reporting.docx:p2:0.304, pptx:Information Session on 2025 Technical Reporting.pptx:s2:0.299, docx:Guidance on reporting outputs or outcomes.docx:p22:0.263, docx:Engagement Plan 2025 Technical Reporting.docx:p59:0.244, pdf:CGIAR_ImpactReport_2022-24.pdf:p1:0.239, docx:Engagement Plan 2025 Technical Reporting.docx:p31:0.208, pptx:Engagement Plan 2025 Technical Reporting.pptx:s1:0.202, docx:CGSpace.docx:p3:0.201, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5:0.200, docx:General information on Technical Reporting .docx:p1:0.196, pptx:Information Session on 2025 Technical Reporting.pptx:s15:0.184, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1:0.176, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23:0.166, docx:Guidance on reporting outputs or outcomes.docx:p21:0.163, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4:0.160, docx:Guidance on reporting outputs or outcomes.docx:p30:0.160, docx:2025 Technical Reporting Information (Session 2).docx:p5:0.152, docx:2025 Technical Reporting Information (Session 2).docx:p32:0.138, docx:Guidance on reporting outputs or outcomes.docx:p24:0.138, pdf:Type3_2024Report.pdf:p1:0.136, pptx:Information Session on 2025 Technical Reporting.pptx:s13:0.134, docx:Using the PRMS Reporting Tool.docx:p12:0.133, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7:0.133, docx:Guidance on reporting outputs or outcomes.docx:p31:0.133, docx:General information on Technical Reporting .docx:p4:0.131, pptx:Information Session on 2025 Technical Reporting.pptx:s7:0.128, pdf:Type3_2024Report.pdf:p5:0.124, pptx:Information Session on 2025 Technical Reporting.pptx:s5:0.124, pdf:Portfolio Narrative_2024.pdf:p1:0.124, pdf:Portfolio Narrative_2024.pdf:p5:0.124, pptx:Information Session on 2025 Technical Reporting.pptx:s3:0.123, docx:Innovation use.docx:p7:0.121, pptx:Information Session on 2025 Technical Reporting.pptx:s6:0.121, docx:Innovation development.docx:p31:0.120, docx:2025 Technical Reporting Information (Session 1).docx:p26:0.119, pptx:Information Session on 2025 Technical Reporting.pptx:s10:0.118, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16:0.118, docx:2025 Technical Reporting Information (Session 1).docx:p7:0.117, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6:0.116, pdf:Portfolio Narrative_2024.pdf:p6:0.110, docx:2025 Technical Reporting Information (Session 2).docx:p1:0.110, docx:2025 Technical Reporting Information (Session 1).docx:p1:0.110, docx:Guidance on reporting outputs or outcomes.docx:p26:0.109, docx:Innovation development.docx:p13:0.108, docx:Submitting evidence.docx:p3:0.108, docx:Guidance on complementary innnov.docx:p38:0.107, docx:Engagement Plan 2025 Technical Reporting.docx:p61:0.106, docx:Engagement Plan 2025 Technical Reporting.docx:p27:0.102, pptx:Information Session on 2025 Technical Reporting.pptx:s1:0.099, pdf:Type3_2024Report.pdf:p11:0.099, pdf:Type3_2024Report.pdf:p4:0.099, docx:General information on Technical Reporting .docx:p5:0.098, docx:Engagement Plan 2025 Technical Reporting.docx:p39:0.097, docx:Guidance on complementary innnov.docx:p10:0.097, pptx:Information Session on 2025 Technical Reporting.pptx:s4:0.094, pptx:Information Session on 2025 Technical Reporting.pptx:s11:0.092, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2:0.092, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18:0.090, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22:0.089, docx:2025 Technical Reporting Information (Session 2).docx:p26:0.089, docx:Using the PRMS Reporting Tool.docx:p1:0.089, docx:2025 Technical Reporting MELIA glossary.docx:p6:0.089, docx:Engagement Plan 2025 Technical Reporting.docx:p106:0.088, pdf:Type3_2024Report.pdf:p6:0.087, docx:Engagement Plan 2025 Technical Reporting.docx:p42:0.086, docx:General reporting guidance.docx:p1:0.085, docx:General reporting guidance.docx:p5:0.084, docx:2025 Technical Reporting Information (Session 1).docx:p30:0.084, docx:Engagement Plan 2025 Technical Reporting.docx:p17:0.083, docx:Guidance on reporting outputs or outcomes.docx:p2:0.082, docx:2025 Technical Reporting Information (Session 2).docx:p11:0.081, docx:Engagement Plan 2025 Technical Reporting.docx:p69:0.080, pdf:CGIAR_ImpactReport_2022-24.pdf:p2:0.080, docx:Engagement Plan 2025 Technical Reporting.docx:p25:0.079, docx:Reporting the geographic location of results.docx:p1:0.078, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3:0.074, docx:Engagement Plan 2025 Technical Reporting.docx:p45:0.072, docx:Innovation use.docx:p22:0.072, pdf:Portfolio Narrative_2024.pdf:p37:0.071, docx:General reporting guidance.docx:p3:0.071, docx:2025 Technical Reporting Information (Session 2).docx:p41:0.071, docx:Engagement Plan 2025 Technical Reporting.docx:p8:0.071, docx:Engagement Plan 2025 Technical Reporting.docx:p10:0.070, docx:2025 Technical Reporting Information (Session 1).docx:p41:0.068, docx:Guidance on ensuring quality over quantity.docx:p3:0.066, docx:Engagement Plan 2025 Technical Reporting.docx:p55:0.066, pdf:Type3_2024Report.pdf:p3:0.066, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9:0.066, docx:Innovation development.docx:p40:0.066, docx:Guidance on ensuring quality over quantity.docx:p5:0.066, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15:0.065, docx:Knowledge products.docx:p11:0.065, pdf:Portfolio Narrative_2024.pdf:p72:0.065, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25:0.065, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p2:0.064, docx:2025 Technical Reporting Information (Session 2).docx:p7:0.064, docx:2025 Technical Reporting Information (Session 1).docx:p15:0.064, docx:2025 Technical Reporting Information (Session 2).docx:p14:0.063, docx:2025 Technical Reporting Information (Session 1).docx:p33:0.063</t>
   </si>
   <si>
@@ -310,6 +337,15 @@
   </si>
   <si>
     <t>pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.321, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.276, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.272, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.256, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.252, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.231, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.216, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.198, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.196, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.186, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.184, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3:0.166, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.163, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.157, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.146, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.138, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.137, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1:0.137, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3:0.130, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.124, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2:0.121, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.120, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3:0.118, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4:0.118, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2:0.116, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2:0.112, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2:0.112, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p32pt1:0.106, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt2:0.106, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4:0.104, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2:0.104, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.103, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.103, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2:0.102, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2:0.101, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4:0.100, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1:0.097, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.096, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.096, pdf:CGI21-507032-PORB-Climate Action.pdf:p21pt3:0.094, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt3:0.092, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt3:0.091, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1:0.088, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt4:0.087, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1:0.087, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.083, pdf:Portfolio Narrative_2024.pdf:p47pt3:0.082, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt2:0.082, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4:0.081, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt4:0.081, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2:0.079, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt2:0.078, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt4:0.078, pdf:Portfolio Narrative_2024.pdf:p47pt4:0.075, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p7pt4:0.075, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt1:0.075, pdf:CGIAR_ImpactReport_2022-24.pdf:p56pt2:0.073, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3:0.072, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.072, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p23pt1:0.072, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p53pt4:0.070, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt2:0.070, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3:0.068, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt1:0.067, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p29pt1:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p54pt3:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt3:0.065, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt2:0.064, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt3:0.063, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt2:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3:0.062, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt4:0.062, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt3:0.061, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt1:0.060, docx:Standard Provisions 2026.docx:u22-25:0.060, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt1:0.059, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p10pt4:0.059, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt3:0.058, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt4:0.058, docx:Standard Provisions 2026.docx:u115-118:0.057, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p28pt3:0.057, pdf:Climate Action_Inception Report 30-06-2025.pdf:p11pt3:0.057, pdf:Portfolio Narrative_2024.pdf:p47pt2:0.056, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p25pt4:0.056, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt4:0.056, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt2:0.056, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt1:0.054, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.054, docx:2025 Technical Reporting Information (Session 2).docx:u52-56:0.054, docx:Standard Provisions 2026.docx:u127-130:0.053, docx:2025 Technical Reporting Information (Session 1).docx:u43-45:0.051, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt4:0.050, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.049, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt1:0.049, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p30pt1:0.048, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt4:0.048, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt4:0.048, docx:Standard Provisions 2026.docx:u100-103:0.048, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt2:0.047, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt1:0.047, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt1:0.045, pdf:CGIAR_ImpactReport_2022-24.pdf:p34pt1:0.045, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt2:0.045, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt4:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p43pt4:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p44pt4:0.044, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4:0.044, pdf:Type3_2024Report.pdf:p2pt4:0.043, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt3:0.043, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p40pt4:0.042, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt2:0.042, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p18pt2:0.042, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt2:0.041, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p22pt2:0.041, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt2:0.041, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt3:0.041, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt1:0.041, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt1:0.040, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p52pt3:0.040, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt1:0.040, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt3:0.040, pdf:Climate Action_Inception Report 30-06-2025.pdf:p8pt4:0.040, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt2:0.040, pdf:Portfolio Narrative_2024.pdf:p83pt1:0.040, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt2:0.040, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt1:0.040, pdf:Type3_2024Report.pdf:p8pt4:0.039, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p9pt4:0.038, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt2:0.038, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3:0.038, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.038, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt2:0.038, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt3:0.037, docx:Standard Provisions 2026.docx:u103-106:0.037, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p13pt4:0.037, pdf:Portfolio Narrative_2024.pdf:p28pt4:0.037, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt4:0.036, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt2:0.036, pdf:CGIAR_ImpactReport_2022-24.pdf:p45pt4:0.035, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p22pt1:0.035, pdf:Portfolio Narrative_2024.pdf:p19pt1:0.035, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p26pt1:0.035, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p29pt4:0.034, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt2:0.034, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt1:0.034, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p30pt3:0.033, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p51pt1:0.033, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt2:0.033, docx:Standard Provisions 2026.docx:u85-88:0.033, docx:Standard Provisions 2026.docx:u172-175:0.033, docx:Standard Provisions 2026.docx:u124-127:0.032, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p20pt2:0.032, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt3:0.032, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt3:0.031, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p13pt1:0.031, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt3:0.030, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt4:0.030, pdf:CGIAR_ImpactReport_2022-24.pdf:p23pt4:0.030, pdf:Type3_2024Report.pdf:p10pt4:0.030, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt3:0.030, docx:Standard Provisions 2026.docx:u82-85:0.029, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt3:0.029, docx:Standard Provisions 2026.docx:u97-100:0.029, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p22pt2:0.028, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p39pt2:0.028, pdf:CGIAR_ImpactReport_2022-24.pdf:p41pt4:0.028, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt2:0.028, docx:Standard Provisions 2026.docx:u52-55:0.027, pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt2:0.027, pdf:Portfolio Narrative_2024.pdf:p82pt4:0.026, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p6pt4:0.026, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt3:0.026, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt3:0.026, docx:Standard Provisions 2026.docx:u112-115:0.026, pdf:CGI21-507032-PORB-Climate Action.pdf:p24pt2:0.026, docx:Standard Provisions 2026.docx:u106-109:0.025, pdf:CGI21-507032-PORB-Climate Action.pdf:p24pt3:0.025, pdf:CGIAR_ImpactReport_2022-24.pdf:p40pt1:0.025, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.024, docx:Standard Provisions 2026.docx:u7-10:0.024, docx:Standard Provisions 2026.docx:u130-133:0.024, docx:Standard Provisions 2026.docx:u4-7:0.024, pdf:Type3_2024Report.pdf:p7pt2:0.024, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.024, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p22pt2:0.024, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.024, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt4:0.023, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3:0.023, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt3:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p22pt1:0.023, docx:Standard Provisions 2026.docx:u34-37:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p14pt3:0.023, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p22pt2:0.023, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.023, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p18pt1:0.022, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt4:0.022, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt4:0.022, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt2:0.022, pdf:Quick style guide Feb 2024 (1).pdf:p5pt1:0.022, pdf:Climate Action_Inception Report 30-06-2025.pdf:p28pt3:0.022</t>
+  </si>
+  <si>
+    <t>pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.450, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.393, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.359, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.347, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.308, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.272, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.271, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.252, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.249, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.249, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.249, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.223, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2:0.218, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.217, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.209, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.186, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.186, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3:0.176, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3:0.175, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.172, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1:0.169, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.166, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2:0.147, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.146, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3:0.145, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2:0.141, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.139, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1:0.133, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1:0.131, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1:0.131, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.127, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4:0.124, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4:0.123, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2:0.123, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2:0.120, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2:0.119, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2:0.119, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.114, docx:2025 Technical Reporting Information (Session 2).docx:u52-56:0.114, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.113, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p32pt1:0.112, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt2:0.112, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4:0.110, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3:0.110, docx:2025 Technical Reporting Information (Session 1).docx:u43-45:0.109, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2:0.108, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4:0.105, pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3:0.103, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.101, pdf:CGI21-507032-PORB-Climate Action.pdf:p21pt3:0.099, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt3:0.097, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt3:0.096, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p53pt4:0.095, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt3:0.095, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt4:0.092, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.091, pdf:Portfolio Narrative_2024.pdf:p47pt3:0.087, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt2:0.086, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt4:0.086, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p16pt2:0.084, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt2:0.083, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p42pt4:0.082, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.079, pdf:Portfolio Narrative_2024.pdf:p47pt4:0.079, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p7pt4:0.079, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p28pt1:0.079, pdf:CGIAR_ImpactReport_2022-24.pdf:p56pt2:0.077, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p23pt1:0.076, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt1:0.074, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt2:0.074, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt1:0.071, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p29pt1:0.070, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p54pt3:0.070, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p48pt3:0.069, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt2:0.067, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt3:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt2:0.066, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt4:0.065, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt1:0.064, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p21pt1:0.062, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt3:0.062, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt4:0.062, pdf:Climate Action_Inception Report 30-06-2025.pdf:p11pt3:0.060, pdf:Portfolio Narrative_2024.pdf:p47pt2:0.059, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p25pt4:0.059, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt4:0.059, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt1:0.057, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p23pt2:0.057, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p28pt4:0.053, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt4:0.051, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt4:0.051, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt1:0.049, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt1:0.048, pdf:CGIAR_ImpactReport_2022-24.pdf:p34pt1:0.047, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt2:0.047, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt4:0.047, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p43pt4:0.046, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p44pt4:0.046, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p41pt3:0.045, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt2:0.044, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p18pt2:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p22pt2:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p38pt2:0.043, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p27pt1:0.043, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt3:0.042, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt2:0.042, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt1:0.042, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p9pt4:0.040, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt2:0.040, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt3:0.039, pdf:Portfolio Narrative_2024.pdf:p28pt4:0.039, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt4:0.038, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt2:0.038, pdf:CGIAR_ImpactReport_2022-24.pdf:p45pt4:0.037, pdf:Portfolio Narrative_2024.pdf:p19pt1:0.037, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p26pt1:0.036, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p39pt2:0.036, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p40pt4:0.036, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p30pt3:0.035, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p51pt1:0.035, pdf:CGIAR_ImpactReport_2022-24.pdf:p61pt2:0.035, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p20pt2:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt3:0.033, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p47pt3:0.033, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt3:0.032, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt4:0.032, pdf:CGIAR_ImpactReport_2022-24.pdf:p23pt4:0.032, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p49pt3:0.031, pdf:CGIAR_ImpactReport_2022-24.pdf:p53pt3:0.031, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p22pt2:0.030, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p39pt2:0.030, pdf:CGIAR_ImpactReport_2022-24.pdf:p41pt4:0.030, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt2:0.030, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt3:0.027, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p32pt3:0.027, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p32pt2:0.027, pdf:CGIAR_ImpactReport_2022-24.pdf:p40pt1:0.026, pdf:Type3_2024Report.pdf:p7pt2:0.025, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt4:0.025, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p37pt3:0.024, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p17pt4:0.024, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p47pt2:0.023, pdf:Quick style guide Feb 2024 (1).pdf:p5pt1:0.023, pdf:CGIAR_ImpactReport_2022-24.pdf:p58pt1:0.023, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p22pt4:0.022, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p29pt1:0.022, pdf:CGIAR_ImpactReport_2022-24.pdf:p25pt1:0.022, pdf:CGIAR_ImpactReport_2022-24.pdf:p10pt3:0.020</t>
+  </si>
+  <si>
+    <t>docx:Standard Provisions 2026.docx:u19-22:0.692, docx:Standard Provisions 2026.docx:u16-19:0.656, docx:Standard Provisions 2026.docx:u181-184:0.470, docx:Standard Provisions 2026.docx:u28-31:0.467, docx:Standard Provisions 2026.docx:u178-181:0.421, docx:Standard Provisions 2026.docx:u31-34:0.413, docx:Standard Provisions 2026.docx:u13-16:0.406, docx:Standard Provisions 2026.docx:u22-25:0.379, docx:Standard Provisions 2026.docx:u34-37:0.332, docx:Standard Provisions 2026.docx:u172-175:0.314, docx:Standard Provisions 2026.docx:u25-28:0.307, docx:Standard Provisions 2026.docx:u55-58:0.277, docx:Standard Provisions 2026.docx:u46-49:0.240, docx:Standard Provisions 2026.docx:u184-189:0.235, docx:Standard Provisions 2026.docx:u175-178:0.234, docx:Standard Provisions 2026.docx:u4-7:0.231, docx:Standard Provisions 2026.docx:u106-109:0.212, docx:Standard Provisions 2026.docx:u58-61:0.209, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4:0.187, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2:0.184, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt2:0.183, docx:Standard Provisions 2026.docx:u10-13:0.179, docx:Standard Provisions 2026.docx:u67-70:0.169, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p3pt1:0.168, docx:Standard Provisions 2026.docx:u163-166:0.163, docx:Standard Provisions 2026.docx:u157-160:0.162, docx:Standard Provisions 2026.docx:u64-67:0.160, docx:Standard Provisions 2026.docx:u73-76:0.159, docx:Standard Provisions 2026.docx:u37-40:0.159, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt1:0.152, docx:Standard Provisions 2026.docx:u121-124:0.147, docx:Standard Provisions 2026.docx:u52-55:0.147, docx:Standard Provisions 2026.docx:u70-73:0.146, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.142, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt2:0.140, docx:Standard Provisions 2026.docx:u133-136:0.140, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p3pt2:0.136, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt4:0.135, docx:Standard Provisions 2026.docx:u103-106:0.133, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.128, pdf:Climate Action_Inception Report 30-06-2025.pdf:p16pt3:0.127, docx:Standard Provisions 2026.docx:u43-46:0.124, docx:Standard Provisions 2026.docx:u61-64:0.123, docx:Guidance on reporting outputs or outcomes.docx:u10-13:0.123, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p4pt4:0.122, docx:Standard Provisions 2026.docx:u109-112:0.121, docx:Standard Provisions 2026.docx:u166-169:0.120, docx:Standard Provisions 2026.docx:u130-133:0.114, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p2pt3:0.113, docx:Standard Provisions 2026.docx:u160-163:0.113, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt1:0.111, docx:Standard Provisions 2026.docx:u82-85:0.105, docx:Standard Provisions 2026.docx:u97-100:0.105, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.100, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt4:0.099, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p16pt1:0.098, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt3:0.098, docx:Standard Provisions 2026.docx:u145-148:0.097, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p2pt4:0.096, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt3:0.094, docx:Standard Provisions 2026.docx:u94-97:0.093, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p20pt1:0.093, docx:Standard Provisions 2026.docx:u112-115:0.092, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt2:0.090, docx:2025 Technical Reporting Information (Session 1).docx:u40-43:0.089, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt3:0.089, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt4:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.087, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt1:0.087, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.086, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt2:0.085, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt3:0.085, docx:Standard Provisions 2026.docx:u1-4:0.084, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p16pt1:0.084, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt2:0.084, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p19pt1:0.083, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt2:0.083, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p2pt2:0.083, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt2:0.082, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt2:0.082, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt2:0.082, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt2:0.082, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt2:0.082, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1:0.082, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p2pt2:0.081, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p2pt2:0.081, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p2pt2:0.081, docx:Standard Provisions 2026.docx:u76-79:0.078, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p22pt4:0.077, pdf:Portfolio Narrative_2024.pdf:p37pt4:0.076, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p6pt3:0.075, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt1:0.075, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p2pt2:0.074, pdf:Type3_2024Report.pdf:p5pt1:0.074, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p3pt4:0.073, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt2:0.072, pdf:Genebanks_Inception Report 30-06-2025.pdf:p8pt2:0.072, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p3pt3:0.071, docx:Standard Provisions 2026.docx:u88-91:0.071, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p23pt1:0.070, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4:0.070, pdf:Genebanks_Inception Report 30-06-2025.pdf:p3pt4:0.067, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p21pt1:0.067, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p2pt1:0.067, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p23pt3:0.066, pdf:Genebanks_Inception Report 30-06-2025.pdf:p8pt3:0.066, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt2:0.066, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p21pt1:0.060, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p14pt2:0.060, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4:0.060, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p23pt2:0.060, docx:Standard Provisions 2026.docx:u7-10:0.059, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p26pt1:0.059, docx:Standard Provisions 2026.docx:u85-88:0.059, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt2:0.059, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p4pt3:0.058, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt4:0.057, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt1:0.057, pdf:Genebanks_Inception Report 30-06-2025.pdf:p29pt1:0.056, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p29pt4:0.056, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.055, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p24pt2:0.054, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p4pt2:0.054, docx:Standard Provisions 2026.docx:u148-151:0.053, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt1:0.053, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p3pt3:0.052, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p9pt2:0.051, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt1:0.051, docx:2025 Technical Reporting Information (Session 2).docx:u28-31:0.051, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p6pt4:0.051, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt1:0.050, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt1:0.050, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt2:0.049, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p32pt4:0.049, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p6pt4:0.049, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p3pt2:0.049, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p15pt2:0.048, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p14pt3:0.048, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p4pt2:0.047, docx:Engagement Plan 2025 Technical Reporting.docx:u55-58:0.046, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p25pt2:0.046, pdf:Type3_2024Report.pdf:p2pt4:0.046, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt3:0.046, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p16pt4:0.046, pdf:Genebanks_Inception Report 30-06-2025.pdf:p29pt2:0.045, docx:Standard Provisions 2026.docx:u169-172:0.044, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p17pt2:0.044, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p16pt3:0.044, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p17pt3:0.044, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p10pt4:0.043, docx:Guidance on reporting outputs or outcomes.docx:u7-10:0.043, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p13pt4:0.043, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p8pt1:0.043, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p5pt2:0.043, docx:Standard Provisions 2026.docx:u100-103:0.043, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p22pt1:0.043, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p6pt2:0.043, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt2:0.042, docx:Standard Provisions 2026.docx:u151-154:0.042, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt2:0.041, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p10pt4:0.041, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p11pt1:0.041, pdf:Genebanks_Inception Report 30-06-2025.pdf:p39pt3:0.040, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p14pt4:0.040, pdf:Portfolio Narrative_2024.pdf:p14pt2:0.040, pdf:Genebanks_Inception Report 30-06-2025.pdf:p17pt4:0.040, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p25pt4:0.040, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p25pt3:0.040, pdf:Portfolio Narrative_2024.pdf:p7pt3:0.040, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt4:0.039, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.039, pdf:Portfolio Narrative_2024.pdf:p20pt1:0.039, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p22pt1:0.039, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p17pt4:0.039, pdf:Genebanks_Inception Report 30-06-2025.pdf:p9pt3:0.039, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p11pt2:0.038, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt4:0.038, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt2:0.038, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p33pt4:0.038, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p14pt4:0.038, docx:Guidance on reporting outputs or outcomes.docx:u4-7:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p21pt3:0.037, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.037, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt2:0.037, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p14pt3:0.037, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p36pt4:0.037, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.037, pdf:Genebanks_Inception Report 30-06-2025.pdf:p37pt2:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p21pt2:0.037, pdf:CGIAR_ImpactReport_2022-24.pdf:p10pt2:0.036, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p6pt1:0.036, pdf:Portfolio Narrative_2024.pdf:p41pt1:0.036, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p27pt3:0.036, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p15pt2:0.035, pdf:CGIAR_ImpactReport_2022-24.pdf:p67pt3:0.035, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p11pt3:0.035, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p15pt2:0.035, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt1:0.035, pdf:Genebanks_Inception Report 30-06-2025.pdf:p18pt1:0.035, pdf:Genebanks_Inception Report 30-06-2025.pdf:p36pt4:0.034</t>
+  </si>
+  <si>
+    <t>docx:Standard Provisions 2026.docx:u19-22:0.155, docx:Standard Provisions 2026.docx:u16-19:0.145, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2:0.090, docx:Standard Provisions 2026.docx:u31-34:0.085, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.078, docx:Standard Provisions 2026.docx:u28-31:0.078, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.077, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.075, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.074, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p52pt1:0.069, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.067, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.067, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.066, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.064, docx:Standard Provisions 2026.docx:u70-73:0.063, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p37pt3:0.062, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.061, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.060, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.059, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.057, docx:Standard Provisions 2026.docx:u163-166:0.057, docx:Standard Provisions 2026.docx:u67-70:0.056, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt3:0.055, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt2:0.053, pdf:Type3_2024Report.pdf:p6pt3:0.052, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.052, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt2:0.051, pdf:Type3_2024Report.pdf:p6pt4:0.051, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p10pt2:0.051, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt3:0.051, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.049, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.048, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt2:0.048, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p35pt2:0.047, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p17pt2:0.047, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p31pt2:0.047, pdf:Genebanks_Inception Report 30-06-2025.pdf:p38pt1:0.046, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p6pt1:0.045, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4:0.045, pdf:Type3_2024Report.pdf:p3pt2:0.045, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt2:0.044, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt2:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.044, pdf:Climate Action_Inception Report 30-06-2025.pdf:p22pt2:0.043, pdf:Type3_2024Report.pdf:p6pt2:0.043, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p19pt4:0.043, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2:0.043, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.043, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p1pt2:0.042, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.042, pdf:Type3_2024Report.pdf:p5pt1:0.042, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt3:0.041, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p26pt3:0.041, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.041, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.041, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.041, docx:User Roles and Rules for the PRMS Reporting.docx:u4-7:0.040, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p30pt4:0.040, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4:0.039, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p20pt4:0.039, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p22pt3:0.039, pdf:Portfolio Narrative_2024.pdf:p29pt3:0.039, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p10pt2:0.039, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p51pt1:0.039, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt2:0.039, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.039, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt3:0.038, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p4pt4:0.038, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.038, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt2:0.038, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt2:0.038, pdf:Portfolio Narrative_2024.pdf:p82pt2:0.038, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.038, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt3:0.038, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt3:0.038, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt2:0.038, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p24pt1:0.037, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p6pt2:0.037, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.037, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p16pt4:0.037, pdf:Portfolio Narrative_2024.pdf:p89pt4:0.037, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.037, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt4:0.037, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.037, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt1:0.037, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt2:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt2:0.036, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p4pt1:0.036, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p31pt4:0.036, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.036, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt2:0.036, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p22pt3:0.036, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p5pt3:0.036, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p8pt2:0.036, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p26pt4:0.035, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p31pt1:0.035, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.035, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt2:0.035, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p11pt4:0.035, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p12pt2:0.035, docx:Standard Provisions 2026.docx:u58-61:0.035, pdf:Portfolio Narrative_2024.pdf:p29pt4:0.035, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt3:0.035, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt4:0.034, pdf:CGIAR_ImpactReport_2022-24.pdf:p28pt1:0.034, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p26pt4:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt4:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p26pt3:0.034, pdf:Genebanks_Inception Report 30-06-2025.pdf:p15pt2:0.034, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt1:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p11pt2:0.034, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt4:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt1:0.034, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p7pt4:0.034, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p22pt4:0.034, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p1pt2:0.034, pdf:Climate Action_Inception Report 30-06-2025.pdf:p22pt3:0.034, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt3:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p13pt2:0.034, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p36pt3:0.034, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p15pt4:0.034, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p17pt3:0.034, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p9pt4:0.034, pdf:Climate Action_Inception Report 30-06-2025.pdf:p17pt3:0.034, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p29pt1:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p9pt3:0.034, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p3pt2:0.034, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt2:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p10pt4:0.033, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt1:0.033, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p13pt2:0.033, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt1:0.033, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p4pt4:0.033, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.033, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p11pt2:0.033, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p12pt3:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.033, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.033, pdf:Portfolio Narrative_2024.pdf:p17pt1:0.033, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt1:0.033, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p35pt1:0.033, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.033, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p33pt4:0.033, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p24pt4:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p3pt1:0.033, pdf:Portfolio Narrative_2024.pdf:p82pt3:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p13pt3:0.033, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p10pt2:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt4:0.033, pdf:Type3_2024Report.pdf:p7pt1:0.032, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p18pt1:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt2:0.032, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p26pt1:0.032, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p56pt3:0.032, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt1:0.032, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p30pt4:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p32pt3:0.032, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p10pt2:0.032, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt1:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p9pt2:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt3:0.032, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt3:0.032, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt3:0.032, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p18pt4:0.032, pdf:Type3_2024Report.pdf:p8pt3:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt3:0.032, pdf:Portfolio Narrative_2024.pdf:p53pt4:0.032, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt3:0.032, pdf:Genebanks_Inception Report 30-06-2025.pdf:p17pt4:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt2:0.032, docx:Standard Provisions 2026.docx:u73-76:0.032, pdf:Portfolio Narrative_2024.pdf:p38pt4:0.032, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p53pt3:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p8pt1:0.032, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt2:0.032, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt1:0.031, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p22pt3:0.031, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt1:0.031, pdf:Type3_2024Report.pdf:p7pt4:0.031, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt3:0.031, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt2:0.031, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p7pt2:0.031, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p4pt4:0.031, pdf:Portfolio Narrative_2024.pdf:p47pt4:0.031, docx:Standard Provisions 2026.docx:u4-7:0.031, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p12pt3:0.031, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt4:0.031, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p31pt3:0.031, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt4:0.031, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt4:0.031, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p14pt4:0.031, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p16pt2:0.031, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p13pt4:0.031, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt1:0.031, pdf:Climate Action_Inception Report 30-06-2025.pdf:p19pt3:0.031</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -647,6 +683,57 @@
 Standard Provisions 2026.docx — section 'Monitoring and Evaluations' paragraph 115 — docx:Standard Provisions 2026.docx:u103-106</t>
   </si>
   <si>
+    <t>I cannot find information in the provided chunks to answer this. The documents do not specify who holds fiduciary responsibility over the funds of Ventanas 1 and 2 or what guarantees are required. For detailed information on fiduciary responsibilities and guarantees related to these funds, further context or specific documents may be necessary. 
+Sources:
+File — Location — Cited IDs
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1
+CGI21_508012_PORB_Genebanks.pdf — page 10 part 2 — pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2</t>
+  </si>
+  <si>
+    <t>La responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 recae en el CGIAR (Grupo Consultivo sobre Investigación Agrícola Internacional). Este organismo debe garantizar que los fondos se utilicen de manera eficiente y efectiva para la conservación y el uso sostenible de los recursos genéticos de cultivos, así como para el desarrollo de soluciones innovadoras que aborden los desafíos de la seguridad alimentaria y la sostenibilidad agrícola.
+En particular, el CGIAR tiene la obligación de asegurar que los proyectos financiados bajo estas ventanas contribuyan a los resultados deseados en términos de conservación de la biodiversidad agrícola, mejora de la calidad de la dieta y adaptación al cambio climático, entre otros objetivos estratégicos. Esto implica una gestión cuidadosa de los recursos, la rendición de cuentas y la transparencia en el uso de los fondos asignados.</t>
+  </si>
+  <si>
+    <t>I cannot find information in the provided chunks to answer this. 
+Sources:
+File — Location — Cited IDs
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 9 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1
+CGI21_508012_PORB_Genebanks.pdf — page 10 part 2 — pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2
+CGIAR_PORB_Scaling_4Impact.pdf — page 23 part 3 — pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3
+CGIAR_PORB_Breeding_Tomorrow.pdf — page 45 part 3 — pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3
+2025 Technical Reporting Information (Session 1).docx — paragraph 1 to paragraph 4 — docx:2025 Technical Reporting Information (Session 1).docx:u1-4
+Genebanks_Inception Report 30-06-2025.pdf — page 22 part 4 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 22 part 1 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1
+docx:2025 Technical Reporting Information (Session 2).docx — paragraph 1 to paragraph 4 — docx:2025 Technical Reporting Information (Session 2).docx:u1-4
+CGI21-507031-PORB-Food Frontiers and Security.pdf — page 22 part 3 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3
+CGI21-507032-PORB-Climate Action.pdf — page 11 part 2 — pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2
+CGI21_508012_PORB_Genebanks.pdf — page 11 part 2 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2
+CGIAR_PORB_Breeding_Tomorrow.pdf — page 42 part 3 — pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3
+CGIAR_PORB_Breeding_Tomorrow.pdf — page 46 part 3 — pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3
+CGIAR_PORB_Scaling_4Impact.pdf — page 22 part 4 — pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4
+Climate Action_Inception Report 30-06-2025.pdf — page 4 part 3 — pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3</t>
+  </si>
+  <si>
+    <t>The fiduciary responsibility over Window 1 and Window 2 Funds is held by the System Organization toward the Funders, while each Center has fiduciary responsibility toward the System Organization for the funds it receives. This means that the System Organization must ensure that the funds are used for their intended purposes and in accordance with relevant agreements, while Centers must manage the funds they receive in a similar manner. Both entities are required to monitor, evaluate, and report on the use of these funds to ensure compliance with established standards. 
+Sources:
+File — Location — Cited IDs
+docx:Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — u19-22
+docx:Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — u16-19</t>
+  </si>
+  <si>
+    <t>The fiduciary responsibility for the use of Window 1 and Window 2 Funds lies with the System Organization towards the Funders, while each Center holds fiduciary responsibility towards the System Organization for the funds it receives. They must ensure that these funds are used exclusively for their intended purposes and administered in accordance with the CGIAR System Charter, the CGIAR System Framework, and applicable Fund Use Agreements. Additionally, they are required to monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by these resources. 
+Sources:
+File — Location — Cited IDs
+Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22
+Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -684,6 +771,12 @@
   </si>
   <si>
     <t>https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543 — page 9 part 2 — pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1 — page 22 part 1 — pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1, CGI21_508012_PORB_Genebanks.pdf — page 11 part 1 — pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1</t>
+  </si>
+  <si>
+    <t>Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22, Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19, Standard Provisions 2026.docx — section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198 to section 'Misused Fund' paragraph 202 — docx:Standard Provisions 2026.docx:u181-184</t>
+  </si>
+  <si>
+    <t>Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22, Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19, https://cgspace.cgiar.org/items/a88f8775-4ba9-41b6-9525-0d698d83cfb4 — page 72 part 2 — pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -1628,6 +1721,381 @@
 Research Organization Centre de coopération internationale en recherche agronomique pour le développement Wageningen University and Research Centre Cornell University Zambia Agriculture Research Institute Ethiopian Institute of Agricultural Research Agricultural Research Institute - Tanzania Food and Agriculture Organization of the United Nations Indian Council of Agricultural Research 176 118 135 111 106 87 98 80 79 78 Food and Agriculture Organization of the United Nations Agricultural Research Institute - Tanzania National Agricultural Research Organisation (Uganda) Ministry of Agriculture and Rural Development (Vietnam) Kenya Agricultural and Livestock Research Organization Instituto de Investigacao Agraria de Mozambique Department of Agriculture Extension (Bangladesh) Indian Council of Agricultural Research Zambia Agric</t>
   </si>
   <si>
+    <t>[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]
+el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]
+Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]
+- 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness" 411,914 "Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 "Andean Crop Diversity for Climate Change P-1560-DGUL" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 "Youth, Citizen Science and E-commerce:
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]
+Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]
+Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]
+2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]
+nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]
+2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]
+at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]
+II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]
+business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]
+de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW
+---
+[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]
+Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]
+de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 "Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]
+(INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]
+C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L.
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]
+to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p55pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 55 of 86 External collaborations/partners Center Area of Work Title and Number High level output (If Available) Arab Center for the Studies of Arid Zones and Dry Areas - ACSAD ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de la Recherche Agronomique de Tunisie; National Agricultural Research Institute of Tunisia - INRAT ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing Institut National de Recherche Agronomique de Tunisie. INRAT. ICARDA AoW2, AoW3 HLO: Accelerate - Stage2 &amp; Stage 3 testing &amp; Deploy Ankara University, Faculty of Agriculture ICARDA AoW2 HLO: Accelerate Stage2 &amp; Stage 3 testing
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4]
+del Bienestar (SEBIEN) de Quintana Roo CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Secretaría de Desarrollo Agropecuario (SEDAGRO) de Morelos CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Ministerio de Agricultura, Ganadería y Alimentación (MAGA) de Guatemala CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio CGI21-508007-PORB-Scaling for Impact.indd 31CGI21-508007-PORB-Scaling for Impact.indd 31
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt2]
+(SME) Private Ltd CIMMYT ID DEPLOY IFFA Seed Co Ltd CIMMYT ID DEPLOY Indian Institute of Maize Research CIMMYT AB, ID DEPLOY Indo American Hybrid Seeds (India) Pvt. Ltd CIMMYT ID DEPLOY Institut de Recherche Agricole pour le Développement (IRAD) CIMMYT AB, ID DEPLOY Institut des Sciences Agronomiques du Burundi (ISABU) CIMMYT AB, ID DEPLOY Institut National de la Recherche Agronomique du Niger (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 32 of 90 August 2025 | CGIAR Contracted partner Center Current Status of Partnership Area of Work Title and Number High level output (If Available) Dirección de Coordinación Regional y Extensión Rural (DICORER) CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Fundación para la Innovación Tecnológica Agropecuaria y Forestal
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p27pt3]
+Bolivia CIMMYT Phenotyping ZARI - Zambia Agricultural Research Institute, Zambia CIMMYT Phenotyping INIA Chile -Instituto de Investigaciones Agropecuarias, Chile CIMMYT Phenotyping INIA Uruguay -Instituto Ncional de Investigacion Agropecuaria, Uruguay CIMMYT Phenotyping IRESA - Institution de la Recherche et de l’Enseignement Supérieur Agricoles, Tunisia CIMMYT Phenotyping TAGEM - Ministry of Food Agriculture and Livestock, Turkey CIMMYT Phenotyping KALRO- Kenya Agricultural &amp; Livestock Research Organization, Kenya ARIA, Afghanistan CIMMYT Phenotyping-Int Nurseries ITGC, Algeria CIMMYT Phenotyping-Int
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt2]
+la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics (Breeding for Tomorrow) ● T-PJ-003670- Long-term funding of Ex Situ collections of germplasm (IITA) (Breeding for Tomorrow and CapSha) ● L-LTG001-Long term funding of ex situ collections of germplasm (ILRI) (Breeding for Tomorrow) ● R-A-2023-9-Genebank-AI (Breeding for Tomorrow) ● T-PJ-003575: Cassava Allele Mining Project: (IITA) Mining useful alleles for climate change adaptation in the cassava from CGIAR Genebanks (Breeding for Tomorrow and Climate Action) ● T-PJ-003576- (IITA) Mining useful alleles for climate change adaptation cowpea (Cowpea Allele mining project: Mining useful alleles for climate change adaptation in cowpea from CGIAR Genebanks (year 2022-26) (Breeding for Tomorrow, CapSha, and Climate Acti on) ● T-PJ-004017-VACS (IITA): Vision for Adapted Crops and Soil: Bambara Groundnut (Breeding for Tomorrow, CapSha and
+---
+[ID: pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 13 of 86 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) Alliance Bioversity CIAT AoW 3-Markets and Business Models; AoW 5-Gender Equality, Social Inclusion and Fairness Intermediate Outcome - AOW-IOC 3.2. Local producer organizations, national and sub-national public actors and private sector actors co-design or strengthen inclusive business models; 2030 Outcome - 2030 OC-4. Marginalized people participate in implementing innovations; 2030 Outcome - 2030 OC-3 Government, market and finance actors implement
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p25pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 25 of 44 Partner Center Area of Work Title and Number High level output (If Available) Local Governments for Sustainability, Nairobi City County, Dhaka North City Corporation, Local Government of Quezon City (Philippines), RUAF Foundation International Potato Center / Centro Internacional de la Papa 3.5.5 Urban food systems governance - Delivering knowledge products, evidence and capacity sharing with policy makers to guide interventions aimed at strengthening
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt1]
+Capacity Sharing Accelerator Inception Report 4 ISNAR International Service for National Agricultural Research ISRA Institut Sénégalais de la Recherche Agricole (Senegalese Agricultural Research Institute) ITU International Telecommunication Union KOICA Korea International Cooperation Agency KPIs Key Performance Indicators. MELIA Monitoring, Evaluation, Learning, and Impact Assessment NARES National Agricultural Research and Extension Systems NARS National Agricultural Research System PCT Program Coordination Team
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p36pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 36 of 86 August 2025 | CGIAR External collaborations/partners Center Area of Work Title and Number High level output (If Available) L’Institut Tchadien de Recherche Agronomique pour le Développement – ITRAD – Chad CIMMYT AB, ID, MI, Enable l’Institut National de la Recherche Agronomique du Niger – INRAN – Niger CIMMYT AB, ID, MI, Enable Ministry of Agriculture and Food Security – MAFS – Sudan CIMMYT AB, ID, MI, Enable MyAgro – USA CIMMYT ID National Agricultural Research Organization
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2]
+(SLARI) Africa Rice Potential AoW 4 - Achieving Impact by Unlocking Finance and Partnerships GrainPro Inc Africa Rice Potential AoW 2 - Pathways to Scale in Agrifood Systems African Development Bank Africa Rice Contracted AoW 4 - Achieving Impact by Unlocking Finance and Partnerships Seed Development and Certification Agency, Liberia Africa Rice Potential AoW 3 - Enabling Environment Lab Central de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p35pt4]
+Senegalais de Recherches Agricoles – ISRA – Senegal CIMMYT AB, ID, MI, Enable Instituto de Investigacao Agraria de Mocambique – IIAM – Mozambique CIMMYT AB, ID, MI, Enable International Institute of Tropical Agriculture – IITA – Nigeria CIMMYT AB, ID, MI, Enable Kenya Agricultural and Livestock Research Organization – KALRO – Kenya CIMMYT AB, ID, MI, Enable Lake Chad Research Institute – LCRI – Nigeria CIMMYT AB, ID, MI, Enable L’Institut de l’Environnement et de Recherches Agricoles – INERA – Burkina Faso CIMMYT AB, ID, MI, Enable CGI21-508008-PORB-Breeding for Tomorrow.indd 35CGI21-508008-PORB-Breeding for Tomorrow.indd 35 08/08/2025 16:0208/08/2025
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p36pt4]
+metrics, monitoring and evaluations. HLO 5.3: Curated analytics for innovation portfolio management and decision-making, including Scaling Readiness evaluations and customized assessment tools for target countries, both ongoing and as part of the annual adaptive management process, to ensure continuous learning and improvement Foundation SpectAct, Morocco ICARDA Existing AoW 3 - Enabling Environment Lab Institut National de la Recherche Agronomique a Tunisie (INRAT) ICARDA Existing AoW 3 - Enabling Environment Lab CGI21-508007-PORB-Scaling for Impact.indd 36CGI21-508007-PORB-Scaling for Impact.indd 36 07/08/2025 13:2407/08/2025 13:24
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt2]
+capacity AfriSeed, Zambia CIMMYT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact HLO 5.2: Insights for CGIAR scaling success through impact assessments.HLO 2.2: Co-designed scaling pathways for regional and national agrifood systems through improved stakeholder capacity Secretaría de Agricultura y Desarrollo Rural (SADER) de México CIMMYT Potential AoW1 - Engage and Empower HLO 1.1: A toolbox of methods, data, and dashboards HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Agencia Mexicana de Cooperación Internacional para el Desarrollo (AMEXCID) CIMMYT Potential AoW1 - Engage and Empower HLO
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt2]
+Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The World Bank, German Red Cross (Germany), Dhaka City North Corporation, Nairobi City County, International Water Management Institute, WorldFish International Food Policy Research Institute 1.2.2 Evidence Synthesis and Adaptive Learning - Co-develop knowledge products and action plans, and identify key investment and innovation priorities for stakeholders and partners to guide interventions aimed at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National
+---
+[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2]
+system Provincial govt. AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Colombian Roundtable for Sustainable Cattle AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Universidad del Cauca AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system Universidad de los Andes AOW 4 Market Systems, Policy Solutions and Scaling OP 4.2. Decision-support tools for efficient animal and aquatic food system EAFIT University Colombia AOW 4 Market Systems, Policy Solutions and
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p1pt2]
+Report June 2025 Contact: Nicoline de Haan (n.dehaan@cgiar.org)
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4]
+Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations, and evidence-based programs for enhancing inclusive informal food markets that effectively create quality jobs for young women and men and deliver safe and healthy foods in urban environments University of Peradeniya, Wayamba University of Sri Lanka, Asian Development Bank, World Food Programme International Food Policy Research Institute 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents CGI21-507031-PORB-Food Frontiers and Security.indd 24CGI21-507031-PORB-Food Frontiers and Security.indd 24 29/07/2025 19:3929/07/2025 19:39
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u52-56]
+Aryal, Bishal (IFPRI) 44:47 Thank you. Thank you. Nirmal, Rajalakshmi (IFPRI) 44:50 Thank you. Bye, bye. Trifa, Nicoleta (CGIAR System Organization) 44:53 Hi. Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1]
+23 Bilateral Contribution to Multifunctional Landscapes MELIA Studies UK FCDO - Seed to tree: value chains and partnerships for resilient restored forests in Malaysia • Actor engagement and outcome tracking UK – GCBC (UK-Defra) - Deploying Diversity as a Strategic Asset for Scaling of Ethiopia’s Green Legacy Initiative for Climate Change Resilience and Livelihoods • Program learning review • Actor engagement and outcome tracking FRANCE – FFEM Promover Oportunidades Sostenibles en la Cadena de Valor del Cacao de Excelencia (IA Lead of A1537) • Actor engagement and outcome tracking CoIMPACT INDIA • Program learning review Fruitful Lands India Phase II • Actor engagement and outcome tracking Sustainable Investments for Large-scale Rangeland R • Actor engagement and outcome tracking Building Community
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p32pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 32 of 72 July 2025 | CGIAR Contracted partner Center Area of Work Title and Number High level output (If Available) University of Los Andes CIAT Governance and Political Economy (AOW03) 3.3: New communities of practice, political economy and policy process tools are developed and strengthened, bringing together decision makers and diverse stakeholders to strengthen science diplomacy, science policy engagement, design, and implementation. Tegemeo Institute in Kenya IFPRI Governance and Political Economy (AOW03) 3.3: New communities of practice, political economy
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p21pt2]
+Research for Development (IRAD) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems Centre National de Recherche Agronomique (CNRA) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems The Council for Scientific and Industrial Research – Savannah Agricultural Research Institute (CSIR- SARI) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems Centre National de Recherche Appliqué au Développement Rural (FOFIFA/CENRADERU) Africa Rice Contracted AoW 2 - Pathways to Scale in Agrifood Systems L’Institut Sénégalais de Recherches
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4]
+for delivering SAAF outputs and outcomes. These organizations are either think tanks and consultancy firms (e.g. MacKenzie), governmental extension services (Fisheries Commission Ghana), or NGOs (Heifer International, CARE). In those instances, CGIAR is well-positioned to undertake the work. Still, stakeholder engagement can be pursued with stakeholders to transition toward sustainability and scaling. The remaining 80% have been rated as moderately efficient and impactful in undertaking HLO work. This group encompasses NARES (KALRO, IFReDI), NGOs (Vétérinaires Sans Frontières); private sector organizations (EON Aquaculture Limited, Githunguri Dairy Cooperative); international organizations (FAO, World Bank, AfDB); universities from the Global North (Corwell, Kiel) or targeted countries (Universidad de los Andes, University of Nairobi, Hanoi University of Public Health). While CGIAR is well or moderately positioned in most instances, there are significant opportunities for collaboration, stakeholder engagement, and in some instances, formal partnerships. Sustainable Animal &amp; Aquatic Food Science Program Comparative Advantage analysis
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt3]
+International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations, and evidence- based programs for enhancing inclusive informal food markets that effectively create quality jobs for young women and men and deliver safe and healthy foods in urban environments $454,738 T-PJ-003812-ETH/IITA - CITY REGIONS FOOD SYSTEMS, RUNRES (TH International Institute of Tropical Agriculture Urban Food Systems - AOW3 3.1.1 Safe urban food production - Evidence- based innovations and business models to improve safe, nutritious, and
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u43-45]
+Colomer, Julien (One CGIAR - France) 48:19 Thanks. Hurt, Chris (ILRI) 48:19 Thank you. Trifa, Nicoleta (CGIAR System Organization) ha detenido la transcripción
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt2]
+National Agricultural Research and Extension Systems NARS National Agricultural Research System PCT Program Coordination Team PMU Program Management Unit PORB Plans of Results and Budgets RAB Rwanda Agriculture and Animal Resources Development Board RELASER Red Latinoamericana de Servicios de Extensión Rural (Latin American Network for Rural Extension Services) RUFORUM Regional Universities Forum for Capacity Building in Agriculture SAARC South Asian
+---
+[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p4pt4]
+Cooperation TAP Tropical Agriculture Platform ToC Theory of Change ToR Terms of References TPI The Partnering Initiative UM6P Université Mohammed VI Polytechnique UNCTAD United Nations Conference on Trade and Development UNESCO United Nations Educational, Scientific and Cultural Organization. UNICEF United Nations International Children's Emergency Fund UPLB University of the Philippines Los Baños W3 Window 3 WCDI Wageningen Centre for Development
+---
+[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt3]
+ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance Contract IITA AOW02 Digital Advisories and Climate Risk Management T-PJ-003517: Chicken, Fish and Pigs Feed and Organic Fertilizer Value Chain Development Using BSF-Based Urban Biowaste Processing in Ghana, Mali, Niger and the Democratic Republic of Congo IITA AOW03 Locally-led Adaptation, AOW04 Low- emission Transitions $470,249 L-CIA023-Accelerating Impacts of CGIAR Climate Research for Africa II ILRI AOW01 Prioritization
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3]
+management of research &amp; scaling activities across CGIAR’s portfolio Agencia Mexicana de</t>
+  </si>
+  <si>
+    <t>[ID: docx:Standard Provisions 2026.docx:u19-22]
+Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.
+---
+[ID: docx:Standard Provisions 2026.docx:u16-19]
+Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:
+---
+[ID: docx:Standard Provisions 2026.docx:u181-184]
+Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Misused Fund Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, refund any portion of Window 1 and Window 2 Funds not used in accordance with the applicable Fund Use Agreements, and such funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.
+---
+[ID: docx:Standard Provisions 2026.docx:u28-31]
+ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.
+---
+[ID: docx:Standard Provisions 2026.docx:u178-181]
+appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center. Return of Funds. Unexpended or Uncommitted Funding. Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, promptly return any portion of Window 1 and Window 2 Funds that is unexpended or uncommitted at the completion of a CGIAR Program or activities under the CGIAR Program for which it was provided (including approved extensions) or at the termination of a Financial Framework Agreement between the System Organization and a Center, unless decided otherwise by the System Council. Such returned funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.
+---
+[ID: docx:Standard Provisions 2026.docx:u31-34]
+The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such
+---
+[ID: docx:Standard Provisions 2026.docx:u13-16]
+In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational level, as may be adopted from time to time. Responsibilities over Window 1 and Window 2 Funds Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research.
+---
+[ID: docx:Standard Provisions 2026.docx:u22-25]
+monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions. Window 3 Funds. Window 3 Funds are directed by Funders to individual Centers. Funders may designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization.
+---
+[ID: docx:Standard Provisions 2026.docx:u34-37]
+in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center. Window 3 Side Agreements or Arrangements. Nothing in the Funding Agreements or Arrangements is intended to preclude Funders and Centers from entering into Window 3 Side Agreements or Arrangements in regard to the terms governing the administration and use of Window 3 Funds. Funders may choose to make a Contribution to a Center through Window 3 without entering into a Window 3 Side Agreement or Arrangement, provided that such Contribution is made without any additional conditions attached to it. Any Window 3 Side Agreement or Arrangement will be consistent with these Standard Provisions and substantially in the form of Schedule 1 (Form of Window 3 Side Agreement or Arrangement) attached to these Standard Provisions, as may be amended from time to time. Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4,
+---
+[ID: docx:Standard Provisions 2026.docx:u172-175]
+Acknowledgement of Funders All communications products on CGIAR Research funded by Window 1, 2 and 3 Funds, whether online or in hard copy form (e.g., publications, press releases, newsletters, website stories, blogs, posters, etc.), must acknowledge support received from Funders in accordance with applicable CGIAR Policies and Procedures on branding and communication. Suspending Transfers of Funding from Window 1 and 2 Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement.
+---
+[ID: docx:Standard Provisions 2026.docx:u25-28]
+designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization. Centers receiving Window 3 Funds are responsible for the use of such funds and will: ensure that Window 3 Funds are used exclusively for their intended purposes; ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements;
+---
+[ID: docx:Standard Provisions 2026.docx:u55-58]
+Efficiency. The System Organization and each Center will, respectively: ensure that Window 1, 2 and 3 Funds are used with due regard to economy and efficiency, and that the highest standards of integrity in the administration of the funds are upheld; and ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures on cost allocation, which set forth the principles of allowability, allocability, and reasonableness. Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council.
+---
+[ID: docx:Standard Provisions 2026.docx:u46-49]
+Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund. Requirements on the Use of Window 1, 2 and 3 Funds CGIAR Policies and Procedures. The System Organization and each Center will, respectively ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures and the relevant entity's own policies and procedures. All CGIAR Policies and Procedures will be available on the System Organization's web site. Standard of care.
+---
+[ID: docx:Standard Provisions 2026.docx:u184-189]
+Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Inconsistency In the event of any inconsistency between the Cover Pages and these Standard Provisions, these Standard Provisions will prevail. Amendments Amendments These Standard Provisions may only be amended by approval of the System Council subject to concurrence of the Integrated Partnership Board. The System Organization will promptly notify the Funders and Centers in writing of any such amendments to these Standard Provisions.
+---
+[ID: docx:Standard Provisions 2026.docx:u175-178]
+Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement. Before taking such action under paragraph 13.1, the System Organization will notify the relevant Center in writing, and consult with the System Council as well as the relevant Center with a view to identify ways and means to manage the suspension and mitigate the impact on the implementation of CGIAR Research until such time that the suspension may be lifted. If such suspension is lifted by the System Organization, it will notify the relevant Center in writing. Request by a Funder. If a Funder has a credible concern: (a) that Window 1, 2 and 3 Funds are not used by a Center in accordance with the applicable Fund Use Agreement or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) of a non-compliance by a Center with any of its obligations under an applicable Fund Use Agreement, the Funder may request, through the System Council, the System Organization to review the specific concern and, as relevant, to take appropriate corrective action. The System Organization will report to the System Council on the outcome of the review and, as appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center.
+---
+[ID: docx:Standard Provisions 2026.docx:u4-7]
+the Financial Framework Agreement between the System Organization and each Center with respect to Window 1, 2 and 3 Funds; and any Window 3 Side Agreement or Arrangement between a Funder and a Center with respect to Window 3 Funds. Interpretation of the Standard Provisions. Unless the context requires otherwise, the terms of these Standard Provisions governing the roles and responsibilities: between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization;
+---
+[ID: docx:Standard Provisions 2026.docx:u106-109]
+Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder. If an individual Funder wishes to request, on an exceptional basis, a review or evaluation of any activities financed with Window 1 and Window 2 Funds, such Funder will consult with a designated representative from the System Organization on the most appropriate scope and terms of reference of such review or evaluation. The designated representative will assist in arranging for such review or evaluation in accordance with the applicable CGIAR Policies and Procedures. The costs of any such review or evaluation, including the internal costs of the System Organization or Center with respect to such review or evaluation, will be paid by the requesting Funder. The System Organization and each Center will, respectively collaborate on any monitoring or evaluations conducted in connection with CGIAR Research activities funded with Window 1, 2 and 3 Funds. Monitoring
+---
+[ID: docx:Standard Provisions 2026.docx:u58-61]
+Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council. Procurement. In the event that consultants are employed or services or goods are procured with Window 1, 2 and 3 Funds, the System Organization and each Center will, respectively, ensure that the employment and supervision of such consultants and the procurement of such services or goods will be the responsibility of each entity employing or contracting such consultants or carrying out such procurement and will be conducted in conformity with applicable CGIAR Policies and Procedures on procurement, in line with the following basic principles of equal treatment and non-discrimination on grounds of nationality, competition, predictability, transparency, verifiability, and proportionality. No taxation. The System Organization and each Center will, respectively, use best efforts, to the extent allowed by applicable agreements, such as those signed with host governments, and applicable laws, to ensure that the use of Window 1, 2 and 3 Funds will be free from any taxation or fees imposed under local laws. Insurance. The System Organization and each Center will, respectively, maintain insurance coverage sufficient to cover the activities, risks, and potential omissions of the activities funded by Window 1, 2 and 3 Funds in accordance with generally accepted industry standards and as required by law.
+---
+[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4]
+the continuity of prior work that is less fit for purpose in the Program’s ToC. Windows 1, 2, 3 and bilateral funding: Approximately half of S4I’s 2025 funding is from Window 1, with the remainder from Window 2, including two $1.25 million designated W2 allocations specifically for AoWs 4 and 5. The PORB also reflects stronger alignment of Window 3 and bilateral funding with Program logic: in 2025, 47 mapped W3 and bilateral investments totaling $44.8 million support the Program ($0.42M, $26.47M, $1.55M, $15.37M, and $0.99M across AoWs 1 through 5, respectively), with 74% of these funds active in Africa, 19% in Asia, and 7% in Latin America. Engage and Empower (AoW 1): This AoW is allocated $2.98 million in W1/W2 funding and supported by $0.42 million in W3/bilaterals. It anchors S4I’s stakeholder demand intelligence 9 The section on AoW 4 in the PORB description highlights major inception period successes in leveraging Window 3 investments, with an anticipated, two-year bilateral investment in HLO 4.1 to transition TAAT into the Scaling Program that will support new work that was not part of the RIIs or NPS.
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2]
+reducing producers' incomes and ability to invest in innovations; iv. Adverse national policy shifts regarding inclusion and equality; and v. Increased frequency of extreme climate events, which could undermine social progress and resilience. Please refer to the following link with the Program/Accelerator's full risk register. This link is open to ISDC colleagues and others will be granted access, on request. Category Risk Description Current Risk Level Target Risk Level Actions to Manage Risk Funding Reduced Window 1 &amp; 2 Funds Reduced Window 1 &amp; 2 funds caused by political changes from national governments which donate the bulk of CGIAR funds or other changes in donor priorities. This could result in outcome achievements failing to reach the
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt2]
+CGIAR Centers, and cross-cutting functions. Additional Window 3 and bilateral funds (~$8.8 million) complement this, especially enhancing research on socio-technical innovations and inclusion. Key risks identified include inadequate funding, insufficient in-house
+---
+[ID: docx:Standard Provisions 2026.docx:u10-13]
+Use and administration of the Contributions General Provisions in Respect of the Contributions The Contributions, including the funds, assets and receipts thereof, held in the Trust Fund are administered in accordance with the terms of the CGIAR Trustee Agreement and each Contribution Agreement or Arrangement. In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational
+---
+[ID: docx:Standard Provisions 2026.docx:u67-70]
+Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and
+---
+[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p3pt1]
+Inception Report: Policy Innovations Science Program 3 Acronyms FLW Food, Land, and Water MELIA Monitoring, Evaluation, Learning, and Impact Assessment HLO High-Level Output W3 Window 3 (bilateral
+---
+[ID: docx:Standard Provisions 2026.docx:u163-166]
+In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations
+---
+[ID: docx:Standard Provisions 2026.docx:u157-160]
+Change in Reporting Requirements. Unless decided otherwise by the System Council and/or the Integrated Partnership Board as the case may be, any change in the form or substance or periodicity of a technical or financial report will become effective only in the following calendar year. Additional Audits / Financial Reviews / Technical Reporting Funders will manage their audits, financial reviews and technical reporting with respect to the Window 1, 2 and 3 Funds collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to require duplicative reporting, provided that a Funder may require supplemental audits, financial reviews and technical reporting with respect to Window 3 Funds pursuant to its Window 3 Side Agreement or Arrangement, the costs of which would be paid by the requesting Funder. If a Funder wishes to request, on an exceptional basis, that the System Organization or a Center has an external audit or provides additional financial reviews or technical reports with respect to Window 1 and Window 2 Funds, and the requesting Funder has a statutory, regulatory or policy environment requiring such Funder's ability to make such a request unilaterally, such Funder will decide with the System Organization or the relevant Center on the most appropriate scope and terms of such audit, review or reporting. The costs of which, including the internal costs of the System Organization or any Center with respect to such additional audits, reviews or reporting, will be paid by the requesting Funder.
+---
+[ID: docx:Standard Provisions 2026.docx:u64-67]
+ensure, consistent with its governing arrangements, CGIAR Policies and Procedures and the respective entities’ policies and procedures, including those pertaining to combating financing for terrorists, that Window 1, 2 and 3 Funds are used for their intended purposes and are not diverted to individuals or entities associated with terrorism, as identified in accordance with relevant United Nations Security Council Sanctions resolution; and not use such Window 1, 2 and 3 Funds for the purpose of any payment to persons or entities, or for the import of goods, if such payment or import, to its knowledge or belief is prohibited by a decision of the United Nations Security Council taken under Chapter VII of the Charter of the United Nations or directed to a person or entity, appearing on the Consolidated United Nations Security Council Sanctions List. Lobbying. The System Organization and each Center will, respectively, ensure that none of Window 1, 2 and 3 Funds is earmarked for lobbying activity, defined as attempting to influence legislation (i) through affecting the opinion of the general public or any segment thereof (i.e. grassroots lobbying), or (ii) through communications with any member or employee of a legislative body, except in the case of both (i) and (ii) to the extent such activities arise inherently in relation to CGIAR Research comprising policy development. Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive.
+---
+[ID: docx:Standard Provisions 2026.docx:u73-76]
+The System Organization and each Center will, respectively, take all necessary precautions to avoid or manage any Conflicts of Interest in all matters related to Window 1, 2 and 3 Funds. If a Conflict of Interest occurs, the System Organization and each Center will, respectively take, without delay, all necessary measures to resolve the conflict, e.g. by replacing the person in question or by obtaining independent verification of the terms of the proposed decision or transaction. Environmental and Social Standards. The System Organization and each Center will, respectively ensure: that Window 1, 2 and 3 Funds are used with due regard to environmental sustainability; and
+---
+[ID: docx:Standard Provisions 2026.docx:u37-40]
+Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4, 9.1.1, 9.1.2, 9.2-9.4 and 13-15. Due Diligence. Each Center will conduct due diligence and review of the CGIAR System Partners to which it is disbursing funding from the Window 1, 2 and 3 Funds to the extent deemed necessary or appropriate by such Center. Cooperation. Centers will cooperate with the System Organization in order for the System Organization to fulfill its obligations under the relevant Fund Use Agreements.
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt1]
+Gender Equality and Inclusion Accelerator Inception Report 5 A total of $9 million in pooled funding for 2025 is strategically distributed across AoWs, 12 CGIAR Centers, and cross-cutting functions. Additional Window
+---
+[ID: docx:Standard Provisions 2026.docx:u121-124]
+be prepared in accordance with International Financial Reporting Standards (IFRS) or U.S. Generally Accepted Accounting Principles and in each case audited by an independent certified auditor of international standard in accordance with international audit standards; be prepared as of 31 December of each year to be submitted within six (6) months after the end of each calendar year; and disclose the use of Window 1 and Window 2 Funds in accordance with applicable CGIAR Policies and Procedures on reporting. Financial Reports
+---
+[ID: docx:Standard Provisions 2026.docx:u52-55]
+carry out all regulated research activities under high standards (set with reference to internationally accepted practices) and in accordance with applicable CGIAR Policies and Procedures, and applicable laws and regulations. Responsibility to Inform. Centers will promptly inform the System Organization, and the System Organization will promptly inform Funders through the System Council, should substantial deviation from the CGIAR Research supported with Window 1, 2 and 3 Funds develop. Financial, Economic and Administrative Standards Efficiency. The System Organization and each Center will, respectively:
+---
+[ID: docx:Standard Provisions 2026.docx:u70-73]
+with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of perso</t>
+  </si>
+  <si>
+    <t>[ID: docx:Standard Provisions 2026.docx:u19-22]
+Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.
+---
+[ID: docx:Standard Provisions 2026.docx:u16-19]
+Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2]
+of green bananas on her head.
+---
+[ID: docx:Standard Provisions 2026.docx:u31-34]
+The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]
+Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for
+---
+[ID: docx:Standard Provisions 2026.docx:u28-31]
+ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]
+CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]
+el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p52pt1]
+A pig farmer in Tien Lu district, Hung
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]
+nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt4]
+HLOs
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]
+business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]
+- 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness" 411,914 "Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 "Andean Crop Diversity for Climate Change P-1560-DGUL" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 "Youth, Citizen Science and E-commerce:
+---
+[ID: docx:Standard Provisions 2026.docx:u70-73]
+with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and (viii) respect for the evolving capacities of children with disabilities. Conflicts of Interest. The System Organization and each Center will, respectively, take all necessary precautions to avoid or manage any Conflicts of Interest in all matters related to Window 1, 2 and 3 Funds.
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p37pt3]
+2.2 Better designed emergency response in fragile settings - Government, humanitarian, and NGO actors use evidence and tools in fragile settings to guide emergency responses X X X X High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 180,781.00 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X Total AoW 2 budget 180,781.00 Area of Work 3:
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]
+Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]
+Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]
+protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]
+Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2
+---
+[ID: docx:Standard Provisions 2026.docx:u163-166]
+In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations
+---
+[ID: docx:Standard Provisions 2026.docx:u67-70]
+Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt3]
+in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Mozambi que Surveys and KII CASP 2024 2026 100,000 Evaluate UNHCR’s Sustainable Land Management and Environmental Rehabilitation Project in Bangladesh Adam Savelli (CIAT) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt2]
+for the stud y End date for the stud y Study cost (USD) How related to past evaluations (SG or others) Gendered Labor Impacts of Herder-Related Violence in Nigeria Jeff Bloem (IFPRI) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Nigeria Household survey (panel) n/a 2024 2025 13,100 n/a Analyzing
+---
+[ID: pdf:Type3_2024Report.pdf:p6pt3]
+Evaluation Recommendations are addressed by management. These responses are designed to ensure that Evaluations inform decision-making, enhance organizational effectiveness, promote learning, and strengthen accountability. They include time-bound commitments from management to implement Evaluation Recommendations and are systematically followed up as outlined in the CGIAR Evaluation Policy, which identifies follow-up as a critical component of the evaluative process.5 Since the launch of formal tracking in CGIAR’s 2022 Technical Report, the systematic monitoring and reporting of Management Response Actions has continued to evolve. This 2024 report provides information on (9) Evaluations and one (1) Evaluability Assessment (EA) completed during 2021-24 – all of which are available on the updated Evaluation and Management Response Actions Tracker. These Evaluations generated a total of 319 Recommendations and sub-Recommendations, underscoring the organization’s commitment to learning and continuous improvement. Evaluation title Date completed Date of Management Response No. of Recs. and sub-Recs No. of Actions Max. completion date for Actions Links to Evaluation Reports and Management Responses 2021 Synthesis of Learning from a Decade of CGIAR Research Programs June 2021 June 2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]
+at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt2]
+2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. SP04 and SP078 will implement joint research on natural resources management and rangelands governance. Food Frontiers and Security SP04- Multifunctional Landscapes 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis
+---
+[ID: pdf:Type3_2024Report.pdf:p6pt4]
+2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project Management Approaches and Fit-for-Purpose Information Products December 2022 December 2022 36 19 2024 • Advisory Report GENDER (Generating Evidence and New Directions for Equitable Results) Platform Evaluation December 2023 January 2024 22 21 2024 • Evaluation Report • Management Response CGIAR Genebank Platform Evaluation March 2024 March 2024 32 26 2027 • Evaluation Report • Management Response Evaluability Assessment Review of Four Regional Integrated Initiatives June 2024 June 2024 9 8 2026 • Evaluation Report • Management Response Genetic Innovation Science Group Evaluation August 2024 September 2024 42 28* 2030 • Evaluation Report • Management Response Resilient Agrifood Systems Science Group Evaluation August 2024 September 2024 26 22* 2027 • Evaluation Report • Management Response Systems Transformation Science Group Evaluation August 2024 September 2024 21 12* TBC • Evaluation Report • Management Response Total 319 248 Table 1. Evaluation details and associated Management Responses and Actions *The number of Management Response Actions for the Science Group Evaluations will likely change after Q2, 2025. May 2025 7 6 CGIAR Portfolio Practice Change (Type 3) Report
+---
+[ID: pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p10pt2]
+use cases respond to clear demand from both
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt3]
+settings - Government, humanitarian, and NGO actors use evidence and tools in fragile settings to guide emergency responses X X X X 2.3 Programs and policies to promote recovery and stabilize livelihoods in fragile settings - Government, humanitarian, and NGO actors use evidence and tools in fragile settings to design programs and policies that will promote recovery and stabilize livelihoods X X X X High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 759,052.00 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X 2.3.3 Recover -
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]
+de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4]
+del Bienestar (SEBIEN) de Quintana Roo CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Secretaría de Desarrollo Agropecuario (SEDAGRO) de Morelos CIMMYT Contracted AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio Ministerio de Agricultura, Ganadería y Alimentación (MAGA) de Guatemala CIMMYT Potential AoW1 - Engage and Empower HLO 1.2. Institutional innovations supporting prioritization, feedback, &amp; adaptive management of research &amp; scaling activities across CGIAR’s portfolio CGI21-508007-PORB-Scaling for Impact.indd 31CGI21-508007-PORB-Scaling for Impact.indd 31
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt2]
+erato r(s) Start date for the stud y End date for the stud y Study cost (USD) How related to past evaluations (SG or others) fragile settings Evaluation of UNHCR's climate resilient shelter in Mozambique Adam Savelli (CIAT) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p35pt2]
+use evidence and tools in fragile settings to design programs and policies that will promote recovery and stabilize livelihoods X X X X 1,001,985.01 High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 458,103.86 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X 2.3.3 Recover - Guidance for policymakers and project implementers on programming options to stabilize household and community livelihoods, promote recovery, and build resilience in FCA settings (especially for
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p17pt2]
+the stud y End date for the stud y Stud y cost (USD ) How related to past evaluations (SG or others) From Exchange to Impact: How GHUs Catalyze Genebanks- Breeding Germplasm Exchange for Invasive Cassava Disease Management IITA Intermediat e Outcome CGIAR and internal and external partners exchange genetic resources without the risk of spreading quarantine pests
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p31pt2]
+stabilize livelihoods X X X X 30,000.00 High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 1,031,051.00 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X 2.3.3 Recover - Guidance for policymakers and project implementers on programming options to stabilize household and community livelihoods, promote recovery, and build resilience in FCA settings (especially for the underserved) X X X X Total AoW 2 budget 1,131,051.00 Area of Work 3: Urban Food Systems 2025 Outcome Q1 Q2 Q3
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p38pt1]
+Genebanks Accelerator Inception Report 37 are few alternative sources, especially for roots, tubers and bananas, that can provide the same assurance. AoW1 Emphasize the inclusion of NUS in Genebank collections and clarify measurement criteria for process improvements. Identify specific bottlenecks and establish accountability for targets, along with clear baselines. Provide rationale for chosen technologies and detail how various platforms integrate to enhance effectiveness. Set funding milestones to ensure support for additional activities. See above for response on NUS. Note also that CGIAR genebanks will always be responsible for the conservation and availability of the major staple crops, mandate crops of the Centers that host the genebank, and that resources cannot necessarily be moved from these to other crops especially given the frequency of requests for these crops. Hundreds of small genebank process adjustments and improvements are made annually. These are extremely hard to monitor and document but a better job should be
+---
+[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p6pt1]
+Plan of results and budget 2025 | Page 6 of 44 July 2025 | CGIAR Area of Work 2: Fragile and Conflict-affected Food Systems 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 2,428,987.86 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X 2.3.3 Recover - Guidance for policymakers and project implementers on programming options to stabilize household and community livelihoods, promote recovery, and build resilience in FCA settings (especially for the underserved) X X X X
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4]
+in rural communities and the overall capacity of populations to innovate and to build and maintain resilient livelihoods and landscapes. AoW5 contributes to this vision by: a) developing or strengthen ing participatory research tools and methodologies for understanding the context, history, causes and influences of fairness and GEYSI in each multifunctional landscape; b) co-designing gender transformative approaches to change discourses and norms; c) supporting the gender responsive and fair implementation of innovations and interventions; d) strengthening capacity of partners on transdisciplinary, gender responsive a nd socially inclusive approaches; e) supporting the development and implementation of re sponsible scaling strategies; f) adapting GEYSI -responsive and -transformative approaches to landscape perspective; and g) develop research on emerging (new) topics and generating evidence on new directions for achieving quality of life and social equity r esilience from a human perspective. These lead to two key outputs: GEYSI-responsive and transformative approaches and methodologies from
+---
+[ID: pdf:Type3_2024Report.pdf:p3pt2]
+stakeholders 4 2.2. Close-out of the 2022-24 Portfolio 6 2.3. Transitioning to the 2025-30 Portfolio 6 Section 3: Implementation Status: Management Responses to CGIAR Evaluations 7 3.1. Key developments in 2024 for tracking Evaluation Recommendations and Management Response Actions 10
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt2]
+TOC is pivotal to mapping out the complex connections across a holistic B4T program and enabling clarity in responsibilities for MELIA and accountabilities for outcomes. ISDC Feedback The ISDC Feedback was summarized for the System Council. This summarized feedback is shown in Table 7, along with how the points of feedback have been considered in the revision of the TOC and MELIA framework. Table 7 Response to ISDC Feedback from MELIA perspective Assessment Criteria Comment Response 2. Evidence that the Science Program is demand driven through codesign with key stakeholders and partners (NARES, governments, farmers, private sector, funders) and research collaborators within and outside CGIAR. This Program targets “impactful geographics and user needs,” seeking to identify areas with the lowest 35% impact and reallocate these resources to the top 25% impact. However, more acknowledgement could be given to the crucial role of the NARES and farmers and their local knowledge which should be integrated with modern tools to enhance adoption. While targeting “the highest
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt2]
+evaluate the returns to R&amp;D investments in different regions and different crop and anima</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -1671,6 +2139,21 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who coordinates funders’ M&amp;E requirements across the CGIAR Portfolio and how is duplication avoided? \n\nContext:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23 part 4\nContent: additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 2 part 4\nContent: report is part of the CGIAR System Organisations’ technical reporting arrangement. We would like to thank all funders who supported this work through their contributions to the CGIAR Trust Fund, and those who supported bilaterally: https://www.cgiar .org/funders. The report was led by the Portfolio Performance Unit, with expert technical support from the Food Security Evidence Brokerage. We gratefully acknowledge the contributions and insights from many CGIAR staff who provided access to source materials, selected prominent themes, and reviewed drafts. This included Impact Area Platform Directors, regional leaders, CGIAR Center assessment and monitoring specialists, the Independent Advisory and Evaluation Services, the Donor Relations and Business Development unit, the Communications and Advocacy unit, CGIAR research leaders and senior\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p29pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 29 part 2\nContent: of information on how climate mitigation is covered in the Portfolio. There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. There is a lack of information on how orphan and opportunity crops and pulses are covered in the Portfolio. There is a lack of information on how\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p33pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 33 part 2\nContent: is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. N/A There is a lack of information on how orphan and opportunity crops and pulses are covered in the Portfolio. N/A There is a lack of information on how youth and social inclusion (that does not relate to gender) is covered in the Portfolio. N/A There is a lack of information on how capacity sharing (as it relates to internal learning and decolonization of research) is covered in the Portfolio. Capacity sharing is foundational to\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p39pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 39 part 4\nContent: more details on ToC, Areas of Work, etc. We have significantly reworked and streamlined the research questions. They are now underpinned by the assumptions formulated in the revised ToC these also serve as hypotheses (in terms of fulfilled assumptions) for the research questions. Linkages with other Programs and Accelerators A concern is how the accelerator will effectively work with and build on other capacity sharing activities at CGIAR (with other Programs and Accelerators) without duplication or competition (pp. 85). The Accelerator will include a matrix analysis of Programs and other Accelerator during inception, to map Programs’ AoW and its own AoW, in order to define common interests in research questions or challenges, synergies, alignments, complementarities, and avoid duplication of actions. Section 8 of the inception report details how the accelerator would work with other programs to ensure synergy, and avoid duplication and support complementarity in terms of delivery of its service portfolio.\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 1\nContent: 2.2. Close-out of the 2022-24 Portfolio As the 2022-24 Portfolio closed, close-out guidelines were designed to ensure a smooth transition to the new Portfolio, building on past achievements while maintaining continuity in science and innovation delivery. The close-out process focused on the timely preparation and submission of 2024 technical and financial reports, ensuring all CGIAR teams and partners met Portfolio deliverables, and facilitating effective engagement and continuous communication with stakeholders. Proactive mitigation measures were identified to manage risks associated with the transition to the new research Portfolio. Focus was placed on sustaining partnerships beyond the conclusion of the 2022-24 Portfolio to ensure ongoing collaboration. The guidelines included a section on SGPs to ensure alignment. This structured approach ensures that the achievements and collaborations of the 2022-24 cycle are seamlessly integrated into the new Portfolio. 2.3. Transitioning to the 2025-30 Portfolio Support was provided to the CGIAR Portfolio Transition Team, which included the development of Inception Guidelines that outlined the principles and processes to assist Transition Teams in planning and achieving inception deliverables for the 2025-30 CGIAR Portfolio. In 2024 work began on developing a new Technical Reporting Arrangement for 2025-30 (TRA 25-30) to define the Technical Reporting requirements for the next CGIAR Portfolio. A cross-CGIAR working group – comprising Center experts and System functions – led its development. The TRA 25-30 will promote progressive alignment between reporting requirements for pooled and non-pooled\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p30pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 30 part 4\nContent: S4I will map scaling efforts across Programs to reduce duplication, achieve synergies, and strengthen system-wide coherence.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 3 part 2\nContent: outcomes and i mpacts of the whole portfolio through progressive alignment of reporting on w3/bilaterally funded components with a common framework. • Line of sight: The TRA is designed to meet the needs of diverse funders, ensuring transparency and accountability by linking investment to results, both for pooled and non-pooled funds. • Impact focus: Research results will be better linked to CGIAR’s 2030 targets using enhanced impact area indicators. Impact assessments will be integrated into Program/Accelerator design. The use of geographically-bounded targets will be explored for priority locations. A robust approach to project cross-Portfolio benefits by Impact Area for different funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified reporting: Overly complex requirements will be avoided, aiming to\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p2pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 2 part 4\nContent: reviewed and validated by the authors to ensure accuracy, coherence, and alignment with the original intent. Acknowledgements This work is part of the CGIAR System Organization. We would like to thank all funders who supported this research through their contributions to the CGIAR Trust Fund:\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p32pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 32 part 1\nContent: Genebanks Accelerator Inception Report 31 10. Addressing feedback on selects topics Concise summary of feedback Details on how the Program/ Accelerator has addressed or will address this feedback (in the Inception Phase or beyond) There is a lack of information on how water systems are covered in the Portfolio. N/A There is a lack of information on how climate mitigation is covered in the Portfolio. N/A There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how environmental health and biodiversity is covered in the Portfolio. The Genebanks proposal noted that activities will lead to a stronger overall global system of international and national institutions, policies, and mechanisms contributing\n\n---\n\n[ID: pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p25pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_Inception Report 30-06-2025.pdf\nLocation: page 25 part 1\nContent: Food Frontiers and Security Program | Inception Report 25 operational efficiency, avoid duplication, and generate broader, more context-responsive insights than either program could produce alone, delivering greater value to partners and stakeholders across the CGIAR portfolio. Together with The Climate Action SP,\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 3 part 3\nContent: funding scenarios will be developed; these projections will be used to set the targets and milestones against which progress will be reported. • Simplified reporting: Overly complex requirements will be avoided, aiming to reduce the reporting burden on Centers. Technical Report products include the following: • A Results Dashboard including AI functionalities will be updated several times a year (e.g. quarterly) to offer funders and partners closer to real-time data. • Annual Program/Accelerator Technical Reports will be complemented by an Annual Portfolio Report which will convey progress by Impact Area, geographic and thematic priorities and include information on CGIAR’s internal practice change and learning. • Portfolio outcomes and impacts will be consolidated in a specific report every 3 years. Evidence of CGIAR contributions to impact will be synthesized and regularly updated through an\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u103-106]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use of Materials' paragraph 108 to section 'Monitoring and Evaluations' paragraph 115\nContent: Intellectual Property rights. The System Organization and each Center will, respectively, ensure that necessary intellectual property rights are obtained to allow the rights referred to under this paragraph 6 to be granted. If third party copyright restrictions or attribution requirements apply to such documents, this will be indicated on the documents. Monitoring and Evaluations General Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p8pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 8 part 4\nContent: other organizations as well as by funders. “CGIAR’s efforts to mainstream scaling put it at the cutting edge …” compared to other research and innovation organizations, and development organizations generally (Global Scaling Community of Practice). Figure 5: A pile of LEGO pieces that represents CGIAR’s innovation portfolio management pre-2022. What was once a fragmented system is now becoming more structured and strategic. Until 2022, there was no efficient way to manage ‘’CGIAR’s innovation portfolio’’. Innovation data was scattered, not up-to-date and lacked evidence. Furthermore, there was no operational framework to track or support scaling for impact. It led to organizational risks and inefficiencies as leadership, partners and funders could not easily access CGIAR innovations. This changed under the CGIAR 2030 Research and Innovation Strategy that embraced a more systematic and evidence-based innovation management based on principles of the Scaling Readiness approach. Currently, information on more than 1,325 innovations under development or use are now easily accessible on the CGIAR Results Dashboard, which is widely used by partners and funders. The World Bank Group, FAO, Gates Foundation, GIZ, ENABEL, and the African Development Bank are among organizations that have embraced (elements of) the CGIAR innovation management approach. CGIAR is actively sharing its innovation portfolio management journey with other organizations. The Gates Foundation partnered with CGIAR to co-develop a protocol for scaling strategies aimed at high-impact innovations. Internally, CGIAR Centers such as the Alliance of Bioversity and CIAT (ABC) and the International Livestock Research Institute (ILRI) and CGIAR projects such as the Accelerate for Impact Platform (A4IP), Technologies for African Agricultural Transformation (TAAT) and HarvestPlus Solutions have adopted elements of innovation portfolio management. May 2025 1110 CGIAR Portfolio Practice Change (Type 3)\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 2\nContent: 2025-30 CGIAR Portfolio. In 2024 work began on developing a new Technical Reporting Arrangement for 2025-30 (TRA 25-30) to define the Technical Reporting requirements for the next CGIAR Portfolio. A cross-CGIAR working group – comprising Center experts and System functions – led its development. The TRA 25-30 will promote progressive alignment between reporting requirements for pooled and non-pooled funding components, and sets expectations for transparency, performance tracking, and accountability across CGIAR and with funders. It will also operationalize the PRMF , inform decision-making, and provide direction for Portfolio-level monitoring, evaluation, learning and impact assessment (MELIA) and the design of the next version of the PRMS. The TRA 25-30 is expected to be endorsed in the first half of 2025. A durum wheat field at Toluca Station. Credit: Alfonso Cortés/CIMMYT Section 3: Implementation Status: Management Responses to CGIAR Evaluations 5. For more information see the CGIAR Evaluation Policy, the CGIAR Evaluation Guidelines, and the Process Note on Developing, Tracking and Reporting on Management Responses to Evaluations. A Management Response is a formal mechanism through which Evaluation Recommendations are addressed by management. These responses are designed to ensure that Evaluations inform decision-making, enhance organizational effectiveness, promote learning, and strengthen accountability. They include time-bound commitments from management to implement Evaluation Recommendations and are systematically followed up as outlined in the CGIAR Evaluation Policy, which identifies follow-up as a critical component of the evaluative process.5 Since\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p87pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 87 part 2\nContent: 2025–2030 The creation of a Scaling for Impact Program in CGIAR’s Portfolio 2025–2030 creates even more space and resources for innovation and scaling work. The Scaling for Impact Program plays an important role in catalyzing innovation scaling on the ground with CGIAR colleagues and partners while more System-wide innovation portfolio management functions continue to be delivered by CGIAR’s Portfolio Performance Unit. In CGIAR’s 2025–2030 Portfolio (Figure 6.4), innovation management is not just a process or tool — it is the central instrument for driving coherence and collaboration between the Science Programs and the Scaling for Impact Program while also aligning demand with supply and guiding strategic Portfolio priorities. Figure 6.4. Schematic overview of the CGIAR 2025–2030 Portfolio. CGIAR’s Portfolio Performance Unit and Project Coordination Unit work closely with the Scaling for Impact Program to deliver key innovation portfolio management functions for the 2025–2030 Portfolio. These two units continue to mainstream innovation and scaling tracking and performance across the\n\n---\n\n[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations_Inception Report 30-06-2025.pdf\nLocation: page 26 part 2\nContent: to national policy research ecosystems through coordinated capacity sharing activities. A prime example of this effective coordination and the efficiencies it generates is the policy program hub in Kenya. This hub actively coordinates with other CGIAR Programs, Accelerators, and individual CGIAR Centers building on efforts that the CGIAR country convener for Kenya had started. It therefore also provides an integration mechanism with W3/bilateral projects. Coordination is fundamental for avoiding duplication of efforts: They serve as a critical platform to share research plans, identify synergies, and proactively prevent overlapping activities, thereby ensuring a highly efficient deployment of collective resources across various CGIAR programs in Kenya. Beyond internal CGIAR coordination, the Kenya hub takes a leading role in planning joint policy dialogue series, country policy notes, bringing diverse stakeholders together for impactful co- design and co-implementation.\n\n---\n\n[ID: pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p33pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_Inception Report 30-06-2025.pdf\nLocation: page 33 part 1\nContent: Capacity Sharing Accelerator Inception Report 33 10. Addressing feedback on select topics Only one feedback (lack of information on how capacity sharing) applies directly to the CapSha Accelerator. Concise summary of feedback Details on how the Program/ Accelerator has addressed or will address this feedback (in the Inception Phase or beyond) There is a lack of information on how water systems are covered in the Portfolio. N/A There is a lack of information on how climate mitigation is covered in the Portfolio. N/A There is a lack of information on how tradeoffs and synergies in mixed systems are covered in the Portfolio. N/A There is a lack of information on how\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 45 part 3\nContent: Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]\nLink: https://cgspace.cgiar.org/items/8acc660f-7305-4e4b-ab21-1c192611b017\nFile: CGI21-507032-PORB-Climate Action.pdf\nLocation: page 11 part 2\nContent: II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 3\nContent: de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW\n\n---\n\n[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_Inception Report 30-06-2025.pdf\nLocation: page 4 part 3\nContent: Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 2\nContent: de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 \"Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735\" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 42 part 3\nContent: (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 46 part 3\nContent: C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L.\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 4\nContent: to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "deeper research"}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 45 part 3\nContent: Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]\nLink: https://cgspace.cgiar.org/items/8acc660f-7305-4e4b-ab21-1c192611b017\nFile: CGI21-507032-PORB-Climate Action.pdf\nLocation: page 11 part 2\nContent: II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 3\nContent: de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW\n\n---\n\n[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_Inception Report 30-06-2025.pdf\nLocation: page 4 part 3\nContent: Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 2\nContent: de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 \"Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735\" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 42 part 3\nContent: (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 46 part 3\nContent: C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L.\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 4\nContent: to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Use all the chunks that you receive. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?\n\nContext:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 45 part 3\nContent: Seed Ltd CIMMYT ID DEPLOY PROASE Productores Asociados de Semillas S.C. de R.L. de C.V. CIMMYT ID DEPLOY Productora de Semillas Azteca S.P .R. de R.L. CIMMYT ID DEPLOY PRODUCTORA DE SEMILLAS SMART SEEDS SAS DE CV CIMMYT ID DEPLOY Productora de Semillas Zarco S.P .R. de R.L. CIMMYT ID DEPLOY Productores de Semilla de Copandaro S.P .R. de R.L. CIMMYT ID DEPLOY Productos y Servicios Agrícolas S.P .R. de R.L. CIMMYT ID DEPLOY QualiBasic Seed Company (QBS) CIMMYT AB, ID\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507032-PORB-Climate Action.pdf:p11pt2]\nLink: https://cgspace.cgiar.org/items/8acc660f-7305-4e4b-ab21-1c192611b017\nFile: CGI21-507032-PORB-Climate Action.pdf\nLocation: page 11 part 2\nContent: II) ICRISAT AOW02 Digital Advisories and Climate Risk Management $89,064 N-343001-GCAN INITIATIVE IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $1,321,123 N-601158-SPIR II IFPRI AOW01 Prioritization and Coordination of Climate Action, AOW05 Finance and Policy for Scaling Solutions $201,213 PJ-003953: APPUI A LA TRANSFORMATION ET A LA RESILIENCE DES SYSTEMES ALIMENTAIRES DE MADAGASCAR A TRAVERS LA RECHERCHE POUR LE DEVELOPPEMENT IITA AOW03 Locally-led Adaptation $82,949 PJ-004108: ACRESAL Technical Assistance\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 3\nContent: de Cajas Rurales de Ahorro y Crédito Comunidades de Oriente (CECRUCSO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organización para el Desarrollo del Corquin (ODECO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Organismo Cristiano de Desarrollo Integral de Honduras (OCDIH) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW\n\n---\n\n[ID: pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_Inception Report 30-06-2025.pdf\nLocation: page 4 part 3\nContent: Frameworks for Climate Services PLACA Climate Action Platform for Agriculture in Latin America and the Caribbean / La Plataforma de Acción Climática en Agricultura de Latinoamérica y el Caribe PMU Program Management Unit PPU Portfolio Performance Unit PRMS Performance and Results Management System REMET Reducing Methane Emissions from Rice project ROI Return on investment S4I Scaling for Impact (Program) SA South Asia SB\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 2\nContent: de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation Globally (AOW05) High Level Output 5.4. Unique crop diversity under threat is safeguarded through the integration of in situ and ex situ conservation strategies 50,000 \"Revealing the Diversity of Barley Quality Traits through Synergies between On-farm Practices and Technological Innovations D-100735\" ICARDA Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 237,008 Long Term Partnership Agreement ICARDA Biodiversity\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p42pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 42 part 3\nContent: (INRAN) CIMMYT AB, ID DEPLOY Institut National de Recherché pour l’Agriculture, la Pêche et l’Environnement (INRAPE) - Comoros CIMMYT AB, ID DEPLOY Institut National pour l'Etude et la Recherche Agronomiques (INERA) - RDC CIMMYT AB, ID DEPLOY Instituto de Investigação Agronómica (IIA) - Angola CIMMYT AB, ID DEPLOY Instituto de Investigación Agropecuaria de Panamá CIMMYT AB, ID STRATEGIZE/REFOCUS, PARTNER / TRANSFORM, OPTIMIZE / ACCELERATE, CREATE Invicta Agritech India Private Limited CIMMYT ID DEPLOY JAMSONI COMPANY LIMITED CIMMYT ID DEPLOY Jardins da Yoba CIMMYT ID\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p46pt3]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 46 part 3\nContent: C.V. CIMMYT ID DEPLOY Semillas Barriga S.R.P . de R.L. CIMMYT ID DEPLOY Semillas Berentsen S.A. de C.V. CIMMYT ID DEPLOY Semillas Cinteotl S.P .R de R.L. CIMMYT ID DEPLOY Semillas Iyadilpro y Ya S.A. de C.V. CIMMYT ID DEPLOY SEMILLAS MEJORADAS S.A. CIMMYT ID DEPLOY Semillas Ocso S.P .R. de R.L. CIMMYT ID DEPLOY Semillas Proseso SA DE CV CIMMYT ID DEPLOY Semillas y Agroinsumos Golden S.P .R. de R.L. de C.V. CIMMYT ID DEPLOY Semillas PROSASOL S.P .R. de R.L.\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 22 part 4\nContent: to Scale in Agrifood Systems Mancomunidad de Municipios del Parque Nacional Montaña de Celaque (MAPANCE) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación Regionalde Servicios Agropecuarios de Oriente (ARSAGRO) - Honduras CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Cooperación para el Desarrollo Rural de Occidente-CDRO - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems CGI21-508007-PORB-Scaling for Impact.indd 22CGI21-508007-PORB-Scaling for Impact.indd 22 07/08/2025 13:2407/08/2025 13:24"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who holds fiduciary responsibility over Window 1 and Window 2 Funds?\n\nContext:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u19-22]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24\nContent: Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u16-19]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21\nContent: Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u181-184]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198 to section 'Misused Fund' paragraph 202\nContent: Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Misused Fund Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, refund any portion of Window 1 and Window 2 Funds not used in accordance with the applicable Fund Use Agreements, and such funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u28-31]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33\nContent: ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u178-181]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 194 to section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198\nContent: appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center. Return of Funds. Unexpended or Uncommitted Funding. Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, promptly return any portion of Window 1 and Window 2 Funds that is unexpended or uncommitted at the completion of a CGIAR Program or activities under the CGIAR Program for which it was provided (including approved extensions) or at the termination of a Financial Framework Agreement between the System Organization and a Center, unless decided otherwise by the System Council. Such returned funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u31-34]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 33 to section 'Window 3 Funds.' paragraph 36\nContent: The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u13-16]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 15 to section 'Use and administration of the Contributions' paragraph 18\nContent: In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational level, as may be adopted from time to time. Responsibilities over Window 1 and Window 2 Funds Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u22-25]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 24 to section 'Window 3 Funds.' paragraph 27\nContent: monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions. Window 3 Funds. Window 3 Funds are directed by Funders to individual Centers. Funders may designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u34-37]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 36 to section 'Window 3 Funds.' paragraph 39\nContent: in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center. Window 3 Side Agreements or Arrangements. Nothing in the Funding Agreements or Arrangements is intended to preclude Funders and Centers from entering into Window 3 Side Agreements or Arrangements in regard to the terms governing the administration and use of Window 3 Funds. Funders may choose to make a Contribution to a Center through Window 3 without entering into a Window 3 Side Agreement or Arrangement, provided that such Contribution is made without any additional conditions attached to it. Any Window 3 Side Agreement or Arrangement will be consistent with these Standard Provisions and substantially in the form of Schedule 1 (Form of Window 3 Side Agreement or Arrangement) attached to these Standard Provisions, as may be amended from time to time. Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4,\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u172-175]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 187 to section 'Acknowledgement of Funders' paragraph 191\nContent: Acknowledgement of Funders All communications products on CGIAR Research funded by Window 1, 2 and 3 Funds, whether online or in hard copy form (e.g., publications, press releases, newsletters, website stories, blogs, posters, etc.), must acknowledge support received from Funders in accordance with applicable CGIAR Policies and Procedures on branding and communication. Suspending Transfers of Funding from Window 1 and 2 Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u25-28]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 27 to section 'Window 3 Funds.' paragraph 30\nContent: designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization. Centers receiving Window 3 Funds are responsible for the use of such funds and will: ensure that Window 3 Funds are used exclusively for their intended purposes; ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements;\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u55-58]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 59 to section 'Financial, Economic and Administrative Standards' paragraph 62\nContent: Efficiency. The System Organization and each Center will, respectively: ensure that Window 1, 2 and 3 Funds are used with due regard to economy and efficiency, and that the highest standards of integrity in the administration of the funds are upheld; and ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures on cost allocation, which set forth the principles of allowability, allocability, and reasonableness. Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u46-49]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Cost Sharing Percentage' paragraph 49 to section 'Standard of care.' paragraph 53\nContent: Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund. Requirements on the Use of Window 1, 2 and 3 Funds CGIAR Policies and Procedures. The System Organization and each Center will, respectively ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures and the relevant entity's own policies and procedures. All CGIAR Policies and Procedures will be available on the System Organization's web site. Standard of care.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u184-189]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Misused Fund' paragraph 202 to section 'Inconsistency' paragraph 207\nContent: Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Inconsistency In the event of any inconsistency between the Cover Pages and these Standard Provisions, these Standard Provisions will prevail. Amendments Amendments These Standard Provisions may only be amended by approval of the System Council subject to concurrence of the Integrated Partnership Board. The System Organization will promptly notify the Funders and Centers in writing of any such amendments to these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u175-178]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 191 to section 'Acknowledgement of Funders' paragraph 194\nContent: Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement. Before taking such action under paragraph 13.1, the System Organization will notify the relevant Center in writing, and consult with the System Council as well as the relevant Center with a view to identify ways and means to manage the suspension and mitigate the impact on the implementation of CGIAR Research until such time that the suspension may be lifted. If such suspension is lifted by the System Organization, it will notify the relevant Center in writing. Request by a Funder. If a Funder has a credible concern: (a) that Window 1, 2 and 3 Funds are not used by a Center in accordance with the applicable Fund Use Agreement or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) of a non-compliance by a Center with any of its obligations under an applicable Fund Use Agreement, the Funder may request, through the System Council, the System Organization to review the specific concern and, as relevant, to take appropriate corrective action. The System Organization will report to the System Council on the outcome of the review and, as appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u4-7]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Introductory Provisions' paragraph 5 to section 'Introductory Provisions' paragraph 8\nContent: the Financial Framework Agreement between the System Organization and each Center with respect to Window 1, 2 and 3 Funds; and any Window 3 Side Agreement or Arrangement between a Funder and a Center with respect to Window 3 Funds. Interpretation of the Standard Provisions. Unless the context requires otherwise, the terms of these Standard Provisions governing the roles and responsibilities: between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization;\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u106-109]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Monitoring and Evaluations' paragraph 115 to section 'Monitoring' paragraph 118\nContent: Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder. If an individual Funder wishes to request, on an exceptional basis, a review or evaluation of any activities financed with Window 1 and Window 2 Funds, such Funder will consult with a designated representative from the System Organization on the most appropriate scope and terms of reference of such review or evaluation. The designated representative will assist in arranging for such review or evaluation in accordance with the applicable CGIAR Policies and Procedures. The costs of any such review or evaluation, including the internal costs of the System Organization or Center with respect to such review or evaluation, will be paid by the requesting Funder. The System Organization and each Center will, respectively collaborate on any monitoring or evaluations conducted in connection with CGIAR Research activities funded with Window 1, 2 and 3 Funds. Monitoring\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u58-61]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 62 to section 'Financial, Economic and Administrative Standards' paragraph 65\nContent: Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council. Procurement. In the event that consultants are employed or services or goods are procured with Window 1, 2 and 3 Funds, the System Organization and each Center will, respectively, ensure that the employment and supervision of such consultants and the procurement of such services or goods will be the responsibility of each entity employing or contracting such consultants or carrying out such procurement and will be conducted in conformity with applicable CGIAR Policies and Procedures on procurement, in line with the following basic principles of equal treatment and non-discrimination on grounds of nationality, competition, predictability, transparency, verifiability, and proportionality. No taxation. The System Organization and each Center will, respectively, use best efforts, to the extent allowed by applicable agreements, such as those signed with host governments, and applicable laws, to ensure that the use of Window 1, 2 and 3 Funds will be free from any taxation or fees imposed under local laws. Insurance. The System Organization and each Center will, respectively, maintain insurance coverage sufficient to cover the activities, risks, and potential omissions of the activities funded by Window 1, 2 and 3 Funds in accordance with generally accepted industry standards and as required by law.\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 24 part 4\nContent: the continuity of prior work that is less fit for purpose in the Program’s ToC. Windows 1, 2, 3 and bilateral funding: Approximately half of S4I’s 2025 funding is from Window 1, with the remainder from Window 2, including two $1.25 million designated W2 allocations specifically for AoWs 4 and 5. The PORB also reflects stronger alignment of Window 3 and bilateral funding with Program logic: in 2025, 47 mapped W3 and bilateral investments totaling $44.8 million support the Program ($0.42M, $26.47M, $1.55M, $15.37M, and $0.99M across AoWs 1 through 5, respectively), with 74% of these funds active in Africa, 19% in Asia, and 7% in Latin America. Engage and Empower (AoW 1): This AoW is allocated $2.98 million in W1/W2 funding and supported by $0.42 million in W3/bilaterals. It anchors S4I’s stakeholder demand intelligence 9 The section on AoW 4 in the PORB description highlights major inception period successes in leveraging Window 3 investments, with an anticipated, two-year bilateral investment in HLO 4.1 to transition TAAT into the Scaling Program that will support new work that was not part of the RIIs or NPS.\n\n---\n\n[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP03%20%2D%20Sustainable%20Animal%20and%20Aquatic%20Foods%2FSustainable%20Animal%20and%20Aquatic%20Foods%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP03%20%2D%20Sustainable%20Animal%20and%20Aquatic%20Foods&amp;p=true&amp;ga=1\nFile: Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf\nLocation: page 21 part 2\nContent: reducing producers' incomes and ability to invest in innovations; iv. Adverse national policy shifts regarding inclusion and equality; and v. Increased frequency of extreme climate events, which could undermine social progress and resilience. Please refer to the following link with the Program/Accelerator's full risk register. This link is open to ISDC colleagues and others will be granted access, on request. Category Risk Description Current Risk Level Target Risk Level Actions to Manage Risk Funding Reduced Window 1 &amp; 2 Funds Reduced Window 1 &amp; 2 funds caused by political changes from national governments which donate the bulk of CGIAR funds or other changes in donor priorities. This could result in outcome achievements failing to reach the"}]</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?\n\nContext:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u19-22]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24\nContent: Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u16-19]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21\nContent: Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:\n\n---\n\n[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2]\nLink: https://cgspace.cgiar.org/items/a88f8775-4ba9-41b6-9525-0d698d83cfb4\nFile: CGI21-507033-PORB-Policy Innovations.pdf\nLocation: page 72 part 2\nContent: of green bananas on her head.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u31-34]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 33 to section 'Window 3 Funds.' paragraph 36\nContent: The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u28-31]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33\nContent: ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p52pt1]\nLink: https://cgspace.cgiar.org/items/302ea600-c601-403e-8b29-e65bfa501e95\nFile: CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf\nLocation: page 52 part 1\nContent: A pig farmer in Tien Lu district, Hung\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 15 part 4\nContent: HLOs\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u70-73]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 74 to section 'Conflicts of Interest.' paragraph 77\nContent: with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and (viii) respect for the evolving capacities of children with disabilities. Conflicts of Interest. The System Organization and each Center will, respectively, take all necessary precautions to avoid or manage any Conflicts of Interest in all matters related to Window 1, 2 and 3 Funds.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p37pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 37 part 3\nContent: 2.2 Better designed emergency response in fragile settings - Government, humanitarian, and NGO actors use evidence and tools in fragile settings to guide emergency responses X X X X High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 180,781.00 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X Total AoW 2 budget 180,781.00 Area of Work 3:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 5 part 1\nContent: Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 31 part 2\nContent: protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u163-166]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Limitation of Liabilities' paragraph 176 to section 'No Additional Obligations' paragraph 180\nContent: In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u67-70]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 71 to section 'Ethical Standards' paragraph 74\nContent: Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 29 part 3\nContent: in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Mozambi que Surveys and KII CASP 2024 2026 100,000 Evaluate UNHCR’s Sustainable Land Management and Environmental Rehabilitation Project in Bangladesh Adam Savelli (CIAT) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 21 part 2\nContent: for the stud y End date for the stud y Study cost (USD) How related to past evaluations (SG or others) Gendered Labor Impacts of Herder-Related Violence in Nigeria Jeff Bloem (IFPRI) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Nigeria Household survey (panel) n/a 2024 2025 13,100 n/a Analyzing\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 3\nContent: Evaluation Recommendations are addressed by management. These responses are designed to ensure that Evaluations inform decision-making, enhance organizational effectiveness, promote learning, and strengthen accountability. They include time-bound commitments from management to implement Evaluation Recommendations and are systematically followed up as outlined in the CGIAR Evaluation Policy, which identifies follow-up as a critical component of the evaluative process.5 Since the launch of formal tracking in CGIAR’s 2022 Technical Report, the systematic monitoring and reporting of Management Response Actions has continued to evolve. This 2024 report provides information on (9) Evaluations and one (1) Evaluability Assessment (EA) completed during 2021-24 – all of which are available on the updated Evaluation and Management Response Actions Tracker. These Evaluations generated a total of 319 Recommendations and sub-Recommendations, underscoring the organization’s commitment to learning and continuous improvement. Evaluation title Date completed Date of Management Response No. of Recs. and sub-Recs No. of Actions Max. completion date for Actions Links to Evaluation Reports and Management Responses 2021 Synthesis of Learning from a Decade of CGIAR Research Programs June 2021 June 2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 17 part 2\nContent: 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. SP04 and SP078 will implement joint research on natural resources management and rangelands governance. Food Frontiers and Security SP04- Multifunctional Landscapes 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 4\nContent: 2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project Management Approaches and Fit-for-Purpose Information Products December 2022 December 2022 36 19 2024 • Advisory Report GENDER (Generating Evidence and New Directions for Equitable Results) Platform Evaluation December 2023 January 2024 22 21 2024 • Evaluation Report • Management Response CGIAR Genebank Platform Evaluation March 2024 March 2024 32 26 2027 • Evaluation Report • Management Response Evaluability Assessment Review of Four Regional Integrated Initiatives June 2024 June 2024 9 8 2026 • Evaluation Report • Management Response Genetic Innovation Science Group Evaluation August 2024 September 2024 42 28* 2030 • Evaluation Report • Management Response Resilient Agrifood Systems Science Group Evaluation August 2024 September 2024 26 22* 2027 • Evaluation Report • Management Response Systems Transformation Science Group Evaluation August 2024 September 2024 21 12* TBC • Evaluation Report • Management Response Total 319 248 Table 1. Evaluation details and associated Management Responses and Actions *The number of Management Response Actions for the Science Group Evaluations will likely change after Q2, 2025. May 2025 7 6 CGIAR Portfolio Practice Change (Type 3) Report\n\n---\n\n[ID: pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p10pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_Inception Report 30-06-2025.pdf\nLocation: page 10 part 2\nContent: use cases respond to clear demand from both\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-98</t>
   </si>
 </sst>
 </file>
@@ -2041,7 +2524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2084,7 +2567,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -2096,16 +2579,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G2" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I2" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2113,7 +2596,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -2125,16 +2608,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G3" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="H3" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2142,7 +2625,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -2154,16 +2637,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="H4" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="I4" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2171,7 +2654,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -2183,16 +2666,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="G5" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="H5" t="s">
-        <v>99</v>
+        <v>111</v>
       </c>
       <c r="I5" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2200,7 +2683,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -2212,16 +2695,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G6" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="H6" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="I6" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -2229,7 +2712,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -2241,16 +2724,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H7" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="I7" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -2258,7 +2741,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -2270,16 +2753,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G8" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="H8" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="I8" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2287,7 +2770,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -2299,16 +2782,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="G9" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="H9" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="I9" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2316,7 +2799,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -2328,16 +2811,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G10" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="H10" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="I10" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2345,7 +2828,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -2357,16 +2840,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G11" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H11" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I11" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2374,7 +2857,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -2386,16 +2869,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G12" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H12" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="I12" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2403,7 +2886,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -2415,16 +2898,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G13" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H13" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="I13" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2432,7 +2915,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -2444,16 +2927,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G14" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H14" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="I14" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2461,7 +2944,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C15">
         <v>100</v>
@@ -2473,16 +2956,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G15" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H15" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="I15" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2490,7 +2973,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -2502,16 +2985,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G16" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H16" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="I16" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2519,7 +3002,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -2531,16 +3014,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G17" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H17" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="I17" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2548,7 +3031,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -2560,16 +3043,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H18" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="I18" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2577,7 +3060,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -2589,16 +3072,16 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="G19" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H19" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I19" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2606,7 +3089,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -2618,16 +3101,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G20" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H20" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I20" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2635,7 +3118,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -2647,22 +3130,22 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G21" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H21" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I21" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J21" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="K21" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2670,7 +3153,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -2682,22 +3165,22 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G22" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H22" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I22" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J22" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="K22" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2705,7 +3188,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -2717,22 +3200,22 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G23" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H23" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I23" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J23" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="K23" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2740,7 +3223,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C24">
         <v>200</v>
@@ -2752,22 +3235,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G24" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="H24" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I24" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J24" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="K24" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2775,7 +3258,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C25">
         <v>200</v>
@@ -2787,22 +3270,22 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G25" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="H25" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="I25" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J25" t="s">
-        <v>152</v>
+        <v>171</v>
       </c>
       <c r="K25" t="s">
-        <v>161</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2810,7 +3293,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C26">
         <v>200</v>
@@ -2822,22 +3305,22 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G26" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="H26" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="I26" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="J26" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="K26" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2845,7 +3328,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C27">
         <v>200</v>
@@ -2857,22 +3340,22 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G27" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="H27" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="I27" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="J27" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="K27" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2880,7 +3363,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C28">
         <v>200</v>
@@ -2892,22 +3375,22 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G28" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="H28" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="I28" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="J28" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="K28" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2915,7 +3398,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C29">
         <v>200</v>
@@ -2927,22 +3410,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G29" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="H29" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="I29" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="J29" t="s">
-        <v>153</v>
+        <v>172</v>
       </c>
       <c r="K29" t="s">
-        <v>162</v>
+        <v>184</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2950,7 +3433,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -2962,22 +3445,22 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G30" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="H30" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I30" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="J30" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="K30" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2985,7 +3468,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -2997,22 +3480,22 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G31" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="H31" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="I31" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="J31" t="s">
-        <v>154</v>
+        <v>173</v>
       </c>
       <c r="K31" t="s">
-        <v>163</v>
+        <v>185</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -3020,7 +3503,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -3032,22 +3515,22 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G32" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H32" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="I32" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="J32" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K32" t="s">
-        <v>164</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -3055,7 +3538,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -3067,22 +3550,22 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G33" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H33" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J33" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K33" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -3090,7 +3573,7 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -3102,22 +3585,22 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G34" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H34" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J34" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K34" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -3125,7 +3608,7 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -3137,22 +3620,22 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G35" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H35" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J35" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K35" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3160,7 +3643,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -3172,22 +3655,22 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G36" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H36" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J36" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K36" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -3195,7 +3678,7 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -3207,22 +3690,22 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G37" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H37" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J37" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K37" t="s">
-        <v>165</v>
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -3230,7 +3713,7 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -3242,22 +3725,22 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G38" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="H38" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="J38" t="s">
-        <v>155</v>
+        <v>174</v>
       </c>
       <c r="K38" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -3265,7 +3748,7 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -3277,22 +3760,22 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G39" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H39" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I39" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J39" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K39" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -3300,7 +3783,7 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -3312,22 +3795,22 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G40" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H40" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I40" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J40" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K40" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -3335,7 +3818,7 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -3347,22 +3830,22 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G41" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H41" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I41" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J41" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K41" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -3370,7 +3853,7 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C42">
         <v>100</v>
@@ -3382,22 +3865,22 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G42" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H42" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I42" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J42" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K42" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -3405,7 +3888,7 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -3417,22 +3900,22 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G43" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H43" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="I43" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J43" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K43" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -3440,7 +3923,7 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -3452,22 +3935,22 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G44" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H44" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="I44" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J44" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K44" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -3484,13 +3967,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H45" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="K45" t="s">
-        <v>168</v>
+        <v>190</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3498,7 +3981,7 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -3510,22 +3993,22 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G46" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H46" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="I46" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J46" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K46" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3533,7 +4016,7 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -3545,22 +4028,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G47" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H47" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="I47" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J47" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K47" t="s">
-        <v>167</v>
+        <v>189</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3568,7 +4051,7 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -3580,22 +4063,22 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G48" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="H48" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="J48" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="K48" t="s">
-        <v>169</v>
+        <v>191</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3603,7 +4086,7 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C49">
         <v>200</v>
@@ -3615,22 +4098,22 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="G49" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="H49" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="J49" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="K49" t="s">
-        <v>170</v>
+        <v>192</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3638,7 +4121,7 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C50">
         <v>200</v>
@@ -3650,22 +4133,22 @@
         <v>1</v>
       </c>
       <c r="F50" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="G50" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H50" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="J50" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="K50" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3673,7 +4156,7 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C51">
         <v>200</v>
@@ -3685,22 +4168,22 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="G51" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H51" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="J51" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="K51" t="s">
-        <v>171</v>
+        <v>193</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3708,7 +4191,7 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C52">
         <v>200</v>
@@ -3720,22 +4203,22 @@
         <v>1</v>
       </c>
       <c r="F52" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G52" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="H52" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="J52" t="s">
-        <v>158</v>
+        <v>177</v>
       </c>
       <c r="K52" t="s">
-        <v>172</v>
+        <v>194</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3743,7 +4226,7 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C53">
         <v>200</v>
@@ -3755,22 +4238,22 @@
         <v>1</v>
       </c>
       <c r="F53" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G53" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="H53" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="J53" t="s">
-        <v>159</v>
+        <v>178</v>
       </c>
       <c r="K53" t="s">
-        <v>173</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3778,7 +4261,7 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C54">
         <v>200</v>
@@ -3790,22 +4273,22 @@
         <v>1</v>
       </c>
       <c r="F54" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G54" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="H54" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="J54" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="K54" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -3813,7 +4296,7 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C55">
         <v>200</v>
@@ -3825,22 +4308,22 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G55" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="H55" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="J55" t="s">
-        <v>160</v>
+        <v>179</v>
       </c>
       <c r="K55" t="s">
-        <v>174</v>
+        <v>196</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -3848,7 +4331,7 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C56">
         <v>200</v>
@@ -3860,22 +4343,197 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G56" t="s">
+        <v>102</v>
+      </c>
+      <c r="H56" t="s">
+        <v>150</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="J56" t="s">
+        <v>176</v>
+      </c>
+      <c r="K56" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11">
+      <c r="A57" t="s">
+        <v>66</v>
+      </c>
+      <c r="B57" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57">
+        <v>200</v>
+      </c>
+      <c r="D57">
+        <v>148</v>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+      <c r="F57" t="s">
+        <v>91</v>
+      </c>
+      <c r="G57" t="s">
+        <v>106</v>
+      </c>
+      <c r="H57" t="s">
+        <v>151</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J57" t="s">
+        <v>180</v>
+      </c>
+      <c r="K57" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11">
+      <c r="A58" t="s">
+        <v>67</v>
+      </c>
+      <c r="B58" t="s">
+        <v>82</v>
+      </c>
+      <c r="C58">
+        <v>200</v>
+      </c>
+      <c r="D58">
+        <v>148</v>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+      <c r="F58" t="s">
+        <v>92</v>
+      </c>
+      <c r="G58" t="s">
+        <v>106</v>
+      </c>
+      <c r="H58" t="s">
+        <v>152</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J58" t="s">
+        <v>180</v>
+      </c>
+      <c r="K58" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11">
+      <c r="A59" t="s">
+        <v>68</v>
+      </c>
+      <c r="B59" t="s">
+        <v>82</v>
+      </c>
+      <c r="C59">
+        <v>200</v>
+      </c>
+      <c r="D59">
+        <v>148</v>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+      <c r="F59" t="s">
         <v>93</v>
       </c>
-      <c r="H56" t="s">
-        <v>138</v>
-      </c>
-      <c r="I56" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="J56" t="s">
-        <v>157</v>
-      </c>
-      <c r="K56" t="s">
-        <v>175</v>
+      <c r="G59" t="s">
+        <v>106</v>
+      </c>
+      <c r="H59" t="s">
+        <v>153</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="J59" t="s">
+        <v>180</v>
+      </c>
+      <c r="K59" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11">
+      <c r="A60" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" t="s">
+        <v>83</v>
+      </c>
+      <c r="C60">
+        <v>200</v>
+      </c>
+      <c r="D60">
+        <v>200</v>
+      </c>
+      <c r="E60" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" t="s">
+        <v>91</v>
+      </c>
+      <c r="G60" t="s">
+        <v>107</v>
+      </c>
+      <c r="H60" t="s">
+        <v>154</v>
+      </c>
+      <c r="I60" t="s">
+        <v>169</v>
+      </c>
+      <c r="J60" t="s">
+        <v>181</v>
+      </c>
+      <c r="K60" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11">
+      <c r="A61" t="s">
+        <v>70</v>
+      </c>
+      <c r="B61" t="s">
+        <v>82</v>
+      </c>
+      <c r="C61">
+        <v>200</v>
+      </c>
+      <c r="D61">
+        <v>200</v>
+      </c>
+      <c r="E61" t="b">
+        <v>1</v>
+      </c>
+      <c r="F61" t="s">
+        <v>91</v>
+      </c>
+      <c r="G61" t="s">
+        <v>108</v>
+      </c>
+      <c r="H61" t="s">
+        <v>155</v>
+      </c>
+      <c r="I61" t="s">
+        <v>170</v>
+      </c>
+      <c r="J61" t="s">
+        <v>182</v>
+      </c>
+      <c r="K61" t="s">
+        <v>202</v>
       </c>
     </row>
   </sheetData>
@@ -3895,6 +4553,9 @@
     <hyperlink ref="I54" r:id="rId13"/>
     <hyperlink ref="I55" r:id="rId14"/>
     <hyperlink ref="I56" r:id="rId15"/>
+    <hyperlink ref="I57" r:id="rId16"/>
+    <hyperlink ref="I58" r:id="rId17"/>
+    <hyperlink ref="I59" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Generated new Q&A list with Python and achieved 98% accuracy
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="210">
   <si>
     <t>timestamp</t>
   </si>
@@ -229,6 +229,9 @@
     <t>2025-09-25T00:45:44.397869</t>
   </si>
   <si>
+    <t>2025-09-25T01:18:56.051769</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -266,6 +269,9 @@
   </si>
   <si>
     <t>Who holds fiduciary responsibility over Window 1 and Window 2 Funds?</t>
+  </si>
+  <si>
+    <t>Who has fiduciary responsibility over the Windows 1 and 2 funds, and what must they guarantee?</t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -346,6 +352,9 @@
   </si>
   <si>
     <t>docx:Standard Provisions 2026.docx:u19-22:0.155, docx:Standard Provisions 2026.docx:u16-19:0.145, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2:0.090, docx:Standard Provisions 2026.docx:u31-34:0.085, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1:0.078, docx:Standard Provisions 2026.docx:u28-31:0.078, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1:0.077, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1:0.075, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2:0.074, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p52pt1:0.069, pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4:0.067, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.067, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3:0.066, pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2:0.064, docx:Standard Provisions 2026.docx:u70-73:0.063, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p37pt3:0.062, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1:0.061, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.060, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.059, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3:0.057, docx:Standard Provisions 2026.docx:u163-166:0.057, docx:Standard Provisions 2026.docx:u67-70:0.056, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt3:0.055, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt2:0.053, pdf:Type3_2024Report.pdf:p6pt3:0.052, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3:0.052, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt2:0.051, pdf:Type3_2024Report.pdf:p6pt4:0.051, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p10pt2:0.051, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt3:0.051, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt3:0.049, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt4:0.048, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt2:0.048, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p35pt2:0.047, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p17pt2:0.047, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p31pt2:0.047, pdf:Genebanks_Inception Report 30-06-2025.pdf:p38pt1:0.046, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p6pt1:0.045, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4:0.045, pdf:Type3_2024Report.pdf:p3pt2:0.045, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt2:0.044, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt2:0.044, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p50pt4:0.044, pdf:Climate Action_Inception Report 30-06-2025.pdf:p22pt2:0.043, pdf:Type3_2024Report.pdf:p6pt2:0.043, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p19pt4:0.043, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p28pt2:0.043, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.043, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p1pt2:0.042, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.042, pdf:Type3_2024Report.pdf:p5pt1:0.042, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt3:0.041, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p26pt3:0.041, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p31pt3:0.041, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt4:0.041, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt4:0.041, docx:User Roles and Rules for the PRMS Reporting.docx:u4-7:0.040, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p30pt4:0.040, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p13pt4:0.039, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p20pt4:0.039, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p22pt3:0.039, pdf:Portfolio Narrative_2024.pdf:p29pt3:0.039, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p10pt2:0.039, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p51pt1:0.039, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt2:0.039, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.039, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt3:0.038, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p4pt4:0.038, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p45pt3:0.038, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt2:0.038, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt2:0.038, pdf:Portfolio Narrative_2024.pdf:p82pt2:0.038, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt1:0.038, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt3:0.038, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt3:0.038, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt2:0.038, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p24pt1:0.037, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p6pt2:0.037, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.037, pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt2:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p16pt4:0.037, pdf:Portfolio Narrative_2024.pdf:p89pt4:0.037, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.037, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt4:0.037, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.037, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p30pt1:0.037, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt2:0.037, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt2:0.036, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p4pt1:0.036, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p31pt4:0.036, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.036, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt2:0.036, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p22pt3:0.036, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p5pt3:0.036, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p8pt2:0.036, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p26pt4:0.035, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p31pt1:0.035, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.035, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt2:0.035, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p11pt4:0.035, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p12pt2:0.035, docx:Standard Provisions 2026.docx:u58-61:0.035, pdf:Portfolio Narrative_2024.pdf:p29pt4:0.035, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt3:0.035, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt4:0.034, pdf:CGIAR_ImpactReport_2022-24.pdf:p28pt1:0.034, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p26pt4:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt4:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p26pt3:0.034, pdf:Genebanks_Inception Report 30-06-2025.pdf:p15pt2:0.034, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt1:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p11pt2:0.034, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt4:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt1:0.034, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p7pt4:0.034, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p22pt4:0.034, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p1pt2:0.034, pdf:Climate Action_Inception Report 30-06-2025.pdf:p22pt3:0.034, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p18pt3:0.034, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p13pt2:0.034, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p36pt3:0.034, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p15pt4:0.034, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p17pt3:0.034, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p9pt4:0.034, pdf:Climate Action_Inception Report 30-06-2025.pdf:p17pt3:0.034, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p29pt1:0.034, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p9pt3:0.034, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p3pt2:0.034, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt2:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p10pt4:0.033, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt1:0.033, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p13pt2:0.033, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt1:0.033, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p4pt4:0.033, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.033, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p11pt2:0.033, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p12pt3:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.033, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p22pt2:0.033, pdf:Portfolio Narrative_2024.pdf:p17pt1:0.033, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt1:0.033, pdf:Climate Action_Inception Report 30-06-2025.pdf:p4pt3:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p35pt1:0.033, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p32pt2:0.033, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p33pt4:0.033, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p24pt4:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p3pt1:0.033, pdf:Portfolio Narrative_2024.pdf:p82pt3:0.033, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p13pt3:0.033, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p10pt2:0.033, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt4:0.033, pdf:Type3_2024Report.pdf:p7pt1:0.032, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p18pt1:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt2:0.032, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p26pt1:0.032, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p56pt3:0.032, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p6pt1:0.032, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p30pt4:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p32pt3:0.032, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p10pt2:0.032, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt1:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p9pt2:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt3:0.032, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt3:0.032, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt3:0.032, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p18pt4:0.032, pdf:Type3_2024Report.pdf:p8pt3:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt3:0.032, pdf:Portfolio Narrative_2024.pdf:p53pt4:0.032, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt3:0.032, pdf:Genebanks_Inception Report 30-06-2025.pdf:p17pt4:0.032, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt2:0.032, docx:Standard Provisions 2026.docx:u73-76:0.032, pdf:Portfolio Narrative_2024.pdf:p38pt4:0.032, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.032, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p53pt3:0.032, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p8pt1:0.032, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt2:0.032, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt1:0.031, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p22pt3:0.031, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt1:0.031, pdf:Type3_2024Report.pdf:p7pt4:0.031, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt3:0.031, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p23pt2:0.031, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p7pt2:0.031, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p4pt4:0.031, pdf:Portfolio Narrative_2024.pdf:p47pt4:0.031, docx:Standard Provisions 2026.docx:u4-7:0.031, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p12pt3:0.031, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt4:0.031, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p31pt3:0.031, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt4:0.031, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt4:0.031, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p14pt4:0.031, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p16pt2:0.031, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p13pt4:0.031, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt1:0.031, pdf:Climate Action_Inception Report 30-06-2025.pdf:p19pt3:0.031</t>
+  </si>
+  <si>
+    <t>docx:Standard Provisions 2026.docx:u19-22:0.500, docx:Standard Provisions 2026.docx:u16-19:0.437, docx:Standard Provisions 2026.docx:u28-31:0.324, docx:Standard Provisions 2026.docx:u31-34:0.319, docx:Standard Provisions 2026.docx:u181-184:0.262, docx:Standard Provisions 2026.docx:u13-16:0.242, docx:Standard Provisions 2026.docx:u178-181:0.234, docx:Standard Provisions 2026.docx:u22-25:0.214, docx:Standard Provisions 2026.docx:u172-175:0.211, docx:Standard Provisions 2026.docx:u4-7:0.200, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.198, docx:Standard Provisions 2026.docx:u46-49:0.196, docx:Standard Provisions 2026.docx:u55-58:0.195, docx:Standard Provisions 2026.docx:u25-28:0.191, docx:Standard Provisions 2026.docx:u34-37:0.182, docx:Standard Provisions 2026.docx:u163-166:0.181, docx:Standard Provisions 2026.docx:u58-61:0.179, docx:Standard Provisions 2026.docx:u106-109:0.167, docx:Standard Provisions 2026.docx:u175-178:0.167, docx:Standard Provisions 2026.docx:u184-189:0.160, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.159, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1:0.157, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4:0.156, docx:Standard Provisions 2026.docx:u67-70:0.155, docx:Standard Provisions 2026.docx:u157-160:0.154, docx:Standard Provisions 2026.docx:u43-46:0.148, docx:Standard Provisions 2026.docx:u70-73:0.147, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2:0.146, docx:Standard Provisions 2026.docx:u160-163:0.140, docx:Standard Provisions 2026.docx:u10-13:0.139, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.136, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt2:0.136, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p4pt4:0.134, docx:Standard Provisions 2026.docx:u112-115:0.133, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt3:0.132, docx:Standard Provisions 2026.docx:u103-106:0.132, docx:2025 Technical Reporting Information (Session 1).docx:u40-43:0.131, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.129, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt2:0.129, docx:Standard Provisions 2026.docx:u52-55:0.128, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p4pt1:0.127, pdf:Climate Action_Inception Report 30-06-2025.pdf:p30pt2:0.125, docx:Standard Provisions 2026.docx:u109-112:0.125, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt3:0.124, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.123, docx:Standard Provisions 2026.docx:u73-76:0.121, docx:Standard Provisions 2026.docx:u64-67:0.121, pdf:Climate Action_Inception Report 30-06-2025.pdf:p30pt3:0.120, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt2:0.118, docx:Standard Provisions 2026.docx:u37-40:0.118, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt1:0.118, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt2:0.118, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt4:0.118, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt2:0.118, docx:2025 Technical Reporting MELIA glossary.docx:u55-58:0.118, docx:Standard Provisions 2026.docx:u166-169:0.117, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt1:0.117, pdf:Type3_2024Report.pdf:p5pt1:0.116, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt2:0.116, docx:Standard Provisions 2026.docx:u97-100:0.116, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt4:0.116, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt2:0.115, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt2:0.115, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p2pt2:0.115, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt4:0.115, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt2:0.115, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt2:0.115, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt2:0.115, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt2:0.114, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt3:0.113, docx:Standard Provisions 2026.docx:u1-4:0.112, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.112, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt3:0.110, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt4:0.110, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.110, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p32pt1:0.108, pdf:Climate Action_Inception Report 30-06-2025.pdf:p16pt3:0.107, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt3:0.107, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p2pt1:0.107, docx:User Roles and Rules for the PRMS Reporting.docx:u4-7:0.106, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt2:0.105, docx:Standard Provisions 2026.docx:u61-64:0.105, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt3:0.104, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt2:0.103, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.103, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p30pt2:0.103, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt1:0.103, docx:Standard Provisions 2026.docx:u76-79:0.103, docx:User Roles and Rules for the PRMS Reporting.docx:u16-19:0.102, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt1:0.102, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.102, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt4:0.101, pdf:Genebanks_Inception Report 30-06-2025.pdf:p18pt1:0.101, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p18pt3:0.100, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt3:0.100, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.100, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4:0.099, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.099, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt4:0.099, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt4:0.098, docx:Standard Provisions 2026.docx:u100-103:0.097, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p25pt4:0.097, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt2:0.097, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p29pt2:0.097, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt2:0.096, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt1:0.096, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt2:0.095, docx:Standard Provisions 2026.docx:u148-151:0.095, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p19pt1:0.095, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p3pt3:0.095, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p11pt4:0.095, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.095, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p2pt1:0.095, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt1:0.094, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt1:0.094, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p8pt4:0.094, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt1:0.094, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.094, docx:Standard Provisions 2026.docx:u133-136:0.094, docx:Standard Provisions 2026.docx:u130-133:0.093, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt1:0.093, docx:Standard Provisions 2026.docx:u88-91:0.093, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt1:0.093, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt1:0.093, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt1:0.093, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p15pt1:0.093, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p24pt1:0.093, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt3:0.093, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p13pt4:0.093, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt3:0.093, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p32pt4:0.092, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt1:0.092, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt2:0.092, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p19pt2:0.092, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt2:0.092, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.092, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p20pt4:0.092, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt4:0.092, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt1:0.091, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt1:0.091, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt3:0.091, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.091, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.091, pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt3:0.091, pptx:Information Session on 2025 Technical Reporting.pptx:s12pt3:0.091, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt1:0.091, pdf:Portfolio Narrative_2024.pdf:p2pt4:0.091, docx:Standard Provisions 2026.docx:u151-154:0.090, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt1:0.090, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt1:0.090, docx:Guidance on reporting outputs or outcomes.docx:u10-13:0.090, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p15pt2:0.089, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt4:0.089, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt2:0.089, docx:Standard Provisions 2026.docx:u145-148:0.089, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt2:0.089, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt3:0.089, docx:Standard Provisions 2026.docx:u82-85:0.089, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p35pt3:0.088, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt1:0.088, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt1:0.088, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.088, pdf:Portfolio Narrative_2024.pdf:p82pt2:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u46-49:0.088, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt2:0.088, pdf:Genebanks_Inception Report 30-06-2025.pdf:p9pt2:0.088, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt3:0.088, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p2pt1:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt2:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p35pt4:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u25-28:0.088, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt2:0.087, docx:Standard Provisions 2026.docx:u94-97:0.087, pdf:Genebanks_Inception Report 30-06-2025.pdf:p24pt2:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4:0.087, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.087, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt3:0.087, docx:Standard Provisions 2026.docx:u169-172:0.086, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.086, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p32pt2:0.086, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt2:0.086, pdf:Genebanks_Inception Report 30-06-2025.pdf:p8pt3:0.086, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p5pt2:0.086, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p23pt1:0.086, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt2:0.086, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.086, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.085, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p25pt3:0.085, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p4pt2:0.085, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p40pt4:0.084, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p33pt4:0.084, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt1:0.084, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt3:0.084, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p31pt2:0.084, docx:Standard Provisions 2026.docx:u85-88:0.084, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p2pt1:0.084, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p2pt1:0.084, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.084, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p24pt4:0.084</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -734,6 +743,13 @@
 Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19</t>
   </si>
   <si>
+    <t>The fiduciary responsibility over the Window 1 and Window 2 funds lies with the System Organization, which is accountable to the Funders, while each Center has fiduciary responsibility toward the System Organization for the funds it receives. They must guarantee that these funds are used exclusively for their intended purposes and administered in accordance with the CGIAR System Charter, the CGIAR System Framework, and the applicable Fund Use Agreements. Additionally, they are required to monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by these windows. 
+Sources:
+File — Location — Cited IDs
+docx:Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — u19-22
+docx:Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — u16-19</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -777,6 +793,9 @@
   </si>
   <si>
     <t>Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22, Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19, https://cgspace.cgiar.org/items/a88f8775-4ba9-41b6-9525-0d698d83cfb4 — page 72 part 2 — pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2</t>
+  </si>
+  <si>
+    <t>Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22, Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19, Standard Provisions 2026.docx — section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33 — docx:Standard Provisions 2026.docx:u28-31</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -2096,6 +2115,100 @@
 evaluate the returns to R&amp;D investments in different regions and different crop and anima</t>
   </si>
   <si>
+    <t>[ID: docx:Standard Provisions 2026.docx:u19-22]
+Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.
+---
+[ID: docx:Standard Provisions 2026.docx:u16-19]
+Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:
+---
+[ID: docx:Standard Provisions 2026.docx:u28-31]
+ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.
+---
+[ID: docx:Standard Provisions 2026.docx:u31-34]
+The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such
+---
+[ID: docx:Standard Provisions 2026.docx:u181-184]
+Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Misused Fund Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, refund any portion of Window 1 and Window 2 Funds not used in accordance with the applicable Fund Use Agreements, and such funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.
+---
+[ID: docx:Standard Provisions 2026.docx:u13-16]
+In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational level, as may be adopted from time to time. Responsibilities over Window 1 and Window 2 Funds Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research.
+---
+[ID: docx:Standard Provisions 2026.docx:u178-181]
+appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center. Return of Funds. Unexpended or Uncommitted Funding. Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, promptly return any portion of Window 1 and Window 2 Funds that is unexpended or uncommitted at the completion of a CGIAR Program or activities under the CGIAR Program for which it was provided (including approved extensions) or at the termination of a Financial Framework Agreement between the System Organization and a Center, unless decided otherwise by the System Council. Such returned funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.
+---
+[ID: docx:Standard Provisions 2026.docx:u22-25]
+monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions. Window 3 Funds. Window 3 Funds are directed by Funders to individual Centers. Funders may designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization.
+---
+[ID: docx:Standard Provisions 2026.docx:u172-175]
+Acknowledgement of Funders All communications products on CGIAR Research funded by Window 1, 2 and 3 Funds, whether online or in hard copy form (e.g., publications, press releases, newsletters, website stories, blogs, posters, etc.), must acknowledge support received from Funders in accordance with applicable CGIAR Policies and Procedures on branding and communication. Suspending Transfers of Funding from Window 1 and 2 Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement.
+---
+[ID: docx:Standard Provisions 2026.docx:u4-7]
+the Financial Framework Agreement between the System Organization and each Center with respect to Window 1, 2 and 3 Funds; and any Window 3 Side Agreement or Arrangement between a Funder and a Center with respect to Window 3 Funds. Interpretation of the Standard Provisions. Unless the context requires otherwise, the terms of these Standard Provisions governing the roles and responsibilities: between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization;
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]
+protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the
+---
+[ID: docx:Standard Provisions 2026.docx:u46-49]
+Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund. Requirements on the Use of Window 1, 2 and 3 Funds CGIAR Policies and Procedures. The System Organization and each Center will, respectively ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures and the relevant entity's own policies and procedures. All CGIAR Policies and Procedures will be available on the System Organization's web site. Standard of care.
+---
+[ID: docx:Standard Provisions 2026.docx:u55-58]
+Efficiency. The System Organization and each Center will, respectively: ensure that Window 1, 2 and 3 Funds are used with due regard to economy and efficiency, and that the highest standards of integrity in the administration of the funds are upheld; and ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures on cost allocation, which set forth the principles of allowability, allocability, and reasonableness. Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council.
+---
+[ID: docx:Standard Provisions 2026.docx:u25-28]
+designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization. Centers receiving Window 3 Funds are responsible for the use of such funds and will: ensure that Window 3 Funds are used exclusively for their intended purposes; ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements;
+---
+[ID: docx:Standard Provisions 2026.docx:u34-37]
+in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center. Window 3 Side Agreements or Arrangements. Nothing in the Funding Agreements or Arrangements is intended to preclude Funders and Centers from entering into Window 3 Side Agreements or Arrangements in regard to the terms governing the administration and use of Window 3 Funds. Funders may choose to make a Contribution to a Center through Window 3 without entering into a Window 3 Side Agreement or Arrangement, provided that such Contribution is made without any additional conditions attached to it. Any Window 3 Side Agreement or Arrangement will be consistent with these Standard Provisions and substantially in the form of Schedule 1 (Form of Window 3 Side Agreement or Arrangement) attached to these Standard Provisions, as may be amended from time to time. Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4,
+---
+[ID: docx:Standard Provisions 2026.docx:u163-166]
+In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations
+---
+[ID: docx:Standard Provisions 2026.docx:u58-61]
+Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council. Procurement. In the event that consultants are employed or services or goods are procured with Window 1, 2 and 3 Funds, the System Organization and each Center will, respectively, ensure that the employment and supervision of such consultants and the procurement of such services or goods will be the responsibility of each entity employing or contracting such consultants or carrying out such procurement and will be conducted in conformity with applicable CGIAR Policies and Procedures on procurement, in line with the following basic principles of equal treatment and non-discrimination on grounds of nationality, competition, predictability, transparency, verifiability, and proportionality. No taxation. The System Organization and each Center will, respectively, use best efforts, to the extent allowed by applicable agreements, such as those signed with host governments, and applicable laws, to ensure that the use of Window 1, 2 and 3 Funds will be free from any taxation or fees imposed under local laws. Insurance. The System Organization and each Center will, respectively, maintain insurance coverage sufficient to cover the activities, risks, and potential omissions of the activities funded by Window 1, 2 and 3 Funds in accordance with generally accepted industry standards and as required by law.
+---
+[ID: docx:Standard Provisions 2026.docx:u106-109]
+Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder. If an individual Funder wishes to request, on an exceptional basis, a review or evaluation of any activities financed with Window 1 and Window 2 Funds, such Funder will consult with a designated representative from the System Organization on the most appropriate scope and terms of reference of such review or evaluation. The designated representative will assist in arranging for such review or evaluation in accordance with the applicable CGIAR Policies and Procedures. The costs of any such review or evaluation, including the internal costs of the System Organization or Center with respect to such review or evaluation, will be paid by the requesting Funder. The System Organization and each Center will, respectively collaborate on any monitoring or evaluations conducted in connection with CGIAR Research activities funded with Window 1, 2 and 3 Funds. Monitoring
+---
+[ID: docx:Standard Provisions 2026.docx:u175-178]
+Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement. Before taking such action under paragraph 13.1, the System Organization will notify the relevant Center in writing, and consult with the System Council as well as the relevant Center with a view to identify ways and means to manage the suspension and mitigate the impact on the implementation of CGIAR Research until such time that the suspension may be lifted. If such suspension is lifted by the System Organization, it will notify the relevant Center in writing. Request by a Funder. If a Funder has a credible concern: (a) that Window 1, 2 and 3 Funds are not used by a Center in accordance with the applicable Fund Use Agreement or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) of a non-compliance by a Center with any of its obligations under an applicable Fund Use Agreement, the Funder may request, through the System Council, the System Organization to review the specific concern and, as relevant, to take appropriate corrective action. The System Organization will report to the System Council on the outcome of the review and, as appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center.
+---
+[ID: docx:Standard Provisions 2026.docx:u184-189]
+Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Inconsistency In the event of any inconsistency between the Cover Pages and these Standard Provisions, these Standard Provisions will prevail. Amendments Amendments These Standard Provisions may only be amended by approval of the System Council subject to concurrence of the Integrated Partnership Board. The System Organization will promptly notify the Funders and Centers in writing of any such amendments to these Standard Provisions.
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]
+Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results
+---
+[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4]
+the continuity of prior work that is less fit for purpose in the Program’s ToC. Windows 1, 2, 3 and bilateral funding: Approximately half of S4I’s 2025 funding is from Window 1, with the remainder from Window 2, including two $1.25 million designated W2 allocations specifically for AoWs 4 and 5. The PORB also reflects stronger alignment of Window 3 and bilateral funding with Program logic: in 2025, 47 mapped W3 and bilateral investments totaling $44.8 million support the Program ($0.42M, $26.47M, $1.55M, $15.37M, and $0.99M across AoWs 1 through 5, respectively), with 74% of these funds active in Africa, 19% in Asia, and 7% in Latin America. Engage and Empower (AoW 1): This AoW is allocated $2.98 million in W1/W2 funding and supported by $0.42 million in W3/bilaterals. It anchors S4I’s stakeholder demand intelligence 9 The section on AoW 4 in the PORB description highlights major inception period successes in leveraging Window 3 investments, with an anticipated, two-year bilateral investment in HLO 4.1 to transition TAAT into the Scaling Program that will support new work that was not part of the RIIs or NPS.
+---
+[ID: docx:Standard Provisions 2026.docx:u67-70]
+Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and
+---
+[ID: docx:Standard Provisions 2026.docx:u157-160]
+Change in Reporting Requirements. Unless decided otherwise by the System Council and/or the Integrated Partnership Board as the case may be, any change in the form or substance or periodicity of a technical or financial report will become effective only in the following calendar year. Additional Audits / Financial Reviews / Technical Reporting Funders will manage their audits, financial reviews and technical reporting with respect to the Window 1, 2 and 3 Funds collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to require duplicative reporting, provided that a Funder may require supplemental audits, financial reviews and technical reporting with respect to Window 3 Funds pursuant to its Window 3 Side Agreement or Arrangement, the costs of which would be paid by the requesting Funder. If a Funder wishes to request, on an exceptional basis, that the System Organization or a Center has an external audit or provides additional financial reviews or technical reports with respect to Window 1 and Window 2 Funds, and the requesting Funder has a statutory, regulatory or policy environment requiring such Funder's ability to make such a request unilaterally, such Funder will decide with the System Organization or the relevant Center on the most appropriate scope and terms of such audit, review or reporting. The costs of which, including the internal costs of the System Organization or any Center with respect to such additional audits, reviews or reporting, will be paid by the requesting Funder.
+---
+[ID: docx:Standard Provisions 2026.docx:u43-46]
+The Cost Sharing Percentage or CSP will be collected by the System Organization in accordance with applicable CGIAR Policies and Procedures on System Costs financing. Until and unless amended by CGIAR Policies and Procedures on System Costs financing, Centers will pay the CSP to the System Organization on any Bilateral Funding received for the implementation of CGIAR Research unless this requirement is exceptionally waived by the System Council. The System Organization will transfer the corresponding funds to the Trust Fund. Unless otherwise agreed by the System Council, if a Center does not pay any CSP which is due, the amount of such CSP which is due may be offset, after the Center has been adequately consulted, against Window 1 Funds that are otherwise to be disbursed to such Center. Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund.
+---
+[ID: docx:Standard Provisions 2026.docx:u70-73]
+with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and (viii) respect for the evolving capacities of children with disabilities. Conflicts of Interest. The System Organization and each Center will, respectively, take all necessary precautions to avoid or manage any Conflicts of Interest in all matters related to Window 1, 2 and 3 Funds.
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2]
+reducing producers' incomes and ability to invest in innovations; iv. Adverse national policy shifts regarding inclusion and equality; and v. Increased frequency of extreme climate events, which could undermine social progress and resilience. Please refer to the following link with the Program/Accelerator's full risk register. This link is open to ISDC colleagues and others will be granted access, on request. Category Risk Description Current Risk Level Target Risk Level Actions to Manage Risk Funding Reduced Window 1 &amp; 2 Funds Reduced Window 1 &amp; 2 funds caused by political changes from national governments which donate the bulk of CGIAR funds or other changes in donor priorities. This could result in outcome achievements failing to reach the
+---
+[ID: docx:Standard Provisions 2026.docx:u160-163]
+If a Funder wishes to request, on an exceptional basis, that the System Organization or a Center has an external audit or provides additional financial reviews or technical reports with respect to Window 1 and Window 2 Funds, and the requesting Funder has a statutory, regulatory or policy environment requiring such Funder's ability to make such a request unilaterally, such Funder will decide with the System Organization or the relevant Center on the most appropriate scope and terms of such audit, review or reporting. The costs of which, including the internal costs of the System Organization or any Center with respect to such additional audits, reviews or reporting, will be paid by the requesting Funder. The System Organization and each Center will, respectively, collaborate on any audits, financial reviews or technical reporting conducted in connection with CGIAR Research activities. Limitation of Liabilities In providing funds under:
+---
+[ID: docx:Standard Provisions 2026.docx:u10-13]
+Use and administration of the Contributions General Provisions in Respect of the Contributions The Contributions, including the funds, assets and receipts thereof, held in the Trust Fund are administered in accordance with the terms of the CGIAR Trustee Agreement and each Contribution Agreement or Arrangement. In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of chan</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -2154,6 +2267,9 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: ¿Quién tiene la responsabilidad fiduciaria sobre los fondos de Ventanas 1 y 2 y qué debe garantizar?\n\nContext:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u19-22]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24\nContent: Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u16-19]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21\nContent: Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:\n\n---\n\n[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p72pt2]\nLink: https://cgspace.cgiar.org/items/a88f8775-4ba9-41b6-9525-0d698d83cfb4\nFile: CGI21-507033-PORB-Policy Innovations.pdf\nLocation: page 72 part 2\nContent: of green bananas on her head.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u31-34]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 33 to section 'Window 3 Funds.' paragraph 36\nContent: The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 1\nContent: Genebanks Accelerator Inception Report 21 ● GCDT-Long-term conservation and sustainable use of plant genetic resources (Alliance Bioversity - CIAT) ● 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales ● P-1560-DGUL-Andean Crop Diversity for Climate Change ● 1571-FAO0 - Youth, Citizen Science and E-commerce: scaling integrated conservation solutions and farmers’ rights by connecting key diversity hotspots: Bolivia, Chile, and Peru ● P-1530-GIZ0-Construction and implementation of a new Cryobank ● Conservation of ICRISAT genetic resources for food and nutrition security in the semi -arid tropics The following Genebanks projects were erroneously listed as belonging to other Science Programs/Accelerators: ● 1572-MIPO (CIP) Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP, a través de la Bioeconomía y los Alimentos Funcionales (Better Diets and Nutrition) ● P-1560-DGUL (CIP)-Andean Crop Diversity for Climate Change (Better Diets and Nutrition) ● Conservation of ICRISAT genetic resources for\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u28-31]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33\nContent: ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 1\nContent: CGIAR | July 2025 Plan of results and budget 2025 | W3 Mapping | Page 9 of 44 W3 Mapping W3/Bilateral project mapping to Food Frontiers and Security W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD 1572-MIPO Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p11pt1]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 11 part 1\nContent: CGIAR | August 2025 Plan of results and budget 2025 | W3 Mapping | Page 11 of 52 W3/Bilateral project mapping to P/As W3/Bilateral project name Center Area of Work Title and Number High level output or Outcome (If Available) Total AoW Proposed W3/Bilateral budget (Jan- Dec 2025), USD Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo- Puno CIP Strengthening Capacity for In Situ and Ex Situ Conservation\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p9pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 9 part 2\nContent: el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.4.4 Healthy diets - Innovations, adaptation of tools and assessments, and evidence generation to support interventions for improving diet quality for urban residents $84,231 P-1529-UNGP-Technical Assistance for Sweetpotato processing International Potato Center / Centro Internacional de la Papa Urban Food Systems - AOW3 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p52pt1]\nLink: https://cgspace.cgiar.org/items/302ea600-c601-403e-8b29-e65bfa501e95\nFile: CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf\nLocation: page 52 part 1\nContent: A pig farmer in Tien Lu district, Hung\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p22pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 22 part 4\nContent: nevertheless important for the core functions of the genebanks as well as to track relevant indicators associated with the Accelerator’s theory of change. • Long Term Partnership Grant for conservation of the rice biodiversity at AfricaRice genebank (AfricaRice) • Long Term Partnership Grant (CIP) • Fortalecimiento de la conservación y uso sostenible de variedades locales de raíces y tubérculos andinos libres de enfermedades en la Zona de Agrobiodiversidad Andenes de Cuyocuyo - Puno (CIP) • Long Term Partnership Agreement (ICARDA) • Providing for the long-term funding of ex situ collections of germplasm (Bioversity) • Long Term Partnership Grant (ICRISAT) • Defining new phynotypes for forage and crop residue improvement based on rumen function and greenhouse gas emissions (UK-CGIAR) Finally, there are projects which are crucial to the work of Genebanks but were either not assigned to a Science Program/Accelerator during the mapping exercise, or that have no budget assigned to the Genebanks but are still relevant in terms of work and objectives for the Genebanks team.\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 15 part 4\nContent: HLOs\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p24pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 24 part 3\nContent: business models for circular bioeconomy, integrating organic waste recycling and wastewater reuse for urban production United Nations High Commissioner for Refugees, Kanya Dairy Board, Global Alliance for Improved Nutrition, Food and Agriculture Organization of the United Nations, Work for Better Bangladesh Trust, Dhaka North City Corporation, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, Welthungerhilfe, Consortium for Health, Environment, and Development / Consorcio por la Salud, Ambiente y Desarrollo, Food and Nutrition Research Institute Philippines, Quezon City University, Local Government of Quezon City (Philippines), Kenya Dairy Board, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina International Livestock Research Institute 3.3.3 Informal food markets - Guidelines, innovations,\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p10pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 10 part 2\nContent: - 1.1. Crop Trust signs Long-Term Partnership Agreements with CGIAR Intermediate Outcome - 1.2. CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness\" 411,914 \"Impulsando la Agroindustria Rural y el Uso de la Diversidad del Yacón conservada en Pataz y CIP , a través de la Bioeconomía y los Alimentos Funcionales 1572-MIPO\" CIP Strategic User Engagement (AOW02) High Level Output 2.2. Enhanced germplasm information for more precise accession targeting 84,231 \"Andean Crop Diversity for Climate Change P-1560-DGUL\" CIP Strategic User Engagement (AOW02) High Level Ouput 2.2 Enhanced germplasm information for more precise accession targeting 674,036 \"Youth, Citizen Science and E-commerce:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u70-73]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 74 to section 'Conflicts of Interest.' paragraph 77\nContent: with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and (viii) respect for the evolving capacities of children with disabilities. Conflicts of Interest. The System Organization and each Center will, respectively, take all necessary precautions to avoid or manage any Conflicts of Interest in all matters related to Window 1, 2 and 3 Funds.\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p37pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 37 part 3\nContent: 2.2 Better designed emergency response in fragile settings - Government, humanitarian, and NGO actors use evidence and tools in fragile settings to guide emergency responses X X X X High-Level Outputs 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. X X X X 180,781.00 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis X X X X Total AoW 2 budget 180,781.00 Area of Work 3:\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt1]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 1\nContent: Plan of results and budget 2025 | W3 Mapping | Page 22 of 44 July 2025 | CGIAR Partners (CRAs, sub-grant agreement, LoI, MoU ) Partner Center Area of Work Title and Number High level output (If Available) National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, RUAF Foundation, Alliance of Bioversity and CIAT - Headquarter (Bioversity International) International Potato Center / Centro Internacional de la Papa Future Food Systems Lab - AOW1 1.1.1 Envisioning Food System Futures - Tools and evidence for policymakers and partners to navigate emerging trends and future scenarios within relevant food systems. The\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 5 part 1\nContent: Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 31 part 2\nContent: protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p23pt3]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 23 part 3\nContent: Agrifood Systems Federación de Cafeteros del Valle - Colombia CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems Asociación de Desarrollo Integral de la parte alta de Zacapa (ADIPAZ) - Guatemala CIAT Contracted AoW 2 - Pathways to Scale in Agrifood Systems Universidad de San Carlos de Guatemala (USAC) - Guatemala CIAT Potential AoW 2 - Pathways to Scale in Agrifood Systems AoW 5 - Learning for Impact World Food Program - Guatemala CIAT Potential AoW 2\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u163-166]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Limitation of Liabilities' paragraph 176 to section 'No Additional Obligations' paragraph 180\nContent: In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u67-70]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 71 to section 'Ethical Standards' paragraph 74\nContent: Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p29pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 29 part 3\nContent: in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Mozambi que Surveys and KII CASP 2024 2026 100,000 Evaluate UNHCR’s Sustainable Land Management and Environmental Rehabilitation Project in Bangladesh Adam Savelli (CIAT) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 21 part 2\nContent: for the stud y End date for the stud y Study cost (USD) How related to past evaluations (SG or others) Gendered Labor Impacts of Herder-Related Violence in Nigeria Jeff Bloem (IFPRI) I-OC 2.2 Better designed emergen cy response in fragile settings Respond Policy change instance s and Quantity of new innovatio n uses identified Nigeria Household survey (panel) n/a 2024 2025 13,100 n/a Analyzing\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 3\nContent: Evaluation Recommendations are addressed by management. These responses are designed to ensure that Evaluations inform decision-making, enhance organizational effectiveness, promote learning, and strengthen accountability. They include time-bound commitments from management to implement Evaluation Recommendations and are systematically followed up as outlined in the CGIAR Evaluation Policy, which identifies follow-up as a critical component of the evaluative process.5 Since the launch of formal tracking in CGIAR’s 2022 Technical Report, the systematic monitoring and reporting of Management Response Actions has continued to evolve. This 2024 report provides information on (9) Evaluations and one (1) Evaluability Assessment (EA) completed during 2021-24 – all of which are available on the updated Evaluation and Management Response Actions Tracker. These Evaluations generated a total of 319 Recommendations and sub-Recommendations, underscoring the organization’s commitment to learning and continuous improvement. Evaluation title Date completed Date of Management Response No. of Recs. and sub-Recs No. of Actions Max. completion date for Actions Links to Evaluation Reports and Management Responses 2021 Synthesis of Learning from a Decade of CGIAR Research Programs June 2021 June 2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p22pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 22 part 3\nContent: at strengthening resilience in frontier geographies Council for Scientific and Industrial Research (Ghana), Welthungerhilfe, International Potato Center / Centro Internacional de la Papa, National Agrarian University La Molina/ Universidad Nacional Agraria La Molina, World Food Programme International Water Management Institute 1.3.3 Entrepreneurship Support Program - Technical and business training programs delivered to select number of innovators and entrepreneurs to develop and scale high-potential innovations for resource- constrained food systems GISSE, Mali, UNHCR, Red Cross Red Crescent Climate Centre, Nigerian Ministry of Humanitarian Affairs, ActionAid International, University of Bamako, International Organization for Migration, Government of Jordan, Alliance of Bioversity and\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p17pt2]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-9803-398b74cab543\nFile: CGI21-507031-PORB-Food Frontiers and Security.pdf\nLocation: page 17 part 2\nContent: 2.1.1 Prevent - Guidance on anticipatory action and disaster risk reduction (DRR) for FCA food systems that showcase impacts and scalability. SP04 and SP078 will implement joint research on natural resources management and rangelands governance. Food Frontiers and Security SP04- Multifunctional Landscapes 2.2.2 Respond - Guidance to improve the effectiveness of humanitarian responses to benefit individuals and communities affected by ongoing conflict and crisis\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p6pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 6 part 4\nContent: 2022 41 41 2024 • Synthesis of Learning • Management Response Evaluation of CGIAR Platform for Big Data in Agriculture December 2021 February 2022 43 36 2030 • Evaluation Report • Management Response Evaluation of CGIAR Excellence in Breeding Platform April 2022 May 2022 47 35 2024 • Evaluation Report • Management Response Study of the PRMS Project Management Approaches and Fit-for-Purpose Information Products December 2022 December 2022 36 19 2024 • Advisory Report GENDER (Generating Evidence and New Directions for Equitable Results) Platform Evaluation December 2023 January 2024 22 21 2024 • Evaluation Report • Management Response CGIAR Genebank Platform Evaluation March 2024 March 2024 32 26 2027 • Evaluation Report • Management Response Evaluability Assessment Review of Four Regional Integrated Initiatives June 2024 June 2024 9 8 2026 • Evaluation Report • Management Response Genetic Innovation Science Group Evaluation August 2024 September 2024 42 28* 2030 • Evaluation Report • Management Response Resilient Agrifood Systems Science Group Evaluation August 2024 September 2024 26 22* 2027 • Evaluation Report • Management Response Systems Transformation Science Group Evaluation August 2024 September 2024 21 12* TBC • Evaluation Report • Management Response Total 319 248 Table 1. Evaluation details and associated Management Responses and Actions *The number of Management Response Actions for the Science Group Evaluations will likely change after Q2, 2025. May 2025 7 6 CGIAR Portfolio Practice Change (Type 3) Report\n\n---\n\n[ID: pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p10pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_Inception Report 30-06-2025.pdf\nLocation: page 10 part 2\nContent: use cases respond to clear demand from both\n\n---\n\n[ID: pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p40pt3]\nLink: https://cgspace.cgiar.org/items/3271720b-98a5-4bcb-98</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who has fiduciary responsibility over the Windows 1 and 2 funds, and what must they guarantee?\n\nContext:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u19-22]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24\nContent: Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u16-19]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21\nContent: Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u28-31]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33\nContent: ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u31-34]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 33 to section 'Window 3 Funds.' paragraph 36\nContent: The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u181-184]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198 to section 'Misused Fund' paragraph 202\nContent: Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Misused Fund Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, refund any portion of Window 1 and Window 2 Funds not used in accordance with the applicable Fund Use Agreements, and such funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u13-16]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 15 to section 'Use and administration of the Contributions' paragraph 18\nContent: In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational level, as may be adopted from time to time. Responsibilities over Window 1 and Window 2 Funds Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u178-181]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 194 to section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198\nContent: appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center. Return of Funds. Unexpended or Uncommitted Funding. Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, promptly return any portion of Window 1 and Window 2 Funds that is unexpended or uncommitted at the completion of a CGIAR Program or activities under the CGIAR Program for which it was provided (including approved extensions) or at the termination of a Financial Framework Agreement between the System Organization and a Center, unless decided otherwise by the System Council. Such returned funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u22-25]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 24 to section 'Window 3 Funds.' paragraph 27\nContent: monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions. Window 3 Funds. Window 3 Funds are directed by Funders to individual Centers. Funders may designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u172-175]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 187 to section 'Acknowledgement of Funders' paragraph 191\nContent: Acknowledgement of Funders All communications products on CGIAR Research funded by Window 1, 2 and 3 Funds, whether online or in hard copy form (e.g., publications, press releases, newsletters, website stories, blogs, posters, etc.), must acknowledge support received from Funders in accordance with applicable CGIAR Policies and Procedures on branding and communication. Suspending Transfers of Funding from Window 1 and 2 Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u4-7]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Introductory Provisions' paragraph 5 to section 'Introductory Provisions' paragraph 8\nContent: the Financial Framework Agreement between the System Organization and each Center with respect to Window 1, 2 and 3 Funds; and any Window 3 Side Agreement or Arrangement between a Funder and a Center with respect to Window 3 Funds. Interpretation of the Standard Provisions. Unless the context requires otherwise, the terms of these Standard Provisions governing the roles and responsibilities: between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization;\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 31 part 2\nContent: protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u46-49]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Cost Sharing Percentage' paragraph 49 to section 'Standard of care.' paragraph 53\nContent: Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund. Requirements on the Use of Window 1, 2 and 3 Funds CGIAR Policies and Procedures. The System Organization and each Center will, respectively ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures and the relevant entity's own policies and procedures. All CGIAR Policies and Procedures will be available on the System Organization's web site. Standard of care.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u55-58]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 59 to section 'Financial, Economic and Administrative Standards' paragraph 62\nContent: Efficiency. The System Organization and each Center will, respectively: ensure that Window 1, 2 and 3 Funds are used with due regard to economy and efficiency, and that the highest standards of integrity in the administration of the funds are upheld; and ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures on cost allocation, which set forth the principles of allowability, allocability, and reasonableness. Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u25-28]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 27 to section 'Window 3 Funds.' paragraph 30\nContent: designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization. Centers receiving Window 3 Funds are responsible for the use of such funds and will: ensure that Window 3 Funds are used exclusively for their intended purposes; ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements;\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u34-37]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 36 to section 'Window 3 Funds.' paragraph 39\nContent: in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center. Window 3 Side Agreements or Arrangements. Nothing in the Funding Agreements or Arrangements is intended to preclude Funders and Centers from entering into Window 3 Side Agreements or Arrangements in regard to the terms governing the administration and use of Window 3 Funds. Funders may choose to make a Contribution to a Center through Window 3 without entering into a Window 3 Side Agreement or Arrangement, provided that such Contribution is made without any additional conditions attached to it. Any Window 3 Side Agreement or Arrangement will be consistent with these Standard Provisions and substantially in the form of Schedule 1 (Form of Window 3 Side Agreement or Arrangement) attached to these Standard Provisions, as may be amended from time to time. Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4,\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u163-166]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Limitation of Liabilities' paragraph 176 to section 'No Additional Obligations' paragraph 180\nContent: In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u58-61]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 62 to section 'Financial, Economic and Administrative Standards' paragraph 65\nContent: Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council. Procurement. In the event that consultants are employed or services or goods are procured with Window 1, 2 and 3 Funds, the System Organization and each Center will, respectively, ensure that the employment and supervision of such consultants and the procurement of such services or goods will be the responsibility of each entity employing or contracting such consultants or carrying out such procurement and will be conducted in conformity with applicable CGIAR Policies and Procedures on procurement, in line with the following basic principles of equal treatment and non-discrimination on grounds of nationality, competition, predictability, transparency, verifiability, and proportionality. No taxation. The System Organization and each Center will, respectively, use best efforts, to the extent allowed by applicable agreements, such as those signed with host governments, and applicable laws, to ensure that the use of Window 1, 2 and 3 Funds will be free from any taxation or fees imposed under local laws. Insurance. The System Organization and each Center will, respectively, maintain insurance coverage sufficient to cover the activities, risks, and potential omissions of the activities funded by Window 1, 2 and 3 Funds in accordance with generally accepted industry standards and as required by law.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u106-109]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Monitoring and Evaluations' paragraph 115 to section 'Monitoring' paragraph 118\nContent: Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder. If an individual Funder wishes to request, on an exceptional basis, a review or evaluation of any activities financed with Window 1 and Window 2 Funds, such Funder will consult with a designated representative from the System Organization on the most appropriate scope and terms of reference of such review or evaluation. The designated representative will assist in arranging for such review or evaluation in accordance with the applicable CGIAR Policies and Procedures. The costs of any such review or evaluation, including the internal costs of the System Organization or Center with respect to such review or evaluation, will be paid by the requesting Funder. The System Organization and each Center will, respectively collaborate on any monitoring or evaluations conducted in connection with CGIAR Research activities funded with Window 1, 2 and 3 Funds. Monitoring\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u175-178]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 191 to section 'Acknowledgement of Funders' paragraph 194\nContent: Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement. Before taking such action under paragraph 13.1, the System Organization will notify the relevant Center in writing, and consult with the System Council as well as the relevant Center with a view to identify ways and means to manage the suspension and mitigate the impact on the implementation of CGIAR Research until such time that the suspension may be lifted. If such suspension is lifted by the System Organization, it will notify the relevant Center in writing. Request by a Funder. If a Funder has a credible concern: (a) that Window 1, 2 and 3 Funds are not used by a Center in accordance with the applicable Fund Use Agreement or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) of a non-compliance by a Center with any of its obligations under an applicable Fund Use Agreement, the Funder may request, through the System Council, the System Organization to review the specific concern and, as relevant, to take appropriate corrective action. The System Organization will report to the System Council on the outcome of the review and, as appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u184-189]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Misused Fund' paragraph 202 to section 'Inconsistency' paragraph 207\nContent: Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Inconsistency In the event of any inconsistency between the Cover Pages and these Standard Provisions, these Standard Provisions will prevail. Amendments Amendments These Standard Provisions may only be amended by approval of the System Council subject to concurrence of the Integrated Partnership Board. The System Organization will promptly notify the Funders and Centers in writing of any such amendments to these Standard Provisions.\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 5 part 1\nContent: Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 24 part 4\nContent: the continuity of prior work that is less fit for purpose in the Program’s ToC. Windows 1, 2, 3 and bilateral funding: Approximately half of S4I’s 2025 funding is from Window 1, with the remainder from Window 2, including two $1.25 million designated W2 allocations specifically for AoWs 4 and 5. The PORB also reflects stronger alignment of Window 3 and bilateral funding with Program logic: in 2025, 47 mapped W3 and bilateral investments totaling $44.8 million support the Program ($0.42M, $26.47M, $1.55M, $15.37M, and $0.99M across AoWs 1 through 5, respectively), with 74% of these funds active in Africa, 19% in Asia, and 7% in Latin America. Engage and Empower (AoW 1): This AoW is allocated $2.98 million in W1/W2 funding and supported by $0.42 million in W3/bilaterals. It anchors S4I’s stakeholder demand intelligence 9 The section on AoW 4 in the PORB description highlights major inception period successes in leveraging Window 3 investments, with an anticipated, two-year bilateral investment in HLO 4.1 to transition TAAT into the Scaling Program that will support new work that was not part of the RIIs or NPS.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u67-70]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 71 to section 'Ethical Standards' paragraph 74\nContent: Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u157-160]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Statement of Assurance' paragraph 169 to section 'Additional Audits / Financial Reviews / Technical Reporting' paragraph 172\nContent: Change in Reporting Requirements. Unless decided otherwise by the System Council and/or the Integrated Partnership Board as the case may be, any change in the form or substance or periodicity of a technical or financial report will become effective only in the following calendar year. Additional Audits / Financial Reviews / Technical Reporting Funders will manage their audits, financial reviews and technical reporting with respect to the Window 1, 2 and 3 Funds collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to require duplicative reporting, provided that a Funder may require supplemental audits, financial reviews and technical reporting with respect to Window 3 Funds pursuant to its Window 3 Side Agreement or Arrangement, the costs of which would be paid by the requesting Funder. If a Funder wishes to request, on an exceptional basis, that the System Organization or a Center has an external audit or provides additional financial reviews or technical reports wi</t>
   </si>
 </sst>
 </file>
@@ -2524,7 +2640,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2567,7 +2683,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -2579,16 +2695,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2596,7 +2712,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -2608,16 +2724,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2625,7 +2741,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -2637,16 +2753,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="I4" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2654,7 +2770,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -2666,16 +2782,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H5" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I5" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2683,7 +2799,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -2695,16 +2811,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H6" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I6" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -2712,7 +2828,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -2724,16 +2840,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H7" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="I7" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -2741,7 +2857,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -2753,16 +2869,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I8" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2770,7 +2886,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -2782,16 +2898,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H9" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="I9" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2799,7 +2915,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -2811,16 +2927,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="I10" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2828,7 +2944,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -2840,16 +2956,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H11" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I11" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2857,7 +2973,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -2869,16 +2985,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H12" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I12" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2886,7 +3002,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -2898,16 +3014,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H13" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I13" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2915,7 +3031,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -2927,16 +3043,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G14" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H14" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="I14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2944,7 +3060,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C15">
         <v>100</v>
@@ -2956,16 +3072,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G15" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H15" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I15" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2973,7 +3089,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -2985,16 +3101,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G16" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H16" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I16" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -3002,7 +3118,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -3014,16 +3130,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G17" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H17" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="I17" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -3031,7 +3147,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -3043,16 +3159,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G18" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H18" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I18" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -3060,7 +3176,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -3072,16 +3188,16 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="I19" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -3089,7 +3205,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -3101,16 +3217,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G20" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H20" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I20" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -3118,7 +3234,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -3130,22 +3246,22 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G21" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H21" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I21" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="J21" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K21" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -3153,7 +3269,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -3165,22 +3281,22 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G22" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H22" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I22" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="J22" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K22" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -3188,7 +3304,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -3200,22 +3316,22 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G23" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H23" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I23" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="J23" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K23" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -3223,7 +3339,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C24">
         <v>200</v>
@@ -3235,22 +3351,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G24" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H24" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I24" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="J24" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K24" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -3258,7 +3374,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25">
         <v>200</v>
@@ -3270,22 +3386,22 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G25" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H25" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="I25" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="J25" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="K25" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -3293,7 +3409,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C26">
         <v>200</v>
@@ -3305,22 +3421,22 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G26" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H26" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I26" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="J26" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K26" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -3328,7 +3444,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C27">
         <v>200</v>
@@ -3340,22 +3456,22 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H27" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="I27" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="J27" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K27" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -3363,7 +3479,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C28">
         <v>200</v>
@@ -3375,22 +3491,22 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G28" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H28" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I28" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="J28" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K28" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -3398,7 +3514,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C29">
         <v>200</v>
@@ -3410,22 +3526,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G29" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H29" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="I29" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="J29" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="K29" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -3433,7 +3549,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -3445,22 +3561,22 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G30" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H30" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I30" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="J30" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="K30" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -3468,7 +3584,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -3480,22 +3596,22 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G31" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H31" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="I31" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="J31" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="K31" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -3503,7 +3619,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -3515,22 +3631,22 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G32" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H32" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I32" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="J32" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K32" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -3538,7 +3654,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -3550,22 +3666,22 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G33" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H33" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="J33" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K33" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -3573,7 +3689,7 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -3585,22 +3701,22 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G34" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H34" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="J34" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K34" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -3608,7 +3724,7 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -3620,22 +3736,22 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G35" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H35" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="J35" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K35" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3643,7 +3759,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -3655,22 +3771,22 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G36" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H36" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="J36" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K36" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -3678,7 +3794,7 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -3690,22 +3806,22 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G37" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H37" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="J37" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K37" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -3713,7 +3829,7 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -3725,22 +3841,22 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G38" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H38" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="J38" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="K38" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -3748,7 +3864,7 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -3760,22 +3876,22 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G39" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I39" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J39" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K39" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -3783,7 +3899,7 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -3795,22 +3911,22 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G40" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H40" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I40" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J40" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K40" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -3818,7 +3934,7 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -3830,22 +3946,22 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G41" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H41" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I41" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J41" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K41" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -3853,7 +3969,7 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C42">
         <v>100</v>
@@ -3865,22 +3981,22 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G42" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H42" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="I42" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J42" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K42" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -3888,7 +4004,7 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -3900,22 +4016,22 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G43" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H43" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I43" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J43" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K43" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -3923,7 +4039,7 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -3935,22 +4051,22 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G44" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H44" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="I44" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J44" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K44" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -3967,13 +4083,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H45" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="K45" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3981,7 +4097,7 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -3993,22 +4109,22 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G46" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H46" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I46" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J46" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K46" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -4016,7 +4132,7 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -4028,22 +4144,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G47" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H47" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="J47" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K47" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -4051,7 +4167,7 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -4063,22 +4179,22 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G48" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H48" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="J48" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="K48" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -4086,7 +4202,7 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C49">
         <v>200</v>
@@ -4098,22 +4214,22 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G49" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H49" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="J49" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="K49" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -4121,7 +4237,7 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C50">
         <v>200</v>
@@ -4133,22 +4249,22 @@
         <v>1</v>
       </c>
       <c r="F50" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G50" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H50" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="J50" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="K50" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -4156,7 +4272,7 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C51">
         <v>200</v>
@@ -4168,22 +4284,22 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G51" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H51" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="J51" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="K51" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -4191,7 +4307,7 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C52">
         <v>200</v>
@@ -4203,22 +4319,22 @@
         <v>1</v>
       </c>
       <c r="F52" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G52" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H52" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="J52" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="K52" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -4226,7 +4342,7 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C53">
         <v>200</v>
@@ -4238,22 +4354,22 @@
         <v>1</v>
       </c>
       <c r="F53" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G53" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H53" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J53" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="K53" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -4261,7 +4377,7 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C54">
         <v>200</v>
@@ -4273,22 +4389,22 @@
         <v>1</v>
       </c>
       <c r="F54" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G54" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H54" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="J54" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="K54" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -4296,7 +4412,7 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C55">
         <v>200</v>
@@ -4308,22 +4424,22 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H55" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="J55" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="K55" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -4331,7 +4447,7 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C56">
         <v>200</v>
@@ -4343,22 +4459,22 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G56" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H56" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="J56" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="K56" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -4366,7 +4482,7 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C57">
         <v>200</v>
@@ -4378,22 +4494,22 @@
         <v>1</v>
       </c>
       <c r="F57" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H57" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J57" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="K57" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -4401,7 +4517,7 @@
         <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C58">
         <v>200</v>
@@ -4413,22 +4529,22 @@
         <v>1</v>
       </c>
       <c r="F58" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G58" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H58" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J58" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="K58" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -4436,7 +4552,7 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C59">
         <v>200</v>
@@ -4448,22 +4564,22 @@
         <v>1</v>
       </c>
       <c r="F59" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G59" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H59" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="J59" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="K59" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -4471,7 +4587,7 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C60">
         <v>200</v>
@@ -4483,22 +4599,22 @@
         <v>1</v>
       </c>
       <c r="F60" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G60" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H60" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I60" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="J60" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="K60" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -4506,7 +4622,7 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C61">
         <v>200</v>
@@ -4518,22 +4634,57 @@
         <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G61" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H61" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="I61" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="J61" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="K61" t="s">
-        <v>202</v>
+        <v>208</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11">
+      <c r="A62" t="s">
+        <v>71</v>
+      </c>
+      <c r="B62" t="s">
+        <v>85</v>
+      </c>
+      <c r="C62">
+        <v>200</v>
+      </c>
+      <c r="D62">
+        <v>200</v>
+      </c>
+      <c r="E62" t="b">
+        <v>1</v>
+      </c>
+      <c r="F62" t="s">
+        <v>93</v>
+      </c>
+      <c r="G62" t="s">
+        <v>111</v>
+      </c>
+      <c r="H62" t="s">
+        <v>159</v>
+      </c>
+      <c r="I62" t="s">
+        <v>175</v>
+      </c>
+      <c r="J62" t="s">
+        <v>188</v>
+      </c>
+      <c r="K62" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added documents from "Home" and modify ctx
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="237">
   <si>
     <t>timestamp</t>
   </si>
@@ -232,6 +232,21 @@
     <t>2025-09-25T01:18:56.051769</t>
   </si>
   <si>
+    <t>2025-09-26T08:47:03.579052</t>
+  </si>
+  <si>
+    <t>2025-09-26T08:54:14.961810</t>
+  </si>
+  <si>
+    <t>2025-09-26T08:56:28.255216</t>
+  </si>
+  <si>
+    <t>2025-09-26T09:00:09.362611</t>
+  </si>
+  <si>
+    <t>2025-09-26T09:07:14.972092</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -272,6 +287,15 @@
   </si>
   <si>
     <t>Who has fiduciary responsibility over the Windows 1 and 2 funds, and what must they guarantee?</t>
+  </si>
+  <si>
+    <t>what is an outcome</t>
+  </si>
+  <si>
+    <t>what is an outcome?</t>
+  </si>
+  <si>
+    <t>what are the different types of outputs in the cgiar results framework?</t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -355,6 +379,18 @@
   </si>
   <si>
     <t>docx:Standard Provisions 2026.docx:u19-22:0.500, docx:Standard Provisions 2026.docx:u16-19:0.437, docx:Standard Provisions 2026.docx:u28-31:0.324, docx:Standard Provisions 2026.docx:u31-34:0.319, docx:Standard Provisions 2026.docx:u181-184:0.262, docx:Standard Provisions 2026.docx:u13-16:0.242, docx:Standard Provisions 2026.docx:u178-181:0.234, docx:Standard Provisions 2026.docx:u22-25:0.214, docx:Standard Provisions 2026.docx:u172-175:0.211, docx:Standard Provisions 2026.docx:u4-7:0.200, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.198, docx:Standard Provisions 2026.docx:u46-49:0.196, docx:Standard Provisions 2026.docx:u55-58:0.195, docx:Standard Provisions 2026.docx:u25-28:0.191, docx:Standard Provisions 2026.docx:u34-37:0.182, docx:Standard Provisions 2026.docx:u163-166:0.181, docx:Standard Provisions 2026.docx:u58-61:0.179, docx:Standard Provisions 2026.docx:u106-109:0.167, docx:Standard Provisions 2026.docx:u175-178:0.167, docx:Standard Provisions 2026.docx:u184-189:0.160, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.159, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1:0.157, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4:0.156, docx:Standard Provisions 2026.docx:u67-70:0.155, docx:Standard Provisions 2026.docx:u157-160:0.154, docx:Standard Provisions 2026.docx:u43-46:0.148, docx:Standard Provisions 2026.docx:u70-73:0.147, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt2:0.146, docx:Standard Provisions 2026.docx:u160-163:0.140, docx:Standard Provisions 2026.docx:u10-13:0.139, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.136, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt2:0.136, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p4pt4:0.134, docx:Standard Provisions 2026.docx:u112-115:0.133, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt3:0.132, docx:Standard Provisions 2026.docx:u103-106:0.132, docx:2025 Technical Reporting Information (Session 1).docx:u40-43:0.131, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.129, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt2:0.129, docx:Standard Provisions 2026.docx:u52-55:0.128, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p4pt1:0.127, pdf:Climate Action_Inception Report 30-06-2025.pdf:p30pt2:0.125, docx:Standard Provisions 2026.docx:u109-112:0.125, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt3:0.124, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.123, docx:Standard Provisions 2026.docx:u73-76:0.121, docx:Standard Provisions 2026.docx:u64-67:0.121, pdf:Climate Action_Inception Report 30-06-2025.pdf:p30pt3:0.120, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt2:0.118, docx:Standard Provisions 2026.docx:u37-40:0.118, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt1:0.118, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt2:0.118, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt4:0.118, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt2:0.118, docx:2025 Technical Reporting MELIA glossary.docx:u55-58:0.118, docx:Standard Provisions 2026.docx:u166-169:0.117, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt1:0.117, pdf:Type3_2024Report.pdf:p5pt1:0.116, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt2:0.116, docx:Standard Provisions 2026.docx:u97-100:0.116, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt4:0.116, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt2:0.115, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt2:0.115, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p2pt2:0.115, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt4:0.115, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt2:0.115, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt2:0.115, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt2:0.115, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt2:0.114, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt3:0.113, docx:Standard Provisions 2026.docx:u1-4:0.112, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.112, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt3:0.110, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p18pt4:0.110, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.110, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p32pt1:0.108, pdf:Climate Action_Inception Report 30-06-2025.pdf:p16pt3:0.107, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p26pt3:0.107, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p2pt1:0.107, docx:User Roles and Rules for the PRMS Reporting.docx:u4-7:0.106, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt2:0.105, docx:Standard Provisions 2026.docx:u61-64:0.105, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p19pt3:0.104, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt2:0.103, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.103, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p30pt2:0.103, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt1:0.103, docx:Standard Provisions 2026.docx:u76-79:0.103, docx:User Roles and Rules for the PRMS Reporting.docx:u16-19:0.102, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt1:0.102, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.102, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt4:0.101, pdf:Genebanks_Inception Report 30-06-2025.pdf:p18pt1:0.101, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p18pt3:0.100, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt3:0.100, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.100, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4:0.099, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.099, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt4:0.099, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt4:0.098, docx:Standard Provisions 2026.docx:u100-103:0.097, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p25pt4:0.097, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p9pt2:0.097, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p29pt2:0.097, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p4pt2:0.096, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt1:0.096, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p5pt2:0.095, docx:Standard Provisions 2026.docx:u148-151:0.095, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p19pt1:0.095, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p3pt3:0.095, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p11pt4:0.095, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.095, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p2pt1:0.095, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt1:0.094, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt1:0.094, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p8pt4:0.094, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p5pt1:0.094, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.094, docx:Standard Provisions 2026.docx:u133-136:0.094, docx:Standard Provisions 2026.docx:u130-133:0.093, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p15pt1:0.093, docx:Standard Provisions 2026.docx:u88-91:0.093, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt1:0.093, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt1:0.093, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt1:0.093, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p15pt1:0.093, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p24pt1:0.093, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt3:0.093, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p13pt4:0.093, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt3:0.093, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p32pt4:0.092, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt1:0.092, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p12pt2:0.092, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p19pt2:0.092, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt2:0.092, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p16pt1:0.092, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p20pt4:0.092, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt4:0.092, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt1:0.091, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt1:0.091, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt3:0.091, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.091, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.091, pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt3:0.091, pptx:Information Session on 2025 Technical Reporting.pptx:s12pt3:0.091, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p21pt1:0.091, pdf:Portfolio Narrative_2024.pdf:p2pt4:0.091, docx:Standard Provisions 2026.docx:u151-154:0.090, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt1:0.090, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt1:0.090, docx:Guidance on reporting outputs or outcomes.docx:u10-13:0.090, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p15pt2:0.089, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt4:0.089, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p7pt2:0.089, docx:Standard Provisions 2026.docx:u145-148:0.089, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt2:0.089, pdf:Genebanks_Inception Report 30-06-2025.pdf:p21pt3:0.089, docx:Standard Provisions 2026.docx:u82-85:0.089, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p35pt3:0.088, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p22pt1:0.088, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt1:0.088, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.088, pdf:Portfolio Narrative_2024.pdf:p82pt2:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u46-49:0.088, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt2:0.088, pdf:Genebanks_Inception Report 30-06-2025.pdf:p9pt2:0.088, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt3:0.088, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p2pt1:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt2:0.088, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p35pt4:0.088, docx:2025 Technical Reporting Information (Session 2).docx:u25-28:0.088, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt2:0.087, docx:Standard Provisions 2026.docx:u94-97:0.087, pdf:Genebanks_Inception Report 30-06-2025.pdf:p24pt2:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt4:0.087, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.087, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.087, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt3:0.087, docx:Standard Provisions 2026.docx:u169-172:0.086, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.086, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p32pt2:0.086, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt2:0.086, pdf:Genebanks_Inception Report 30-06-2025.pdf:p8pt3:0.086, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p5pt2:0.086, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p23pt1:0.086, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt2:0.086, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.086, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p5pt2:0.085, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p25pt3:0.085, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p4pt2:0.085, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p40pt4:0.084, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p33pt4:0.084, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p27pt1:0.084, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p49pt3:0.084, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p31pt2:0.084, docx:Standard Provisions 2026.docx:u85-88:0.084, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p2pt1:0.084, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p2pt1:0.084, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.084, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p24pt4:0.084</t>
+  </si>
+  <si>
+    <t>pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4:0.302, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2:0.290, docx:Innovation use.docx:u1-4:0.281, docx:General reporting guidance.docx:u1-3:0.250, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4:0.240, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3:0.230, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3:0.229, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2:0.228, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4:0.227, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3:0.226, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.226, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.226, docx:Innovation development.docx:u1-4:0.222, docx:2025 Technical Reporting MELIA glossary.docx:u31-34:0.218, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4:0.214, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2:0.214, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4:0.213, pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2:0.213, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1:0.202, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4:0.202, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1:0.200, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.198, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt1:0.197, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1:0.196, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt1:0.193, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3:0.193, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt2:0.193, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt1:0.193, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.192, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2:0.192, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt2:0.192, docx:2025 Technical Reporting MELIA glossary.docx:u28-31:0.191, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.191, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt4:0.191, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p12pt1:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt1:0.189, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt1:0.188, docx:Guidance on reporting outputs or outcomes.docx:u7-10:0.187, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.186, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.185, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt3:0.184, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt2:0.184, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p11pt3:0.184, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p13pt2:0.183, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt1:0.183, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt2:0.183, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt4:0.183, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt4:0.181, pdf:CGI21_508012_PORB_Genebanks.pdf:p24pt1:0.180, pdf:CGI21_508012_PORB_Genebanks.pdf:p31pt3:0.179, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt3:0.178, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p15pt2:0.177, pdf:CGI21_508012_PORB_Genebanks.pdf:p22pt3:0.176, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1:0.176, docx:2025 Technical Reporting Information (Session 1).docx:u25-28:0.173, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p21pt1:0.173, pdf:CGI21_508012_PORB_Genebanks.pdf:p40pt2:0.172, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.168, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.168, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt3:0.168, pdf:Portfolio Narrative_2024.pdf:p7pt1:0.167, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt2:0.167, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4:0.167, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt2:0.166, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt2:0.165, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt2:0.165, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p34pt4:0.164, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.164, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt2:0.163, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p6pt1:0.163, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt2:0.163, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt3:0.163, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p4pt4:0.162, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.162, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt1:0.162, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.161, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt2:0.161, docx:2025 Technical Reporting Information (Session 2).docx:u19-22:0.161, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p51pt1:0.161, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt2:0.160, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt3:0.160, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1:0.160, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt2:0.159, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p1pt4:0.159, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt2:0.159, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt1:0.159, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p11pt4:0.158, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p22pt2:0.157, pdf:Portfolio Narrative_2024.pdf:p53pt2:0.157, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.156, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.156, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt1:0.155, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p40pt1:0.155, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt2:0.155, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt3:0.155, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt3:0.154, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.154, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt3:0.154, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt4:0.153, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p23pt3:0.152, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt2:0.152, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt3:0.151, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt2:0.150, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.150, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p42pt2:0.150, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p18pt2:0.149, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p17pt2:0.149, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p14pt4:0.149, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.148, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt2:0.148, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.148, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt3:0.147, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.147, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt3:0.147, pdf:CGI21_508012_PORB_Genebanks.pdf:p30pt2:0.147, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.146, pdf:CGI21_508012_PORB_Genebanks.pdf:p39pt2:0.146, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt3:0.146, pdf:CGI21_508012_PORB_Genebanks.pdf:p13pt1:0.146, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p28pt3:0.145, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt1:0.145, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt2:0.144, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt3:0.144, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt3:0.143, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt1:0.143, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt4:0.143, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1:0.143, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.143, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p11pt1:0.143, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p10pt1:0.142, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt2:0.142, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p51pt4:0.142, docx:Guidance on reporting outputs or outcomes.docx:u19-22:0.142, pdf:CGI21_508012_PORB_Genebanks.pdf:p48pt2:0.141, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt3:0.141, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p31pt3:0.141, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.141, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3:0.141, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p19pt2:0.141, pdf:CGI21_508012_PORB_Genebanks.pdf:p45pt2:0.141, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p11pt1:0.140, pdf:CGI21_508012_PORB_Genebanks.pdf:p12pt1:0.140, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.140, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt4:0.140, pdf:CGI21_508012_PORB_Genebanks.pdf:p7pt2:0.139, pdf:CGIAR_ImpactReport_2022-24.pdf:p3pt1:0.139, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.139, pdf:CGI21_508012_PORB_Genebanks.pdf:p36pt2:0.139, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt1:0.139, docx:Engagement Plan 2025 Technical Reporting.docx:u61-63:0.139, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt2:0.139, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p18pt4:0.138, docx:2025 Technical Reporting Information (Session 2).docx:u13-16:0.138, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt1:0.138, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p13pt4:0.137, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.137, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt2:0.137, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p12pt2:0.137, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.137, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p12pt3:0.137, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p44pt2:0.136, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt3:0.136, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt4:0.136, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt2:0.136, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.136, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt2:0.135, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt3:0.135, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.135, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt1:0.135, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.134, pdf:Portfolio Narrative_2024.pdf:p60pt1:0.134, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt3:0.134, docx:Innovation use.docx:u13-16:0.134, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.134, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p25pt3:0.134, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.133, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt3:0.133, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt3:0.133, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt1:0.133, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.132, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.132, pdf:CGI21_508012_PORB_Genebanks.pdf:p46pt3:0.132, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p34pt2:0.132, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.132, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.132, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt4:0.131, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt2:0.131, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt3:0.131, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt4:0.131, docx:Guidance on reporting outputs or outcomes.docx:u16-19:0.131</t>
+  </si>
+  <si>
+    <t>pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4:0.301, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2:0.289, docx:Innovation use.docx:u1-4:0.281, docx:General reporting guidance.docx:u1-3:0.250, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4:0.243, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4:0.243, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3:0.230, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3:0.229, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2:0.227, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4:0.227, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.227, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.226, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3:0.226, docx:Innovation development.docx:u1-4:0.221, docx:2025 Technical Reporting MELIA glossary.docx:u31-34:0.218, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4:0.215, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2:0.213, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4:0.213, pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2:0.212, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1:0.202, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4:0.201, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1:0.200, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.199, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt1:0.196, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1:0.196, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt1:0.193, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3:0.193, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.192, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt2:0.192, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt1:0.192, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.192, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2:0.192, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt2:0.191, docx:2025 Technical Reporting MELIA glossary.docx:u28-31:0.191, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt4:0.191, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt1:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt1:0.190, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p12pt1:0.189, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt1:0.187, docx:Guidance on reporting outputs or outcomes.docx:u7-10:0.187, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.186, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.185, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt3:0.183, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p11pt3:0.183, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p13pt2:0.183, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt2:0.183, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt1:0.183, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt2:0.182, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt4:0.182, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt4:0.181, pdf:CGI21_508012_PORB_Genebanks.pdf:p24pt1:0.179, pdf:CGI21_508012_PORB_Genebanks.pdf:p31pt3:0.178, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt3:0.177, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p15pt2:0.176, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1:0.176, pdf:CGI21_508012_PORB_Genebanks.pdf:p22pt3:0.175, docx:2025 Technical Reporting Information (Session 1).docx:u25-28:0.173, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p21pt1:0.172, pdf:CGI21_508012_PORB_Genebanks.pdf:p40pt2:0.171, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.170, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.168, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4:0.167, pdf:Portfolio Narrative_2024.pdf:p7pt1:0.167, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt3:0.167, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt2:0.167, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt2:0.165, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt2:0.165, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt2:0.165, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.165, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p34pt4:0.164, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt2:0.163, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p6pt1:0.162, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt2:0.162, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.162, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt3:0.162, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p4pt4:0.162, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt1:0.161, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt2:0.161, docx:2025 Technical Reporting Information (Session 2).docx:u19-22:0.161, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.161, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p51pt1:0.160, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1:0.160, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p1pt4:0.160, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt1:0.159, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt2:0.159, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt3:0.159, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt2:0.159, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt2:0.158, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p11pt4:0.158, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p22pt2:0.157, pdf:Portfolio Narrative_2024.pdf:p53pt2:0.157, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.156, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.156, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt1:0.155, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.155, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p40pt1:0.155, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt3:0.154, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt2:0.154, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt3:0.154, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt3:0.153, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt4:0.152, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p23pt3:0.152, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt2:0.151, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.150, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt3:0.150, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt2:0.150, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p18pt2:0.149, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p42pt2:0.149, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.149, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p17pt2:0.148, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p14pt4:0.148, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.148, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt2:0.148, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.147, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.147, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt3:0.146, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt3:0.146, pdf:CGI21_508012_PORB_Genebanks.pdf:p30pt2:0.146, pdf:CGI21_508012_PORB_Genebanks.pdf:p39pt2:0.146, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt3:0.145, pdf:CGI21_508012_PORB_Genebanks.pdf:p13pt1:0.145, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p28pt3:0.145, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt1:0.144, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt2:0.144, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt4:0.143, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt4:0.143, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt3:0.143, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1:0.143, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt3:0.143, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt1:0.143, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt1:0.142, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p10pt1:0.142, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt2:0.142, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p11pt1:0.142, docx:Guidance on reporting outputs or outcomes.docx:u19-22:0.142, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.142, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p51pt4:0.141, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3:0.141, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p13pt3:0.141, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p31pt3:0.141, pdf:CGI21_508012_PORB_Genebanks.pdf:p48pt2:0.141, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p19pt2:0.140, pdf:CGI21_508012_PORB_Genebanks.pdf:p45pt2:0.140, pdf:CGI21_508012_PORB_Genebanks.pdf:p12pt1:0.140, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.140, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p11pt1:0.140, docx:Engagement Plan 2025 Technical Reporting.docx:u61-63:0.139, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt4:0.139, pdf:CGIAR_ImpactReport_2022-24.pdf:p3pt1:0.139, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt1:0.139, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.139, pdf:CGI21_508012_PORB_Genebanks.pdf:p7pt2:0.139, pdf:CGI21_508012_PORB_Genebanks.pdf:p36pt2:0.138, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt2:0.138, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.138, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.138, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p18pt4:0.138, docx:2025 Technical Reporting Information (Session 2).docx:u13-16:0.138, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p12pt2:0.137, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.137, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p13pt4:0.137, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt1:0.137, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.137, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt4:0.137, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt4:0.137, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt2:0.136, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p12pt3:0.136, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt3:0.136, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.136, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p44pt2:0.136, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.136, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt2:0.135, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt1:0.135, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt3:0.135, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt2:0.135, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.134, docx:Innovation use.docx:u13-16:0.134, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.134, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4:0.134, pdf:Portfolio Narrative_2024.pdf:p60pt1:0.134, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt3:0.133, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p25pt3:0.133, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt1:0.133, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.132, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.132, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt3:0.132, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt3:0.132, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.132, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p34pt2:0.132, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.132, docx:Guidance on reporting outputs or outcomes.docx:u16-19:0.131, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt3:0.131, pdf:CGI21_508012_PORB_Genebanks.pdf:p46pt3:0.131, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt2:0.131, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt4:0.131, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt2:0.131, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt3:0.131, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p9pt4:0.131, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p12pt2:0.131, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt4:0.130</t>
+  </si>
+  <si>
+    <t>pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4:0.157, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2:0.152, docx:Innovation use.docx:u1-4:0.151, docx:General reporting guidance.docx:u1-3:0.136, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3:0.129, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p18pt4:0.129, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4:0.127, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4:0.124, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.124, docx:2025 Technical Reporting MELIA glossary.docx:u31-34:0.124, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3:0.123, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2:0.123, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4:0.122, docx:Innovation development.docx:u1-4:0.119, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.116, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4:0.116, pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3:0.116, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1:0.112, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2:0.112, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3:0.112, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2:0.111, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1:0.110, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4:0.110, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4:0.110, docx:2025 Technical Reporting MELIA glossary.docx:u28-31:0.109, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3:0.108, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2:0.107, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.107, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p13pt2:0.106, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt1:0.106, pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2:0.105, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.105, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p12pt1:0.105, docx:Guidance on reporting outputs or outcomes.docx:u7-10:0.104, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4:0.103, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt1:0.102, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt1:0.102, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt2:0.102, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1:0.102, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt4:0.100, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt4:0.100, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.099, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1:0.098, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.097, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4:0.097, pdf:Portfolio Narrative_2024.pdf:p7pt1:0.097, docx:2025 Technical Reporting Information (Session 1).docx:u25-28:0.096, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p15pt2:0.096, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt1:0.095, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt1:0.095, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt2:0.095, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt2:0.094, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt4:0.094, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p4pt4:0.094, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.093, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt1:0.093, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt1:0.093, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p1pt4:0.093, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p32pt1:0.092, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.091, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt1:0.091, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt2:0.091, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p29pt4:0.091, pdf:CGI21_508012_PORB_Genebanks.pdf:p31pt3:0.090, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt2:0.090, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt2:0.089, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt1:0.089, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt2:0.089, pdf:CGI21_508012_PORB_Genebanks.pdf:p22pt3:0.089, docx:2025 Technical Reporting Information (Session 2).docx:u19-22:0.089, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt3:0.089, pdf:CGI21_508012_PORB_Genebanks.pdf:p23pt3:0.089, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt2:0.088, pdf:CGI21_508012_PORB_Genebanks.pdf:p24pt1:0.087, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.087, pdf:Portfolio Narrative_2024.pdf:p53pt2:0.087, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt3:0.087, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p34pt4:0.087, pdf:CGI21_508012_PORB_Genebanks.pdf:p40pt2:0.087, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.086, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p14pt4:0.086, pdf:Genebanks_Inception Report 30-06-2025.pdf:p8pt3:0.086, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p46pt3:0.086, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt1:0.086, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt1:0.086, pdf:CGI21_508012_PORB_Genebanks.pdf:p32pt3:0.086, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p17pt2:0.085, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.085, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p11pt3:0.084, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt3:0.083, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p10pt1:0.083, docx:Guidance on reporting outputs or outcomes.docx:u19-22:0.082, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.082, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt3:0.082, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt3:0.082, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt2:0.081, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p21pt1:0.081, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.081, docx:Engagement Plan 2025 Technical Reporting.docx:u61-63:0.081, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt4:0.081, pdf:CGIAR_ImpactReport_2022-24.pdf:p3pt1:0.081, pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt3:0.080, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p18pt4:0.080, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p22pt2:0.080, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p12pt2:0.080, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.080, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p13pt4:0.080, pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt3:0.080, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt4:0.079, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt4:0.079, docx:2025 Technical Reporting Information (Session 2).docx:u13-16:0.079, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1:0.079, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p6pt1:0.079, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.079, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt3:0.079, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.079, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt3:0.078, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt3:0.078, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt1:0.078, docx:Innovation use.docx:u13-16:0.078, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p24pt3:0.077, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt2:0.077, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.077, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p11pt4:0.077, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt1:0.077, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.077, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.076, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p34pt2:0.076, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.076, docx:Guidance on reporting outputs or outcomes.docx:u16-19:0.076, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.076, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt2:0.076, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p18pt2:0.076, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt1:0.075, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p16pt2:0.075, pdf:CGIAR_ImpactReport_2022-24.pdf:p5pt4:0.075, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.075, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4:0.075, pdf:Portfolio Narrative_2024.pdf:p60pt1:0.075, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p11pt1:0.075, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt2:0.075, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt2:0.075, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt2:0.075, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.074, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p19pt3:0.074, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt4:0.074, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt1:0.074, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt1:0.074, pdf:CGI21_508012_PORB_Genebanks.pdf:p41pt2:0.074, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p13pt2:0.074, pdf:Portfolio Narrative_2024.pdf:p15pt4:0.074, pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt1:0.074, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt2:0.074, pdf:CGI21_508012_PORB_Genebanks.pdf:p6pt4:0.073, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p7pt3:0.073, pdf:CGI21_508012_PORB_Genebanks.pdf:p44pt2:0.073, pptx:Information Session on 2025 Technical Reporting.pptx:s13pt1:0.073, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt2:0.073, pdf:CGI21_508012_PORB_Genebanks.pdf:p38pt2:0.073, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p31pt3:0.072, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.072, pdf:CGI21_508012_PORB_Genebanks.pdf:p47pt3:0.072, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p9pt4:0.072, pdf:CGI21_508012_PORB_Genebanks.pdf:p29pt3:0.072, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p11pt1:0.072, docx:2025 Technical Reporting Information (Session 2).docx:u22-25:0.071, docx:2025 Technical Reporting Information (Session 2).docx:u34-37:0.071, pdf:CGI21_508012_PORB_Genebanks.pdf:p30pt2:0.071, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p51pt1:0.071, pdf:CGI21_508012_PORB_Genebanks.pdf:p39pt2:0.071, pdf:CGI21_508012_PORB_Genebanks.pdf:p35pt3:0.071, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt1:0.071, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p40pt1:0.071, pdf:CGIAR_ImpactReport_2022-24.pdf:p36pt3:0.071, pdf:CGI21_508012_PORB_Genebanks.pdf:p26pt3:0.070, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.070, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.070, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt2:0.070, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.070, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt2:0.070, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p4pt1:0.070, pdf:CGI21_508012_PORB_Genebanks.pdf:p33pt1:0.070, pdf:CGI21_508012_PORB_Genebanks.pdf:p46pt3:0.070, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt2:0.070, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1:0.070, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p12pt2:0.070, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt1:0.069, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt2:0.069, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt4:0.069, docx:Guidance on reporting outputs or outcomes.docx:u4-7:0.069, pdf:CGI21_508012_PORB_Genebanks.pdf:p48pt2:0.069, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p23pt3:0.069, pdf:CGI21_508012_PORB_Genebanks.pdf:p28pt3:0.069, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt1:0.068, pdf:CGI21_508012_PORB_Genebanks.pdf:p45pt2:0.068, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p42pt2:0.068, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p13pt3:0.068, pdf:CGI21_508012_PORB_Genebanks.pdf:p7pt2:0.068, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt4:0.068, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p27pt2:0.068</t>
+  </si>
+  <si>
+    <t>pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt1:0.380, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt2:0.339, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4:0.329, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4:0.329, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt2:0.311, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt1:0.292, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1:0.281, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt1:0.281, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3:0.277, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3:0.277, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.276, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p28pt2:0.275, docx:2025 Technical Reporting MELIA glossary.docx:u55-58:0.272, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p9pt2:0.269, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1:0.260, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1:0.255, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1:0.255, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt2:0.247, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p8pt2:0.247, docx:2025 Technical Reporting MELIA glossary.docx:u34-37:0.239, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p32pt3:0.234, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2:0.229, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2:0.229, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p3pt1:0.228, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3:0.227, pdf:Type3_2024Report.pdf:p11pt4:0.226, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p13pt1:0.226, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt2:0.225, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p18pt2:0.225, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt1:0.222, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt1:0.222, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt1:0.218, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p9pt2:0.216, docx:2025 Technical Reporting MELIA glossary.docx:u31-34:0.213, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt3:0.213, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3:0.212, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt1:0.210, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt1:0.210, pptx:Information Session on 2025 Technical Reporting.pptx:s14pt1:0.208, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p1pt1:0.207, pdf:Genebanks_Inception Report 30-06-2025.pdf:p18pt4:0.199, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p3pt1:0.196, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt3:0.196, pdf:CGIAR_ImpactReport_2022-24.pdf:p9pt1:0.195, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p37pt4:0.195, docx:2025 Technical Reporting MELIA glossary.docx:u28-31:0.194, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p10pt1:0.194, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.193, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.193, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p4pt4:0.191, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p3pt2:0.190, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p12pt4:0.189, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1:0.189, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p1pt1:0.188, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p2pt1:0.188, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.186, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p3pt1:0.183, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2:0.182, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p3pt2:0.182, pdf:CGI21_508012_PORB_Genebanks.pdf:p1pt1:0.180, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p1pt1:0.180, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p1pt1:0.180, docx:Guidance on reporting outputs or outcomes.docx:u7-10:0.180, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.180, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt2:0.180, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt2:0.180, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt1:0.178, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt4:0.176, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p20pt1:0.176, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.176, pdf:Genebanks_Inception Report 30-06-2025.pdf:p13pt4:0.175, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p24pt1:0.174, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p9pt1:0.173, docx:Guidance on ensuring quality over quantity.docx:u4-7:0.173, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p28pt3:0.172, pdf:Type3_2024Report.pdf:p4pt4:0.171, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2:0.171, pdf:Genebanks_Inception Report 30-06-2025.pdf:p18pt3:0.171, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3:0.170, pdf:Portfolio Narrative_2024.pdf:p11pt3:0.169, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p14pt1:0.168, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p19pt1:0.167, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p20pt1:0.167, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p33pt3:0.166, pdf:Type3_2024Report.pdf:p4pt1:0.166, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p9pt4:0.164, pdf:Genebanks_Inception Report 30-06-2025.pdf:p13pt1:0.164, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt2:0.164, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt1:0.163, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.163, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4:0.163, pdf:CGIAR_ImpactReport_2022-24.pdf:p42pt1:0.162, docx:2025 Technical Reporting MELIA glossary.docx:u52-55:0.161, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1:0.161, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt1:0.161, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.161, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.160, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p32pt4:0.160, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p10pt3:0.159, docx:Guidance on complementary innnov.docx:u4-7:0.159, pdf:Portfolio Narrative_2024.pdf:p30pt3:0.159, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p22pt4:0.159, pdf:Portfolio Narrative_2024.pdf:p11pt4:0.158, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p13pt2:0.157, pdf:Portfolio Narrative_2024.pdf:p75pt4:0.157, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.157, docx:Guidance on reporting outputs or outcomes.docx:u1-4:0.157, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt2:0.157, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt1:0.156, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p7pt1:0.156, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.156, docx:Standard Provisions 2026.docx:u136-139:0.155, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt3:0.155, pdf:CGIAR_ImpactReport_2022-24.pdf:p27pt1:0.154, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p20pt4:0.154, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p20pt4:0.154, pdf:Portfolio Narrative_2024.pdf:p62pt3:0.154, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p13pt3:0.153, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt3:0.153, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt3:0.153, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p16pt3:0.153, pdf:Portfolio Narrative_2024.pdf:p18pt1:0.153, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.153, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.153, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p15pt2:0.152, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p17pt4:0.152, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt4:0.152, pdf:CGI21-507032-PORB-Climate Action.pdf:p1pt1:0.151, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p21pt3:0.151, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p21pt3:0.151, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p8pt2:0.151, pdf:Portfolio Narrative_2024.pdf:p68pt2:0.151, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p2pt1:0.151, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p9pt1:0.150, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p55pt1:0.150, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p4pt1:0.150, pdf:Portfolio Narrative_2024.pdf:p75pt3:0.150, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p28pt1:0.150, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt3:0.148, pdf:Climate Action_Inception Report 30-06-2025.pdf:p15pt3:0.148, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p16pt3:0.148, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p72pt1:0.148, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p21pt4:0.148, pdf:CGIAR_ImpactReport_2022-24.pdf:p18pt1:0.148, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p14pt2:0.147, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt2:0.147, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p20pt4:0.146, pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt1:0.146, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.146, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p30pt4:0.145, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt3:0.145, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p25pt3:0.145, pdf:Quick style guide Feb 2024 (1).pdf:p7pt4:0.145, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p14pt4:0.145, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p14pt4:0.145, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p18pt2:0.145, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p30pt1:0.145, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.145, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt4:0.145, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p15pt3:0.144, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p22pt1:0.144, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p1pt1:0.144, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p5pt4:0.144, pdf:Portfolio Narrative_2024.pdf:p58pt2:0.143, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.143, pdf:Portfolio Narrative_2024.pdf:p54pt4:0.143, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt3:0.142, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt3:0.142, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p10pt3:0.142, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p12pt1:0.142, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p23pt1:0.141, docx:Guidance on reporting outputs or outcomes.docx:u4-7:0.141, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.141, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p5pt1:0.141, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p28pt4:0.141, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt3:0.141, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p50pt1:0.141, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p19pt3:0.140, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt1:0.139, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt1:0.139, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt3:0.139, pdf:Portfolio Narrative_2024.pdf:p15pt4:0.139, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p14pt4:0.139, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt2:0.139, pdf:Portfolio Narrative_2024.pdf:p67pt4:0.139, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p5pt3:0.139, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt4:0.139, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt4:0.138, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p25pt4:0.138, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt3:0.138, docx:Standard Provisions 2026.docx:u109-112:0.138, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p3pt1:0.137, docx:General reporting guidance.docx:u1-3:0.137, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p3pt1:0.136, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt4:0.136, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt1:0.136, docx:Innovation use.docx:u1-4:0.136, docx:2025 Technical Reporting Information (Session 1).docx:u19-22:0.136, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt1:0.136, pdf:Portfolio Narrative_2024.pdf:p74pt4:0.136</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -750,6 +786,47 @@
 docx:Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — u16-19</t>
   </si>
   <si>
+    <t>An outcome refers to the specific results or changes that occur as a result of a program or initiative. In the context of the provided documents, outcomes can be categorized into various levels, such as intermediate outcomes and 2030 outcomes, which represent the final goals to be achieved by a certain date. For example, an outcome might involve the successful marketing of improved seed varieties to farmers or the strengthening of institutional capacities to guide policy decisions. These outcomes are essential for measuring the effectiveness and impact of initiatives within the CGIAR framework.
+Sources:
+- Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf — page 48 part 4 — pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1)
+- Policy Innovations_Inception Report 30-06-2025.pdf — page 13 part 2 — pdf:Policy Innovations_Inception Report 30-06-2025
+- Innovation use.docx — section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7 — docx:Innovation use
+- General reporting guidance.docx — section 'General reporting guidance' paragraph 1 to section 'General reporting guidance' paragraph 5 — docx:General reporting guidance
+- CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 22 part 4 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30</t>
+  </si>
+  <si>
+    <t>An outcome refers to the final results or impacts achieved as a result of specific initiatives or actions. In the context of the provided documents, outcomes can be seen as the higher-level changes that occur after outputs have been delivered, such as improved capacities, policy changes, or increased access to resources. For example, one document mentions a specific outcome related to seed producers successfully marketing new varieties to farmers, highlighting the practical implications of breeding initiatives. Outcomes are often linked to broader goals, such as achieving Sustainable Development Goals (SDGs) or enhancing food security.
+Sources:
+File — Location — Cited IDs
+Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf — page 48 part 4 — pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4
+Policy Innovations_Inception Report 30-06-2025.pdf — page 13 part 2 — pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2
+Innovation use.docx — section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7 — docx:Innovation use.docx:u1-4
+General reporting guidance.docx — section 'General reporting guidance' paragraph 1 to section 'General reporting guidance' paragraph 5 — docx:General reporting guidance.docx:u1-3
+CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 22 part 4 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4</t>
+  </si>
+  <si>
+    <t>An outcome refers to a change in knowledge, attitudes, skills, and/or relationships (KASR) that results from research and its outputs, manifesting as a change in behavior among external actors. This can include the adoption of new technologies by farmers or the use of research-based knowledge by policy actors to inform decisions. Outcomes are influenced by the research but are not directly controlled by the researchers, distinguishing them from outputs, which are tangible products or services produced by the research process. The focus on outcomes emphasizes the broader impact of research initiatives on stakeholders and systems. 
+Sources:
+File: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf — page 9 part 1 — [ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1]
+File: 2025 Technical Reporting MELIA glossary.docx — table 1 row 28 to table 1 row 31 — [ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+File: Guidance on reporting outputs or outcomes.docx — paragraph 10 to paragraph 17 — [ID: docx:Guidance on reporting outputs or outcomes.docx:u7-10]
+File: CGIAR_ImpactReport_2022-24.pdf — page 11 part 1 — [ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt1]</t>
+  </si>
+  <si>
+    <t>An outcome refers to a change in knowledge, attitudes, skills, and/or relationships (KASR) that results from research outputs and activities. It signifies a behavioral change that occurs outside the research team, influenced by the research but not directly controlled by it. Examples of outcomes include the adoption of new technologies by farmers or the use of research-based knowledge by policy actors to inform decisions. In the context of CGIAR, outcomes are often linked to broader goals such as improving food security, enhancing livelihoods, and promoting sustainable practices. 
+Sources:
+File: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf — page 9 part 1 — [ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt1]
+File: 2025 Technical Reporting MELIA glossary.docx — table 1 row 28 to table 1 row 31 — [ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+File: Guidance on reporting outputs or outcomes.docx — paragraph 10 to paragraph 17 — [ID: docx:Guidance on reporting outputs or outcomes.docx:u7-10]</t>
+  </si>
+  <si>
+    <t>The CGIAR Results Framework categorizes outputs into three distinct types: outputs, outcomes, and impacts. Outputs refer to tangible products or services generated from CGIAR research, such as knowledge advancements, technical innovations, or capacity development activities. Outcomes represent changes in knowledge, attitudes, skills, or relationships that occur as a result of these outputs, while impacts reflect the long-term changes in conditions for people and their environments that result from the cumulative effects of outputs and outcomes. Each of these categories is essential for tracking progress and ensuring accountability within CGIAR's strategic goals.
+Sources:
+- File: CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf — Location: page 7 part 1 — Cited IDs: [ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt1]
+- File: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — Location: page 11 part 4 — Cited IDs: [ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4]
+- File: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf — Location: page 19 part 1 — Cited IDs: [ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt1]</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -796,6 +873,12 @@
   </si>
   <si>
     <t>Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24 — docx:Standard Provisions 2026.docx:u19-22, Standard Provisions 2026.docx — section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21 — docx:Standard Provisions 2026.docx:u16-19, Standard Provisions 2026.docx — section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33 — docx:Standard Provisions 2026.docx:u28-31</t>
+  </si>
+  <si>
+    <t>https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1 — page 48 part 4 — pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1 — page 13 part 2 — pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2, https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0 — section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7 — docx:Innovation use.docx:u1-4</t>
+  </si>
+  <si>
+    <t>https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1 — page 19 part 1 — pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt1, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1 — page 6 part 2 — pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt2, https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 22 part 4 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -2209,6 +2292,415 @@
 Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of chan</t>
   </si>
   <si>
+    <t xml:space="preserve">[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]
+breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in
+---
+[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]
+leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes
+---
+[ID: docx:Innovation use.docx:u1-4]
+Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?
+---
+[ID: docx:General reporting guidance.docx:u1-3]
+General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]
+the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]
+Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Number and type
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]
+in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]
+in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]
+of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]
+Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]
+been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?
+---
+[ID: docx:Innovation development.docx:u1-4]
+Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]
+four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the "challenges and megatrends" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]
+capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]
+Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2]
+2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intemediate Outcome: Crop Trust signs Long-Term Partnerships with CGIAR X X X X - Intermediate Outcome: CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness X X X X 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]
+RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4]
+intermediate outcomes that are not covered by any MELIA studies under the cross-cutting section should be entered under the relevant AoW-level outcome in the PORB
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1]
+27 Impact assessment efforts at the behavioral change level will focus on the 2030 Program Outcomes but also on unintended or unexpected significant outcomes highlighted through mid- term and final Outcome Evaluations and Policy change analyses (see Evaluation section). Data on behavioral changes will be monitored yearly through participatory outcome identification workshops with all partners engaged at the country/site level and outcome journals (see monitoring section). These yearly workshops at the country/site level are budgeted on the 20% non- assigned budget per center and have already been set aside by centers. The System Based Theory of Change approach will be applied to identify areas of success and prioritize the Outcome Evaluations (see
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]
+the misuse of funds for purposes outside what is set up in the
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 50 of 52 August 2025 | CGIAR Area of Work 2: Strategic User Engagement 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X - 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1]
+Learnings This review of CGIAR’s real-world outcomes and impacts provides valuable insights into how CGIAR generates and reports evidence. The experience of developing this report provided valuable learning opportunities to strengthen CGIAR’s evidence-generation and -aggregation processes so that future versions of this report may provide additional evidence. These insights are presented by topic. The 2022–2024 Results Framework At the outcome level, CGIAR Initiatives and Platforms report three types of outcomes: innovation use, policy change, and “other” outcomes. Although relatively few “other” outcomes were expected, well over 300 (28 percent) were reported. These correspond mainly to external engagement. In the future, consideration should be given to defining additional categories to reduce the number of “other” outcomes. In addition, CGIAR’s three Science Groups formulated a few key outcomes for their theories of change to which reported outcomes were mapped.
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt1]
+31 IA studies Result Level Countries MELIA Study Type Frequency MELIA study and tools Evaluation questions Multifunctional Landscapes Results Dashboard Potential Indicators Program 2030 Outcomes Colombia, Peru, Tunisia, Kenya, India, Vietnam Outcome Evaluation Mid term (2028) Endline (2030) Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent do multistakeholder engagement processes and co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Through which mechanisms does the multidisciplinary and transdisciplinary science promoted by the Multifunctional Landscapes program generate adoption of bundles of
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3]
+gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets, contributes to Agenda setting for our partners through research outputs. These Outcomes contributes to all of CGIAR Impact Areas, though the empahsis is on i) nutrition, health and food security; ii) poverty reduction, livelihoods and jobs; iii) climate adaptation and mitigation and iv) gender equality, Youth and social inclusion and to SDGs 1 (No Poverty), 8 (Decent Work and Economic Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt2]
+(Approved Budget) Intermediate Outcome: National partners apply skills to the management and exchange of agrobiodiversity X X X X - 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 27 of 52 Area of Work 4: Germplasm Health 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intermediate Outcome: CGIAR and internal and external partners exchange genetic resources without the risk of spreading quarantine pests or diseases X X X X - 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and more targeted
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4]
+system that allow to capture outputs and outcomes real-time, based on an Output Tracker and an Actor Engagement and Outcome Journal, currently under development. These two tools will be filled on the go by the team of MELIA friends for reporting at the country level, and by AoW leads/co-leads for what concerns activities not specific to the country sites. We will follow recommendations from the CGIAR Technical Reporting Arrangement (TRA) 2025 –30 and input all required reporting information in the
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2]
+foods? 2. How can animal and aquatic food systems support empowerment and create business opportunities and jobs for women, youth and marginalized groups? 3. What are the most effective scaling pathways to achieve SAAF outcomes combining effective partnerships, proven innovations, capacity sharing and supportive policies? 4. What are the best approaches to co-designing innovations and capacity-sharing approaches in specific contexts? 5. How do we most effectively influence, engage with and communicate to investors and policymakers the solutions, trade-offs and synergies of animal and aquatic sourced foods at the global, regional and national levels? After the CGIAR Science Week, we engaged with the Evaluability Assessment (EA) team by providing revised Theory of Change (ToC) diagrams. These revisions highlighted changes to the High -Level Outcomes (HLOs), intermediate outcomes, and 2030 outcomes. Since the overall logic of the ToC remained consistent, we did not share the narrative from the original
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt2]
+through which mechanisms agroecological and nature positive approaches, within a multifunctional landscape lens, optimize landscape multifunctionality? • What are the behavioral outcomes of such a multifunctional landscapes approach? For whom? Under what conditions? Behavior change studies are indispensable in understanding and addressing the human dimensions of agroecological transitions. By integrating socio -cultural, economic, and institutional insights, these studies ensure that interventions are not only scientifically robust but also socially acceptable and economically viable. Without excluding the analysis of other outcome generating processes, we will provide particular attention to the following outcome generating processes underlying the Program ToC: •
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u28-31]
+Key result story | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. Knowledge products | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. Outcome | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different.
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like </t>
+  </si>
+  <si>
+    <t>[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]
+breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in
+---
+[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]
+leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes
+---
+[ID: docx:Innovation use.docx:u1-4]
+Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?
+---
+[ID: docx:General reporting guidance.docx:u1-3]
+General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]
+the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]
+Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Number and type
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]
+in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]
+in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]
+Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]
+been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]
+of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian
+---
+[ID: docx:Innovation development.docx:u1-4]
+Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]
+four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the "challenges and megatrends" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]
+capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]
+Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2]
+2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intemediate Outcome: Crop Trust signs Long-Term Partnerships with CGIAR X X X X - Intermediate Outcome: CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness X X X X 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]
+RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4]
+intermediate outcomes that are not covered by any MELIA studies under the cross-cutting section should be entered under the relevant AoW-level outcome in the PORB
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1]
+27 Impact assessment efforts at the behavioral change level will focus on the 2030 Program Outcomes but also on unintended or unexpected significant outcomes highlighted through mid- term and final Outcome Evaluations and Policy change analyses (see Evaluation section). Data on behavioral changes will be monitored yearly through participatory outcome identification workshops with all partners engaged at the country/site level and outcome journals (see monitoring section). These yearly workshops at the country/site level are budgeted on the 20% non- assigned budget per center and have already been set aside by centers. The System Based Theory of Change approach will be applied to identify areas of success and prioritize the Outcome Evaluations (see
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]
+the misuse of funds for purposes outside what is set up in the
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p50pt1]
+Plan of results and budget 2025 | System Organization and center allocations | Page 50 of 52 August 2025 | CGIAR Area of Work 2: Strategic User Engagement 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X - 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1]
+Learnings This review of CGIAR’s real-world outcomes and impacts provides valuable insights into how CGIAR generates and reports evidence. The experience of developing this report provided valuable learning opportunities to strengthen CGIAR’s evidence-generation and -aggregation processes so that future versions of this report may provide additional evidence. These insights are presented by topic. The 2022–2024 Results Framework At the outcome level, CGIAR Initiatives and Platforms report three types of outcomes: innovation use, policy change, and “other” outcomes. Although relatively few “other” outcomes were expected, well over 300 (28 percent) were reported. These correspond mainly to external engagement. In the future, consideration should be given to defining additional categories to reduce the number of “other” outcomes. In addition, CGIAR’s three Science Groups formulated a few key outcomes for their theories of change to which reported outcomes were mapped.
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p31pt1]
+31 IA studies Result Level Countries MELIA Study Type Frequency MELIA study and tools Evaluation questions Multifunctional Landscapes Results Dashboard Potential Indicators Program 2030 Outcomes Colombia, Peru, Tunisia, Kenya, India, Vietnam Outcome Evaluation Mid term (2028) Endline (2030) Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent do multistakeholder engagement processes and co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Through which mechanisms does the multidisciplinary and transdisciplinary science promoted by the Multifunctional Landscapes program generate adoption of bundles of
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3]
+gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets, contributes to Agenda setting for our partners through research outputs. These Outcomes contributes to all of CGIAR Impact Areas, though the empahsis is on i) nutrition, health and food security; ii) poverty reduction, livelihoods and jobs; iii) climate adaptation and mitigation and iv) gender equality, Youth and social inclusion and to SDGs 1 (No Poverty), 8 (Decent Work and Economic Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4]
+system that allow to capture outputs and outcomes real-time, based on an Output Tracker and an Actor Engagement and Outcome Journal, currently under development. These two tools will be filled on the go by the team of MELIA friends for reporting at the country level, and by AoW leads/co-leads for what concerns activities not specific to the country sites. We will follow recommendations from the CGIAR Technical Reporting Arrangement (TRA) 2025 –30 and input all required reporting information in the
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p51pt2]
+(Approved Budget) Intermediate Outcome: National partners apply skills to the management and exchange of agrobiodiversity X X X X - 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and
+---
+[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p27pt1]
+CGIAR | August 2025 Plan of results and budget 2025 | System Organization and center allocations | Page 27 of 52 Area of Work 4: Germplasm Health 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intermediate Outcome: CGIAR and internal and external partners exchange genetic resources without the risk of spreading quarantine pests or diseases X X X X - 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and more targeted
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2]
+foods? 2. How can animal and aquatic food systems support empowerment and create business opportunities and jobs for women, youth and marginalized groups? 3. What are the most effective scaling pathways to achieve SAAF outcomes combining effective partnerships, proven innovations, capacity sharing and supportive policies? 4. What are the best approaches to co-designing innovations and capacity-sharing approaches in specific contexts? 5. How do we most effectively influence, engage with and communicate to investors and policymakers the solutions, trade-offs and synergies of animal and aquatic sourced foods at the global, regional and national levels? After the CGIAR Science Week, we engaged with the Evaluability Assessment (EA) team by providing revised Theory of Change (ToC) diagrams. These revisions highlighted changes to the High -Level Outcomes (HLOs), intermediate outcomes, and 2030 outcomes. Since the overall logic of the ToC remained consistent, we did not share the narrative from the original
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p24pt2]
+through which mechanisms agroecological and nature positive approaches, within a multifunctional landscape lens, optimize landscape multifunctionality? • What are the behavioral outcomes of such a multifunctional landscapes approach? For whom? Under what conditions? Behavior change studies are indispensable in understanding and addressing the human dimensions of agroecological transitions. By integrating socio -cultural, economic, and institutional insights, these studies ensure that interventions are not only scientifically robust but also socially acceptable and economically viable. Without excluding the analysis of other outcome generating processes, we will provide particular attention to the following outcome generating processes underlying the Program ToC: •
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u28-31]
+Key result story | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. Knowledge products | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. Outcome | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods a</t>
+  </si>
+  <si>
+    <t>[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]
+breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in
+---
+[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]
+leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes
+---
+[ID: docx:Innovation use.docx:u1-4]
+Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?
+---
+[ID: docx:General reporting guidance.docx:u1-3]
+General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]
+the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p18pt4]
+better understand farmer perspectives, motivations, and constraints concerning the adoption of SFP innovations. 4. Adoption or diffusion studies addressing learning questions on the TOC The baseline surveys conducted in Ghana, Malawi, and Ethiopia focusing on sustainable intensification technologies will form the basis for the adoption and impacts studies. These studies will seek to answer the following causal impact learning questions: ( 1) What factors are constraining/enabling the scaling and adoption as well as the intensity of use of the SFP innovations? and (2) How does adoption of the SFP innovations impact yield, farm income and household income? (3) What are the most promising inte grated farm -level innovation bundles to improve sustainability, equity, and agronomic gain at scale within the selected geographies of the program? To answer these questions, adoption and impact studies build up on the baseline studies (panel survey) to assess the extent, pathways, and determinants of
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]
+been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]
+four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the "challenges and megatrends" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]
+Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]
+of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]
+in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]
+in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.
+---
+[ID: docx:Innovation development.docx:u1-4]
+Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3]
+activities of the CapSha Accelerator, its products and services, contribute to improved capacity development practices, resulting in more equitable partnerships? • Are CGIAR NARES partners, donors and CapSha expert institutions making use of CapSha products and services? • Are CGIAR NARES partners, donors and CapSha expert institutions member of the CapSha Cop? • To what extent are the CapSha Accelerator’s objectives aligned with the needs and priorities of Southern partners? • What elements of the partnership model have the potential to be scaled or replicated in other regions or contexts? What are the enabling and limiting factors affecting scalability? How have Southern partners contributed to or led scaling efforts, and what support mechanisms have been most effective? • What measurable
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]
+Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support
+---
+[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]
+the misuse of funds for purposes outside what is set up in the
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]
+RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]
+capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]
+Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Number and type
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p6pt2]
+foods? 2. How can animal and aquatic food systems support empowerment and create business opportunities and jobs for women, youth and marginalized groups? 3. What are the most effective scaling pathways to achieve SAAF outcomes combining effective partnerships, proven innovations, capacity sharing and supportive policies? 4. What are the best approaches to co-designing innovations and capacity-sharing approaches in specific contexts? 5. How do we most effectively influence, engage with and communicate to investors and policymakers the solutions, trade-offs and synergies of animal and aquatic sourced foods at the global, regional and national levels? After the CGIAR Science Week, we engaged with the Evaluability Assessment (EA) team by providing revised Theory of Change (ToC) diagrams. These revisions highlighted changes to the High -Level Outcomes (HLOs), intermediate outcomes, and 2030 outcomes. Since the overall logic of the ToC remained consistent, we did not share the narrative from the original
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1]
+Learnings This review of CGIAR’s real-world outcomes and impacts provides valuable insights into how CGIAR generates and reports evidence. The experience of developing this report provided valuable learning opportunities to strengthen CGIAR’s evidence-generation and -aggregation processes so that future versions of this report may provide additional evidence. These insights are presented by topic. The 2022–2024 Results Framework At the outcome level, CGIAR Initiatives and Platforms report three types of outcomes: innovation use, policy change, and “other” outcomes. Although relatively few “other” outcomes were expected, well over 300 (28 percent) were reported. These correspond mainly to external engagement. In the future, consideration should be given to defining additional categories to reduce the number of “other” outcomes. In addition, CGIAR’s three Science Groups formulated a few key outcomes for their theories of change to which reported outcomes were mapped.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u28-31]
+Key result story | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. | In-depth accounts of results that provide insight into CGIAR contribution to outcomes and/or impact. Each year, Programs and Accelerators are asked to report at least one key result story. Knowledge products | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. | Knowledge products are intellectual assets generated from research and development activities such as articles, briefs, reports, extension and training content, databases, software, and multimedia elements that contribute to behavioural changes in particular actors. Outcome | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. | A change in knowledge, attitudes, skills, and/or relationships (KASR), which manifests as a change in behaviour within the spheres of influence and interest, that results in whole or in part from the research and its outputs. Examples: use of a new technology (including outputs like a seed variety) by farmers; policy actors using research-based knowledge to inform policy decisions; participants in a CGIAR-supported process agree to new germplasm conservation and exchange protocols; researchers use CGIAR generated methods and/or databases. Key outcomes: Who will do what differently as a result of the Program/Accelerator/Project. Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different.
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt3]
+gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets, contributes to Agenda setting for our partners through research outputs. These Outcomes contributes to all of CGIAR Impact Areas, though the empahsis is on i) nutrition, health and food security; ii) poverty reduction, livelihoods and jobs; iii) climate adaptation and mitigation and iv) gender equality, Youth and social inclusion and to SDGs 1 (No Poverty), 8 (Decent Work and Economic Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p31pt2]
+has CGIAR-NARES prioritization of products encouraged targeted investment for breeding? (AOW2 AB) RQ9 To what extent has the amount and quality of active collaboration on products increased? (AOW5 E) RQ11 To what extent has B4T influenced more equitable access to improved varieties by marginalized groups? (AOW3 ID) RQ27 To what extent have interoperable tools and services
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.
+---
+[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p13pt2]
+agrifood system actors use metrics and analytics to understand and monitor progress in addressing structural barriers to gender equality and social inclusion; and ultimately; 4. Women, youth, and socially excluded groups have equitably benefited from innovations designed to enhance sustainability and outcomes from agrifood systems. These outcomes are interconnected and interdependent, and the achievement of each is not linear. The achievement of the first three outcomes is also a precondition to the achievement of the fourth 2030 outcome. The 2030 outcomes will be achieved through the two interconnected AoWs. Since the original proposal, we have updated the high-level outputs across the two AoWs, to harmonize and clarify what key offerings the Accelerator will produce by the end of 2030. AoW on Solutions: The Accelerator’s first impact pathway will mostly be pursued through this AoW by working with partners on the ground. The AoW on Solutions builds on a conceptual framework that surfaces four
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt1]
+Program and Accelerator MELIA Plan Update Template and Guidance I March 2025 9 1. Monitoring plan for HLOs and outcomes This section outlines how the Policy Program will monitor delivery of HLOs and progress towards outcomes. For tracking progress, the high -level outputs (HLOs) and intermediate outcomes, are each supported by specific activities detailed in the Program of Work and Budget (POWB). This framework serves as the foundation for monitoring progress, ensuring not only the implementation of activities but also the validation of underlying assumptio ns to achieve the anticipated changes. Targets were developed consultatively within the AoWs but also corroborated at the Program level since this determines the overall targets committed for the 2030 Outcomes. Data collection strategy The Results Framework details the HLOs , Intermediate Outcomes and 2030 Outcomes they c</t>
+  </si>
+  <si>
+    <t>[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt1]
+Results framework The program result
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt2]
+Work 2.3 Results framework The CapSha Accelerator results framework has been
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4]
+CGIAR Results Framework – Portfolio Outcome
+---
+[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt2]
+types For reference only, the current MELIA study types defined in
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt1]
+CGIAR Performance and Results Management Framework 2022-2030 CGIAR System Organization Page 7 of 20 4. Results framework CGIAR’s results framework is directly aligned to the five impact areas and Sustainable Development Goals. Three distinct result types: outputs, outcomes and impacts are mapped to the spheres of Control, Influence and Interest, respectively. • Output: Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples of outputs include new research methods, policy analyses, gene maps, new crop varieties and breeds, or other products of research work. • Outcome: A change in knowledge, skills, attitudes and/or relationships, which manifests as a change in behavior of users of outputs, to which a combination of research outputs and related activities have contributed. •
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3]
+portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3]
+portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.
+---
+[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt3]
+Results Framework Please refer
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p28pt2]
+4. MELIA study types For reference only, the current MELIA study types
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u55-58]
+Policy change | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. Portfolio | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. Program | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. Result | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact. | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact. | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact.
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p9pt2]
+Mitigation, Nutrition, Poverty Reduction and Livelihoods, Gender Equality and Social Inclusion, and Environmental Health and Biodiversity. The SFP results framework operationalizes this contribution by aligning program indicators and learning activities with CGIAR’s Performance and Results Management Framework (PRMF) and systematically collect evidence across the eight AoWs. Each AoW is designed to deliver results that directly or indirectly support one or more CGIAR Impact Areas. The framework provides a coherent roadmap for measuring the SFP contributions. Open Access link for both the ToC and the Results Framework . (Download the Results Framework as part of several other worksheets-e.g., assumptions, research questions, etc using the 3rd icon on the top left conner of the page). 3. Monitoring plan for HLOs and outcomes This section outlines how the Program will monitor delivery of HLOs and progress towards
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1]
+7 Results framework The Result Framework presents a structured articulation of the intended results under CGIAR’s strategic Areas of Work (AOWs) for the period 2025 to 2030. It distinguishes between two types of results: High-Level Outputs (HLOs), which represent tangible, near-term deliverables from research eƯorts, and Intermediate Outcomes (IOCs), which indicate progress toward longer- term development goals and systemic change. Each result entry captures several key variables—among many others—that collectively deﬁne the pathway from research to impact. These include the thematic Area of Work to which the result contributes, the classiﬁcation of the result as either an output or outcome, and a short title paired with a detailed result statement that describes the intended change, innovation, or contribution. The responsible organization(s), often CGIAR centers, are identiﬁed alongside any listed partners and outcome actors, with additional information on whether those actors are directly engaged and what
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt2]
+result framework is accessible from
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p8pt2]
+the Program and Area of Work levels. This link gives the ToC tables-overall and AoW ToCs) and Open Access link for both the ToC and the Results Framework . (Zoom out to see the linkages of the various AoW ToCs and download the ToC tables using the 4 th icon on the top left conner of the page). Figure 1. Sustainable Farming Program level Theory of Change Results framework The SFP Results Framework reflects the logical sequence from high-level outputs to intermediate outcomes, aligned with the program’s Theory of Change. It captures the intended contributions of each AoW,
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u34-37]
+High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). Partner | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. Partner typology (CGIAR) | CGIAR uses a partner typology to define partner types. Definitions are presented below. | CGIAR uses a partner typology to define partner types. Definitions are presented below. | CGIAR uses a partner typology to define partner types. Definitions are presented below. Partner typology (CGIAR) | CGIAR type | CGIAR type definition
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p32pt3]
+tab in the program result s framework accessible
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2]
+Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2]
+Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p3pt1]
+3 1. Reviewing guidance for developing the MELIA Plan Developing the Sustainable Farming program (SFP) MELIA plan, started with the review of the ISDC feedback on the overall program Theory of Change (ToC) and the Area of Work (AoW) ToCs. This feedback has been used in updating the ToC, (example, creating indicators for AoW 8 - Program Efficiency and Delivery . In addition, the core assessment criteria from the IAES evaluability assessment guide were used as reference checks in developing the MELIA plan. 2. Program overview and results framework This section provides a n overview of the Sustainable Farming Program (SFP), outlining its intervention logic and the results framework. It also details the alignment of the Program’s results framework with the CGIAR Performance and Results Management Framework (PRMF) and Portfolio outcomes, ensuring system thinking. Program overview SFP is designed to respond to
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3]
+2030 Outcome, or Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framework Provide the assumption( s) statem ent from the Results Framework Indicate the location(s) where the study will be conducted Indicate the methods and design approaches that will be used for the study List the Program(s) and Accelerator( s ) you will collaborate with or coordinate for the implementati on of this study. Indicate the Start
+---
+[ID: pdf:Type3_2024Report.pdf:p11pt4]
+System (PRMS): The PRMS serves as the central reporting platform, powering the Results Dashboard and supporting the development of Type 1 Reports with real-time data aggregation and analysis. These components were instrumental in driving the 2024 Technical Reporting process, and key elements will be carried forward to shape Technical Reporting in the next CGIAR Portfolio, ensuring continuity, alignment, and continuous improvement. Monitoring tools tailored to suit core indicators Non-pooled projects Type 1 Type 3 Science Group Projects Research and Performance and Results Management Framework Arrangement CGIAR Results Framework Standard Indicator Theory of Change and Scaling Readiness (IPSR) Quality Assurance criteria, process Performance and Results Management System Type 2 Triennial Outcome/Impact Report Annual Technical Report Results Dashboard $771M Revenue 2% 23% 44% 31% Revenue by Funding Source Windows 1&amp;2 | Window 3 | Bilateral | Other 1 2 3 4 5 6 7 8 9 10 13 12 11 6. CGIAR 2030 Research and Innovation Strategy 7. Performance and Results Management Framework 8. Technical Reporting Arrangement 9. CGIAR Results Framework 10. Standard Indicator Description Sheets: • Output level • Outcome level 11. Theory of Change 12. IPSR • Output level • Outcome level • IPM for responsible food systems transformation • Scaling Readiness website • Online course on Innovation and Scaling • Scaling Readiness calculator • Scaling Directory 13. Adaptive Management 14. Quality Assurance 15. PRMS &amp; TOC board 16. Results Dashboard 17. 2022 &amp; 2023 Annual Technical Reports 18. Type 2 report Grass pea production in Odisha. Credit: IRRI May 2025 17 16 CGIAR Portfolio Practice Change (Type 3) Report
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p13pt1]
+Genebank Accelerator MELIA Plan 13 The Annual Genebank Meetings (AGMs) are an important forum to review and reflect on the CGIAR Genebanks past year’s activities, progress and achievements, and to make plans for the next year. National partners, CGIAR programs, and technical and scientific experts are represented in the AGMs, and the location of the meeting is in a different region each year to assure better interaction with multiple stakeholders from different regions. By doing this, we are constantly consulting with partners in different regions of the world, understanding their realities and needs so we can better plan the
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt2]
+we will approach this as a learning journey with stakeholders, building on existing expertise, studies and approaches to land on an approach that is meaningful and cost-effective. Linking $ to results CGIAR aims to establish a fit for purpose solution that provides intelligence on how financial inputs connect to different types of outputs, outcomes and impacts across CGIAR's portfolio. This is crucial for improving transparency and accountability, as well as for resource prioritization and portfolio man agement. The primary objective is to establish a transparent link , at an appropriate level of granularity, between financial investments and the tangible results they yield. Having such linkages will also allow CGIAR to better: 1. Ensure successful CGIAR 2030 Research and Innovation Strategy implementation under different funding scenarios 2. Make
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p18pt2]
+we will approach this as a learning journey with stakeholders, building on existing expertise, studies and approaches to land on an approach that is meaningful and cost-effective. Linking $ to results CGIAR aims to establish a fit for purpose solution that provides intelligence on how financial inputs connect to different types of outputs, outcomes and impacts across CGIAR's portfolio. This is crucial for improving transparency and accountability, as well as for resource prioritization and portfolio man agement. The primary objective is to establish a transparent link , at an appropriate level of granularity, between financial investments and the tangible results they yield. Having such linkages will also allow CGIAR to better: 1. Ensure successful CGIAR 2030 Research and Innovation Strategy implementation under different funding scenarios 2. Make
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 13 operational plans. They will underpin geography and impact pathway -specific outcome and impact assessments at different levels. They will provide more consistent information for future evaluations and other studies. • There are in the order of 10,000 indicators in use across CGIAR’s 900+ active projects with limited consistency among them. Most indicators (around 80%) map well to existing CGIAR Results Framework categories but are defined and measured in different ways, meaning that effective transfer of data and learning between extant and successive generations of Portfolio components is suboptimal. The resulting high rate of single use results data in the CGIAR hampers effective delivery and learning at all levels. If standard indicators, data collection tools, protocols, and collected data are integrated into new w3 and
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 13 operational plans. They will underpin geography and impact pathway -specific outcome and impact assessments at different levels. They will provide more consistent information for future evaluations and other studies. • There are in the order of 10,000 indicators in use across CGIAR’s 900+ active projects with limited consistency among them. Most indicators (around 80%) map well to existing CGIAR Results Framework categories but are defined and measured in different ways, meaning that effective transfer of data and learning between extant and successive generations of Portfolio components is suboptimal. The resulting high rate of single use results data in the CGIAR hampers effective delivery and learning at all levels. If standard indicators, data collection tools, protocols, and collected data are integrated into new w3 and
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt1]
+7 Results framework Aligned with the Program’s updated ToC, the results framework outlines the identiﬁed indicators per result and corresponding targets. It further speciﬁes monitoring, and evaluation approaches that document and assess progress toward each indicator target to inform performance review and adaptive management. This guides the overall MELIA Plan, particularly the data collection strategy, MELIA studies, and other MELIA activities in target countries in close collaboration with other Programs, Accelerators, and bilateral projects. Refer to the Results Framework attachment for additional information. 2. Monitoring plan for high-level outputs (HLOs) and outcomes Data collection strategy The Climate Action Program will adopt a monitoring-for-learning approach grounded in results-based management (RBM) principles and aligned with CGIAR’s Performance and Results Management Framework (PRMF). Progress will be tracked against deﬁned indicators and targets as outlined in
+---
+[ID: pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p9pt2]
+the municipal market in Tucuru, Guatemala. Using several different strategies tailored to different contexts, the Better Diets and Nutrition program aims to
+---
+[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]
+Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p15pt3]
+AOW results and
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3]
+Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framewo rk Provid e the assu mptio n(s) state ment from the Resul ts Fram ework Indicate the location( s) where the study will be conducte d Indicate the methods and design approache s that will be used for the study List the Progr am(s) and Accel erato
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt1]
+2. Monitoring plan for HLOs and outcomes This section outlines how Better Diets and Nutrition will monitor the delivery of high-level outputs (HLOs) and progress toward defined outcomes. The monitoring approach reflects the Program's decentralized structure with strong central coordination, ensuring that routine tracking of indicators against the logical framework is feasible, relevant, and aligned with resource availability. Indicators will be reviewed annually and revised as necessary, based on implementation progress, emerging priorities, and feedback from AoW teams and partners. The Program ToC and result s framework comprises 22 HLOs and 30 outcomes . The results framework for the program will be submitted through the Performance and Results Management System (PRMS) ToC Board, and exported in Excel format for review, as per guidance. HLOs represent results such as tools, guidelines, datasets, and tested solutions; outcomes represent the behavioral and systemic changes these outputs are expected to generate. We will use the
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt1]
+Results framework Program/Accelerator results framework Please refer to the Results Framework attachment 2. Monitoring plan for HLOs and outcomes The genebanks will continue to use an online reporting tool (ORT), which was set up in 2014 to monitor the status of individual collections with respect to performance targets. Through the QMS adopted in AoW 1, genebank operations, data, and accession numbers are audit ed internally and externally and are subject to regular review by the Crop Trust. The audits ensure that international standards are complied with, and deviations and risks are documented and managed. FAO’s monitoring of UN SDG 2.5, State of the World of PGRFA, and the Global Plan of Action</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -2270,6 +2762,18 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who has fiduciary responsibility over the Windows 1 and 2 funds, and what must they guarantee?\n\nContext:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u19-22]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 21 to section 'Use and administration of the Contributions' paragraph 24\nContent: Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively: ensure that such Window 1 and Window 2 Funds are used exclusively for their intended purposes; ensure that such Window 1 and Window 2 Funds are administered, used and expended in accordance with the CGIAR System Charter, the CGIAR System Framework and the applicable Fund Use Agreements entered into by it, including by taking corrective action with respect to Window 1 and Window 2 Funds not used in accordance with the relevant Fund Use Agreement; and monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u16-19]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 18 to section 'Use and administration of the Contributions' paragraph 21\nContent: Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research. Disbursement to Centers. The System Organization may, from time to time, initiate disbursements of Window 1 and Window 2 Funds to a Center for approved CGIAR Programs. Disbursement to a Program Participant. Subject to paragraph 2.4 of the Standard Provisions, Centers receiving Window 1 and Window 2 Funds may make further disbursements of such funds to Program Participants for the relevant CGIAR Program under Subagreements. Fiduciary Responsibility for the Use of Window 1 and Window 2 Funds. The System Organization has fiduciary responsibility toward Funders for the use of Window 1 and Window 2 Funds. Each Center has fiduciary responsibility toward the System Organization for the use of the Window 1 and Window 2 Funds it receives. With respect to the funds for which they have fiduciary responsibility, the System Organization and each Center will, respectively:\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u28-31]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 30 to section 'Window 3 Funds.' paragraph 33\nContent: ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements; monitor, evaluate as applicable, and provide quality assurance and financial and technical reporting for activities funded by Window 3 Funds in accordance with the relevant terms of these Standard Provisions; and if the Window 3 Funds are mapped to a CGIAR Program (i.e. provided for CGIAR Research activities that are aligned to the CGIAR Program's high-level outcomes and theory of change), continuously inform the System Organization and the project management unit of such CGIAR Program of the receipt of any Window 3 Funds and their use. The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u31-34]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 33 to section 'Window 3 Funds.' paragraph 36\nContent: The System Organization will not have fiduciary or programmatic responsibility over, or responsibility to supervise or monitor, Window 3 Funds. The System Organization may, however: upon request of a Funder providing Window 3 Funds and acting through the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center; or in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u181-184]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198 to section 'Misused Fund' paragraph 202\nContent: Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Misused Fund Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, refund any portion of Window 1 and Window 2 Funds not used in accordance with the applicable Fund Use Agreements, and such funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u13-16]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 15 to section 'Use and administration of the Contributions' paragraph 18\nContent: In addition to the designation of contributions to the Trust Fund in accordance with the CGIAR Trustee Agreement and the Contribution Agreements or Arrangements, Funders may further designate Window 1 Funds and/or Window 2 Funds for specific purposes at the operational level subject to a decision of the System Council enabling such designations, and in accordance with a procedure for designation of funds at operational level, as may be adopted from time to time. Responsibilities over Window 1 and Window 2 Funds Disbursement to the System Organization. Window 1 and Window 2 Funds will be disbursed from time to time for the activities of the System Organization (including System Costs) and for CGIAR Research.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u178-181]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 194 to section 'Return of Funds. Unexpended or Uncommitted Funding.' paragraph 198\nContent: appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center. Return of Funds. Unexpended or Uncommitted Funding. Window 1 and Window 2 Funds. The System Organization and each Center will, respectively, promptly return any portion of Window 1 and Window 2 Funds that is unexpended or uncommitted at the completion of a CGIAR Program or activities under the CGIAR Program for which it was provided (including approved extensions) or at the termination of a Financial Framework Agreement between the System Organization and a Center, unless decided otherwise by the System Council. Such returned funds will be deposited to Window 1 of the Trust Fund. Window 3 Funds. At the written direction of an individual Funder, the System Organization will require Centers to promptly return any portion of Window 3 Funds that are unexpended or uncommitted at the completion of the CGIAR Research for which it was provided (including approved extensions). Such returned funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u22-25]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Use and administration of the Contributions' paragraph 24 to section 'Window 3 Funds.' paragraph 27\nContent: monitor, evaluate, and provide quality assurance and financial and technical reporting for activities funded by Window 1 and Window 2 Funds in accordance with the relevant terms and requirements of these Standard Provisions. Window 3 Funds. Window 3 Funds are directed by Funders to individual Centers. Funders may designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u172-175]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 187 to section 'Acknowledgement of Funders' paragraph 191\nContent: Acknowledgement of Funders All communications products on CGIAR Research funded by Window 1, 2 and 3 Funds, whether online or in hard copy form (e.g., publications, press releases, newsletters, website stories, blogs, posters, etc.), must acknowledge support received from Funders in accordance with applicable CGIAR Policies and Procedures on branding and communication. Suspending Transfers of Funding from Window 1 and 2 Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u4-7]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Introductory Provisions' paragraph 5 to section 'Introductory Provisions' paragraph 8\nContent: the Financial Framework Agreement between the System Organization and each Center with respect to Window 1, 2 and 3 Funds; and any Window 3 Side Agreement or Arrangement between a Funder and a Center with respect to Window 3 Funds. Interpretation of the Standard Provisions. Unless the context requires otherwise, the terms of these Standard Provisions governing the roles and responsibilities: between Funders and the System Organization apply to each Funding Agreement or Arrangement between a Funder and the System Organization;\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p31pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 31 part 2\nContent: protocols for data anonymization and access requests Implementation and oversight Data management responsibilities will be integrated into research staff roles with the ultimate responsibility being the\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u46-49]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Cost Sharing Percentage' paragraph 49 to section 'Standard of care.' paragraph 53\nContent: Window 1, 2 and 3 Funds. Centers will not have any obligation to collect or otherwise pay the CSP on funds disbursed through Windows 1, 2 or 3. The Funders, the System Organization and the Centers recognize that the Trustee of the CGIAR Trust Fund will collect the CSP before such funds are disbursed from the Trust Fund. Requirements on the Use of Window 1, 2 and 3 Funds CGIAR Policies and Procedures. The System Organization and each Center will, respectively ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures and the relevant entity's own policies and procedures. All CGIAR Policies and Procedures will be available on the System Organization's web site. Standard of care.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u55-58]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 59 to section 'Financial, Economic and Administrative Standards' paragraph 62\nContent: Efficiency. The System Organization and each Center will, respectively: ensure that Window 1, 2 and 3 Funds are used with due regard to economy and efficiency, and that the highest standards of integrity in the administration of the funds are upheld; and ensure that Window 1, 2 and 3 Funds are used in accordance with applicable CGIAR Policies and Procedures on cost allocation, which set forth the principles of allowability, allocability, and reasonableness. Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u25-28]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 27 to section 'Window 3 Funds.' paragraph 30\nContent: designate specific amounts to specific Centers for use by the Center; provided such funds are used to implement aspects of the Strategy and Research Framework and provided further that such funds are used in accordance with applicable CGIAR Policies and Procedures. Designations of Window 3 Funds by Funders to Centers are not subject to review, allocation or approval by the System Organization. Centers receiving Window 3 Funds are responsible for the use of such funds and will: ensure that Window 3 Funds are used exclusively for their intended purposes; ensure that Window 3 Funds are administered, used and expended in accordance with the applicable Fund Use Agreements entered into by them, including by taking corrective action with respect to those funds not used in accordance with such Fund Use Agreements;\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u34-37]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Window 3 Funds.' paragraph 36 to section 'Window 3 Funds.' paragraph 39\nContent: in consultation with the relevant Funder providing Window 3 Funds and the System Council, take corrective action vis-â-vis a Center in the event such Window 3 Funds are not used in accordance with any applicable Fund Use Agreement entered into by such Center. Window 3 Side Agreements or Arrangements. Nothing in the Funding Agreements or Arrangements is intended to preclude Funders and Centers from entering into Window 3 Side Agreements or Arrangements in regard to the terms governing the administration and use of Window 3 Funds. Funders may choose to make a Contribution to a Center through Window 3 without entering into a Window 3 Side Agreement or Arrangement, provided that such Contribution is made without any additional conditions attached to it. Any Window 3 Side Agreement or Arrangement will be consistent with these Standard Provisions and substantially in the form of Schedule 1 (Form of Window 3 Side Agreement or Arrangement) attached to these Standard Provisions, as may be amended from time to time. Program Participants. In engaging a Program Participant with respect to Window 1, 2 and 3 Funds, Centers will incorporate in the relevant Subagreements, and cause, and monitor, compliance with the obligations set out in the Standard Provisions, including but not limited to those set out in paragraphs 2.5-2.6, 4-6, 7.2.2, 7.1.3, 7.3.2, 8.3, 8.4.4,\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u163-166]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Limitation of Liabilities' paragraph 176 to section 'No Additional Obligations' paragraph 180\nContent: In providing funds under: Funding Agreements or Arrangements, or Window 3 Side Agreements or Arrangements, Funders do not accept any responsibility or liability towards any third parties including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund; and Financial Framework Agreements, the System Organization does not accept, any responsibility or liability towards any third parties, including any claims, debts, demands, damage or loss as a result of the implementation of activities with funds from the Trust Fund. No Additional Obligations\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u58-61]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Financial, Economic and Administrative Standards' paragraph 62 to section 'Financial, Economic and Administrative Standards' paragraph 65\nContent: Investment Income. The System Organization and each Center will, respectively, ensure that any investment income generated by the portions of the Window 1, 2 and 3 Funds they receive, including currency conversion gains, will be used for CGIAR Research or, if not needed for such purposes, returned to the Trustee for deposit into Window 1 to be made available for allocation by the System Council. Procurement. In the event that consultants are employed or services or goods are procured with Window 1, 2 and 3 Funds, the System Organization and each Center will, respectively, ensure that the employment and supervision of such consultants and the procurement of such services or goods will be the responsibility of each entity employing or contracting such consultants or carrying out such procurement and will be conducted in conformity with applicable CGIAR Policies and Procedures on procurement, in line with the following basic principles of equal treatment and non-discrimination on grounds of nationality, competition, predictability, transparency, verifiability, and proportionality. No taxation. The System Organization and each Center will, respectively, use best efforts, to the extent allowed by applicable agreements, such as those signed with host governments, and applicable laws, to ensure that the use of Window 1, 2 and 3 Funds will be free from any taxation or fees imposed under local laws. Insurance. The System Organization and each Center will, respectively, maintain insurance coverage sufficient to cover the activities, risks, and potential omissions of the activities funded by Window 1, 2 and 3 Funds in accordance with generally accepted industry standards and as required by law.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u106-109]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Monitoring and Evaluations' paragraph 115 to section 'Monitoring' paragraph 118\nContent: Funders will manage their monitoring and evaluation requirements with respect to the CGIAR Portfolio, collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to conduct duplicative evaluations, provided that Funders providing Window 3 Funds may require supplemental monitoring and evaluations with respect to Window 3 Funds, the costs of which, including the internal costs to the System Organization or Center, would be paid by the requesting Funder. If an individual Funder wishes to request, on an exceptional basis, a review or evaluation of any activities financed with Window 1 and Window 2 Funds, such Funder will consult with a designated representative from the System Organization on the most appropriate scope and terms of reference of such review or evaluation. The designated representative will assist in arranging for such review or evaluation in accordance with the applicable CGIAR Policies and Procedures. The costs of any such review or evaluation, including the internal costs of the System Organization or Center with respect to such review or evaluation, will be paid by the requesting Funder. The System Organization and each Center will, respectively collaborate on any monitoring or evaluations conducted in connection with CGIAR Research activities funded with Window 1, 2 and 3 Funds. Monitoring\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u175-178]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Acknowledgement of Funders' paragraph 191 to section 'Acknowledgement of Funders' paragraph 194\nContent: Suspension by the System Organization. The System Organization may, at any time, suspend transfers of Window 1 and Window 2 Funds allocated to a specific Center by providing a written notice to the relevant Center: (a) if the System Organization has a credible concern that the Window 1, 2 and 3 Funds are not used in accordance with the applicable Fund Use Agreements, or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) in the event of non-compliance by the Center with any of its obligations under an applicable Fund Use Agreement. Before taking such action under paragraph 13.1, the System Organization will notify the relevant Center in writing, and consult with the System Council as well as the relevant Center with a view to identify ways and means to manage the suspension and mitigate the impact on the implementation of CGIAR Research until such time that the suspension may be lifted. If such suspension is lifted by the System Organization, it will notify the relevant Center in writing. Request by a Funder. If a Funder has a credible concern: (a) that Window 1, 2 and 3 Funds are not used by a Center in accordance with the applicable Fund Use Agreement or of an interpersonal misconduct in connection with the implementation of activities financed by Window 1, 2 and 3 Funds; and/or (b) of a non-compliance by a Center with any of its obligations under an applicable Fund Use Agreement, the Funder may request, through the System Council, the System Organization to review the specific concern and, as relevant, to take appropriate corrective action. The System Organization will report to the System Council on the outcome of the review and, as appropriate, the corrective action undertaken to address the concern, which may include suspension of transfer of Window 1 and Window 2 Funds to the Center.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u184-189]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Misused Fund' paragraph 202 to section 'Inconsistency' paragraph 207\nContent: Window 3 Funds. Subject to paragraph 2.3.4 of these Standard Provisions, the System Organization will require Centers to refund any portion of Window 3 Funds not used in accordance with the applicable Fund Use Agreement, and such Funds will be deposited to Window 1, Window 2 or Window 3 of the Trust Fund as directed by the Funder that contributed such funding. Inconsistency In the event of any inconsistency between the Cover Pages and these Standard Provisions, these Standard Provisions will prevail. Amendments Amendments These Standard Provisions may only be amended by approval of the System Council subject to concurrence of the Integrated Partnership Board. The System Organization will promptly notify the Funders and Centers in writing of any such amendments to these Standard Provisions.\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p5pt1]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 5 part 1\nContent: Section 1: Connecting impact and insight: The 2024 CGIAR Portfolio Narrative 1. SGPs are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance, and fiduciary oversight. 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022–2024. 3. EiB II reported through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they provided a concise, high- level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the Technical Reports. The 2024 CGIAR Portfolio Narrative is a cornerstone of CGIAR’s Technical Reporting Arrangement. It offers a synthesis of Portfolio coherence, synergies, and collective progress across Initiatives, Impact Platforms, and Science Group Projects (SGPs)1, which represent approximately 40 percent of CGIAR’s Portfolio by dollar value. The report does not include Center-managed bilateral projects. As a key\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p24pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 24 part 4\nContent: the continuity of prior work that is less fit for purpose in the Program’s ToC. Windows 1, 2, 3 and bilateral funding: Approximately half of S4I’s 2025 funding is from Window 1, with the remainder from Window 2, including two $1.25 million designated W2 allocations specifically for AoWs 4 and 5. The PORB also reflects stronger alignment of Window 3 and bilateral funding with Program logic: in 2025, 47 mapped W3 and bilateral investments totaling $44.8 million support the Program ($0.42M, $26.47M, $1.55M, $15.37M, and $0.99M across AoWs 1 through 5, respectively), with 74% of these funds active in Africa, 19% in Asia, and 7% in Latin America. Engage and Empower (AoW 1): This AoW is allocated $2.98 million in W1/W2 funding and supported by $0.42 million in W3/bilaterals. It anchors S4I’s stakeholder demand intelligence 9 The section on AoW 4 in the PORB description highlights major inception period successes in leveraging Window 3 investments, with an anticipated, two-year bilateral investment in HLO 4.1 to transition TAAT into the Scaling Program that will support new work that was not part of the RIIs or NPS.\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u67-70]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Ethical Standards' paragraph 71 to section 'Ethical Standards' paragraph 74\nContent: Electioneering. The System Organization and each Center will, respectively, ensure that Window 1, 2 and 3 Funds will not be used to influence the outcome of any specific public election or to directly or indirectly carry on any voter registration drive. Drug trafficking. The System Organization and each Center, respectively, confirms that they have no reasonable basis to suspect that Window 1, 2 and 3 Funds would be diverted in support of drug trafficking. Discrimination against people with disabilities. The System Organization and each Center will, respectively, agree not to discriminate against persons with disabilities in the implementation of activities financed by Window 1, 2 and 3 Funds, and to make every effort to respect the principles of the UN Convention on the Rights of Persons with Disabilities in performing such activities. To that end, and to the extent this goal can be accomplished within the scope of the objectives of CGIAR Research, the System Organization and Centers involved in an activity financed by Window 1, 2 and 3 Funds should demonstrate a comprehensive and consistent approach for including men, women and children with disabilities consistent with such principles: (i) respect for inherent dignity, individual autonomy including the freedom to make one's own choices, and independence of persons; (ii) non-discrimination; (iii) full and effective participation and inclusion in society; (iv) respect for difference and acceptance of persons with disabilities as part of human diversity and humanity; (v) equality of opportunity; (vi) accessibility; (vii) equality between men and women; and\n\n---\n\n[ID: docx:Standard Provisions 2026.docx:u157-160]\nLink: N/A\nFile: Standard Provisions 2026.docx\nLocation: section 'Statement of Assurance' paragraph 169 to section 'Additional Audits / Financial Reviews / Technical Reporting' paragraph 172\nContent: Change in Reporting Requirements. Unless decided otherwise by the System Council and/or the Integrated Partnership Board as the case may be, any change in the form or substance or periodicity of a technical or financial report will become effective only in the following calendar year. Additional Audits / Financial Reviews / Technical Reporting Funders will manage their audits, financial reviews and technical reporting with respect to the Window 1, 2 and 3 Funds collectively through the System Council, including relying on applicable CGIAR Policies and Procedures, thereby endeavoring not to require duplicative reporting, provided that a Funder may require supplemental audits, financial reviews and technical reporting with respect to Window 3 Funds pursuant to its Window 3 Side Agreement or Arrangement, the costs of which would be paid by the requesting Funder. If a Funder wishes to request, on an exceptional basis, that the System Organization or a Center has an external audit or provides additional financial reviews or technical reports wi</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: what is an outcome\n\nContext:\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 48 part 4\nContent: breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in\n\n---\n\n[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations_Inception Report 30-06-2025.pdf\nLocation: page 13 part 2\nContent: leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes\n\n---\n\n[ID: docx:Innovation use.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation use.docx\nLocation: section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7\nContent: Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?\n\n---\n\n[ID: docx:General reporting guidance.docx:u1-3]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General reporting guidance.docx\nLocation: section 'General reporting guidance' paragraph 1 to section 'General reporting guidance' paragraph 5\nContent: General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 3\nContent: the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 32 part 3\nContent: Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Number and type\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 2\nContent: in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 60 part 4\nContent: in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 47 part 3\nContent: of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 23 part 1\nContent: Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 8 part 4\nContent: been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?\n\n---\n\n[ID: docx:Innovation development.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation development.docx\nLocation: section 'Innovation development' paragraph 1 to section 'Innovation development' paragraph 7\nContent: Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?\n\n---\n\n[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]\nLink: https://docs.google.com/document/d/19V8HwQN50riKrU7GomHQ4J8_aBuyngrh/edit\nFile: 2025 Technical Reporting MELIA glossary.docx\nLocation: table 1 row 28 to table 1 row 31\nContent: Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 4\nContent: four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the \"challenges and megatrends\" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 2\nContent: capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 4\nContent: Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 5 part 2\nContent: 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intemediate Outcome: Crop Trust signs Long-Term Partnerships with CGIAR X X X X - Intermediate Outcome: CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness X X X X 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 30 part 1\nContent: RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 15 part 4\nContent: intermediate outcomes that are not covered by any MELIA studies under the cross-cutting section should be entered under the relevant AoW-level outcome in the PORB\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 27 part 1\nContent: 27 Impact assessment efforts at the behavioral change level will focus on the 2030 Program Outcomes but also on unintended or unexpected significant outcomes highlighted through mid- term and final Outcome Evaluations and Policy change analyses (see Evaluation section). Data on behavioral changes will be monitored yearly through participatory outcome identification workshops with all partners engaged at the country/site level and outcome journals (see monitoring section). These yearly workshops at the country/site level are budgeted on the 20% non- assigned budget per center and have already been set aside by centers. The System Based Theory of Change approach will be applied to identify areas of success and prioritize the Outcome Evaluations (see\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsi</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: what is an outcome\n\nContext:\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 48 part 4\nContent: breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in\n\n---\n\n[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations_Inception Report 30-06-2025.pdf\nLocation: page 13 part 2\nContent: leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes\n\n---\n\n[ID: docx:Innovation use.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation use.docx\nLocation: section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7\nContent: Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?\n\n---\n\n[ID: docx:General reporting guidance.docx:u1-3]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General reporting guidance.docx\nLocation: section 'General reporting guidance' paragraph 1 to section 'General reporting guidance' paragraph 5\nContent: General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 3\nContent: the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 32 part 3\nContent: Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co -design of science-based processes and tools lead to ownership of results by landscape stakeholders and therefore to the sustainable uptake of solutions? • Number and type\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 2\nContent: in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 60 part 4\nContent: in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 23 part 1\nContent: Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 8 part 4\nContent: been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 47 part 3\nContent: of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian\n\n---\n\n[ID: docx:Innovation development.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation development.docx\nLocation: section 'Innovation development' paragraph 1 to section 'Innovation development' paragraph 7\nContent: Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?\n\n---\n\n[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]\nLink: https://docs.google.com/document/d/19V8HwQN50riKrU7GomHQ4J8_aBuyngrh/edit\nFile: 2025 Technical Reporting MELIA glossary.docx\nLocation: table 1 row 28 to table 1 row 31\nContent: Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 4\nContent: four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the \"challenges and megatrends\" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 2\nContent: capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 4\nContent: Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support\n\n---\n\n[ID: pdf:CGI21_508012_PORB_Genebanks.pdf:p5pt2]\nLink: N/A\nFile: CGI21_508012_PORB_Genebanks.pdf\nLocation: page 5 part 2\nContent: 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) Intemediate Outcome: Crop Trust signs Long-Term Partnerships with CGIAR X X X X - Intermediate Outcome: CGIAR genebanks conserve and make available crop diversity in perpetuity with greater efficiency and effectiveness X X X X 2030 Outcome 1: National and International genebanks conserve and make diversity more widely available in a strengthened global system of enabling policies and increased capacities X X X X 2030 Outcome 2: Researchers, farmers, and students access diversity and associated data in a smarter and\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 30 part 1\nContent: RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p15pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 15 part 4\nContent: intermediate outcomes that are not covered by any MELIA studies under the cross-cutting section should be entered under the relevant AoW-level outcome in the PORB\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p27pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 27 part 1\nContent: 27 Impact assessment efforts at the behavioral change level will focus on the 2030 Program Outcomes but also on unintended or unexpected significant outcomes highlighted through mid- term and final Outcome Evaluations and Policy change analyses (see Evaluation section). Data on behavioral changes will be monitored yearly through participatory outcome identification workshops with all partners engaged at the country/site level and outcome journals (see monitoring section). These yearly workshops at the country/site level are budgeted on the 20% non- assigned budget per center and have already been set aside by centers. The System Based Theory of Change approach will be applied to identify areas of success and prioritize the Outcome Evaluations (see\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%2</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: what is an outcome?\n\nContext:\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p48pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 48 part 4\nContent: breeding endeavors. While an earlier TOC showed the relationship between the outcomes of the initiatives, the revised TOC showed only one outcome of breeding. This outcome was ‘Seed producers successfully market new demand-driven improved varieties to more farmers’. The GI TOC essentially elevated the final output of the breeding pipeline to an outcome3, reverting to the breeding pipeline engineering view that dominates in breeding. In elevating the output to an outcome, any outcomes outside of breeding itself are diminished. Outcomes related to the quality of how breeding is done, with strategic prioritization, collaborative partnerships and efficiency have been omitted. It is these qualities of how breeding is done that build empowerment of regional partners and legacy beyond the lifecycle of a variety. 3 Note that it could be argued this is an outcome of Seed Equal. Regardless, it is not an outcome of GI, but one of the initiatives and this outcome could be achieved without investment or action in\n\n---\n\n[ID: pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p13pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations_Inception Report 30-06-2025.pdf\nLocation: page 13 part 2\nContent: leading to Intermediate Outcomes and finally to three 2030Outcomes, that correspond broadly to the three pillars. The first 2030 outcome focuses on Pillar C on capacity sharing; the 2nd outcome corresponds to Pillar B while the 3rd one addresses Pillar A.  2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs,  2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessment and governance to guide pro-poor, gender-inclusive and climate smart policies and investments  2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more coherent and sustainable development processes that deliver positive outcomes across a range of SDG targets. The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidates outputs from the 20 High-level outputs of the Policy Program. Multiple Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes\n\n---\n\n[ID: docx:Innovation use.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation use.docx\nLocation: section 'Innovation use' paragraph 1 to section 'Innovation use' paragraph 7\nContent: Innovation use How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome levels. The development of an innovation (at various stages) is an output. The scaling, uptake and use of an innovation can be reported as outcome. In PRMS the results can be linked. What are the two ways to report innovation use results (outcomes)?\n\n---\n\n[ID: docx:General reporting guidance.docx:u1-3]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General reporting guidance.docx\nLocation: section 'General reporting guidance' paragraph 1 to section 'General reporting guidance' paragraph 5\nContent: General reporting guidance Is there guidance on what should be reported as a result? Yes, this document provides some principles for ensuring a focus on quality, rather than quantity, in terms of results reporting: Guidance on ensuring quality over quantity. Is there guidance available on how to distinguish between outputs and outcomes? Yes, information on what to report as an output or outcome can be found here: Guidance on reporting outputs or outcomes.\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 3\nContent: the Theories of Change (overall, Areas of Work and sub-Areas) for consistency and alignment with stated objectives. (more details in Section 3.1 of this report) We have revised the HLOs at sub-area of work level, to harmonize the approach, remove duplications, and prioritize. There are now 26 HLOs. − We have harmonized the intermediate outcomes across sub-AoWs, AoWs, and Accelerator level. There are now five intermediate outcomes for AoW on Solutions and three for AoW on Change. − We have moved one outcome from the intermediate level to the end-of-program level and there are now four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p18pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 18 part 4\nContent: better understand farmer perspectives, motivations, and constraints concerning the adoption of SFP innovations. 4. Adoption or diffusion studies addressing learning questions on the TOC The baseline surveys conducted in Ghana, Malawi, and Ethiopia focusing on sustainable intensification technologies will form the basis for the adoption and impacts studies. These studies will seek to answer the following causal impact learning questions: ( 1) What factors are constraining/enabling the scaling and adoption as well as the intensity of use of the SFP innovations? and (2) How does adoption of the SFP innovations impact yield, farm income and household income? (3) What are the most promising inte grated farm -level innovation bundles to improve sustainability, equity, and agronomic gain at scale within the selected geographies of the program? To answer these questions, adoption and impact studies build up on the baseline studies (panel survey) to assess the extent, pathways, and determinants of\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p8pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 8 part 4\nContent: been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E) Effectiveness (the extent that the intended results or outcomes are achieved) High This criterion directly relates to the MELIA objectives. Assessing the effectiveness of the Intermediate Outcomes will inform contribution analysis and inform the design requirements of future programs. KEQ2. To what extent has B4T and its AOWs effectively achieved the intended intermediate outcomes? RQ2 How did prioritization using the Design Standard contribute to maximized impact (AOW1 MI)? RQ7 To what extent has B4T increased uptake of varieties by scaling partners who have a widespread reach (collectively)? (AOW3 ID) RQ8 To what extent has CGIAR-NARES prioritization of products encouraged targeted investment for breeding?\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p31pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_Inception Report 30-06-2025.pdf\nLocation: page 31 part 4\nContent: four 2030 outcomes. − We have updated the indicators and targets for HLOs and outcomes, ensuring it is clear what the Accelerator will deliver, what changes it aims to influence, and how those would be measured. − We have revised and clearly defined assumptions that underpin each individual HLO and outcome, as well as explaining the connections between the HLOs and outcomes. Bill and Melinda Gates Foundation High-level vision lacks any data points. The FAO data on women's increase in hunger (vis- a-vis men's) would seem to fit well with the \"challenges and megatrends\" for example. More recent FAO data points on gender issues in climate change might help set the table for Data points have been added in the final version of the proposal.\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 23 part 1\nContent: Key Evaluation Questions Some guiding questions that will inform future evaluations include: • Are the Program’s assumptions about actor behavior, incentives, and influence valid for the specific stakeholders identified, and are they likely to lead to the intended outcomes? • How do differences in AoW presence across countries affect the Program’s ability to deliver its intended outcomes? • Are the current configurations of AoWs efficient and synergistic, or are there opportunities to increase impact through structural changes? • What mechanisms exist (or are lacking) to integrate bilateral and W3-funded results into core program planning and reporting? • To what extent is MELIA evidence used to inform planning, learning, and adaptation across the Program? • How well do program assumptions and outcome pathways reflect national priorities and systems capacities in each geography? • • What types of MELIA findings\n\n---\n\n[ID: docx:2025 Technical Reporting MELIA glossary.docx:u31-34]\nLink: https://docs.google.com/document/d/19V8HwQN50riKrU7GomHQ4J8_aBuyngrh/edit\nFile: 2025 Technical Reporting MELIA glossary.docx\nLocation: table 1 row 28 to table 1 row 31\nContent: Intermediate outcome | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. | Intermediate outcomes are necessary steps towards achieving the 2030 outcomes. Intermediate outcomes will lead to the 2030 outcomes, although the actors and units of measure may be different. 2030 outcome | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. | 2030 outcomes are the final, highest-level outcomes to be achieved by the end of 2030 by the Programs/Accelerators/Projects. It is expected that these 2030 outcomes would lead to measurable impacts. Output | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. | Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples: new research methods, policy analyses, gene maps, new crop varieties and breeds, institutional innovations or other products of research work, partnerships because of a signed memorandum of understanding. High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on).\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt3]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 47 part 3\nContent: of this report. Comparison with 2017–2021 Retrospective analysis of CGIAR’s 2017 to 2021 reporting cycle provides a reference point for assessing progress in outcome reporting and portfolio management under the current Results Framework. While differences in the reporting systems limit direct comparability, several structural patterns from the previous cycle remain relevant. Policy outcomes Learnings from CGIAR’s 2017 to 2021 reporting cycle demonstrate that policy outcomes were mostly oriented toward policies and strategies (75 percent), and the rest influenced budget and investment decisions or legal instruments.29 The majority reflected early uptake of research results, but 39 percent of policy outcomes were concrete decisions, policies, or programs taken or enacted. In the current 2022 to 2024 cycle, there was a slight increase in the percentage of reported policy changes that were actual policies or programs put into place (43 percent of policy outcomes). Moreover , the type of policy outcome differed, with the percentage of policy outcomes leading to modified programs or investments jumping to 29 percent. The thematic and geographic orientations of policy outcomes are similar across the two periods, generally displaying CGIAR effectiveness in all of its priority countries and across most of its Impact Areas. However , the percentage of policy outcomes which were aimed primarily at gender equality was low in both periods. Partners were critical to CGIAR’s success in informing policies. Critical partners included national and subnational governments, civil society organizations, private sector , regional bodies, and international organizations. The review of 2017 to 2021 policy outcomes also revealed that very few were evaluated for their impacts, yet many appeared to be significant. Some examples of those are in Table 3. Impacts of CGIAR’s policy research remain underanalyzed. Policy outcome type What the evidence shows Illustrative cases CGIAR partners Outcomes Policy and strategy outcomes, mainly at national level 60% of outcomes were national and 37% reached formal enactment— often when a ministry or regulatory body was part of the design team Ethiopian\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p9pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 2\nContent: in breeding contribute to increased rate of genetic gain, as captured in the extent of improvement and impact achieved by products. Efficiency is included in an intermediate outcome so any effectiveness evaluation of intermediate outcomes will be duplicative. This criterion is most relevant to AOW4 as it is designed to support efficient access and use of modernized breeding. An AOW level outcome has captured this so any effectiveness evaluation of outcomes will duplicate efficiency. Research questions will contribute to KEQ2 on effectiveness: To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? RQ12 How has the use of interoperable, scaled breeding tools and services increased\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p60pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 60 part 4\nContent: in thriving Multifunctional Landscapes • Number of policy innovations that support the transition to sustained MFLs what was the contribution of the MFL Program interventions to these changes. This will allow us to identify the most impactful Outcomes related to the Impact Areas and orient Outcome Evidencing studies for efficient use of MELIA resources.\n\n---\n\n[ID: docx:Innovation development.docx:u1-4]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Innovation development.docx\nLocation: section 'Innovation development' paragraph 1 to section 'Innovation development' paragraph 7\nContent: Innovation development How do I determine if I should report an innovation as an output (innovation development) or an outcome (innovation use)? Innovations can be reported at both the output and outcome level. The development of an innovation (at various stages of design, testing and validation) is an output. The scaling or use of an innovation is an outcome. You may first report an innovation at the output level. If the innovation advances and starts to be used, it should then be reported as an outcome. Do I need to update innovations that were submitted during previous reporting periods?\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 3\nContent: activities of the CapSha Accelerator, its products and services, contribute to improved capacity development practices, resulting in more equitable partnerships? • Are CGIAR NARES partners, donors and CapSha expert institutions making use of CapSha products and services? • Are CGIAR NARES partners, donors and CapSha expert institutions member of the CapSha Cop? • To what extent are the CapSha Accelerator’s objectives aligned with the needs and priorities of Southern partners? • What elements of the partnership model have the potential to be scaled or replicated in other regions or contexts? What are the enabling and limiting factors affecting scalability? How have Southern partners contributed to or led scaling efforts, and what support mechanisms have been most effective? • What measurable\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 4\nContent: Growth) and 10 (Reduced Inequalities). The progress towards the 2030 Outcomes is operationalized via six AoWs, contributing to 11 Intermediate outcomes which consolidate outputs from the 20 High -level outputs of the Policy Program. All Intermediate Outcomes contribute towards the 2030 Outcomes. For example, Intermediate outcomes 1.2.1 (Partners use outlook reports to inform and enhance design of their strategies and policies), 4.2.1 (Partners achieve a shared understanding of emerging ch allenges in WEFE systems and foresight data, tools and analysis), 5.2.1 (Countries co-create national strategies and policies) and 6.2.2 (CGIAR researchers and partners have enh anced capacity) all address the capacity challenge and contribute to the impact pathway achieving 2030 Outcome1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs. This 2030 Outcome in turn, also addresses CGIAR Portfolio Outcome #1: Implementation partners (e.g. NARES, NGOs, private companies) actively support\n\n---\n\n[ID: pdf:Genebanks_Inception Report 30-06-2025.pdf:p31pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_Inception Report 30-06-2025.pdf\nLocation: page 31 part 3\nContent: the misuse of funds for purposes outside what is set up in the\n\n---\n\n[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p30pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow%2FBreeding%20for%20Tomorrow%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP01%20%2D%20Breeding%20for%20Tomorrow&amp;p=true&amp;ga=1\nFile: Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 30 part 1\nContent: RQ17 What proportion of marginalized beneficiaries in each market segment have accessed improved varieties? (AOW3 ID) RQ29 What extent of value proposition is needed to motivate adoption? KEQ2. To what extent has B4T and its AOW effectively achieved the intended intermediate outcomes? Coherence RQ4 How have the network strategies improved coherence with region x crop investments? (AOW5 E) RQ5 How have bottlenecks or barriers between variety development and seed systems been overcome to improve smallholder access to seed? (AOW3 ID) RQ6 How has B4T’s work with other CGIAR investments increased or improved the achievement of 2030 outcomes? (AOW5 E)\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p5pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 5 part 2\nContent: capacity &amp; tools. . The Program’s Theory of Change works through six interconnected Areas of Work (AoWs), their High- level Outputs (HLOs), leading to Intermediate Outcomes and finally to three 2030 Outcomes. During the inception phase the Policy Program align ed the Intermediate Outcomes and 2030 Outcomes to these 3 pillars. The 2030 Outcomes were revised to contribute to our impact around these. 2030 Outcome 1: National think tanks analytical and institutional capacity strengthened to guide policy and investment decisions considering trade-offs between SDGs: represents the Capacity and tools pillar, 2030 Outcome 2: Global, regional institutions and governments use knowledge products on foresight, impact assessm ent and governance to guide pro -poor, gender-inclusive and climate smart policies and investments, represents Rapid Response and policy guidance pillar while 2030 Outcome 3: Governments and partners adopt policy responses to address local, national, regional and global challenges and shocks, contributing to more\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p32pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 32 part 3\nContent: Outcome Evidencing/ Outcome Trajectory evaluation instruments: Document review, workshops, key informant interviews, secondary data System-based Theory of Change Actor engagement and outcome tracker AoW6 assessments AoW7 partner capacity evaluation • To what extent does co</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: what are the different types of outputs in the cgiar results framework?\n\nContext:\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 19 part 1\nContent: Results framework The program result\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 6 part 2\nContent: Work 2.3 Results framework The CapSha Accelerator results framework has been\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt4]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 4\nContent: CGIAR Results Framework – Portfolio Outcome\n\n---\n\n[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 2\nContent: types For reference only, the current MELIA study types defined in\n\n---\n\n[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt1]\nLink: N/A\nFile: CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf\nLocation: page 7 part 1\nContent: CGIAR Performance and Results Management Framework 2022-2030 CGIAR System Organization Page 7 of 20 4. Results framework CGIAR’s results framework is directly aligned to the five impact areas and Sustainable Development Goals. Three distinct result types: outputs, outcomes and impacts are mapped to the spheres of Control, Influence and Interest, respectively. • Output: Knowledge, technical or institutional advancement produced by CGIAR research, engagement and/or capacity development activities. Examples of outputs include new research methods, policy analyses, gene maps, new crop varieties and breeds, or other products of research work. • Outcome: A change in knowledge, skills, attitudes and/or relationships, which manifests as a change in behavior of users of outputs, to which a combination of research outputs and related activities have contributed. •\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 5 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 11 part 3\nContent: portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 11 part 3\nContent: portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.\n\n---\n\n[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 9 part 3\nContent: Results Framework Please refer\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p28pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf\nLocation: page 28 part 2\nContent: 4. MELIA study types For reference only, the current MELIA study types\n\n---\n\n[ID: docx:2025 Technical Reporting MELIA glossary.docx:u55-58]\nLink: https://docs.google.com/document/d/19V8HwQN50riKrU7GomHQ4J8_aBuyngrh/edit\nFile: 2025 Technical Reporting MELIA glossary.docx\nLocation: table 1 row 52 to table 1 row 55\nContent: Policy change | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. | Policies, strategies, legal instruments, programs, budgets, or investments at different scales (local to global) that have been modified in design or implementation, with evidence that the change was informed by CGIAR research. Portfolio | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. | The CGIAR System Framework approved by the System’s Funders and Centers in June 2016, and then amended in October 2024, defines “CGIAR Portfolio” as the research programs and/or platforms carried out by the Centers and the CGIAR System Partners in support of the CGIAR Strategy and Results Framework and which are supported by (i) the CGIAR Trust Fund and/or (ii) bilateral sources contractually aligned to such programs and/or platforms. Program | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. | CGIAR Programs are the main vehicle for delivery of research and innovation by CGIAR from 2025 to 2030. Programs serve as entry points to describe CGIAR’s offer on a key topic, elevating CGIAR’s visibility in global agendas and facilitating the continuation and formation of inclusive alliances and partnerships. They state quantitatively what impacts and outcomes they intend to achieve, along a theory of change. They come with evaluable results frameworks and clear reporting of results against investment. Bilateral and window 3 projects are aligned to Programs and Accelerators and their results are reported as part of Program and Accelerator reporting. Result | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact. | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact. | The product of an activity by CGIAR staff or due in part to CGIAR staff, described as an output, outcome or impact.\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p9pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 9 part 2\nContent: Mitigation, Nutrition, Poverty Reduction and Livelihoods, Gender Equality and Social Inclusion, and Environmental Health and Biodiversity. The SFP results framework operationalizes this contribution by aligning program indicators and learning activities with CGIAR’s Performance and Results Management Framework (PRMF) and systematically collect evidence across the eight AoWs. Each AoW is designed to deliver results that directly or indirectly support one or more CGIAR Impact Areas. The framework provides a coherent roadmap for measuring the SFP contributions. Open Access link for both the ToC and the Results Framework . (Download the Results Framework as part of several other worksheets-e.g., assumptions, research questions, etc using the 3rd icon on the top left conner of the page). 3. Monitoring plan for HLOs and outcomes This section outlines how the Program will monitor delivery of HLOs and progress towards\n\n---\n\n[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_MELIA Plan 30-06-2025.pdf\nLocation: page 7 part 1\nContent: 7 Results framework The Result Framework presents a structured articulation of the intended results under CGIAR’s strategic Areas of Work (AOWs) for the period 2025 to 2030. It distinguishes between two types of results: High-Level Outputs (HLOs), which represent tangible, near-term deliverables from research eƯorts, and Intermediate Outcomes (IOCs), which indicate progress toward longer- term development goals and systemic change. Each result entry captures several key variables—among many others—that collectively deﬁne the pathway from research to impact. These include the thematic Area of Work to which the result contributes, the classiﬁcation of the result as either an output or outcome, and a short title paired with a detailed result statement that describes the intended change, innovation, or contribution. The responsible organization(s), often CGIAR centers, are identiﬁed alongside any listed partners and outcome actors, with additional information on whether those actors are directly engaged and what\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p19pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 19 part 2\nContent: result framework is accessible from\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p8pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 8 part 2\nContent: the Program and Area of Work levels. This link gives the ToC tables-overall and AoW ToCs) and Open Access link for both the ToC and the Results Framework . (Zoom out to see the linkages of the various AoW ToCs and download the ToC tables using the 4 th icon on the top left conner of the page). Figure 1. Sustainable Farming Program level Theory of Change Results framework The SFP Results Framework reflects the logical sequence from high-level outputs to intermediate outcomes, aligned with the program’s Theory of Change. It captures the intended contributions of each AoW,\n\n---\n\n[ID: docx:2025 Technical Reporting MELIA glossary.docx:u34-37]\nLink: https://docs.google.com/document/d/19V8HwQN50riKrU7GomHQ4J8_aBuyngrh/edit\nFile: 2025 Technical Reporting MELIA glossary.docx\nLocation: table 1 row 31 to table 1 row 34\nContent: High-level output | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). | High-level outputs are aggregated clusters of outputs which are linked by the intention to achieve a specific outcome. The high-level outputs should be relatively downstream – i.e. ready to be used by next/end users – and would often be composed of various different types of outputs (e.g. knowledge products, innovations, capacity sharing activities and so on). Partner | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. | Organizations or individual stakeholders that CGIAR collaborates with to achieve its goals for which proof exists, i.e., memorandum of understanding, joint code of practice, a contract under a joint proposal. Partners can also be beneficiaries of CGIAR’s interventions. Examples: demand partner, innovation partner and scaling partner. Partner typology (CGIAR) | CGIAR uses a partner typology to define partner types. Definitions are presented below. | CGIAR uses a partner typology to define partner types. Definitions are presented below. | CGIAR uses a partner typology to define partner types. Definitions are presented below. Partner typology (CGIAR) | CGIAR type | CGIAR type definition\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p32pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 32 part 3\nContent: tab in the program result s framework accessible\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 11 part 2\nContent: Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 11 part 2\nContent: Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p3pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 3 part 1\nContent: 3 1. Reviewing guidance for developing the MELIA Plan Developing the Sustainable Farming program (SFP) MELIA plan, started with the review of the ISDC feedback on the overall program Theory of Change (ToC) and the Area of Work (AoW) ToCs. This feedback has been used in updating the ToC, (example, creating indicators for AoW 8 - Program Efficiency and Delivery . In addition, the core assessment criteria from the IAES evaluability assessment guide were used as reference checks in developing the MELIA plan. 2. Program overview and results framework This section provides a n overview of the Sustainable Farming Program (SFP), outlining its intervention logic and the results framework. It also details the alignment of the Program’s results framework with the CGIAR Performance and Results Management Framework (PRMF) and Portfolio outcomes, ensuring system thinking. Program overview SFP is designed to respond to\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf\nLocation: page 18 part 3\nContent: 2030 Outcome, or Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framework Provide the assumption( s) statem ent from the Results Framework Indicate the location(s) where the study will be conducted Indicate the methods and design approaches that will be used for the study List the Program(s) and Accelerator( s ) you will collaborate with or coordinate for the implementati on of this study. Indicate the Start\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p11pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/05/Type3_2024Report.pdf\nFile: Type3_2024Report.pdf\nLocation: page 11 part 4\nContent: System (PRMS): The PRMS serves as the central reporting platform, powering the Results Dashboard and supporting the development of Type 1 Reports with real-time data aggregation and analysis. These components were instrumental in driving the 2024 Technical Reporting process, and key elements will be carried forward to shape Technical Reporting in the next CGIAR Portfolio, ensuring continuity, alignment, and continuous improvement. Monitoring tools tailored to suit core indicators Non-pooled projects Type 1 Type 3 Science Group Projects Research and Performance and Results Management Framework Arrangement CGIAR Results Framework Standard Indicator Theory of Change and Scaling Readiness (IPSR) Quality Assurance criteria, process Performance and Results Management System Type 2 Triennial Outcome/Impact Report Annual Technical Report Results Dashboard $771M Revenue 2% 23% 44% 31% Revenue by Funding Source Windows 1&amp;2 | Window 3 | Bilateral | Other 1 2 3 4 5 6 7 8 9 10 13 12 11 6. CGIAR 2030 Research and Innovation Strategy 7. Performance and Results Management Framework 8. Technical Reporting Arrangement 9. CGIAR Results Framework 10. Standard Indicator Description Sheets: • Output level • Outcome level 11. Theory of Change 12. IPSR • Output level • Outcome level • IPM for responsible food systems transformation • Scaling Readiness website • Online course on Innovation and Scaling • Scaling Readiness calculator • Scaling Directory 13. Adaptive Management 14. Quality Assurance 15. PRMS &amp; TOC board 16. Results Dashboard 17. 2022 &amp; 2023 Annual Technical Reports 18. Type 2 repo</t>
   </si>
 </sst>
 </file>
@@ -2640,7 +3144,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K62"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2683,7 +3187,7 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -2695,16 +3199,16 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H2" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I2" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2712,7 +3216,7 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -2724,16 +3228,16 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G3" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H3" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I3" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2741,7 +3245,7 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C4">
         <v>100</v>
@@ -2753,16 +3257,16 @@
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="G4" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H4" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="I4" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2770,7 +3274,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -2782,16 +3286,16 @@
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G5" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="I5" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2799,7 +3303,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C6">
         <v>100</v>
@@ -2811,16 +3315,16 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="G6" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H6" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
       <c r="I6" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -2828,7 +3332,7 @@
         <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C7">
         <v>100</v>
@@ -2840,16 +3344,16 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="G7" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H7" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="I7" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -2857,7 +3361,7 @@
         <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C8">
         <v>100</v>
@@ -2869,16 +3373,16 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="G8" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="H8" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="I8" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2886,7 +3390,7 @@
         <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C9">
         <v>100</v>
@@ -2898,16 +3402,16 @@
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="G9" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="H9" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="I9" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2915,7 +3419,7 @@
         <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C10">
         <v>100</v>
@@ -2927,16 +3431,16 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G10" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="I10" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2944,7 +3448,7 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C11">
         <v>100</v>
@@ -2956,16 +3460,16 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G11" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H11" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I11" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2973,7 +3477,7 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C12">
         <v>100</v>
@@ -2985,16 +3489,16 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G12" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H12" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="I12" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -3002,7 +3506,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C13">
         <v>100</v>
@@ -3014,16 +3518,16 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G13" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H13" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="I13" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -3031,7 +3535,7 @@
         <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C14">
         <v>100</v>
@@ -3043,16 +3547,16 @@
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G14" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H14" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="I14" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -3060,7 +3564,7 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C15">
         <v>100</v>
@@ -3072,16 +3576,16 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G15" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H15" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="I15" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -3089,7 +3593,7 @@
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -3101,16 +3605,16 @@
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G16" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H16" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="I16" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -3118,7 +3622,7 @@
         <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C17">
         <v>100</v>
@@ -3130,16 +3634,16 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G17" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H17" t="s">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="I17" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -3147,7 +3651,7 @@
         <v>27</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C18">
         <v>100</v>
@@ -3159,16 +3663,16 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G18" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H18" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="I18" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -3176,7 +3680,7 @@
         <v>28</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C19">
         <v>100</v>
@@ -3188,16 +3692,16 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="G19" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H19" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="I19" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -3205,7 +3709,7 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C20">
         <v>100</v>
@@ -3217,16 +3721,16 @@
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G20" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H20" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I20" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -3234,7 +3738,7 @@
         <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C21">
         <v>100</v>
@@ -3246,22 +3750,22 @@
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G21" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H21" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I21" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="J21" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K21" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -3269,7 +3773,7 @@
         <v>31</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C22">
         <v>100</v>
@@ -3281,22 +3785,22 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H22" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I22" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="J22" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K22" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -3304,7 +3808,7 @@
         <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C23">
         <v>100</v>
@@ -3316,22 +3820,22 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G23" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="H23" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I23" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="J23" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K23" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -3339,7 +3843,7 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C24">
         <v>200</v>
@@ -3351,22 +3855,22 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G24" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H24" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I24" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="J24" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K24" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -3374,7 +3878,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C25">
         <v>200</v>
@@ -3386,22 +3890,22 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G25" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H25" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="I25" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="J25" t="s">
-        <v>176</v>
+        <v>195</v>
       </c>
       <c r="K25" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -3409,7 +3913,7 @@
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C26">
         <v>200</v>
@@ -3421,22 +3925,22 @@
         <v>1</v>
       </c>
       <c r="F26" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G26" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="H26" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="I26" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="J26" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="K26" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -3444,7 +3948,7 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C27">
         <v>200</v>
@@ -3456,22 +3960,22 @@
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G27" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="H27" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="I27" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="J27" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="K27" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -3479,7 +3983,7 @@
         <v>37</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C28">
         <v>200</v>
@@ -3491,22 +3995,22 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G28" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="I28" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="J28" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="K28" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -3514,7 +4018,7 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C29">
         <v>200</v>
@@ -3526,22 +4030,22 @@
         <v>1</v>
       </c>
       <c r="F29" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G29" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="H29" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="I29" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="J29" t="s">
-        <v>177</v>
+        <v>196</v>
       </c>
       <c r="K29" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -3549,7 +4053,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C30">
         <v>100</v>
@@ -3561,22 +4065,22 @@
         <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G30" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="H30" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="I30" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="J30" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="K30" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -3584,7 +4088,7 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C31">
         <v>100</v>
@@ -3596,22 +4100,22 @@
         <v>1</v>
       </c>
       <c r="F31" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G31" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="H31" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="I31" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="J31" t="s">
-        <v>178</v>
+        <v>197</v>
       </c>
       <c r="K31" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -3619,7 +4123,7 @@
         <v>41</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C32">
         <v>100</v>
@@ -3631,22 +4135,22 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G32" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H32" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="I32" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="J32" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K32" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -3654,7 +4158,7 @@
         <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C33">
         <v>100</v>
@@ -3666,22 +4170,22 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G33" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H33" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J33" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K33" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -3689,7 +4193,7 @@
         <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C34">
         <v>100</v>
@@ -3701,22 +4205,22 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G34" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H34" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J34" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K34" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -3724,7 +4228,7 @@
         <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C35">
         <v>100</v>
@@ -3736,22 +4240,22 @@
         <v>1</v>
       </c>
       <c r="F35" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G35" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H35" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J35" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K35" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3759,7 +4263,7 @@
         <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C36">
         <v>100</v>
@@ -3771,22 +4275,22 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G36" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H36" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J36" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K36" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -3794,7 +4298,7 @@
         <v>46</v>
       </c>
       <c r="B37" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C37">
         <v>100</v>
@@ -3806,22 +4310,22 @@
         <v>1</v>
       </c>
       <c r="F37" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G37" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H37" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J37" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K37" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -3829,7 +4333,7 @@
         <v>47</v>
       </c>
       <c r="B38" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C38">
         <v>100</v>
@@ -3841,22 +4345,22 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G38" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="H38" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="J38" t="s">
-        <v>179</v>
+        <v>198</v>
       </c>
       <c r="K38" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -3864,7 +4368,7 @@
         <v>48</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C39">
         <v>100</v>
@@ -3876,22 +4380,22 @@
         <v>1</v>
       </c>
       <c r="F39" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G39" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H39" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I39" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J39" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K39" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -3899,7 +4403,7 @@
         <v>49</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C40">
         <v>100</v>
@@ -3911,22 +4415,22 @@
         <v>1</v>
       </c>
       <c r="F40" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G40" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H40" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I40" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J40" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K40" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -3934,7 +4438,7 @@
         <v>50</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C41">
         <v>100</v>
@@ -3946,22 +4450,22 @@
         <v>1</v>
       </c>
       <c r="F41" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G41" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H41" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I41" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J41" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K41" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -3969,7 +4473,7 @@
         <v>51</v>
       </c>
       <c r="B42" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C42">
         <v>100</v>
@@ -3981,22 +4485,22 @@
         <v>1</v>
       </c>
       <c r="F42" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G42" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H42" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I42" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J42" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K42" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -4004,7 +4508,7 @@
         <v>52</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C43">
         <v>100</v>
@@ -4016,22 +4520,22 @@
         <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G43" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H43" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="I43" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J43" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K43" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -4039,7 +4543,7 @@
         <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C44">
         <v>100</v>
@@ -4051,22 +4555,22 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G44" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H44" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="I44" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J44" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K44" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -4083,13 +4587,13 @@
         <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H45" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K45" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -4097,7 +4601,7 @@
         <v>55</v>
       </c>
       <c r="B46" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C46">
         <v>100</v>
@@ -4109,22 +4613,22 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G46" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H46" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="I46" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J46" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K46" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -4132,7 +4636,7 @@
         <v>56</v>
       </c>
       <c r="B47" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C47">
         <v>100</v>
@@ -4144,22 +4648,22 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G47" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H47" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="I47" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="J47" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K47" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -4167,7 +4671,7 @@
         <v>57</v>
       </c>
       <c r="B48" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C48">
         <v>100</v>
@@ -4179,22 +4683,22 @@
         <v>1</v>
       </c>
       <c r="F48" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="G48" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H48" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="J48" t="s">
-        <v>180</v>
+        <v>199</v>
       </c>
       <c r="K48" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -4202,7 +4706,7 @@
         <v>58</v>
       </c>
       <c r="B49" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="C49">
         <v>200</v>
@@ -4214,22 +4718,22 @@
         <v>1</v>
       </c>
       <c r="F49" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="G49" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="H49" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="J49" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="K49" t="s">
-        <v>198</v>
+        <v>221</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -4237,7 +4741,7 @@
         <v>59</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C50">
         <v>200</v>
@@ -4249,22 +4753,22 @@
         <v>1</v>
       </c>
       <c r="F50" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="G50" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="H50" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="J50" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="K50" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -4272,7 +4776,7 @@
         <v>60</v>
       </c>
       <c r="B51" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C51">
         <v>200</v>
@@ -4284,22 +4788,22 @@
         <v>1</v>
       </c>
       <c r="F51" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="G51" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="H51" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="J51" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="K51" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -4307,7 +4811,7 @@
         <v>61</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C52">
         <v>200</v>
@@ -4319,22 +4823,22 @@
         <v>1</v>
       </c>
       <c r="F52" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G52" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="H52" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="J52" t="s">
-        <v>182</v>
+        <v>201</v>
       </c>
       <c r="K52" t="s">
-        <v>200</v>
+        <v>223</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -4342,7 +4846,7 @@
         <v>62</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C53">
         <v>200</v>
@@ -4354,22 +4858,22 @@
         <v>1</v>
       </c>
       <c r="F53" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G53" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="H53" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="J53" t="s">
-        <v>183</v>
+        <v>202</v>
       </c>
       <c r="K53" t="s">
-        <v>201</v>
+        <v>224</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -4377,7 +4881,7 @@
         <v>63</v>
       </c>
       <c r="B54" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C54">
         <v>200</v>
@@ -4389,22 +4893,22 @@
         <v>1</v>
       </c>
       <c r="F54" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G54" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H54" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="J54" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="K54" t="s">
-        <v>202</v>
+        <v>225</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -4412,7 +4916,7 @@
         <v>64</v>
       </c>
       <c r="B55" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C55">
         <v>200</v>
@@ -4424,22 +4928,22 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G55" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H55" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="J55" t="s">
-        <v>184</v>
+        <v>203</v>
       </c>
       <c r="K55" t="s">
-        <v>202</v>
+        <v>225</v>
       </c>
     </row>
     <row r="56" spans="1:11">
@@ -4447,7 +4951,7 @@
         <v>65</v>
       </c>
       <c r="B56" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C56">
         <v>200</v>
@@ -4459,22 +4963,22 @@
         <v>1</v>
       </c>
       <c r="F56" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G56" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="H56" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="J56" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="K56" t="s">
-        <v>203</v>
+        <v>226</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -4482,7 +4986,7 @@
         <v>66</v>
       </c>
       <c r="B57" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C57">
         <v>200</v>
@@ -4494,22 +4998,22 @@
         <v>1</v>
       </c>
       <c r="F57" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G57" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="H57" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="I57" s="2" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="J57" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="K57" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -4517,7 +5021,7 @@
         <v>67</v>
       </c>
       <c r="B58" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C58">
         <v>200</v>
@@ -4529,22 +5033,22 @@
         <v>1</v>
       </c>
       <c r="F58" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G58" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="H58" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="I58" s="2" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="J58" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="K58" t="s">
-        <v>205</v>
+        <v>228</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -4552,7 +5056,7 @@
         <v>68</v>
       </c>
       <c r="B59" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C59">
         <v>200</v>
@@ -4564,22 +5068,22 @@
         <v>1</v>
       </c>
       <c r="F59" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G59" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="H59" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="I59" s="2" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="J59" t="s">
-        <v>185</v>
+        <v>204</v>
       </c>
       <c r="K59" t="s">
-        <v>206</v>
+        <v>229</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -4587,7 +5091,7 @@
         <v>69</v>
       </c>
       <c r="B60" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C60">
         <v>200</v>
@@ -4599,22 +5103,22 @@
         <v>1</v>
       </c>
       <c r="F60" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G60" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H60" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="I60" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="J60" t="s">
-        <v>186</v>
+        <v>205</v>
       </c>
       <c r="K60" t="s">
-        <v>207</v>
+        <v>230</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -4622,7 +5126,7 @@
         <v>70</v>
       </c>
       <c r="B61" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C61">
         <v>200</v>
@@ -4634,22 +5138,22 @@
         <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="G61" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="H61" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="I61" t="s">
-        <v>174</v>
+        <v>191</v>
       </c>
       <c r="J61" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="K61" t="s">
-        <v>208</v>
+        <v>231</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -4657,7 +5161,7 @@
         <v>71</v>
       </c>
       <c r="B62" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C62">
         <v>200</v>
@@ -4669,22 +5173,197 @@
         <v>1</v>
       </c>
       <c r="F62" t="s">
+        <v>101</v>
+      </c>
+      <c r="G62" t="s">
+        <v>119</v>
+      </c>
+      <c r="H62" t="s">
+        <v>171</v>
+      </c>
+      <c r="I62" t="s">
+        <v>192</v>
+      </c>
+      <c r="J62" t="s">
+        <v>207</v>
+      </c>
+      <c r="K62" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11">
+      <c r="A63" t="s">
+        <v>72</v>
+      </c>
+      <c r="B63" t="s">
+        <v>91</v>
+      </c>
+      <c r="C63">
+        <v>190</v>
+      </c>
+      <c r="D63">
+        <v>190</v>
+      </c>
+      <c r="E63" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" t="s">
+        <v>101</v>
+      </c>
+      <c r="G63" t="s">
+        <v>120</v>
+      </c>
+      <c r="H63" t="s">
+        <v>172</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J63" t="s">
+        <v>208</v>
+      </c>
+      <c r="K63" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11">
+      <c r="A64" t="s">
+        <v>73</v>
+      </c>
+      <c r="B64" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64">
+        <v>200</v>
+      </c>
+      <c r="D64">
+        <v>200</v>
+      </c>
+      <c r="E64" t="b">
+        <v>1</v>
+      </c>
+      <c r="F64" t="s">
+        <v>101</v>
+      </c>
+      <c r="G64" t="s">
+        <v>121</v>
+      </c>
+      <c r="H64" t="s">
+        <v>173</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J64" t="s">
+        <v>209</v>
+      </c>
+      <c r="K64" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11">
+      <c r="A65" t="s">
+        <v>74</v>
+      </c>
+      <c r="B65" t="s">
+        <v>92</v>
+      </c>
+      <c r="C65">
+        <v>200</v>
+      </c>
+      <c r="D65">
+        <v>200</v>
+      </c>
+      <c r="E65" t="b">
+        <v>1</v>
+      </c>
+      <c r="F65" t="s">
+        <v>101</v>
+      </c>
+      <c r="G65" t="s">
+        <v>122</v>
+      </c>
+      <c r="H65" t="s">
+        <v>174</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J65" t="s">
+        <v>210</v>
+      </c>
+      <c r="K65" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11">
+      <c r="A66" t="s">
+        <v>75</v>
+      </c>
+      <c r="B66" t="s">
+        <v>92</v>
+      </c>
+      <c r="C66">
+        <v>200</v>
+      </c>
+      <c r="D66">
+        <v>200</v>
+      </c>
+      <c r="E66" t="b">
+        <v>1</v>
+      </c>
+      <c r="F66" t="s">
+        <v>101</v>
+      </c>
+      <c r="G66" t="s">
+        <v>122</v>
+      </c>
+      <c r="H66" t="s">
+        <v>175</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J66" t="s">
+        <v>210</v>
+      </c>
+      <c r="K66" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11">
+      <c r="A67" t="s">
+        <v>76</v>
+      </c>
+      <c r="B67" t="s">
         <v>93</v>
       </c>
-      <c r="G62" t="s">
-        <v>111</v>
-      </c>
-      <c r="H62" t="s">
-        <v>159</v>
-      </c>
-      <c r="I62" t="s">
-        <v>175</v>
-      </c>
-      <c r="J62" t="s">
-        <v>188</v>
-      </c>
-      <c r="K62" t="s">
-        <v>209</v>
+      <c r="C67">
+        <v>200</v>
+      </c>
+      <c r="D67">
+        <v>200</v>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+      <c r="F67" t="s">
+        <v>101</v>
+      </c>
+      <c r="G67" t="s">
+        <v>123</v>
+      </c>
+      <c r="H67" t="s">
+        <v>176</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="J67" t="s">
+        <v>211</v>
+      </c>
+      <c r="K67" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -4707,6 +5386,11 @@
     <hyperlink ref="I57" r:id="rId16"/>
     <hyperlink ref="I58" r:id="rId17"/>
     <hyperlink ref="I59" r:id="rId18"/>
+    <hyperlink ref="I63" r:id="rId19"/>
+    <hyperlink ref="I64" r:id="rId20"/>
+    <hyperlink ref="I65" r:id="rId21"/>
+    <hyperlink ref="I66" r:id="rId22"/>
+    <hyperlink ref="I67" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Implementing SNAP script on usage of language models for embeddings
</commit_message>
<xml_diff>
--- a/Logs/interaction_log.xlsx
+++ b/Logs/interaction_log.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="293">
   <si>
     <t>timestamp</t>
   </si>
@@ -250,6 +250,33 @@
     <t>2025-09-26T11:34:52.334743</t>
   </si>
   <si>
+    <t>2025-10-21T21:10:52.199161</t>
+  </si>
+  <si>
+    <t>2025-10-21T21:11:32.363581</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:06:51.646914</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:07:07.376371</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:08:02.191148</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:09:02.001442</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:09:32.046759</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:11:19.352493</t>
+  </si>
+  <si>
+    <t>2025-10-22T00:12:20.343462</t>
+  </si>
+  <si>
     <t>What funding did 2024 Technical Reporting cover?</t>
   </si>
   <si>
@@ -302,6 +329,21 @@
   </si>
   <si>
     <t xml:space="preserve">Who is responsible for approving changes to reporting categories and for balancing the benefits of collecting detailed information against the reporting burden on P/A? </t>
+  </si>
+  <si>
+    <t>What are the 2025 reporting timelines?</t>
+  </si>
+  <si>
+    <t>What are the technical reporting timelines for 2025?</t>
+  </si>
+  <si>
+    <t>When does PRMS opens?</t>
+  </si>
+  <si>
+    <t>What is impact?</t>
+  </si>
+  <si>
+    <t>What is impact? in the context of technical reporting and the Results Framework</t>
   </si>
   <si>
     <t xml:space="preserve">You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:
@@ -339,6 +381,15 @@
     <t>You are a RAG assistant for deeper research. Use all the chunks that you receive. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.</t>
   </si>
   <si>
+    <t>You are a helpful assistant that answers very detailedly to user questions</t>
+  </si>
+  <si>
+    <t>You are a helpful assistant</t>
+  </si>
+  <si>
+    <t>You are a helpful assistant that answer user questions in a very detailed and comprehensive way</t>
+  </si>
+  <si>
     <t>pptx:Information Session on 2025 Technical Reporting.pptx:s9:0.307, docx:Engagement Plan 2025 Technical Reporting.docx:p2:0.304, pptx:Information Session on 2025 Technical Reporting.pptx:s2:0.299, docx:Guidance on reporting outputs or outcomes.docx:p22:0.263, docx:Engagement Plan 2025 Technical Reporting.docx:p59:0.244, pdf:CGIAR_ImpactReport_2022-24.pdf:p1:0.239, docx:Engagement Plan 2025 Technical Reporting.docx:p31:0.208, pptx:Engagement Plan 2025 Technical Reporting.pptx:s1:0.202, docx:CGSpace.docx:p3:0.201, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5:0.200, docx:General information on Technical Reporting .docx:p1:0.196, pptx:Information Session on 2025 Technical Reporting.pptx:s15:0.184, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1:0.176, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23:0.166, docx:Guidance on reporting outputs or outcomes.docx:p21:0.163, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4:0.160, docx:Guidance on reporting outputs or outcomes.docx:p30:0.160, docx:2025 Technical Reporting Information (Session 2).docx:p5:0.152, docx:2025 Technical Reporting Information (Session 2).docx:p32:0.138, docx:Guidance on reporting outputs or outcomes.docx:p24:0.138, pdf:Type3_2024Report.pdf:p1:0.136, pptx:Information Session on 2025 Technical Reporting.pptx:s13:0.134, docx:Using the PRMS Reporting Tool.docx:p12:0.133, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7:0.133, docx:Guidance on reporting outputs or outcomes.docx:p31:0.133, docx:General information on Technical Reporting .docx:p4:0.131, pptx:Information Session on 2025 Technical Reporting.pptx:s7:0.128, pdf:Type3_2024Report.pdf:p5:0.124, pptx:Information Session on 2025 Technical Reporting.pptx:s5:0.124, pdf:Portfolio Narrative_2024.pdf:p1:0.124, pdf:Portfolio Narrative_2024.pdf:p5:0.124, pptx:Information Session on 2025 Technical Reporting.pptx:s3:0.123, docx:Innovation use.docx:p7:0.121, pptx:Information Session on 2025 Technical Reporting.pptx:s6:0.121, docx:Innovation development.docx:p31:0.120, docx:2025 Technical Reporting Information (Session 1).docx:p26:0.119, pptx:Information Session on 2025 Technical Reporting.pptx:s10:0.118, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16:0.118, docx:2025 Technical Reporting Information (Session 1).docx:p7:0.117, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6:0.116, pdf:Portfolio Narrative_2024.pdf:p6:0.110, docx:2025 Technical Reporting Information (Session 2).docx:p1:0.110, docx:2025 Technical Reporting Information (Session 1).docx:p1:0.110, docx:Guidance on reporting outputs or outcomes.docx:p26:0.109, docx:Innovation development.docx:p13:0.108, docx:Submitting evidence.docx:p3:0.108, docx:Guidance on complementary innnov.docx:p38:0.107, docx:Engagement Plan 2025 Technical Reporting.docx:p61:0.106, docx:Engagement Plan 2025 Technical Reporting.docx:p27:0.102, pptx:Information Session on 2025 Technical Reporting.pptx:s1:0.099, pdf:Type3_2024Report.pdf:p11:0.099, pdf:Type3_2024Report.pdf:p4:0.099, docx:General information on Technical Reporting .docx:p5:0.098, docx:Engagement Plan 2025 Technical Reporting.docx:p39:0.097, docx:Guidance on complementary innnov.docx:p10:0.097, pptx:Information Session on 2025 Technical Reporting.pptx:s4:0.094, pptx:Information Session on 2025 Technical Reporting.pptx:s11:0.092, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2:0.092, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18:0.090, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22:0.089, docx:2025 Technical Reporting Information (Session 2).docx:p26:0.089, docx:Using the PRMS Reporting Tool.docx:p1:0.089, docx:2025 Technical Reporting MELIA glossary.docx:p6:0.089, docx:Engagement Plan 2025 Technical Reporting.docx:p106:0.088, pdf:Type3_2024Report.pdf:p6:0.087, docx:Engagement Plan 2025 Technical Reporting.docx:p42:0.086, docx:General reporting guidance.docx:p1:0.085, docx:General reporting guidance.docx:p5:0.084, docx:2025 Technical Reporting Information (Session 1).docx:p30:0.084, docx:Engagement Plan 2025 Technical Reporting.docx:p17:0.083, docx:Guidance on reporting outputs or outcomes.docx:p2:0.082, docx:2025 Technical Reporting Information (Session 2).docx:p11:0.081, docx:Engagement Plan 2025 Technical Reporting.docx:p69:0.080, pdf:CGIAR_ImpactReport_2022-24.pdf:p2:0.080, docx:Engagement Plan 2025 Technical Reporting.docx:p25:0.079, docx:Reporting the geographic location of results.docx:p1:0.078, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3:0.074, docx:Engagement Plan 2025 Technical Reporting.docx:p45:0.072, docx:Innovation use.docx:p22:0.072, pdf:Portfolio Narrative_2024.pdf:p37:0.071, docx:General reporting guidance.docx:p3:0.071, docx:2025 Technical Reporting Information (Session 2).docx:p41:0.071, docx:Engagement Plan 2025 Technical Reporting.docx:p8:0.071, docx:Engagement Plan 2025 Technical Reporting.docx:p10:0.070, docx:2025 Technical Reporting Information (Session 1).docx:p41:0.068, docx:Guidance on ensuring quality over quantity.docx:p3:0.066, docx:Engagement Plan 2025 Technical Reporting.docx:p55:0.066, pdf:Type3_2024Report.pdf:p3:0.066, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9:0.066, docx:Innovation development.docx:p40:0.066, docx:Guidance on ensuring quality over quantity.docx:p5:0.066, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15:0.065, docx:Knowledge products.docx:p11:0.065, pdf:Portfolio Narrative_2024.pdf:p72:0.065, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25:0.065, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p2:0.064, docx:2025 Technical Reporting Information (Session 2).docx:p7:0.064, docx:2025 Technical Reporting Information (Session 1).docx:p15:0.064, docx:2025 Technical Reporting Information (Session 2).docx:p14:0.063, docx:2025 Technical Reporting Information (Session 1).docx:p33:0.063</t>
   </si>
   <si>
@@ -400,6 +451,24 @@
   </si>
   <si>
     <t>docx:Questions and Answers from Tech reporting info sessions.docx:u7-10:0.538, pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4:0.379, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2:0.311, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt2:0.303, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt2:0.303, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.284, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.283, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.280, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt1:0.266, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt1:0.266, docx:Questions and Answers from Tech reporting info sessions.docx:u10-13:0.255, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.245, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2:0.244, docx:Engagement Plan 2025 Technical Reporting.docx:u16-19:0.243, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt4:0.242, pdf:Type3_2024Report.pdf:p5pt2:0.241, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p8pt3:0.240, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4:0.238, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt1:0.237, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt1:0.237, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4:0.236, docx:General information on Technical Reporting .docx:u1-6:0.233, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p14pt3:0.231, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.231, pdf:Type3_2024Report.pdf:p4pt1:0.229, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.225, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt3:0.223, docx:Guidance on ensuring quality over quantity.docx:u4-7:0.223, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p11pt3:0.223, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p9pt2:0.222, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.220, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.219, pdf:Type3_2024Report.pdf:p11pt2:0.217, docx:Using the PRMS Reporting Tool.docx:u1-4:0.217, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.217, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.217, docx:Engagement Plan 2025 Technical Reporting.docx:u13-16:0.217, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3:0.216, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt3:0.216, pdf:Portfolio Narrative_2024.pdf:p6pt4:0.215, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt1:0.214, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p8pt2:0.214, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.213, pdf:Type3_2024Report.pdf:p4pt3:0.212, pdf:Type3_2024Report.pdf:p11pt3:0.212, docx:Engagement Plan 2025 Technical Reporting.docx:u19-22:0.211, pdf:Type3_2024Report.pdf:p5pt3:0.211, docx:2025 Technical Reporting MELIA glossary.docx:u61-66:0.210, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p13pt4:0.210, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p9pt1:0.209, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.208, pdf:Type3_2024Report.pdf:p5pt1:0.208, docx:Engagement Plan 2025 Technical Reporting.docx:u4-7:0.207, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.206, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.206, pdf:Type3_2024Report.pdf:p5pt4:0.205, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p18pt1:0.205, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p18pt1:0.205, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt1:0.205, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p19pt1:0.205, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt1:0.204, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p11pt3:0.204, pdf:Type3_2024Report.pdf:p4pt2:0.200, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2:0.199, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2:0.199, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt2:0.198, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p10pt3:0.197, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt2:0.197, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.197, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt1:0.197, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt4:0.196, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt4:0.194, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt3:0.194, pdf:CGIAR_ImpactReport_2022-24.pdf:p67pt3:0.194, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.193, docx:Questions and Answers from Tech reporting info sessions.docx:u19-22:0.192, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2:0.191, pdf:Type3_2024Report.pdf:p8pt1:0.191, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3:0.190, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt4:0.190, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt4:0.190, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt3:0.190, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt2:0.189, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt1:0.189, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt1:0.189, docx:2025 Technical Reporting Information (Session 1).docx:u34-37:0.189, pdf:Type3_2024Report.pdf:p11pt4:0.189, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p23pt4:0.189, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.188, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt1:0.188, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt2:0.188, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt3:0.187, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt3:0.187, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt2:0.187, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt2:0.186, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p11pt2:0.186, docx:2025 Technical Reporting Information (Session 2).docx:u7-10:0.186, pdf:Type3_2024Report.pdf:p4pt4:0.184, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt1:0.184, docx:Standard Provisions 2026.docx:u157-160:0.183, docx:Standard Provisions 2026.docx:u130-133:0.183, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt1:0.182, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt1:0.182, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.182, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.182, docx:Questions and Answers from Tech reporting info sessions.docx:u1-4:0.181, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p13pt3:0.181, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.180, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt4:0.180, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt4:0.180, pdf:Portfolio Narrative_2024.pdf:p63pt2:0.179, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p12pt3:0.178, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3:0.178, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.178, docx:2025 Technical Reporting Information (Session 1).docx:u19-22:0.178, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt2:0.178, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt2:0.177, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt2:0.177, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt1:0.177, pdf:Type3_2024Report.pdf:p1pt2:0.176, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p62pt3:0.176, docx:Capacity sharing for development.docx:u1-6:0.175, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p19pt3:0.175, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.175, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3:0.174, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt3:0.174, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p10pt2:0.174, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p6pt4:0.174, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p14pt3:0.174, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.173, pdf:Portfolio Narrative_2024.pdf:p5pt1:0.173, docx:General reporting guidance.docx:u1-3:0.173, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt2:0.173, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt2:0.173, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p7pt3:0.172, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p37pt2:0.172, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.172, pdf:Better Diets and Nutrition_Inception Report 30-06-2025.pdf:p13pt2:0.172, pdf:Type3_2024Report.pdf:p6pt2:0.172, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p21pt1:0.172, docx:2025 Technical Reporting Information (Session 1).docx:u40-43:0.171, pdf:Portfolio Narrative_2024.pdf:p5pt2:0.170, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt3:0.170, pdf:Genebanks_Inception Report 30-06-2025.pdf:p35pt2:0.170, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p18pt2:0.169, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt4:0.169, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt1:0.169, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt1:0.169, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p16pt2:0.169, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.168, pdf:CGIAR_ImpactReport_2022-24.pdf:p6pt4:0.168, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt4:0.168, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt4:0.168, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt3:0.168, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt2:0.168, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt2:0.168, docx:Standard Provisions 2026.docx:u133-136:0.167, pdf:Portfolio Narrative_2024.pdf:p1pt2:0.167, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt2:0.167, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt1:0.166, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p8pt4:0.165, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.165, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt1:0.165, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt1:0.165, docx:Questions and Answers from Tech reporting info sessions.docx:u13-16:0.165, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p29pt3:0.165, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt1:0.165, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p8pt1:0.164, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt2:0.164, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1:0.164, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt3:0.163, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt4:0.163, docx:2025 Technical Reporting Information (Session 2).docx:u10-13:0.163, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p14pt4:0.163, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p24pt3:0.163, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p11pt2:0.162, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt3:0.162, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt3:0.162, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p17pt1:0.162, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p24pt1:0.161, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p24pt1:0.161, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p11pt1:0.161, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.161, docx:Innovation development.docx:u4-7:0.160, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p13pt1:0.160, docx:Questions and Answers from Tech reporting info sessions.docx:u16-19:0.160, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p14pt1:0.159, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p14pt1:0.159, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt3:0.159, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt1:0.159, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt2:0.159, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt3:0.159, pdf:Portfolio Narrative_2024.pdf:p12pt4:0.159, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt1:0.159, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt1:0.159, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p19pt4:0.159, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p9pt2:0.158, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p7pt2:0.158</t>
+  </si>
+  <si>
+    <t>pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4:0.685, pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4:0.472, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2:0.387, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.349, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.341, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3:0.335, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.333, docx:General information on Technical Reporting .docx:u1-6:0.324, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2:0.317, docx:2025 Technical Reporting Information (Session 2).docx:u4-7:0.309, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3:0.300, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2:0.298, docx:Engagement Plan 2025 Technical Reporting.docx:u13-16:0.296, docx:Questions and Answers from Tech reporting info sessions.docx:u1-4:0.285, docx:2025 Technical Reporting Information (Session 1).docx:u4-7:0.283, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.279, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt1:0.274, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt3:0.269, pdf:Portfolio Narrative_2024.pdf:p6pt4:0.267, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt3:0.263, pdf:Type3_2024Report.pdf:p5pt2:0.259, docx:Engagement Plan 2025 Technical Reporting.docx:u4-7:0.253, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt1:0.250, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt1:0.250, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt1:0.250, pdf:Type3_2024Report.pdf:p4pt1:0.248, pdf:Type3_2024Report.pdf:p1pt2:0.246, docx:Using the PRMS Reporting Tool.docx:u1-4:0.246, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4:0.246, docx:General reporting guidance.docx:u1-3:0.244, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3:0.240, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3:0.240, pdf:Portfolio Narrative_2024.pdf:p1pt2:0.239, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.238, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.238, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.233, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt3:0.232, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p23pt1:0.228, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt4:0.228, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1:0.226, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1:0.226, docx:Engagement Plan 2025 Technical Reporting.docx:u16-19:0.226, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1:0.223, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.217, pdf:Type3_2024Report.pdf:p4pt2:0.215, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.213, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt1:0.213, docx:2025 Technical Reporting Information (Session 1).docx:u28-31:0.212, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.212, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.212, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.211, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.209, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p31pt2:0.209, docx:Questions and Answers from Tech reporting info sessions.docx:u7-10:0.208, pdf:CGI21_508012_PORB_Genebanks.pdf:p42pt2:0.208, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt1:0.207, pdf:CGI21_508012_PORB_Genebanks.pdf:p42pt1:0.206, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2:0.206, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.206, pdf:Type3_2024Report.pdf:p5pt1:0.206, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p11pt3:0.205, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p24pt1:0.205, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p24pt1:0.205, docx:Engagement Plan 2025 Technical Reporting.docx:u10-13:0.205, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p28pt3:0.204, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p19pt3:0.204, docx:Capacity sharing for development.docx:u1-6:0.203, pdf:CGI21-507032-PORB-Climate Action.pdf:p27pt1:0.203, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.203, docx:Questions and Answers from Tech reporting info sessions.docx:u10-13:0.202, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt4:0.202, pdf:Type3_2024Report.pdf:p11pt3:0.201, docx:2025 Technical Reporting Information (Session 1).docx:u25-28:0.201, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt4:0.201, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt4:0.201, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt4:0.200, pdf:Type3_2024Report.pdf:p5pt4:0.199, pdf:CGI21_508012_PORB_Genebanks.pdf:p21pt1:0.199, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p31pt1:0.199, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p35pt1:0.197, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3:0.197, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt1:0.197, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt2:0.197, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.197, pdf:CGI21-507032-PORB-Climate Action.pdf:p41pt1:0.197, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p64pt1:0.197, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p23pt2:0.196, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p20pt1:0.196, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.196, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p11pt1:0.195, docx:2025 Technical Reporting Information (Session 1).docx:u22-25:0.195, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt2:0.195, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p43pt1:0.194, docx:User Roles and Rules for the PRMS Reporting.docx:u10-13:0.193, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p38pt1:0.193, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.193, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p33pt1:0.192, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p82pt1:0.191, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p25pt1:0.191, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p13pt1:0.191</t>
+  </si>
+  <si>
+    <t>pdf:Portfolio Narrative_2024.pdf:p1pt2:0.812, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.749, docx:General information on Technical Reporting .docx:u1-6:0.700, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1:0.691, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3:0.691, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2:0.676, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3:0.666, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3:0.662, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1:0.649, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1:0.649, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.647, docx:Questions and Answers from Tech reporting info sessions.docx:u1-4:0.643, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4:0.637, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.637, pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2:0.608, docx:Engagement Plan 2025 Technical Reporting.docx:u52-55:0.607, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3:0.606, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3:0.606, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.603, pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1:0.602, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1:0.602, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1:0.602, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.600, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1:0.598, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1:0.595, docx:Engagement Plan 2025 Technical Reporting.docx:u4-7:0.594, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2:0.593, docx:Engagement Plan 2025 Technical Reporting.docx:u1-4:0.592, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.591, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1:0.590, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1:0.590, docx:2025 Technical Reporting Information (Session 2).docx:u7-10:0.590, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2:0.589, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2:0.589, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1:0.586, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1:0.586, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.585, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt3:0.583, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt3:0.583, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt3:0.583, pdf:Type3_2024Report.pdf:p5pt2:0.580, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p26pt1:0.576, docx:2025 Technical Reporting Information (Session 2).docx:u13-16:0.574, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt4:0.574, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt4:0.574, docx:Engagement Plan 2025 Technical Reporting.docx:u7-10:0.572, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p4pt1:0.569, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p43pt3:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p24pt1:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p24pt1:0.568, pdf:Portfolio Narrative_2024.pdf:p8pt4:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt2:0.567, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt2:0.567, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p4pt1:0.567, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt3:0.566, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p30pt1:0.565, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt1:0.558, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p4pt1:0.557, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt2:0.557, pdf:Portfolio Narrative_2024.pdf:p6pt2:0.555, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p21pt1:0.554, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p21pt1:0.554, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.553, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p57pt1:0.553, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p49pt1:0.551, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p81pt1:0.551, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p34pt1:0.550, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt4:0.549, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt2:0.547, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt2:0.547, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p13pt1:0.547, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p51pt2:0.546, docx:Engagement Plan 2025 Technical Reporting.docx:u10-13:0.545, docx:Engagement Plan 2025 Technical Reporting.docx:u13-16:0.544, pptx:Information Session on 2025 Technical Reporting.pptx:s13pt1:0.543, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p1pt2:0.541, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt1:0.540, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt1:0.540, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p21pt2:0.539, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt2:0.539, pdf:CGI21-507032-PORB-Climate Action.pdf:p4pt1:0.538, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p9pt1:0.538, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p55pt1:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt1:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt1:0.538, pdf:Type3_2024Report.pdf:p4pt3:0.537, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p16pt1:0.536, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p33pt1:0.535, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p53pt2:0.535, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p32pt1:0.535, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p9pt1:0.534, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.533, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.533, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p52pt2:0.532, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p66pt1:0.532, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p39pt1:0.532, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p6pt1:0.532, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p4pt1:0.531, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p2pt1:0.530, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p2pt1:0.530</t>
+  </si>
+  <si>
+    <t>pptx:Information Session on 2025 Technical Reporting.pptx:s12pt1:0.667, pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt1:0.667, docx:Questions and Answers from Tech reporting info sessions.docx:u40-42:0.604, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt3:0.552, pptx:Information Session on 2025 Technical Reporting.pptx:s13pt2:0.544, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt1:0.538, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt2:0.538, pptx:Information Session on 2025 Technical Reporting.pptx:s7pt3:0.534, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.527, docx:Engagement Plan 2025 Technical Reporting.docx:u55-58:0.504, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4:0.502, docx:2025 Technical Reporting Information (Session 2).docx:u49-52:0.492, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1:0.489, pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1:0.487, docx:Engagement Plan 2025 Technical Reporting.docx:u58-61:0.480, docx:2025 Technical Reporting Information (Session 1).docx:u10-13:0.478, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p16pt3:0.478, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt3:0.474, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p23pt4:0.454, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt3:0.454, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt3:0.446, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p21pt3:0.439, docx:Engagement Plan 2025 Technical Reporting.docx:u34-37:0.435, docx:Using the PRMS Reporting Tool.docx:u7-9:0.431, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4:0.428, docx:Engagement Plan 2025 Technical Reporting.docx:u49-52:0.427, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt3:0.424, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt2:0.400, docx:Submitting evidence.docx:u16-19:0.395, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3:0.394, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p57pt4:0.393, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p86pt4:0.388, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p21pt2:0.387, docx:2025 Technical Reporting Information (Session 1).docx:u22-25:0.385, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt3:0.385, docx:Questions and Answers from Tech reporting info sessions.docx:u4-7:0.379, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt2:0.379, docx:2025 Technical Reporting Information (Session 2).docx:u46-49:0.372, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt4:0.371, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1:0.370, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1:0.370, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p1pt2:0.368, docx:User Roles and Rules for the PRMS Reporting.docx:u1-4:0.367, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4:0.365, pptx:Information Session on 2025 Technical Reporting.pptx:s11pt3:0.363, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p1pt4:0.357, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p1pt2:0.353, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p3pt2:0.352, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p1pt4:0.351, docx:Engagement Plan 2025 Technical Reporting.docx:u46-49:0.349, pdf:Type3_2024Report.pdf:p11pt4:0.349, docx:2025 Technical Reporting Information (Session 1).docx:u37-40:0.347, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p16pt4:0.346, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p1pt1:0.344, docx:Guidance on complementary innnov.docx:u13-16:0.342, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt4:0.342, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3:0.342, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.340, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt1:0.340, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt2:0.338, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.335, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p8pt4:0.335, docx:Submitting evidence.docx:u19-23:0.334, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt4:0.331, docx:2025 Technical Reporting Information (Session 2).docx:u40-43:0.329, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p21pt1:0.328, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p21pt1:0.328, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p6pt1:0.328, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt1:0.327, docx:Guidance on complementary innnov.docx:u10-13:0.326, docx:Engagement Plan 2025 Technical Reporting.docx:u31-34:0.326, docx:2025 Technical Reporting Information (Session 2).docx:u7-10:0.323, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p51pt3:0.321, pptx:Information Session on 2025 Technical Reporting.pptx:s8pt2:0.321, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p19pt3:0.321, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt3:0.320, docx:CGSpace.docx:u7-12:0.320, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt4:0.319, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p9pt3:0.318, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p1pt2:0.317, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p14pt2:0.317, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p9pt4:0.316, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p1pt4:0.314, docx:2025 Technical Reporting Information (Session 2).docx:u25-28:0.314, docx:Submitting evidence.docx:u10-13:0.313, pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p8pt1:0.311, pptx:Information Session on 2025 Technical Reporting.pptx:s13pt1:0.311, pdf:Type3_2024Report.pdf:p6pt4:0.311, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p15pt2:0.311, docx:Questions and Answers from Tech reporting info sessions.docx:u10-13:0.310, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p10pt4:0.306, docx:Using the PRMS Reporting Tool.docx:u1-4:0.305, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p15pt2:0.305, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p52pt2:0.304, docx:Using the PRMS Reporting Tool.docx:u4-7:0.304, docx:2025 Technical Reporting Information (Session 1).docx:u31-34:0.303, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p49pt2:0.302, docx:Innovation development.docx:u19-22:0.301, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p30pt4:0.301, docx:Engagement Plan 2025 Technical Reporting.docx:u7-10:0.301</t>
+  </si>
+  <si>
+    <t>pdf:Portfolio Narrative_2024.pdf:p1pt2:0.812, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.749, docx:General information on Technical Reporting .docx:u1-6:0.700, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1:0.691, pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3:0.691, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2:0.676, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3:0.666, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3:0.662, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1:0.649, pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1:0.649, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2:0.647, docx:Questions and Answers from Tech reporting info sessions.docx:u1-4:0.643, pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4:0.637, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1:0.637, pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2:0.608, docx:Engagement Plan 2025 Technical Reporting.docx:u52-55:0.607, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3:0.606, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3:0.606, docx:2025 Technical Reporting Information (Session 1).docx:u1-4:0.603, pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1:0.602, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1:0.602, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1:0.602, docx:2025 Technical Reporting Information (Session 2).docx:u1-4:0.600, pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1:0.598, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1:0.595, docx:Engagement Plan 2025 Technical Reporting.docx:u4-7:0.594, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2:0.593, docx:Engagement Plan 2025 Technical Reporting.docx:u1-4:0.592, docx:2025 Technical Reporting Information (Session 2).docx:u31-34:0.591, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1:0.590, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1:0.590, docx:2025 Technical Reporting Information (Session 2).docx:u7-10:0.590, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2:0.589, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2:0.589, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1:0.586, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1:0.586, docx:2025 Technical Reporting Information (Session 1).docx:u7-10:0.585, pptx:Information Session on 2025 Technical Reporting.pptx:s4pt3:0.583, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p6pt3:0.583, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p6pt3:0.583, pdf:Type3_2024Report.pdf:p5pt2:0.580, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p26pt1:0.576, docx:2025 Technical Reporting Information (Session 2).docx:u13-16:0.574, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt4:0.574, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt4:0.574, docx:Engagement Plan 2025 Technical Reporting.docx:u7-10:0.572, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p4pt1:0.569, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p43pt3:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p24pt1:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p24pt1:0.568, pdf:Portfolio Narrative_2024.pdf:p8pt4:0.568, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt2:0.567, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt2:0.567, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p4pt1:0.567, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt3:0.566, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p30pt1:0.565, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt1:0.558, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p4pt1:0.557, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt2:0.557, pdf:Portfolio Narrative_2024.pdf:p6pt2:0.555, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p21pt1:0.554, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p21pt1:0.554, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.553, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p57pt1:0.553, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p49pt1:0.551, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p81pt1:0.551, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p34pt1:0.550, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt4:0.549, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt2:0.547, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt2:0.547, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p13pt1:0.547, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p51pt2:0.546, docx:Engagement Plan 2025 Technical Reporting.docx:u10-13:0.545, docx:Engagement Plan 2025 Technical Reporting.docx:u13-16:0.544, pptx:Information Session on 2025 Technical Reporting.pptx:s13pt1:0.543, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p1pt2:0.541, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt1:0.540, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt1:0.540, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p21pt2:0.539, pdf:CGI21_508012_PORB_Genebanks.pdf:p2pt2:0.539, pdf:CGI21-507032-PORB-Climate Action.pdf:p4pt1:0.538, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p9pt1:0.538, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p55pt1:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt1:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt1:0.538, pdf:Type3_2024Report.pdf:p4pt3:0.537, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p16pt1:0.536, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p33pt1:0.535, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p53pt2:0.535, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p32pt1:0.535, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p9pt1:0.534, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.533, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.533, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p52pt2:0.532, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p66pt1:0.532, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p39pt1:0.532, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p6pt1:0.532, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p4pt1:0.531, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p2pt1:0.530, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p2pt1:0.530, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p41pt1:0.530, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p4pt1:0.529, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p30pt1:0.527, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p29pt2:0.526, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p2pt2:0.525, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p1pt1:0.525, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p2pt2:0.522, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p1pt2:0.521, docx:Questions and Answers from Tech reporting info sessions.docx:u4-7:0.521, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p28pt1:0.521, pdf:CGI21-507032-PORB-Climate Action.pdf:p27pt1:0.520, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p1pt2:0.520, pdf:Policy Innovations_Inception Report 30-06-2025.pdf:p1pt2:0.520, pptx:Information Session on 2025 Technical Reporting.pptx:s6pt1:0.519, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt3:0.518, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p59pt1:0.518, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3:0.518, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt3:0.518, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p29pt1:0.517, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt2:0.517, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p17pt1:0.517, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt1:0.516, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt1:0.516, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p46pt1:0.516, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt1:0.516, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p4pt1:0.515, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p1pt1:0.515, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p1pt1:0.515, pdf:CGI21_508012_PORB_Genebanks.pdf:p1pt1:0.515, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p38pt1:0.515, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p2pt2:0.515, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p2pt2:0.515, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p25pt4:0.514, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p25pt4:0.514, pdf:Portfolio Narrative_2024.pdf:p63pt1:0.514, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p37pt1:0.513, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p51pt2:0.513, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p34pt1:0.513, pdf:CGI21_508012_PORB_Genebanks.pdf:p4pt1:0.513, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p71pt1:0.512, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p49pt1:0.512, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt2:0.512, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt2:0.512, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p1pt2:0.511, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p27pt1:0.511, docx:2025 Technical Reporting MELIA glossary.docx:u31-34:0.510, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt1:0.510, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p10pt1:0.510, pdf:CGI21-507033-PORB-Policy Innovations.pdf:p63pt1:0.510, pdf:Capacity Sharing_Inception Report 30-06-2025.pdf:p15pt4:0.510, pdf:Portfolio Narrative_2024.pdf:p6pt1:0.509, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt1:0.508, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt1:0.508, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p37pt1:0.508, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3:0.508, pdf:Type3_2024Report.pdf:p4pt2:0.507, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p14pt1:0.507, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt3:0.507, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt3:0.507, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p4pt1:0.507, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p57pt4:0.507, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt4:0.507, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt4:0.507, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p20pt1:0.506, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p18pt1:0.506, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt1:0.506, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt1:0.506, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p25pt1:0.506, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p38pt1:0.506, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1:0.506, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt1:0.506, pdf:CGI21-507032-PORB-Climate Action.pdf:p46pt1:0.504, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p37pt1:0.503, pdf:CGI21-507032-PORB-Climate Action.pdf:p30pt1:0.503, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p2pt2:0.503, docx:Questions and Answers from Tech reporting info sessions.docx:u34-37:0.503, pdf:CGI21-509002-PORB-Sustainable Farming (1).pdf:p10pt1:0.503, docx:Engagement Plan 2025 Technical Reporting.docx:u16-19:0.503, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p59pt1:0.502, pdf:CGI21-507032-PORB-Climate Action.pdf:p2pt2:0.502, pdf:CGI21-508002-PORB-Sustainable Animal and Aquatic Foods.pdf:p2pt2:0.502, pdf:CGI21-507032-PORB-Better Diets and Nutrition.pdf:p37pt1:0.502, pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p59pt2:0.502, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p24pt1:0.502, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p2pt2:0.502, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p24pt1:0.502, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p15pt1:0.501, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt1:0.501, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt1:0.501, pdf:CGIAR_ImpactReport_2022-24.pdf:p1pt4:0.501, pdf:Portfolio Narrative_2024.pdf:p5pt2:0.500, pdf:CGI21-507032-PORB-Climate Action.pdf:p36pt1:0.500, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt4:0.500, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt4:0.500, pdf:CGI21_508012_PORB_Genebanks.pdf:p42pt2:0.499, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3:0.498, pdf:CGI21-508004-PORB-Capacity Sharing.pdf:p21pt1:0.498, pdf:Portfolio Narrative_2024.pdf:p6pt4:0.498, pdf:CGI21-507031-PORB-Food Frontiers and Security.pdf:p4pt1:0.498, pdf:CGI21-508004-PORB-Digital Transformation.pdf:p19pt1:0.498</t>
+  </si>
+  <si>
+    <t>pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2:0.653, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.653, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.653, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2:0.653, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2:0.653, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2:0.653, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4:0.649, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3:0.610, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p70pt4:0.604, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3:0.595, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2:0.592, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3:0.592, pdf:Portfolio Narrative_2024.pdf:p58pt2:0.591, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1:0.582, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p17pt3:0.568, pdf:Portfolio Narrative_2024.pdf:p11pt3:0.566, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt4:0.563, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt2:0.558, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt1:0.554, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt2:0.551, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt4:0.542, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3:0.541, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p63pt4:0.540, pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt1:0.537, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt2:0.536, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt2:0.536, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4:0.534, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt4:0.534, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p48pt4:0.529, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.524, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p20pt4:0.511, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p23pt3:0.505, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p50pt4:0.504, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p8pt3:0.501, pdf:Portfolio Narrative_2024.pdf:p74pt3:0.499, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt2:0.494, pdf:Portfolio Narrative_2024.pdf:p74pt4:0.493, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3:0.492, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p15pt1:0.492, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p1pt3:0.491, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p1pt2:0.490, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p1pt2:0.489, pdf:Portfolio Narrative_2024.pdf:p50pt2:0.484, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1:0.484, pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt2:0.482, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt3:0.482, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p43pt4:0.480, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p14pt1:0.478, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt1:0.476, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p44pt4:0.476, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4:0.475, pdf:Portfolio Narrative_2024.pdf:p52pt2:0.475, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p90pt3:0.474, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p1pt3:0.473, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p16pt1:0.473, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p83pt4:0.471, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.471, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4:0.471, pdf:CGIAR_ImpactReport_2022-24.pdf:p50pt4:0.471, pdf:Portfolio Narrative_2024.pdf:p71pt4:0.470, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p25pt2:0.470, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p14pt2:0.465, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p44pt3:0.462, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt2:0.461, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt2:0.461, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p9pt1:0.460, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p1pt1:0.459, pdf:Sustainable Farming_Inception Report 30-06-2025.pdf:p34pt3:0.458, pdf:Portfolio Narrative_2024.pdf:p67pt4:0.458, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p2pt3:0.457, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt4:0.455, pdf:Portfolio Narrative_2024.pdf:p4pt1:0.454, pdf:Portfolio Narrative_2024.pdf:p11pt2:0.454, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p44pt2:0.451, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt3:0.451, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p90pt4:0.450, pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt2:0.449, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3:0.448, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.447, pdf:Portfolio Narrative_2024.pdf:p60pt3:0.447, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p7pt4:0.447, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p38pt3:0.446, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p64pt4:0.444, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p42pt4:0.444, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p48pt4:0.444, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p85pt4:0.442, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p47pt4:0.442, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p15pt3:0.441, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p13pt1:0.441, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt4:0.440, pdf:CGI21-508007-PORB-Multifunctional Landscapes.pdf:p80pt4:0.440, pdf:Portfolio Narrative_2024.pdf:p54pt4:0.439, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p50pt1:0.438, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt4:0.438, pdf:CGIAR_ImpactReport_2022-24.pdf:p42pt2:0.438, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p26pt4:0.437, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt2:0.437, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt3:0.436, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p50pt2:0.436, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p14pt2:0.436, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p14pt2:0.436, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p8pt2:0.436, pdf:CGIAR_ImpactReport_2022-24.pdf:p3pt1:0.436, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt4:0.435, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt2:0.435, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p7pt4:0.435, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3:0.435, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3:0.435, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt2:0.434, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p23pt2:0.432, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt1:0.432, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p32pt3:0.432, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p11pt3:0.432, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p2pt3:0.432, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p52pt4:0.430, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt2:0.430, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt3:0.430, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt3:0.430, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt4:0.430, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p50pt3:0.429, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p11pt3:0.429, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt2:0.428, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p9pt3:0.427, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p23pt3:0.427, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p16pt2:0.426, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1:0.425, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt1:0.425, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p14pt1:0.425, pdf:Portfolio Narrative_2024.pdf:p67pt3:0.425, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt4:0.425, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p7pt3:0.424, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt1:0.423, pdf:Climate Action_Inception Report 30-06-2025.pdf:p16pt3:0.422, pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt1:0.421, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p51pt2:0.420, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p25pt2:0.420, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.419, pdf:Portfolio Narrative_2024.pdf:p68pt2:0.419, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p4pt2:0.419, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p14pt1:0.419, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p14pt1:0.419, pdf:Portfolio Narrative_2024.pdf:p11pt1:0.418, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p13pt3:0.418, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p2pt3:0.418, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p4pt3:0.418, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt3:0.417, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt2:0.415, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt2:0.415, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p8pt4:0.415, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p35pt1:0.414, pdf:CGIAR_ImpactReport_2022-24.pdf:p18pt1:0.414, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p4pt2:0.414, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt3:0.414, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.412, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt1:0.412, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p14pt2:0.412, pdf:CGIAR_ImpactReport_2022-24.pdf:p66pt2:0.411, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p74pt4:0.411, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p9pt3:0.411, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p36pt2:0.410, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p31pt2:0.409, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt3:0.409, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p36pt3:0.408, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p24pt4:0.408, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p64pt3:0.407, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p39pt2:0.407, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p8pt3:0.405, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p16pt3:0.405, pdf:CGIAR_ImpactReport_2022-24.pdf:p18pt2:0.405, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p20pt4:0.402, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt2:0.402, pdf:CGIAR_ImpactReport_2022-24.pdf:p30pt3:0.401, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p14pt1:0.401, pdf:CGIAR_ImpactReport_2022-24.pdf:p34pt2:0.401, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p3pt2:0.401, pdf:Portfolio Narrative_2024.pdf:p4pt3:0.400, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p36pt2:0.399, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p47pt2:0.399, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p17pt4:0.399, pdf:CGIAR_ImpactReport_2022-24.pdf:p39pt2:0.399, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p81pt2:0.399, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p81pt4:0.399, pdf:CGIAR_ImpactReport_2022-24.pdf:p32pt3:0.398, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p30pt2:0.398, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p67pt2:0.397, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p42pt4:0.397, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p87pt4:0.397, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p34pt2:0.397, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p71pt4:0.396, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.396, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p15pt2:0.395, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p15pt2:0.394, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p19pt2:0.394, pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p22pt4:0.394, pdf:Gender Equality and Inclusion_Inception Report 30-06-2025.pdf:p20pt2:0.393, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p63pt3:0.393, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt2:0.392, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p39pt4:0.392, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt1:0.392, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p28pt3:0.391</t>
+  </si>
+  <si>
+    <t>pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3:0.766, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3:0.724, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3:0.690, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1:0.649, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3:0.644, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4:0.638, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt2:0.638, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3:0.637, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt3:0.637, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4:0.625, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4:0.625, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1:0.625, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2:0.619, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2:0.619, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3:0.615, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3:0.615, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt2:0.614, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt2:0.614, pdf:Portfolio Narrative_2024.pdf:p11pt3:0.614, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4:0.614, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3:0.609, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3:0.609, docx:Guidance on reporting outputs or outcomes.docx:u1-4:0.609, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt4:0.608, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2:0.607, pdf:Portfolio Narrative_2024.pdf:p58pt2:0.604, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4:0.603, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt4:0.603, docx:Guidance on reporting outputs or outcomes.docx:u19-22:0.600, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3:0.599, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4:0.585, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4:0.585, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt2:0.584, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p9pt2:0.584, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt4:0.579, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2:0.579, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt2:0.578, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt2:0.578, pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt1:0.577, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt4:0.577, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p9pt2:0.576, pdf:Type3_2024Report.pdf:p5pt2:0.576, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt4:0.574, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p4pt1:0.574, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt4:0.573, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p44pt3:0.571, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt2:0.569, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p9pt3:0.569, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt4:0.569, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt2:0.569, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt4:0.568, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt3:0.568, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p27pt2:0.566, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p14pt1:0.566, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p14pt1:0.566, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p2pt3:0.563, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p2pt3:0.563, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p14pt2:0.562, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p17pt3:0.561, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt2:0.558, pdf:Portfolio Narrative_2024.pdf:p74pt4:0.558, pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p14pt1:0.557, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt1:0.556, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt4:0.556, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt2:0.555, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt1:0.555, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt1:0.555, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p83pt4:0.554, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p7pt1:0.554, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p11pt3:0.553, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2:0.553, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3:0.553, pdf:Portfolio Narrative_2024.pdf:p52pt2:0.553, pdf:CGIAR_ImpactReport_2022-24.pdf:p64pt1:0.552, docx:Engagement Plan 2025 Technical Reporting.docx:u13-16:0.552, docx:Engagement Plan 2025 Technical Reporting.docx:u10-13:0.551, pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt2:0.551, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt1:0.550, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt1:0.550, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p38pt3:0.550, pdf:Type3_2024Report.pdf:p11pt4:0.550, pdf:Portfolio Narrative_2024.pdf:p6pt3:0.549, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt3:0.549, pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt2:0.548, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p1pt3:0.547, pdf:Portfolio Narrative_2024.pdf:p60pt3:0.547, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt2:0.547, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt2:0.547, pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p1pt1:0.545, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt1:0.544, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt1:0.544, pdf:Portfolio Narrative_2024.pdf:p5pt3:0.544, pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p9pt1:0.543, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt1:0.542, pdf:CGIAR_ImpactReport_2022-24.pdf:p50pt4:0.541, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt4:0.540, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt4:0.540, pdf:Portfolio Narrative_2024.pdf:p67pt4:0.540, docx:Guidance on ensuring quality over quantity.docx:u1-4:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p15pt1:0.538, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p15pt1:0.538, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt1:0.537, pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt2:0.537, pdf:Portfolio Narrative_2024.pdf:p68pt2:0.536, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt1:0.535, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt1:0.535, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4:0.535, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt3:0.535, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p15pt1:0.534, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p9pt3:0.534, pdf:Portfolio Narrative_2024.pdf:p54pt4:0.534, pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.534, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.534, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2:0.534, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2:0.534, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2:0.534, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2:0.534, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5pt2:0.531, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p5pt2:0.531, pdf:Portfolio Narrative_2024.pdf:p50pt2:0.531, pdf:Portfolio Narrative_2024.pdf:p6pt4:0.531, pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt1:0.530, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt4:0.529, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt4:0.529, pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p8pt2:0.528, pptx:Information Session on 2025 Technical Reporting.pptx:s11pt4:0.528, pdf:CGIAR_ImpactReport_2022-24.pdf:p2pt3:0.527, pptx:Information Session on 2025 Technical Reporting.pptx:s15pt2:0.527, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p7pt3:0.526, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt3:0.526, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt3:0.526, pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p10pt4:0.525, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p20pt4:0.524, pdf:Portfolio Narrative_2024.pdf:p71pt4:0.523, pdf:CGIAR_ImpactReport_2022-24.pdf:p42pt2:0.523, pdf:Food Frontiers and Security_Inception Report 30-06-2025.pdf:p15pt4:0.522, pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p18pt2:0.521, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p70pt4:0.520, pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt1:0.519, pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p11pt3:0.518, docx:2025 Technical Reporting MELIA glossary.docx:u19-22:0.518, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt2:0.518, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p3pt3:0.518, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p3pt3:0.518, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p50pt1:0.517, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p13pt4:0.516, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p13pt4:0.516, docx:Engagement Plan 2025 Technical Reporting.docx:u19-22:0.516, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p12pt1:0.516, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p44pt1:0.516, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p10pt1:0.516, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p10pt1:0.516, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p44pt2:0.515, pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1:0.515, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p34pt4:0.515, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt2:0.515, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt2:0.515, pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p36pt2:0.514, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1:0.514, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1:0.514, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p25pt1:0.513, pdf:Multifunctional Landscapes_Inception Report_MFL 30-06-2025.pdf:p2pt3:0.513, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p1pt3:0.513, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p20pt4:0.512, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p20pt4:0.512, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4pt3:0.512, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p4pt3:0.512, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p25pt2:0.512, pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt3:0.511, pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p8pt3:0.511, pdf:Portfolio Narrative_2024.pdf:p4pt1:0.511, pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2:0.510, pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p16pt1:0.510, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p7pt2:0.510, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt3:0.510, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p1pt2:0.510, pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt1:0.509, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p36pt1:0.509, pptx:Information Session on 2025 Technical Reporting.pptx:s3pt2:0.509, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p8pt3:0.508, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p8pt3:0.508, pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p23pt3:0.508, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p8pt2:0.508, pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p27pt3:0.507, pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p15pt2:0.507, pptx:Information Session on 2025 Technical Reporting.pptx:s5pt3:0.506, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p11pt2:0.506, pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt4:0.506, pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt2:0.506, pdf:CGIAR_PORB_Scaling_4Impact.pdf:p74pt4:0.506, pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt4:0.506, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt3:0.504, pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt3:0.504, pdf:CGIAR_ImpactReport_2022-24.pdf:p8pt3:0.504, pdf:Type3_2024Report.pdf:p4pt1:0.504, pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p14pt2:0.503, pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p2pt2:0.503, pptx:Information Session on 2025 Technical Reporting.pptx:s6pt1:0.502, pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt2:0.502, pdf:CGIAR_ImpactReport_2022-24.pdf:p18pt2:0.501</t>
   </si>
   <si>
     <t>I cannot find information in the provided chunks to answer this.  
@@ -844,6 +913,152 @@
 CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf — page 12 part 1 — p12pt1</t>
   </si>
   <si>
+    <t>I cannot find information in the provided chunks to answer this. For specific details regarding the 2025 reporting timelines, please refer to the Performance and Results Hub or the relevant technical reporting documents. These resources will provide the most accurate and updated information on deadlines and requirements for the reporting cycle. 
+Sources:
+File — Location — Cited IDs
+Information Session on 2025 Technical Reporting.pptx — slide 9 part 4 — pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4
+Engagement Plan 2025 Technical Reporting.pptx — slide 1 part 4 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4
+General information on Technical Reporting .docx — paragraph 1 to paragraph 7 — docx:General information on Technical Reporting .docx:u1-6
+2025 Technical Reporting Information (Session 2).docx — paragraph 4 to paragraph 7 — docx:2025 Technical Reporting Information (Session 2).docx:u4-7
+CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 1 part 1 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1</t>
+  </si>
+  <si>
+    <t>The 2025 reporting timelines for the CGIAR Technical Reporting process are structured around several key deliverables and deadlines, reflecting a transition year aimed at streamlining reporting processes. Here’s a detailed breakdown of the timelines and expectations:
+### Key Reporting Timelines for 2025
+1. **Reporting Period Opening**:
+   - The Performance and Results Management System (PRMS) is expected to open for reporting in **November 2025**. This will allow programs and accelerators to begin entering their results for the year.
+2. **Quality Assurance Process**:
+   - The quality assurance of reported results will take place in **February 2026**. This process is crucial for ensuring the reliability and accuracy of the data submitted.
+3. **Reflect Process**:
+   - The Reflect process, which involves reviewing and analyzing the reported results, will also occur in **Q1 2026**.
+4. **Annual Technical Reports Submission**:
+   - Each program and accelerator is responsible for drafting and submitting their **2025 Annual Technical Reports** by **April 2026**. These reports will provide assurance on the delivery against planned results and progress on the theory of change.
+5. **Portfolio Narrative Report**:
+   - A comprehensive **Portfolio Narrative Report** summarizing the overall contributions and performance will be due in **June 2026**.
+### Additional Context and Deliverables
+- **Integration of Projects**: The reporting will include the integration of the top **80% of Window 3 and bilateral projects** by center and dollar value into the technical reporting and planning processes.
+- **Minimum Data Standards**: There will be an application of minimum data standards for Window 3 and bilateral reporting, which will be refined during the pause and reflect process in early **Q1 2026**.
+- **AI-Generated Drafts**: To assist in the reporting process, an AI-generated draft (V0) of the annual technical report will be provided to each program and accelerator, which will include pre-filled text and analytics for each report section.
+### Engagement and Support
+- Throughout the reporting cycle, there will be **bi-weekly emails** sent to keep all stakeholders informed about updates, deadlines, and resources available for technical reporting.
+- **Info Sessions**: Specific information sessions will be scheduled in **September and October 2025** to provide deeper insights into the PRMS, quality assurance processes, and the annual technical report requirements.
+### Summary of Key Dates
+- **November 2025**: PRMS opens for reporting.
+- **February 2026**: Quality assurance of reported results.
+- **Q1 2026**: Reflect process.
+- **April 2026**: Submission of Annual Technical Reports.
+- **June 2026**: Submission of Portfolio Narrative Report.
+These timelines are designed to facilitate a smooth transition into the new reporting framework while ensuring that all programs and accelerators can effectively communicate their results and contributions. For ongoing updates and resources, stakeholders are encouraged to regularly consult the Performance and Results Hub.</t>
+  </si>
+  <si>
+    <t>I cannot find information in the provided chunks to answer this. The technical reporting timelines for 2025 may be detailed in the documents, but specific dates and deadlines are not explicitly mentioned in the excerpts provided. For accurate and comprehensive information, I recommend checking the Performance and Results Hub or the relevant technical reporting documents directly. 
+Sources:
+File — Location — Cited IDs
+Information Session on 2025 Technical Reporting.pptx — slide 4 part 1 — s4pt1
+CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 6 part 3 — p6pt3
+Engagement Plan 2025 Technical Reporting.docx — section 'Objective' paragraph 14 to section 'A single location for all documents and resources' paragraph 25 — u10-13</t>
+  </si>
+  <si>
+    <t>The technical reporting timelines for 2025 are as follows:
+1. **Delivery of 2025 Program and Accelerator Technical Reports**: Due by **April 2026**.
+2. **Delivery of the 2025 Portfolio Narrative**: Due by **June 2026**.
+3. **Integration of the top 80% of W3 and bilateral projects** (by Center portfolio value) into Program/Accelerator Theory of Change, MELIA, Plan of Results and Budget, and Technical Reporting: This integration is part of the phased approach for the 2025 Technical Reporting Arrangement.
+The reporting process is designed to streamline reporting and strengthen linkages across various components, including the Theory of Change and technical reporting. The 2025 reporting cycle is considered a transition year, focusing on aligning reporting with planned and budgeted results.
+For more detailed information, you can refer to the [CGIAR Technical Reporting Arrangement 2025-30 document](https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf).</t>
+  </si>
+  <si>
+    <t>The technical reporting timelines for 2025, as outlined in the CGIAR Technical Reporting Arrangement for 2025-30, indicate a structured approach to reporting that emphasizes integration and efficiency. Here are the key timelines and deliverables for 2025:
+### Key Reporting Timelines and Deliverables for 2025
+1. **Transition Year Focus**: 2025 is designated as a transition year, which means that the reporting processes will be streamlined and integrated with a focus on aligning various components such as the Theory of Change (ToC), Performance and Results Management System (PRMS), and technical reporting.
+2. **Program and Accelerator Technical Reports**:
+   - **Due Date**: April 2026
+   - Each program and accelerator is responsible for drafting and internally validating their technical reports, which will provide assurance on annual delivery against the Plan of Results and Budget.
+3. **Portfolio Narrative**:
+   - **Due Date**: June 2026
+   - This narrative will synthesize the contributions of various programs and accelerators to the overall portfolio.
+4. **Integration of Projects**:
+   - The top 80% of Window 3 (W3) and bilateral projects, based on center portfolio value, will be integrated into the Program/Accelerator Theory of Change, MELIA (Monitoring, Evaluation, Learning, Impact Assessment), Plan of Results and Budget, and Technical Reporting.
+5. **Quality Assurance Process**:
+   - Results reported in the PRMS will undergo a quality assessment process in February 2026. This ensures that the reported data is reliable and consistent.
+6. **Reporting Cycle**:
+   - The reporting cycle will include bi-weekly updates and targeted engagement sessions to support programs and accelerators throughout the reporting process.
+7. **Submission of Results**:
+   - Programs and accelerators are encouraged to report results that were planned and budgeted, with a focus on quality-assured results that will be available on the CGIAR Results Dashboard.
+8. **Engagement and Support**:
+   - An engagement plan will be in place from July 2025 to June 2026 to streamline communication and optimize support for programs and accelerators.
+### Summary of Key Dates
+- **April 2026**: Submission of Program and Accelerator Technical Reports.
+- **June 2026**: Submission of the Portfolio Narrative.
+- **February 2026**: Quality assurance of reported results.
+- **Ongoing**: Bi-weekly updates and targeted info sessions throughout the reporting cycle.
+### Additional Resources
+For more detailed information, including guidance documents and templates, stakeholders are encouraged to visit the Performance and Results Hub, which serves as the central repository for all materials related to technical reporting.
+This structured approach aims to enhance the efficiency and effectiveness of the reporting process while ensuring that all stakeholders are well-informed and supported throughout the cycle.</t>
+  </si>
+  <si>
+    <t>The Performance and Reporting Management System (PRMS) is expected to open for reporting in **November 2025**. This timeline is still subject to confirmation, and updates will be provided as the date approaches. The aim is to ensure that users are informed well in advance of the official opening date for PRMS, allowing them to prepare accordingly.
+During the period leading up to the opening, users may have the opportunity to enter data in an editing mode, but the final submission will only be possible once the system is officially opened for reporting. This approach is intended to facilitate a smoother transition into the reporting phase and to allow users to gather and input their results effectively.
+For any further questions or clarifications regarding the PRMS or the reporting process, users are encouraged to reach out to the designated support channels provided by the CGIAR.</t>
+  </si>
+  <si>
+    <t>The technical reporting timelines for 2025, as outlined in the CGIAR Technical Reporting Arrangement (TRA) for the period 2025-30, include several key deliverables and deadlines that are crucial for the effective reporting of results and progress across various programs and accelerators. Here’s a detailed breakdown of the reporting timelines and expectations:
+### Key Reporting Timelines for 2025
+1. **Annual Technical Reports**:
+   - **Delivery of Program and Accelerator Technical Reports**: These reports are due by **April 2026**. Each program and accelerator is responsible for drafting and internally validating their reports, which will provide assurance on annual delivery against the Plan of Results and Budget.
+   - **Delivery of the Portfolio Narrative**: This overarching narrative report is expected to be delivered by **June 2026**. It will synthesize the contributions of various programs and accelerators to the CGIAR's strategic goals.
+2. **Quality Assurance Process**:
+   - The results reported will undergo a quality assurance (QA) process in **February 2026**. This process is essential to ensure the reliability and consistency of the reported data.
+3. **Integration of Projects**:
+   - The top **80% of Window 3 (W3) and bilateral projects** (by center portfolio value) are to be integrated into the Program/Accelerator Theory of Change, Monitoring, Evaluation, Learning, and Impact Assessment (MELIA) planning, and technical reporting. This integration is part of the phased approach to streamline reporting and enhance linkages across various reporting frameworks.
+4. **Minimum Data Standards**:
+   - The application of initial minimum data standards for W3 and bilateral reporting will be implemented, ensuring that the data collected meets the necessary quality and relevance criteria.
+5. **Engagement and Support**:
+   - Throughout the reporting cycle, there will be ongoing engagement with programs and accelerators through bi-weekly updates, targeted emails, and info sessions. These communications will provide guidance on key aspects of the reporting process and ensure that all stakeholders are informed and supported.
+### Additional Context
+- **Transition Year**: 2025 is designated as a transition year, which means that while the reporting processes are being streamlined, there may be some flexibility in how results are reported, particularly for W3 and bilateral projects. The focus will be on reporting against existing targets rather than introducing new metrics or requirements.
+- **Performance and Results Management System (PRMS)**: The PRMS will be utilized for reporting results, and it is expected to be opened for data entry in **November 2025**. This system will facilitate the tracking of results against plans and ensure that all reported data is accessible for quality assessment and integration into the overall reporting framework.
+### Conclusion
+The technical reporting timelines for 2025 are structured to enhance the efficiency and effectiveness of reporting within the CGIAR framework. By focusing on integration, quality assurance, and stakeholder engagement, the CGIAR aims to provide a comprehensive view of its contributions to global agricultural research and development. Stakeholders are encouraged to stay engaged through the Performance and Results Hub, which will serve as the central repository for all reporting materials and updates.</t>
+  </si>
+  <si>
+    <t>**Impact** refers to the significant and lasting changes that result from specific interventions, programs, or activities. In the context of research and development, particularly within organizations like CGIAR (Consultative Group on International Agricultural Research), impact is often assessed to understand how research outputs and innovations affect people, communities, and environments over time.
+### Key Aspects of Impact:
+1. **Definition**: Impact is defined as a durable change in the condition of people and their environment brought about by a chain of events or changes in how a system functions, to which research, innovations, and related activities have contributed. This can include improvements in agricultural productivity, poverty reduction, enhanced food security, and environmental sustainability.
+2. **Impact Assessment (IA)**: This is a systematic process used to evaluate the effects of an intervention. It estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. IA goes beyond mere monitoring of indicators; it seeks to establish a causal link between the intervention and observed changes, often employing both quantitative and qualitative methods.
+3. **Types of Impact**:
+   - **Direct Impact**: Immediate changes resulting from an intervention, such as increased crop yields from a new agricultural practice.
+   - **Indirect Impact**: Broader changes that occur as a result of direct impacts, such as improved nutrition and health outcomes in a community due to increased food availability.
+   - **Long-term Impact**: Sustained changes that persist over time, such as shifts in agricultural policy or practices that lead to systemic changes in food systems.
+4. **Measurement**: Impact is typically measured using a combination of methods, including:
+   - **Quantitative Methods**: Such as randomized controlled trials (RCTs), surveys, and statistical analyses to quantify changes and establish causality.
+   - **Qualitative Methods**: Including interviews, focus groups, and case studies to gather in-depth insights into the experiences and perceptions of stakeholders affected by the intervention.
+5. **Importance of Context**: The impact of an intervention can vary significantly based on the local context, including socio-economic conditions, cultural factors, and environmental circumstances. Therefore, impact assessments often need to be tailored to specific settings to accurately capture the effects.
+6. **Attribution**: A critical aspect of impact assessment is establishing attribution, which involves isolating the contribution of a specific intervention to the observed changes. This can be challenging, especially in complex systems where multiple factors influence outcomes.
+7. **Learning and Adaptation**: Impact assessments not only serve to evaluate the effectiveness of interventions but also provide valuable insights that can inform future programming and policy decisions. They help organizations learn from past experiences and adapt their strategies to enhance effectiveness.
+### Conclusion:
+Understanding and measuring impact is essential for organizations involved in research and development, as it helps demonstrate the value of their work, informs stakeholders, and guides future initiatives. By systematically assessing impact, organizations like CGIAR can ensure that their interventions lead to meaningful and sustainable changes in the lives of people and the health of ecosystems.</t>
+  </si>
+  <si>
+    <t>In the context of technical reporting and the Results Framework, "impact" refers to the long-term, durable changes that occur in the conditions of people and their environments as a result of specific interventions, research outputs, or innovations. This concept is crucial for organizations like CGIAR (Consultative Group on International Agricultural Research) as they aim to demonstrate the effectiveness and value of their research and development efforts.
+### Understanding Impact in Technical Reporting
+1. **Definition of Impact**:
+   - Impact is defined as the significant and lasting changes that result from a series of events or interventions. It is the ultimate goal of research and development activities, reflecting how these efforts contribute to broader societal goals, such as poverty reduction, improved food security, and enhanced environmental sustainability.
+2. **Impact vs. Outcomes**:
+   - While "impact" refers to long-term changes, "outcomes" are the intermediate effects that occur as a result of outputs. Outcomes can include changes in behavior, knowledge, or skills among stakeholders, which are necessary precursors to achieving the desired impacts. For example, an outcome might be an increase in the adoption of a new agricultural practice, while the impact would be the resulting increase in farmers' incomes over time.
+3. **Linkage to the Results Framework**:
+   - The Results Framework is a structured approach that outlines how specific activities lead to outputs, outcomes, and ultimately impacts. It provides a roadmap for tracking progress and measuring success. In the context of CGIAR, the Results Framework aligns with the Sustainable Development Goals (SDGs) and includes various impact areas that the organization aims to address.
+4. **Indicators for Measuring Impact**:
+   - To assess impact, organizations use specific indicators that are designed to measure the extent of change. These indicators should be SMART (Specific, Measurable, Achievable, Relevant, Time-bound) to ensure they effectively capture the nuances of impact. For instance, an indicator might measure the number of people lifted out of poverty due to improved agricultural practices.
+5. **Impact Assessment**:
+   - Impact assessments are systematic evaluations that aim to determine the causal effects of interventions. They often employ both quantitative and qualitative methods to provide a comprehensive understanding of how and why certain changes occur. This process helps in attributing observed changes directly to the interventions made by CGIAR.
+6. **Reporting and Accountability**:
+   - Technical reporting focuses on providing evidence of impact to stakeholders, including funders and partners. It is essential for accountability and transparency, ensuring that the contributions of CGIAR are clearly communicated and understood. The reports synthesize data from various projects and initiatives, highlighting successes and areas for improvement.
+7. **Continuous Learning and Adaptation**:
+   - The process of measuring impact is not static; it involves continuous learning and adaptation. Feedback from impact assessments can inform future strategies and interventions, allowing CGIAR to refine its approaches and enhance its effectiveness in achieving desired outcomes.
+### Conclusion
+In summary, "impact" in the context of technical reporting and the Results Framework is a critical concept that encapsulates the long-term changes resulting from research and development efforts. It is essential for organizations like CGIAR to effectively measure and report on these impacts to demonstrate their value and ensure accountability to stakeholders. By linking impacts to specific indicators and employing rigorous assessment methods, CGIAR can provide a clear narrative of its contributions to global challenges, ultimately guiding future research and policy decisions.</t>
+  </si>
+  <si>
     <t>Information Session on 2025 Technical Reporting.pptx — slide 9 — pptx:Information Session on 2025 Technical Reporting.pptx:s9, Engagement Plan 2025 Technical Reporting.docx — paragraph 2 — docx:Engagement Plan 2025 Technical Reporting.docx:p2, Information Session on 2025 Technical Reporting.pptx — slide 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s2, Guidance on reporting outputs or outcomes.docx — paragraph 22 — docx:Guidance on reporting outputs or outcomes.docx:p22, Engagement Plan 2025 Technical Reporting.docx — section 'Technical Reporting questions' — docx:Engagement Plan 2025 Technical Reporting.docx:p59, CGIAR_ImpactReport_2022-24.pdf — page 1 — pdf:CGIAR_ImpactReport_2022-24.pdf:p1, Engagement Plan 2025 Technical Reporting.docx — section 'A single location for all documents and resources' — docx:Engagement Plan 2025 Technical Reporting.docx:p31, Engagement Plan 2025 Technical Reporting.pptx — slide 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1, CGSpace.docx — section 'CGSpace' — docx:CGSpace.docx:p3, CGIAR-Technical-Reporting-Arrangement-2025-30.pdf — page 5 — pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5</t>
   </si>
   <si>
@@ -899,6 +1114,18 @@
   </si>
   <si>
     <t>Questions and Answers from Tech reporting info sessions.docx — paragraph 8 to paragraph 11 — docx:Questions and Answers from Tech reporting info sessions.docx:u7-10, https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1 — slide 1 part 4 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4, https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 9 part 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 9 part 4 — pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4, https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1 — slide 1 part 4 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4, https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 9 part 2 — pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2</t>
+  </si>
+  <si>
+    <t>https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e — page 1 part 2 — pdf:Portfolio Narrative_2024.pdf:p1pt2, https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 2 part 1 — pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1, https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0 — paragraph 1 to paragraph 7 — docx:General information on Technical Reporting .docx:u1-6</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 12 part 1 — pptx:Information Session on 2025 Technical Reporting.pptx:s12pt1, https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1 — slide 3 part 1 — pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt1, Questions and Answers from Tech reporting info sessions.docx — paragraph 48 to paragraph 50 — docx:Questions and Answers from Tech reporting info sessions.docx:u40-42</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1 — slide 3 part 3 — pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1 — page 10 part 3 — pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3, https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1 — page 18 part 3 — pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3</t>
   </si>
   <si>
     <t>[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]
@@ -2743,6 +2970,613 @@
 Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories</t>
   </si>
   <si>
+    <t>[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]
+Reporting timeline
+---
+[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4]
+Reporting
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2]
+Reporting High
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]
+Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]
+2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]
+information. Technical Reporting resources HOW Latest updates Timeline
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]
+2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)
+---
+[ID: docx:General information on Technical Reporting .docx:u1-6]
+General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2]
+course correction, while an annual MELIA report (December) documents how learning drives adaptive decisions and improved program performance. 7. Reporting The SFP MELIA plan includes a reporting structure that adheres to the CGIAR Technical Reporting Arrangement and ensures accountability, learning, and adaptive management across the Program. Reporting will be structured around the results framework (which has been aligned with the CGIAR Results Framework and Theory of Change (ToC) which also aligns with the PRMS ToC Board structure, encompassing High-Level Outputs (HLOs), intermediate outcomes, and 2030 outcomes and contributions to Impact Areas and SDGs . The reporting process will be aligned with the CGIAR Technical Reporting Arrangement, adhering to the annual reporting timelines, templates and Performance Results Management System (PRMS) requirements, including results of W3/bilateral projects mapped to SFP . Evidence for reporting will be
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u4-7]
+Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:04 5 minutes and then we will move into. I will leave the floor for your questions if that's OK. OK. Presentation mode. This means I no longer see the chat, the questions in the chat, or if hands are raised. So please interrupt me if you have questions or if you you know you you don't see the deck or anything else. I would like to welcome everyone and thank you for joining today's session on the 2025 Technical Reporting. My name is Nicoletta Trifa. I'm part of the Portfolio Performance Unit, a support unit within the Office of the Chief Scientist. This session is the second of two plan, two session plans for today, planned for today. We had an another session this morning to accommodate colleagues in other time zones. Um. Coming straight to the agenda, here's an overview of of what I'm going to cover in the next couple of minutes. So I will provide an update on the technical reporting arrangements. We'll discuss priorities and changes for 2025 technical reporting. A brief introduction on the annual Technical reports and the enablers, so being the Performance and Reporting Management System and the quality assurance, Technical reporting timeline, available resources and support and also what's what's next and how to stay engaged. This session marks the start of the conversation around 2025 Technical reporting. We want to give you the early look at the key priorities and plans for the months ahead. The goal is to make sure that you all stay informed, prepared and supported. With a clear understanding of deliverables and timelines that it is clear for you who to reach out to in case you have questions or in case you need help along the way. Some of the people in this call are already familiar with the technical reporting arrangements. From the previous portfolio, while for others this might be entirely new. Our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, with this let me kick off. So the technical reporting arrangements for the new portfolio, the 2025 to 2030 portfolio has been approved by CJRGLD, so Global Leadership Team in June 2025. And provides the operational basis to plan, monitor, learn and report on the new portfolio. It is designed to progressively enable programs and accelerators and centres to report on the pooled and the Window 3 Bilateral projects. In an aligned and integrated way without increasing reporting burdens on centers or on the scientist. Main changes compared to previous technical reporting arrangement. So the focus will be on streamlined reporting, less products, more integration, lower transaction costs, stronger impact focus results to be clearly linked. To impact outcomes and their associated indicator targets and also better linkages between the annual program and accelerator theory of change, final results and budget, media and technical reporting. The primary audiences for technical reporting are funders and CGR staff at the Integrated Partnership, Portfolio and Program and Accelerator levels. A secondary audience is the partners. The Annual Technical Reporting covers the program and Accelerators Annual Technical Reports and the Portfolio Narrative report, which provides an overall view to thematic and geographic targets. Relevant components of the technical reporting products are also integrated into the CGR corporate reporting, so CGR annual report. 2025 priorities for technical reporting. So 2025 is a transition year. I believe everyone has a line on this being a transition year with the technical reporting arrangements, implementation focusing again as I mentioned on streamlined reporting. And also on strengthening linkages between the theory of change, the poor media and technical reporting. Many of you know are aware that. These components were not properly linked in the previous portfolio, so it was challenging to demonstrate progress against plans against theory of change. In terms of deliverables for 2025, these are the program and the accelerator technical reports which are due in. April 2026 A Portfolio Narrative report which is due in June 2026 Integration of top 80% window 3 bilateral projects by center and dollar value into technical reporting and planning. Application of the minimum data standards for window 3 and bilateral reporting and mapping refinement which will take place during reflect early Q12026. So as I was mentioning 2025 transition year toward KPI based planning and reporting. So efforts are underway to enable planning and reporting at the KPI level and this is aligned with the System Office objectives and key results for 2026 and 20. 2027 I've listed them here on the slide, but be mindful that these are to be confirmed, so not confirmed yet. So uh for 2026 OK Rs. 100 of Program Accelerator. PRBS and the Annual Technical Reporting starting with the 2026 will provide monitoring of performance and result against Smart KPIs by center, by year, by pooled fund invested. So for 2026, the aim is to have 80% of centers, window free and bilateral projects included in 2025 Technical reports, while for 2027 this will increase to 90% of center window free and bilateral projects included in 2026. Technical reports. Yep. Specifically for programs and accelerators deliverables, here the focus is on three key deliverables. So first one being reporting the 2025 results in the Performance and Reporting Management System, the PRMS. Programs and accelerators are strongly encouraged to report results that were planned and budgeted, so included in their PORB, since the technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of the reported reported results. The 2025 results will be quality assessed following a defined process and timeline. Once this is done, the quality assessed results will be available on the Results dashboard and it will also be available for you to inform, pause and reflect. And to fill into your technical reports and to your annual technical reports. A third deliverable is drafting and submission of the 2025 Annual Technical Report. So each program and accelerators is responsible for drafting and internally validating quality assessing their. Annual Technical Report before submitting it to to us to the PPU. To support this process, this year we will have an AI generated V0 draft of this report which will include pre-filled text, some narrative and analytics for each report section. And this will be available for you as a starting point to further refine and and finalize your annual technical report. On the three deliverables, I want to mention that we will plan in September, October specific info session. So there will be info session on PRMS. Like a deep dive on PRMS, there will be a deep dive on quality assurance and the process timeline, who does what and so on, and also a deep dive on the Annual Technical Report to further make you familiar with its content, the internal approval process. The external approval process, I mean by external, I mean outside of program and accelerator approval process, what will be available, where AI will help and so on. So more information on this will come. For the annual technical report, what are these? These reports provide assurance on the annual program and accelerator delivery against PORP and progress on theory of change. They are short, concise and targeted. They are based on the quality assess results. The requirement is to have this report submitted in April and then the aim is to publish them early May as I was mentioning template guidance and and. A I generated V0 report will be will be provided to You to the right on the right side of the screen You can see that the content areas of the annual Technical report. This is extracted from the Technical reporting arrangements document and IT has it's very similar to what we had for the initiatives and impact platforms in the previous portfolio. So You have a fact sheet, an executive summary, annual progress area for work details. A Results section, Partnerships, Portfolio Linkages, Adaptive Management and then Key Results story. For reference or especially for for People new to Technical reporting, which who want You to have a look at, You know how this this reports might look like in the end. I've I've pasted here the. Annual reports from initiatives, impact platforms and science Group projects from 2024, SO from this year and You also have a link to the Portfolio narrative report. And the Type 2 report, sorry, the Type 2 impact report, which is drafted every three years. The System where this will take Place with reporting will take place. It's called Performance and Results Management System, PRMS in short. We are currently validating the PRMS roles, SO we have reached out to Program Coordinators and asked them to. Give us the name and the role of the People in their teams which will be involved in Technical reporting. A reminder on this will be sent on Thursday to finalize the process and this will enable the Technical Team to. Create proper accesses in the System when the reporting period starts. Similar to previous information, SO we are working to to to draft the new users onboarding deck where You can find relevant information on PRMS and. We will keep You updated on what's new in the pyramids or on the enhancements that we're working on this year as we advance towards Technical reporting to the reporting period later in the year. Quality assurance process what IT is. So Results submitted by programs and accelerators in the PRMS are quality assessed by QA Team in February 2026. Your participation in this process is required. Guidance and resources will be provided and then also as I was mentioning, an info session will be scheduled for September, October. What is QA? It is a process that aims to improve the quality of reported data, to provide consistency across the system, to ensure reliability of reported results, inform learning, and overall improve CGR accountability and transparency. Quality assessed data, SO the Results quality assessed inform the reflect process. They Go into the Results dashboard. They are also featured in the annual reports in the Portfolio narrative and then further into the CJR corporate report. And oh, there's I I only noticed now the title says 2024. Apologies for this. It's 2025 Technical reporting timeline. This is a print screenshot of. Same information that can be seen on the PNR hub. So we have the first info session on Technical reporting now in July, August through November. We will engage Program accelerators and centers, media People in preparation of. Various guidance materials, testing, PRMS enhancement. We'll plan information sessions which will take Place in September, October to make sure that we everyone is properly prepared for the reporting period. Reporting 2025 results. Our intent is to open PRMS in November. Let's see how how well we advance with the changes to the System again 2025. Is a Transition year. There are many changes to be done since we moved from 1 Portfolio to another, many adjustments which need to take Place in the system, but hopefully in November we can open reporting on 2025 results. We will keep You updated on this though. Quality assurance will take Place as mentioned in February 2026. Reflect same thing will take Place in Q 1/20/26. And then the annual Technical reports are due in in April, in March, April for publication early May. The Performance and Results Hub is your one-stop shop for planning, Technical reporting and managing information. You'll find I want to stop sharing this deck for now and I want to. Take You to the PNR hub. Let me know if You see when I switch screens. Rose, Sabrina ( Alliance Bioversity-CIAT) 16:48 Yes, we can see. Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3]
+System (PRMS) Quality Assurance When Technical Reporting timeline How Resources Engagement
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]
+2025 Technical Reporting Portfolio
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u13-16]
+The Performance and Results (P&amp;R) Hub will serve as the central repository for all materials related to Technical Reporting. This includes timelines, guidance documents, templates, updates, frequently asked questions (FAQs), and other relevant resources to support Programs and Accelerators throughout the reporting cycle. The Hub is structured around key phases of the reporting process, with dedicated pages for planning, reporting, and reflect/re-planning, making it easier for users to find what they need at each stage. The content and structure of the P&amp;R Hub have been reviewed and updated based on: Changes to the Technical Reporting process
+---
+[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]
+Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u4-7]
+Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:03 Will be available on the Performance and Results Hub later today and also will be shared by e-mail by the end of this week. Good. OK, so we can start. Welcome everyone. Thank you for joining today's session on the 2025 technical reporting. I'm going to share my screen. As I was mentioning, I have a couple of slides I want to share with you. She moved. I do not see the chat or hands raised or anything, so please let me know if you get if you can see my slide. Colomer, Julien (One CGIAR - France) 0:47 Yep. Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports ar</t>
+  </si>
+  <si>
+    <t>[ID: pdf:Portfolio Narrative_2024.pdf:p1pt2]
+2024 Technical Reporting 2024
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]
+Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What
+---
+[ID: docx:General information on Technical Reporting .docx:u1-6]
+General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1]
+2024 Technical
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]
+information. Technical Reporting resources HOW Latest updates Timeline
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]
+2025 Technical Reporting Portfolio
+---
+[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3]
+defined in the 2024 Technical Reporting Guidance are listed below. An
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3]
+Technical Reporting Arrangement 2025-30 Results
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1]
+2025 Technical reporting priorities (transition year) The TRA will be implemented through a phased approach, with the first phase focusing on streamlined reporting and stronger linkages across Program/Accelerator ToCs, PoRBs, MELIA and technical reporting. Key deliverables in this initial phase include: Delivery of 2025 Program and Accelerator Technical Reports by April 2026. Delivery of the 2025 Portfolio Narrative by June 2026. Integration of the top 80% of W3 and bilateral projects (by Center portfolio value) into Program/Accelerator ToC, MELIA, PoRBs, and Technical Reporting. Application of the
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1]
+Information Session on 2025
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]
+2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)
+---
+[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]
+Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]
+Reporting timeline
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]
+2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2]
+report is available here The 2024 Initiatives, Impact Platforms and Science Group Projects annual technical (Type 1) reports are available here WHAT Annual Technical Reports provide assurance on annual Program/Accelerator delivery against PORBs and
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u52-55]
+Additional emails will be sent out from this email address with any time-sensitive information. Info-sessions A limited number of targeted info-sessions will be held to provide focused guidance on key aspects of the 2025 Technical Reporting process, and will be timed to align with critical points in the reporting timeline. Each session will include a short presentation followed by time for questions and discussion. Invitations and materials will be circulated in advance, and recordings will be made available for those unable to attend live. Monthly drop-ins
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3]
+to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3]
+to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]
+2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]
+Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]
+2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción
+---
+[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]
+Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1]
+Technical Reporting Arrangement (TRA) 2025-30 Approved by the CGIAR Global Leadership Team on 5 June 2025, provides the operational basis to plan, monitor, learn, and report on the 2025-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled and W3/bilateral projects of the 2025-30 portfolio in
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u4-7]
+Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process. Lessons from previous reporting cycles have highlighted the importance of timely, clear, and responsive support to reporting teams. Building on the progress made in recent years, this document outlines a plan to further streamline and optimize communication and engagement mechanisms for the 2025 reporting cycle. Objective
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2]
+results that were planned and budgeted, as the updated technical reporting system will allow for tracking results against plans. QA of reported results 2025 Results will be quality assessed following a defined process and timeline. QA’ed results will be available on the CGIAR Results
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u1-4]
+Engagement Plan: Technical Reporting 2025 Background Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process.
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]
+Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u7-10]
+Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source. Colomer, Julien (One CGIAR - France) 23:53 Nicoletta, maybe I can just say a few words about this one. Thanks. Thanks so much, Nicoletta, for the presentation so far. So the dashboard here is just a a working version. Obviously we can develop a much more polished version. However, at this stage it's going to be sort of a portfolio Explorer. Trifa, Nicoleta (CGIAR System Organization) 23:54 Go ahead. Yes, yes. Mm. Colomer, Julien (One CGIAR - France) 24:11 So really internally facing and the idea is to consolidate all relevant types of information that we can, you know, make available about the portfolios, the program and accelerator result frameworks, Melia studies, I think we'll try and get the proposal inception reports. You know, whatever else we can get on there, that's really to allow you to coordinate with other programs and accelerators. So we'll keep building this out. And yeah, as mentioned, so this is an internally facing dashboard. And we'll keep improving it over time and eventually we'll put it on the Performance and Results Hub. But for the moment, if you wouldn't mind having a poke through and making sure everything looks as good as it should, the two geographic tabs there map and removed and inception just to give we were asked to have a look. At proposal versus inception geographic footprint. So we've done that. Again, those both the proposal and the inception didn't have a, let's say a very strong geographic component. So that that one is probably the diciest I would say in terms of the data quality and completeness, but please do have. Have a look and let us know if you spot anything. Thanks very much.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]
+reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2]
+reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u7-10]
+Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording</t>
+  </si>
+  <si>
+    <t>[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s12pt1]
+PRMS
+---
+[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt1]
+PRMS
+---
+[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u40-42]
+PRMS access Q: When will our role in PRMS change? When I log in, it shows my role in the Initiative? A: You will be able to see your new role assigned to the specific Program/Accelerator once the 2025 reporting phase opens in PRMS.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s8pt3]
+in the PRMS will be quality assessed (QA) by a QA team in February 2026. Your participation in this process is required. Guidance and resources will be provided.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s13pt2]
+on 31 July. Targeted engagement calls for PRMS testing. Info sessions on specific topics (e.g. QA,
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt1]
+PRMS Reporting Tool PRMS
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt2]
+PRMS REPORTING TOOL PRMS
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt3]
+PRMS roles PRMS resources:
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]
+2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u55-58]
+Monthly drop-ins To provide ongoing, accessible support throughout the reporting period, monthly drop-in sessions will be held via Microsoft Teams. These informal sessions will offer Programs and Accelerators the opportunity to raise questions, seek clarification, and engage directly with PPU/PCU. No formal presentations will be given; instead, the focus will be on open dialogue and timely support. Invitations and calendar holds will be shared in advance, with reminders included in the regular update emails. PRMS enhancements and feedback process The PRMS Reporting Tool is continuously improved in response to user needs and feedback. The update process follows these steps:
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4]
+Resources Engagement plan Process for PRMS enhancements What next Upcoming activities
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u49-52]
+Trifa, Nicoleta (CGIAR System Organization) 43:52 Other questions, comments. No, good. Again, we will paste the link to the deck and to the meeting recording and share with you by e-mail. Be available. This will be available on the PNR Hub as well. So if there are no other questions or comments, I want to thank you all for your participation to this session. Yeah, don't hesitate to reach out to us. OK, I see a question there. When does the PRMS open for reporting? This is to be confirmed, Raja. Again, we're aiming for November. It's, you know, we will inform you the closer we get to the date about the the final official. Opening date for PRMS. Thanks everyone. Have a wonderful day. Colomer, Julien (One CGIAR - France) 44:46 Thank you, Nicoleta. Thanks everybody. Ciao. Bye, bye. Trifa, Nicoleta (CGIAR System Organization) 44:47 Bye. Aryal, Bishal (IFPRI) 44:47 Thank you. Thank you.
+---
+[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]
+Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]
+Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u58-61]
+The PRMS Reporting Tool is continuously improved in response to user needs and feedback. The update process follows these steps: The Sounding Board will consist of representatives from: PRMS Team PCU Team
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u10-13]
+Marshall, Karen (ILRI) 25:21 Yeah. Hi, everybody. And thank you for that great update. Just a question, whilst PRMS is being sort of, I think you said streamlined or updated August to November, can we also put results into the system during that time because? You know, a start date from late November, December will will be too late for us. Trifa, Nicoleta (CGIAR System Organization) 25:43 So have them in editing mode. You mean like not submit them just. Marshall, Karen (ILRI) 25:45 Yes, yes. Because I was really hoping that by August we could start putting things into PRMS because you, you know, it would be, we don't want to have like a long period of upgrading PRMS and then very short time for us to to actually put things in there. Yeah. So if we could actually be putting them in where we're tweaking it, that would be very useful or. Trifa, Nicoleta (CGIAR System Organization) 25:48 Yeah.
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p16pt3]
+Target users of the PRMS include CGIAR staff for day-to-day Initiative management and reporting, portfolio management and resource mobilization , and Funders and partners to access evidence of CGIAR thematic and geographic presence and progress against stated objectives such as the SDGs. Security, hosting, maintenance and support The PRMS will incorporate:
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt3]
+critical process for both internal and external communication, ensuring accountability, transparency, and progress tracking. It facilitates decision -making, supports adaptive management, and communicates Program/Accelerator achievements to stakeholders. Relevant information from Program Results Frameworks will be integrated into the PRMS Reporting tool from the PRMS ToC Board to facilitate the
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p23pt4]
+program learning as well as the refinement of the Theory of Change during the annual “Pause and Reflect” sessions. These sessions will also contribute to the overall annual reporting procedures. To facilitate results reporting within the PRMS framework, each Area of Work (AoW) will appoint designated focal persons who will collaborate with the Monitoring, Evaluation, and Learning (MEL) team to upload pertinent r esults and supporting evidence. A comprehensive checklist, in alignment with PRMS metadata requirements, will be employed to guide and standardize the reporting process.
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt3]
+has been developed in the PRMS TOC Board and updated to
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt3]
+and accessible Performance &amp; Results Management System (PRMS) that encompasses planning, monitoring, and reporting will provide robust information upon which to take informed decisions. It will provide: • Practical services aligned to meet learning, accountability and resource mobilization objectives, • Dashboards open to Funders and partners, with access to the full set of underlying quality-checked data , including communications-focused products capturing collated evidence of CGIAR contribution to change (e.g. outcome/impact case reports). • Alignment with international standards such as IATI (International Aid Transparency Initiative). Key PRMS features The CGIAR PRMS will feature: • A common system housing plan of work and budget, theory of change management, stage-gate decision points, and annual reporting processes. It will allow real- time
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p21pt3]
+to guide consistent and credible reporting into the PRMS system. Key elements include: • Use of standardized data collection tools • Training and calibration of enumerators or field staff • Spot-checks and validation missions by MELIA or AoW focal points • Automated consistency checks in digital entry platforms (if used during the program implementation) • Clear metadata documentation for each indicator • Peer review or AoW lead/Director sign-off before data submission (especially at outcome level) 5. Contingency Plan for Data Collection Risks To address potential disruptions, the program will maintain a risk mitigation table that is regularly updated. Initial measures include: Risk Potential Impact Mitigation Strategy Budget constraints Incomplete
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u34-37]
+All questions and comments on Technical Reporting should be sent via email to performanceandresults@cgiar.org. For technical questions related to using the PRMS Reporting Tool, emails should be sent to prmstechsupport@cgiar.org. PPU/PCU will endeavor to reply to queries as soon as possible; please note that delays are usually due to ensuring that responses have been reviewed and align with the latest updates and guidance. Responses will also be posted in real time on the P&amp;R Hub for wider reference. Fortnightly update emails To ensure transparent and regular communication throughout the reporting cycle, a centralized update mechanism will be used.
+---
+[ID: docx:Using the PRMS Reporting Tool.docx:u7-9]
+Yes. The PDF function is always available. The system will generate the PDF with the information that you have entered when you press the button, even if the result entry is not fully complete at the time. What should I do if I encounter a bug in the PRMS Reporting Tool? Please ensure you create technical tickets for the bugs you encounter by sending an email to prmstechsupport@cgiar.org. This will help the PRMS team to track requests and prioritize them.
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4]
+the PRMS Reporting tool from the PRMS ToC Board to facilitate the reporting and evidencing of achievement of both output and outcome indicator targets, as well as links to MELIA studies as sources of evidence. Further details on Technical Reporting processes, products and support will be shared in 2025.
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u49-52]
+PRMS Team PCU Team PPU Team Additional emails will be sent out from this email address with any time-sensitive information.
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt3]
+outlines the types of reports required at diƯerent time intervals. It also aligns with the CGIAR Technical Reporting Arrangement (TRA) 2025–30 (in draft), which standardizes reporting processes and ensures coherence across funding streams. An updated PRMS Outcome Indicator Module will be used to report
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt2]
+criteria: Based on past results plus projected costs and development impact (considerations could include ToC, QoR4D, Scaling Readiness , risk assessment, portfolio risk/reward profile review, Gender in research &amp; Gender, Diversity and Inclusion). Stage-gate delivery and use A Performance and Results Management System (PRMS) will be used to collect relevant data and make it available for use in CGIAR, Action Area, Initiative and component management, including stage-gate decisions. 7. Performance and results management system Building on investments made in the current phase of CGIAR research programming, a comprehensive, mature and accessible Performance &amp; Results Management System (PRMS) that encompasses planning, monitoring, and reporting will provide robust information upon which to take informed decisions. It will provide: • Practical
+---
+[ID: docx:Submitting evidence.docx:u16-19]
+You confirm that all intellectual property rights related to the file have been observed. This includes any rights relevant to the document owner’s Center affiliation and any specific rights tied to content within the document, such as images. You agree to the file link being displayed on the CGIAR Results Dashboard. If you indicate that the file being uploaded to the PRMS is NOT public: You confirm that the file should not be publicly accessible.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3]
+System (PRMS) Quality Assurance When Technical Reporting timeline How Resources Engagement
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p57pt4]
+Tomorrow.indd 57 08/08/2025 16:0208/08/2025
+---
+[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p86pt4]
+Tomorrow.indd 86 08/08/2025 16:0208/08/2025 16:02
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p21pt2]
+not only results, but also key decisions, implementation challenges, and signals of change as they emerge. Data submission will occur on a rolling basis, supported by automated quality checks and centralized review from the MELIA and Program management teams. Quarterly validation and entry into the PRMS system will help maintain momentum and avoid year-end data backlogs, while also enabling continuous insight generation. In line with CGIAR’s Open and FAIR Data Assets Policy, databases generated by research teams will be managed by those teams
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u22-25]
+Trifa, Nicoleta (CGIAR System Organization) 30:25 Mhm. And safe, this is exactly what we're aiming to do this year. So in August in two weeks to three weeks, the the intent is to share with you the PRMS data fields by indicator categories of innovation, policies, capacity sharing and so on. So you know exactly what data fields. Will be capturing PRMS when reporting will open, so you could use those documents to to inform you when gathering information on on your results. And secondly, and Nico also mentioned in the chat here. The intent is to apply the same logic we apply to the out communicator module from the get go, so from the reporting. So we if last year we had that special module at the end of reporting to link results to targets. This will happen now from the get go, so when you enter results you will be asked to link your result to your plans. To your targets. So I hope this answer your question safe, Karen. Marshall, Karen (ILRI) 31:47 Yeah, I I just want to come back to what Enrique said. And Enrique, I really understand that there's quite a lot of, you know, effort and and time put into updating PRMS and it's really getting better every year. But I mean the the problem that happens is that things take long and then we as a scientist are set with a fixed date and we get squeezed to get everything in because. That. It can't be moved because the reports are dependent on it, you know, an ISDC date. So I mean, maybe one way to say is we need so much time for reporting. Yeah, let's say we open it in mid-october or September if we could. Wherever PRMS is there is where it is, yeah, because it cannot be always the people doing the reporting who are the ones who ultimately get squeezed. So I think, you know, really in the initiatives there was, you know, I really had a sense that everything was done from one side and I took the time and then we were just stuck with whatever time was left. It should be the other way around really the people reporting, you know, so let's maybe consider making a deadline saying this is when the reporting has to open, where Pyramus is, is, is where it is. Yeah. Bonaiuti, Enrico (CIP-ICARDA) 32:49 Yeah, yeah, I mean maybe 11 aspect Karen and my reflection the fact of flipping a bit the PRMS using the experience of the outcome module. So you you see first your targets should in theory let programs focus first on. Trifa, Nicoleta (CGIAR System Organization) 32:50 Thanks, Karen.
+---
+[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt3]
+activated only during scheduled meetings and closed immediately after. performanceandresults@cgiar.org is the official communication channel. Full engagement plan available via the P&amp;R Hub and here: Full
+---
+[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u4-7]
+A: The deadline depends on the type of results being reported: Pooled results (reported by P/A under W1/W2 funding): must be submitted by end of January 2026. These results undergo a quality assurance (QA) process in February 2026. W3/bilateral results: since these do not go through QA, they can be reported in PRMS until late February 2026. Governance:
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt2]
+also needs to be verified to maintain quality control and reference relevant documentation for evidence. The PRMS system will be used currently to store and maintain the data collected. Reported HLOs and Intermediate Outcomes from AoWs will be quality checked through the internal review process within AoWs before reporting to the PRMS system. Data repositories will be created and maintained at the AoW level to ensure evidence preservation. Data and reporting on HLOs from bilaterals will be checked by Center delegates for the Program for quality assurance. Data will be cross -checked and validated at the Program level during reporting period. The Program MELIA lead will work closely
+---
+[ID: docx:2025 Technical Reporting Information (Session 2).docx:u46-49]
+Colomer, Julien (One CGIAR - France) 42:25 So that they also understand, you know how how things work. Now there's 1000 plus active grants, 500 new ones already since November. So that's a lot of onboarding sessions. Perhaps what we need is a set of materials that can be shared and accessed easily like a recording and and stuff like that. So I think we'll look. For the most scalable low cost solution that helps people you know understand what we do and perhaps for the for the program and accelerator directors once they come on board then we have the in person you know live one and then for the new projects they get the recorded one, something like that. But it's a it's a good idea. Yeah. Thanks. Trifa, Nicoleta (CGIAR System Organization) 43:04 Good idea. We, as I was mentioning, we are making a drafting a PRMS new user deck if you want. So it's two or three slides with relevant information on PRMS like the access, the roles, guidance on how to report, who needs to report when and so on. So that will be available soon on the PNR Hub. And we will notify you once that's available. So feel free to disseminate that to, you know, colleagues from Windows 3 bathroom projects which have a role in providing information, technical reporting, if not, you know, actually reporting in the system. Nirmal, Rajalakshmi (IFPRI) 43:44 Thanks. Trifa, Nicoleta (CGIAR System Organization) 43:52 Other questions, comments. No, good. Again, we will paste the link to the deck and to the meeting recording and share with you by e-mail. Be available. This will be available on the PNR Hub as well. So if there are no other questions or comments, I want to thank you all for your participation to this session. Yeah, don't hesitate to reach out to us. OK, I see a question there. When does the PRMS open for reporting? This is to be confirmed, Raja. Again, we're aiming for November. It's, you know, we will inform you the closer we get to the date about the the final official. Opening date for PRMS. Thanks everyone. Have a wonderful day.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt4]
+(PPU) 29 July 2025
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1]
+CGIAR Technical Reporting Arrangement 2025-30 June
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_Inception Report 30-06-2025.pdf:p1pt2]
+Program Inception Report June 2025 Contact: Interim
+---
+[ID: docx:User Roles and Rules for the PRMS Reporting.docx:u1-4]
+User Roles and Rules for the PRMS Reporting Tool Roles: Roles define the level of responsibility and permissions a user can have within the PRMS. They determine the role a user has in the submission of results and data management within PRMS, ensuring consistent governance, accountability, and clarity of access across Portfolio (or reporting entities – whichever version you plan to use from now on). Lead and Co-Lead:
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt4]
+An updated PRMS Outcome Indicator Module will be used to report results that evidence the achievement of outcome indicator targets. MELIA studies will contribute to this module and support reporting. Further details on Technical Reporting processes, products and support will be shared in 2025.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt3]
+during scheduled meetings and closed immediately after. performanceandresults@cgiar.org is the official communication channel. Full engagement plan available via the P&amp;R Hub and here: Full engagement plan.
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p1pt4]
+Security Science Program June 2025
+---
+[ID: pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p1pt2]
+April 2021 (Decision reference SB/M19/EDP3). This Policy supersedes and replaces in its entirety the 2013 Open Access and Data Management Policy. It
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p3pt2]
+Transition Consultation Forum, and public consultation feedback received from 28 commentators including CGIAR funders, partners and staff. 2. Introduction This Performance and Results Management Framework (PRMF) describes the processes, systems and measures for managing CGIAR’s performance and results . This will support delivery of the CGIAR 2030 Research and Innovation Strategy. The PRMF is designed to sup port an organizational culture and processes which encourage innovation, deliberately nurture learning and elevate emerging areas of promise. It will help teams to monitor, learn and adapt their Initiatives over time to best navigate towards impact, support leaders to allocate resources towards workstreams with
+---
+[ID: pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p1pt4]
+Director: P.Coaldrake@CGIAR.org Interim Program Manager:
+---
+[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u46-49]
+CGSpace Team Lead KM Managers Curators/Repository Managers PRMS Team
+---
+[ID: pdf:Type3_2024Report.pdf:p11pt4]
+System (PRMS): The PRMS serves as the central reporting platform, powering the Results Dashboard and supporting the development of Type 1 Reports with real-time data aggregation and analysis. These components were instrumental in driving the 2024 Technical Reporting process, and key elements will be carried forward to shape Technical Reporting in the next CGIAR Portfolio, ensuring continuity, alignment, and continuous improvement. Monitoring tools tailored to suit core indicators Non-pooled projects Type 1 Type 3 Science Group Projects Research and Performance and Results Management Framework Arrangement CGIAR Results Framework Standard Indicator Theory of Change and Scaling Readiness (IPSR) Quality Assurance criteria, process Performance and Results Management System Type 2 Triennial Outcome/Impact Report Annual Technical Report Results Dashboard $771M Revenue 2% 23% 44% 31% Revenue by Funding Source Windows 1&amp;2 | Window 3 | Bilateral | Other 1 2 3 4 5 6 7 8 9 10 13 12 11 6. CGIAR 2030 Research and Innovation Strategy 7. Performance and Results Management Framework 8. Technical Reporting Arrangement 9. CGIAR Results Framework 10. Standard Indicator Description Sheets: • Output level • Outcome level 11. Theory of Change 12. IPSR • Output level • Outcome level • IPM for responsible food systems transformation • Scaling Readiness website • Online course on Innovation and Scaling • Scaling Readiness calculator • Scaling Directory 13. Adaptive Management 14. Quality Assurance 15. PRMS &amp; TOC board 16. Results Dashboard 17. 2022 &amp; 2023 Annual Technical Reports 18. Type 2 report Grass pea production in Odisha. Credit: IRRI May 2025 17 16 CGIAR Portfolio Practice Change (Type 3) Report
+---
+[ID: docx:2025 Technical Reporting Information (Session 1).docx:u37-40]
+Colomer, Julien (One CGIAR - France) 42:29 Yeah, thanks. It's just maybe a couple of points there. So one is to Karen's point and just put it in the chat. But I just wanted to also like I I absolutely hear you, Karen, and I think it's good to recognize that over the period 22 to 24, I can't remember the exact state stat. But I think we more than doubled or maybe tripled the number of days that the PRMS was actually open for reporting. And our objective is to really have always on technical reporting so that there's, you know, full flexibility in terms of. Trifa, Nicoleta (CGIAR System Organization) 42:53 Hmm. Colomer, Julien (One CGIAR - France) 43:03 Uh, when the data is able to be entered and like the the period 22 to 24, Nicoletta, we can dig that stat out somewhere, but we've got it um, just in terms of the number of days it was open. Um, so that bit, yeah. Trifa, Nicoleta (CGIAR System Organization) 43:15 I can, I know them by heart. So if you want the first year was first year for initiatives, we start in December. So similar timeline, we had December, January, second year was October and then the third, the third year was July. So yeah, we increased that time.
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p16pt4]
+as the SDGs. Security, hosting, maintenance and support The PRMS will incorporate: • Secured infrastructure, • Cloud hosting, • CGIAR Active Directory integration for user provisioning and account management, • Access control through Multi-Factor Authentication, • Single Sign On, • Tiered support and maintenance approach aligned with CGIAR’s IT support model.
+---
+[ID: pdf:CGIAR Open and FAIR Data Assets Policy.pdf:p1pt1]
+CGIAR Open and FAIR Data Assets Policy Approved by the System Management Board with effect from 16 April 2021 (Decision reference SB/M19/EDP3).
+---
+[ID: docx:Guidance on complementary innnov.docx:u13-16]
+Within the PRMS, you can report complementary innovations/enablers/solutions under innovation packages -&gt; IPSR Innovation use pathway -&gt; Step 2: Innovation Packaging. First, existing complementary innovations/enablers/solutions can be selected from the list of existing innovations reported in the PRMS. If you have finalized adding existing PRMS complementary innovations enablers/solutions, then you can add additional complementary innovations/enablers/solutions manually by clicking on: You can then enter the relevant details:
+---
+[ID: pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt4]
+representatives in early January as part of the quality control process. Following this, the MELIA unit will send the compiled data, including progress and justifications, to the Accelerator Lead for internal approval before incorporation into the PRMS and Type 1
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt3]
+inform reporting outputs. Monitoring data recorded in PRMS will serve as the foundation for compiling evidence in formal reporting, including Annual Technical Reports and dashboard contributions . A periodic export will ensure we can monitor progress against planned targets. Final validation of monitoring data in PRMS will follow CGIAR System Office guidance and will support the Program’s reporting cycles. A dedicated 50% MELIA focal point will focus on outcome actors identification, assumption validation, and outcome monitoring. The program coordinator will ensure that at centralized level all MELIA responsibilities are following SO timeline. Dedicated scientists will instead lead or support the impact assessment work. The program recognizes the need to prioritize baselines for outcome indicators, as most HLOs will be newly developed and do not require a baseline. Baseline planning and data collection will be sequenced based on funding availability, focusing first on cri tical indicators related to early outcome targets. While
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]
+2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt1]
+Program and Accelerator MELIA Plan Update Template and Guidance I March 2025 10 most frequently used for collecting data on HLOs. Focus groups seem to be a recurring methos used by most AoWs to collect data around adoption and policy engagement concurring with the greater qualitative nature of such information. A lot of data also comes from regular meetings with partners and thus will be gathered continuously, but the annual cycle will be followed for most other data collection. Data collected also needs to be verified to maintain quality control and reference relevant documentation for evidence. The PRMS system will be used currently to store and maintain the
+---
+[ID: pdf:Digital Transformation_Inception Report 30-06-2025.pdf:p15pt2]
+will be collected annually. By the end of every November, all AoW leads will be informed and provided with a template outlining their targets, with a submission deadline at the end of December. The collected data will then be compiled
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p20pt2]
+exported in Excel format for review, as per guidance. HLOs represent results such as tools, guidelines, datasets, and tested solutions; outcomes represent the behavioral and systemic changes these outputs are expected to generate. We will use the CGIAR standard indicators for outputs (innovation development, capacity sharing and knowledge product) to measure progress towards the HLOs and for outcomes, we expect to use primarily the CGIAR standard indicators on policy change and innovation use. For the 2030 outcomes, specific indicators will be used. Monitoring efforts will be embedded into a results -based management approach, supported by the PRMS reporting platform. Progress will be tracked through regular data collection cycles to contribute to adaptive management and inform reporting outputs. Monitoring data recorded in PRMS will serve as the foundation for compiling evidence in formal reporting, including Annual Technical Reports and dashboard contributions . A periodic export will ensure we can monitor progress against
+---
+[ID: pdf:CGI21-507033-PORB-Policy Innovations.pdf:p8pt4]
+AoW3, 25% of time Jan-June X X AoW Transition Lead, AoW4, 25% of time Jan-June X X AoW Transition Co-Lead, AoW4, 25% of time Jan-June X X AoW Transition Lead, AoW5, 25% of time Jan-June X X AoW Transition Co-Lead, AoW5, 25% of time Jan-June X X AoW Transition Co-Lead, AoW5, 25% of time Jan-June X X AoW Transition Lead, AoW6, 25% of time Jan-June X X AoW Transition Co-Lead, AoW6, 25% of time Jan-June X X Workshop (Inception period meetings and related costs) X X Other (Support for Comms, MELIA work, others) X X Total AoW 11budget 466,359 CGI21-507033-PORB-Policy Innovations.indd 8CGI21-507033-PORB-Policy Innovations.indd 8 29/07/2025 18:5329/07/2025 18:53
+---
+[ID: docx:Submitting evidence.docx:u19-23]
+You confirm that the file should not be publicly accessible. The file will not be accessible through the CGIAR Results Dashboard. The file will be stored in the PRMS and will only be accessible by CGIAR staff (e.g. quality assurance assessors) with the repository link. Documents uploaded to the PRMS will be view-only and cannot be edited. Documents uploaded to the PRMS will be view-only and cannot be edited.
+---
+[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt4]
+PRMS will feature: • A common system housing plan of work and budget, theory of change management, stage-gate decision points, and annual reporting processes. It will allow real- time data collection and day-to-day portfolio and Initiative management. • Key data sets (results, plan of work and budget, grant, finance, stage -gate specific e.g. Scaling Readiness) will be increasingly linked, for example through CLARISA: CGIAR Level Agricultural Results Inte roperable System Architecture, a web service that harmonizes data from across the CGIAR). • Interface and exchange with b ig data and partner data sets (e.g. WIPO Green and the International Treaty on Plant Genetic Resources for Food and Agriculture ) will increase. CGIAR will publish relevant data through IATI.
+---
+[ID: docx:2025 Technica</t>
+  </si>
+  <si>
+    <t>[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]
+exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. Impact assessments are conducted after an intervention has been completed and are used to substantiate claims of sustained results. They seek to measure impact at scale, i.e., benefits to a large number of people/large areas of land. It employs both quantitative and qualitative methods, often combined for deeper insights. IA goes beyond monitoring indicators to evidenced attribution of observed changes to CGIAR interventions. IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives.
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3]
+Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framewo rk Provid e the assu mptio n(s) state ment from the Resul ts Fram ework Indicate the location( s) where the study will be conducte d Indicate the methods and design approache s that will be used for the study List the Progr am(s) and Accel erato
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p70pt4]
+Impact program to enhance farm productivity and mitigate environmental pressure, making agriculture more efficient, affordable, and sustainable. Credit: Abdul Momin, CIMMYT CGI21-508007-PORB-Scaling for Impact.indd 70CGI21-508007-PORB-Scaling for Impact.indd 70
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3]
+Impact assessment (IA) .............................................................................................................. 13 Program impact overview .................................................................................................................... 13 IA activities and collaboration plans ..................................................................................................... 14 IA studies ........................................................................................................................................... 15 5. Learning and adaptive management ........................................................................................... 16 Learning ............................................................................................................................................. 16 Annual review and adaptive planning ...................................................................................................
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2]
+and Impact Assessment (MELIA)
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3]
+and Impact Assessment (MELIA)
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p58pt2]
+on critically relevant topics. 3,250 6,646 1,708 3,528 3,001 6,709 1,200 1,661 554 2,542 2,500 1,233 2022 results 3,415 2023 results 6,275 2024 results 8,237 Total results 16,605 2 = Principal: Contributing to one or more aspects of the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. 0 = Not targeted: The result has been screened against the Impact Area, but it has not been found to directly contribute to any aspect of the Impact Area as it is outlined in the CGIAR 2030 Research and Innovation strategy. Figure 5.9. Overview
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1]
+Impact Area indicator quantification Given these limitations and opportunities, the Portfolio Performance Unit (PPU) commissioned subject matter experts for each Impact Area to review the Impact Area indicators and the aligned outcomes and impacts reported, with a view to assessing the feasibility of aggregating the reported results to inform on total progress toward the Impact Area indicators during the 2022 to 2024 period. This was very challenging, and partial quantification was attempted in three of the Impact Areas but was not feasible in the remaining two. Several common observations and recommendations emerged from across the different studies: • The Impact Area indicators used in CGIAR’s Results Framework were generally not sufficiently specific, measurable, achievable, relevant, or timebound (SMART).177 They used ambiguous terms such as “benefiting” and “improved management.” Functional units and methods of measurement were often not prescribed, and time or geographic bounds were often not applied. • Potential solution: Revise the Impact Area indicators to ensure full SMART compliance, define methods and tools to be used in data collection, and roll these out through the CGIAR Programs and Accelerators. • The stage along the impact pathway assessed by each Impact Area indicator is highly variable, and different measurements apply at different stages along the impact pathway. For example, in the Poverty Impact Area, an indicator of the ultimate goal is the number of people assisted to exit poverty, but the most common means through which CGIAR affects poverty is by enhancing agricultural productivity, which could be defined as a more proximate goal. • Potential solution: Define proximate and ultimate Impact Area indicators, which relate to stages in the impact pathways and include more studies that attempt to demonstrate the relationships between the two. Defining common impact pathways used in CGIAR programming would also be beneficial. • There is fragmentation in the indicators measured in impact evaluations and the Impact Area indicators required in the Results Framework. There is also a disconnect between studies that
+---
+[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p17pt3]
+private sector impact investments. These efforts will be designed to be consistent with and complement the objectives, priorities, and activities of the CGIAR Standing Panel on Impact Assessment (SPIA). Impact assessment studies are implemented across AoWs and coordinated by S4I’s MELIA unit, with scientific input from AoW 5’s Cluster 5.2 on Dynamic Learning and Impact Assessment. This cluster
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p11pt3]
+the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. Figure 2.3. Number of RAFS results contributing to each Impact Area. Results are tagged as “principal” or “significant” to indicate their contribution to an Impact Area, with principal results shown in the orange and significant results in the yellow. Source: CGIAR Results Dashboard, accessed May 6, 2025. A total of 5,453 results were submitted over the three-year period, with annual
+---
+[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt4]
+Scaling for Impact Program
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt2]
+of the studies that will allow us to answer impact assessment questions (outcomes
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt1]
+Version 1.0 8 evidence is relevant for wider adoption and systemic change. While the exact number of studies is not speciﬁed, the focus on “selected interventions” implies a targeted approach to eƯectively deploy robust methods for evaluating short- and medium-term impacts contributing to the ﬁve CGIAR Impact Areas, prioritizing those with the greatest potential for learning and scaling. CollaboraƟon with other Programs/Accelerators, W3/bilateral projects, and/or partners to deliver the impact assessment work. While speciﬁc details regarding the Frontiers Program’s collaborative impact assessment work are still being formalized, its approach aligns with a broader CGIAR emphasis on synergistic eƯorts. The program is committed to working with other Programs (Policy Innovations and Scaling for Impact SPs), Accelerators,
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt2]
+additional studies from SPIA (see Impact assessments). Most impacts stemmed from earlier work but were published during this period. Some studies were based on one- or two-years’ worth of data, and other studies were based on data spanning up to four decades (Figure 6). Many of these longer-term studies consider the aggregate effects and net returns of large and longstanding CGIAR work streams. Like the outcomes, measured impacts span all the five Impact Areas, though some Impact Areas are more represented than others. Figure 6. Global evidence base of the impacts and outcomes. Top panel: 18 impact assessment studies did not specify the dates covered by their data and so are not represented. Where studies used datasets with different time periods for different indicators, each time period is represented by a horizontal bar . Middle panel: The middle-center panel expresses the methods used by non-causal impact
+---
+[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt4]
+(from farmer to national level) and to assess different assumptions on how impacts are generated through Multifunctional Landscapes approaches based on co-design and systemic thinking. The specific methodologies used include quantitative counterfactual analysis for adoption and impact measurement (where feasible, as well as evaluation methods that allow to capture multidimensional, unintended and unexpected consequences. Given the complexity and breath of the impacts that the Program aims to influence, impact studies will be targeted to the key areas of success of the Program and will therefore be defined by: • Availability of baselines from the three Initiatives • The results of monitoring and evaluation that will provide guidance on the key Outcomes achieved • The collaboration with other Programs/Accelerators • The studies developed in bilaterals mapped to specific outcomes of
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3]
+impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets. Better linkage between annual Program/Accelerator Theory of Change, Plan of Results and Budget, and Technical Reporting. The primary audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary audience is Partners. Annual Technical
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p63pt4]
+program to take these good ideas to scale, reaching more people and places. Credit: Abdul Momin, CIMMYT CGI21-508007-PORB-Scaling for Impact.indd 63CGI21-508007-PORB-Scaling for Impact.indd 63 07/08/2025 13:2407/08/2025
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt1]
+Impacts and outcomes by Impact Area In the following sections, we present evidence of the real- world impacts of CGIAR-supported interventions for each CGIAR Impact Area. Each section starts with an overview of current challenges and CGIAR’s work in that Impact Area. We then summarize the evidence identified pertaining to the Impact Area. Each Impact Area section focuses on the evidence of impact or outcomes on three to four types of work that CGIAR conducts
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt2]
+June 2025 22 Impact level –
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt2]
+June 2025 22 Impact level –
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4]
+and Impact Area indicators. • Once priority Questions identified, engage SPIA &amp; CGIAR Impact Assessment specialists to refine &amp; design delivery approach, • Contribution from across all funding streams, • Adapt existing Program/Accelerator/w3 &amp; bilateral project data collection approach to strengthen linkage between MEL and IA, based on Impact Case study learnings. • Report Impact Case findings as they become available, and compile in Triennial Portfolio Outcome and Impact reports. Additionally, an Impact Compendium will provide stakeholders with ready access to relevant CGIAR impact-related studies and evidence dating back to 2017. Updated annually, users will be able to explore the impact data and syntheses from different perspectives including Impact Area, geography, type of impact study. The Impact compendium will be launched in Q2 2025.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt4]
+and Impact Area indicators. • Once priority Questions identified, engage SPIA &amp; CGIAR Impact Assessment specialists to refine &amp; design delivery approach, • Contribution from across all funding streams, • Adapt existing Program/Accelerator/w3 &amp; bilateral project data collection approach to strengthen linkage between MEL and IA, based on Impact Case study learnings. • Report Impact Case findings as they become available, and compile in Triennial Portfolio Outcome and Impact reports. Additionally, an Impact Compendium will provide stakeholders with ready access to relevant CGIAR impact-related studies and evidence dating back to 2017. Updated annually, users will be able to explore the impact data and syntheses from different perspectives including Impact Area, geography, type of impact study. The Impact compendium will be launched in Q2 2025.
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p48pt4]
+AoW 5 – Learning for Impact 1.1, 1.2, 2.1, 2.2, 2.3, 3.1, 3.2, 3.3, 4.1 CGI21-508007-PORB-Scaling for Impact.indd 48CGI21-508007-PORB-Scaling for Impact.indd 48 07/08/2025 13:2407/08/2025 13:24
+---
+[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p1pt2]
+and Impact Assessment (MELIA) Plan
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p20pt4]
+impact? TBD in WCA, ESA, SA Causal impact assessment Empowerme nt and resilience: research question: what is the TBD in S A and SSA Causal
+---
+[ID: pdf:CGI21-507032-PORB-Gender Equality and Inclusion.pdf:p23pt3]
+engagement, science quality, impact assessment) 2025 Q1 Q2 Q3 Q4 2025 (Approved Budget) Strategic leadership X X X X 68,703.66 Collaborating with Science Programmes to deliver on Impact Area functions X X Total Cross-cutting and Management budget 68,703.66 Area of Work 1: Accelerating Solutions for Impact 2025 Outcome Q1 Q2 Q3 Q4 2025 (Approved Budget) 1.1: Pinpoint and act on restrictive norms X X X X - 1.4: Amplify the voices of
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p50pt4]
+good ideas to scale, reaching more people and places. Credit: Abdul Momin, CIMMYT CGI21-508007-PORB-Scaling for Impact.indd 50CGI21-508007-PORB-Scaling for Impact.indd 50 07/08/2025
+---
+[ID: pdf:Breeding for Tomorrow_Inception Report 30-06-2025.pdf:p8pt3]
+assessment unit which aims to assess the impact
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p74pt3]
+(5 percent) tagged as poverty- principal. This demonstrates that Initiatives, Impact Platforms, and SGPs contributed to poverty reduction, livelihoods, and jobs while simultaneously addressing other Impact Areas and SDGs to maximize synergies. It is also important to note that 2,685 results (33 percent) in 2024 were not tagged as having a significant or principal focus on poverty reduction, livelihoods, and jobs. However, the contributions of these untagged results to the crosscutting dimensions of the Impact Area may have been indirect. 5,109 31% 7,672 46% 873 5%2,951 18% 16,605 Total results 2 = Principal: Contributing to one or more aspects of the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing
+---
+[ID: pdf:Breeding for Tomorrow_MELIA Plan 30-06-2025 (1).pdf:p47pt2]
+in particular continuous improvement Note, impact is an evaluation criterion. Impact Assessments and RCTs are possible methods to evaluate impact. Other methods are available to determine impact. The most appropriate method that provides useful information to improve B4T needs to be determined. E.g. Impact assessment can be used to increase confidence in projection of benefit assumptions. A detailed review of the in-progress Impact Assessment will be required to determine potential use of findings beyond accountability. End of September Learning and adaptive management, including annual review and planning to respond to learnings as emerging Collate list of indicators and research questions that will have data available on an annual basis Review breeding pipeline performance management in Enable
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p74pt4]
+to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. 0 = Not targeted: The result has been screened against the Impact Area, but it has not been found to directly contribute to any aspect of the Impact Area as it is outlined in the CGIAR 2030 Research and Innovation strategy. Not applicable: Pertains to 2022 reported results when only information on Gender and Climate impact area tagging was available. Figure 5.26. Number of reported results tagged as having a principal or significant focus on the Poverty Reduction, Livelihoods and Jobs Impact Area, 2023–2024. Source: CGIAR Results Dashboard, accessed May 6, 2025. Vegetable farmer in Badulla district, Sri Lanka. 70 Annual Technic al
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3]
+2030 Outcome, or Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framework Provide the assumption( s) statem ent from the Results Framework Indicate the location(s) where the study will be conducted Indicate the methods and design approaches that will be used for the study List the Program(s) and Accelerator( s ) you will collaborate with or coordinate for the implementati on of this study. Indicate the Start
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p15pt1]
+13 4. Impact assessment (IA) As detailed above, the Climate Action Science Program will implement a set of formative and summative evaluation studies to document the outcomes and impacts of its interventions across diƯerent levels. The Program’s impact assessment strategy includes studies employing qualitative (primarily), quantitative, and mixed-methods approaches, and, when feasible, methods that allow us to attribute observed results directly to the Program’s actions. The qualitative evaluations—combined with monitoring data and secondary sources—will help us identify early results most likely attributable to the Program’s interventions. This evidence will also inform decisions on where and when to propose and design quantitative adoption studies or causal impact assessments. The quantitative evaluations will, in turn, provide rigorous (causal) evidence on the outcomes and impacts of the Program. The funding mechanism to implement these studies will include a
+---
+[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p1pt3]
+Impact Assessment (MELIA) Plan Digital Transformation
+---
+[ID: pdf:Sustainable Animal and Aquatic Foods_MELIA Plan 30-06-2025.pdf:p1pt2]
+Learning and Impact Assessment (MELIA) Plan
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p1pt2]
+Evaluation, Learning and Impact Assessment (MELIA)
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p50pt2]
+7,6726,069 3,250 6,389 4,822 5,794 1,196 6,858 6,646 Nutrition, health and food security 2,951 1,002876 2,951 2,951 2 = Principal: Contributing to one or more aspects of the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. 0 = Not targeted: The result has been screened against the Impact Area, but it has not been found to directly contribute to any aspect of the Impact Area as it is outlined in the CGIAR 2030 Research and Innovation strategy. Not applicable: Pertains to 2022 reported results when only information on Gender and Climate impact area tagging was available. Figure 5.1.
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1]
+All impact study submissions were reviewed for potential inclusion into the evidence base of the report. The two primary inclusion considerations were relevance and rigor (see Annex A. Selection of evidence). Studies were determined to be relevant if they considered the outcomes and impacts of CGIAR-supported interventions, regardless of the authorship of the study. Outcomes reported into the CGIAR PRMS are quality assessed for relevance (that is, CGIAR’s role in the outcome is validated); therefore, none of these reported outcomes were excluded on the basis of relevance. Studies with unclear or misleading methods were excluded on the basis of rigor. Studies meeting this threshold of clarity were then classed as “impact assessments” or “impact evaluations.” Impact evaluations were the primary study designs of interest. Impact evaluations are studies that use statistical methods (experimental or quasi-experimental) to quantify the causal change in a condition that was achieved by an intervention. Studies using other study designs were included under the umbrella term of impact assessments (including impact evaluations), if they provided information relevant to understanding impacts, such as cost- benefit analyses, reviews of CGIAR work, and measures of the adoption of CGIAR technology. These included the country studies supported by CGIAR’s SPIA. While impact evaluations are necessary to establish causal change linking intervention and impact, they can be limited in scope due to practical constraints, such as resources and measurement challenges. Other types of impact assessments can provide valuable insights into CGIAR’s contributions to real-world change in a wider spatial or temporal context; however , they do c This can be common for power calculations. Authors may have conducted power calculations but not r eported that they did so in-text. Assessment is based on what is reported in-text, not what may have been done but not reported. d See Annex A. Included studies and rigor of
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p4pt2]
+to understanding impacts, including impact evaluations and other study designs, such as cost-benefit analyses, reviews and meta-analyses, and measures of the adoption of technologies. Impact assessment studies of CGIAR innovations cover a range of spatial and temporal scopes (from small geographical areas to global analyses, and various timeframes following dissemination of an innovation) and seek to address a range of questions related to impact, including establishing the amount of impact achieved rather than the causality of the impact. Impact evaluation A subcategory of impact assessments, which use statistical methods (experimental or quasi-experimental) to attribute a change in a condition of interest to an intervention. Outcome A change in knowledge, skills, attitudes, or relationships, manifested as a change in behavior , to which research outputs and related activities have contributed. CGIAR categorizes outcomes as related to innovation use, policy changes, or others. Pooled-funded The financing of CGIAR research activities from the CGIAR Trust Fund. This is in contrast to non-pooled funded activities, which includes finance from bilateral arrangements between Centers and funders, or cases where funders have specified a Center to receive finance from the CGIAR Trust Fund for a specific purpose. Pooled-funded portfolio Within the 2022-2024 period, a portfolio of 32 research Initiatives, five Impact Area Platforms, and six Science Group Projects was operated, subject to a centralized management and technical reporting system. Reach Exposure to, engagement with, or access to an intervention, regardless of the depth of participation or impact. Use Acquisition and adoption of social, institutional, or technological innovations among actors who have been reached. Foreword As CGIAR’s Executive Managing Director , I am proud to present the first ever whole-of-CGIAR impact report.
+---
+[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p12pt3]
+the Policy Program is no exception. Recurring assumptions in the ToC revolve around empowering actors and creating improved knowledge and building capacity to empower these actors. This theme is at the heart of the P olicy Program's operations, encompassing concepts such as co -creation and demand-driven research that build capacity and create the right conditions for policy change to occur. IA activities and collaboration plans The Impact Assessment (IA) strategy employs a combination of quantitative (both experimental and non-experimental) and qualitative (outcome evidencing) research methods to substantiate the Program's contributions to CGIAR's Impact Areas. Additionally, rapid impact assessment methods are utilized when necessary to track achievements and support swift policy responses. Aligned with the learning objectives of the Monitoring, Evaluation, and Learning (MEL) component, the IA strategy provides empirical evidence on the Program's effects, aiming to understand the causal mechanisms underlying both expected and unanticipated outcomes. Each of the 2030
+---
+[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p43pt4]
+Learning for Impact Bahir Dar Unidersity (Ethiopia) IWMI Contracted AoW 5 - Learning for Impact University of Ghana IWMI Contracted AoW 5 - Learning for Impact Africa Group of Negotiators Experts Support (AGNES) IWMI Potential AoW 3 – Enabling Environment Lab TAAT IWMI Contracted AoW 4- Achieving Impact by Unlocking Finance and Partnerships AfDB IWMI Contracted AoW 4- Achieving Impact by Unlocking Finance and Partnerships CGI21-508007-PORB-Scaling for Impact.indd 43CGI21-508007-PORB-Scaling for Impact.indd 43 07/08/2025
+---
+[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p14pt1]
+14 5. Impact assessment Impact Assessment (IA) is a key approach for evaluating the effectiveness and impact of innovations, technologies, or practices on target populations and geographies. By systematically measuring outcomes and impacts, IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives. IA goes beyond monitoring indicators, requiring a rigorous approach to attribut ing observed changes to CGIAR interventions (e.g., innovations, policies). It employs both quantitative and qualitative methods, often combined for deeper insights. Program/Accelerator impact overview The AoWs of the Sustainable Framing Program will collectively contribute to the program’s outcomes and expected impacts by co -developing and delivering whole -farm innovation bundles to at least five million farmers, with positive impacts on socially equitable and sustainable agronomic gain across two million ha of land. At least 50 public and private development partners are expected to facilitate the scaling of solutions to farming communities and integrating innovations in their investments.
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p65pt1]
+not determine what was done or conclusions based on a fundamental misinterpretation of reported results. A few studies provided valuable contextual information regarding the interpretation of included impact assessments but were not impact assessments themselves. These studies were not included in the literature database used to develop the narrative of this report but are presented in the narrative to contextualize findings. Examples of such studies include descriptions of novel methodologies and willingness- to-pay studies. AfricaRice genebank in Mbe, Cote d’Ivoire. Photo credit: Neil Palmer/Crop Trust Include Exclude Impact evaluation inclusion criteria Population Any None Intervention Interventions that were at least partly co-developed by CGIAR and implemented in real-world settings. Real-world settings were defined as settings that could reasonably be expected when a project or scaling up effort is implemented outside of a research context. Interventions are not co-developed by CGIAR or evaluated only in highly controlled (not real-world) settings. Comparator Any comparator , so long as one exists. None Outcome Outcomes must reflect behaviors or effects external to CGIAR and relate to any of CGIAR’s Impact Area indicators
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p44pt4]
+example) loss of employment, livestock, or other productive assets; or through health channels, such as acquisition of persistent, incurable conditions such as HIV. Causal impact assessment learning studies 1 206.25 32,185.87 N/A - 32,185.87
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4]
+against CGIAR’s Results Framework is that, apart from the SPIA country studies, other internal and external studies are designed in an uncoordinated bottom-up way. Because such studies are undertaken to meet specific information needs, opportunities to learn through synthesis or aggregation are missed due to the differences in indicators used and measurement approaches employed. For example, impact assessments are rarely connected with data on innovation use, preventing case study results from being used to extrapolate possible large-scale effects. Thus, moving forward, two areas for improvement are: (1) to collectively undertake strategic impact assessments that will answer high-priority impact assessment questions and (2) to develop and enforce the use of a core set of common indicators and measurement methodsq that should be used in impact assessment studies regardless of who initiates them. In addition, during the 2022 to 2024 period, Initiatives defined targets for outcomes and made commitments to measuring and reporting on those outcomes. They did not have a similar plan or commitment to measuring impacts. As CGIAR evolves to longer-term programs covering the whole of CGIAR, there should be commitments to the consistent measurement of impacts. However , this has been an ongoing challenge within the organization, with similar recommendations from a review of the 2017 to 2021 portfolio.176 Rigor of the evidence All impact evaluations identified were assessed for their rigor based on criteria established by Rao 2025.45 The most common score was a 4 of 9 key elements being present, suggesting moderate overall quality and room for improvement. A high number of impact evaluations used rigorous methods to infer causality between a CGIAR innovation and impacts (see Annex A. Included studies and rigor of evidence). However , many failed to consider heterogeneous treatment effects or report power calculations. Most of the impact evaluations used experimental or quasi-experimental designs with two or more measurement periods. However , a sizeable group of the studies were based on cross-sectional (single measurement) studies. While they are peer-reviewed and employ recommended methods of controlling for unobservable variables to enhance the likelihood of a causal inference, there remain limitations to such designs. In addition to rigor , this study paid attention to the relevance of</t>
+  </si>
+  <si>
+    <t>[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3]
+impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets. Better linkage between annual Program/Accelerator Theory of Change, Plan of Results and Budget, and Technical Reporting. The primary audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary audience is Partners. Annual Technical
+---
+[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3]
+Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framewo rk Provid e the assu mptio n(s) state ment from the Resul ts Fram ework Indicate the location( s) where the study will be conducte d Indicate the methods and design approache s that will be used for the study List the Progr am(s) and Accel erato
+---
+[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p18pt3]
+2030 Outcome, or Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framework Provide the assumption( s) statem ent from the Results Framework Indicate the location(s) where the study will be conducted Indicate the methods and design approaches that will be used for the study List the Program(s) and Accelerator( s ) you will collaborate with or coordinate for the implementati on of this study. Indicate the Start
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1]
+Impact Area indicator quantification Given these limitations and opportunities, the Portfolio Performance Unit (PPU) commissioned subject matter experts for each Impact Area to review the Impact Area indicators and the aligned outcomes and impacts reported, with a view to assessing the feasibility of aggregating the reported results to inform on total progress toward the Impact Area indicators during the 2022 to 2024 period. This was very challenging, and partial quantification was attempted in three of the Impact Areas but was not feasible in the remaining two. Several common observations and recommendations emerged from across the different studies: • The Impact Area indicators used in CGIAR’s Results Framework were generally not sufficiently specific, measurable, achievable, relevant, or timebound (SMART).177 They used ambiguous terms such as “benefiting” and “improved management.” Functional units and methods of measurement were often not prescribed, and time or geographic bounds were often not applied. • Potential solution: Revise the Impact Area indicators to ensure full SMART compliance, define methods and tools to be used in data collection, and roll these out through the CGIAR Programs and Accelerators. • The stage along the impact pathway assessed by each Impact Area indicator is highly variable, and different measurements apply at different stages along the impact pathway. For example, in the Poverty Impact Area, an indicator of the ultimate goal is the number of people assisted to exit poverty, but the most common means through which CGIAR affects poverty is by enhancing agricultural productivity, which could be defined as a more proximate goal. • Potential solution: Define proximate and ultimate Impact Area indicators, which relate to stages in the impact pathways and include more studies that attempt to demonstrate the relationships between the two. Defining common impact pathways used in CGIAR programming would also be beneficial. • There is fragmentation in the indicators measured in impact evaluations and the Impact Area indicators required in the Results Framework. There is also a disconnect between studies that
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p7pt3]
+fully contextualize the results. Are you an implementer? Consider jumping directly to your Impact Area or Continent of interest. But be sure to return and read about the Scope of the Report so that you know what is, and is not, included in this report. Tips on interpretation When interpreting the outcomes reported, be cautious about aggregating across data sources (e.g., as Performance and Results Management System [PRMS] and SPIA country studies), Impact Areas, and continents. Some outcomes are included in more than one of these categories. Pay attention to the specified time period. The report focuses on evidence reported during the 2022 to 2024 period, but outcomes and impacts often developed over much longer periods. Consider the overall weight of the evidence, not individual pieces of evidence. This report presents a body of evidence, drawing on a variety of different epistemological approaches: outcome evidence, impact evaluations, and other types of information, which collectively provide different insights into CGIARs impact. However , only impact evaluations were assessed for the number of best research practices they used, with a composite score of 0 to 9 assigned based on the number of key components of rigor addressed by the study. While weighted equally in this work, these components do not all have equal implications for overall study
+---
+[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]
+exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. Impact assessments are conducted after an intervention has been completed and are used to substantiate claims of sustained results. They seek to measure impact at scale, i.e., benefits to a large number of people/large areas of land. It employs both quantitative and qualitative methods, often combined for deeper insights. IA goes beyond monitoring indicators to evidenced attribution of observed changes to CGIAR interventions. IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives.
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt2]
+additional studies from SPIA (see Impact assessments). Most impacts stemmed from earlier work but were published during this period. Some studies were based on one- or two-years’ worth of data, and other studies were based on data spanning up to four decades (Figure 6). Many of these longer-term studies consider the aggregate effects and net returns of large and longstanding CGIAR work streams. Like the outcomes, measured impacts span all the five Impact Areas, though some Impact Areas are more represented than others. Figure 6. Global evidence base of the impacts and outcomes. Top panel: 18 impact assessment studies did not specify the dates covered by their data and so are not represented. Where studies used datasets with different time periods for different indicators, each time period is represented by a horizontal bar . Middle panel: The middle-center panel expresses the methods used by non-causal impact
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt3]
+Streamline reporting (less products, more integration, lower transaction costs). • Stronger impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets • Better linkage between annual Program and Accelerator Theory of Change , Plan of Results and Budget, and Technical Reporting. Currently these three components are not adequately linked, making it challenging to demonstrate progress against TOCs, or define costs for specific results and subsequent ROI. • Outcome and Impact content from across the Portfolio will be consolidated and delivered through triennial reports, however individual studies will be released as they become available to reduce the wait time for access to outcome and impact-related information. The primary target audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary target audience is
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt3]
+Streamline reporting (less products, more integration, lower transaction costs). • Stronger impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets • Better linkage between annual Program and Accelerator Theory of Change , Plan of Results and Budget, and Technical Reporting. Currently these three components are not adequately linked, making it challenging to demonstrate progress against TOCs, or define costs for specific results and subsequent ROI. • Outcome and Impact content from across the Portfolio will be consolidated and delivered through triennial reports, however individual studies will be released as they become available to reduce the wait time for access to outcome and impact-related information. The primary target audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary target audience is
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt4]
+wait time for access to outcome and impact-related information. The primary target audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary target audience is Partners. Relevant content from Technical Report products will be integrated into CGIAR’s corporate reporting. Annual Technical Reporting will cover individual Program and Accelerator progress towards their respective end of delivery outcomes, as well as provide an overall Portfolio view of aggregate contribution to thematic and geographic targets. The shift to a 6-year Business Cycle will allow CGIAR to address the challenges of outcome and impact reporting in a more holistic manner, looking across individual projects and Business Cycles, including Initiatives and CRPs. This will result in a more complete reporting of CGIAR outcomes and impacts. Changes to the way CGIAR
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt4]
+wait time for access to outcome and impact-related information. The primary target audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary target audience is Partners. Relevant content from Technical Report products will be integrated into CGIAR’s corporate reporting. Annual Technical Reporting will cover individual Program and Accelerator progress towards their respective end of delivery outcomes, as well as provide an overall Portfolio view of aggregate contribution to thematic and geographic targets. The shift to a 6-year Business Cycle will allow CGIAR to address the challenges of outcome and impact reporting in a more holistic manner, looking across individual projects and Business Cycles, including Initiatives and CRPs. This will result in a more complete reporting of CGIAR outcomes and impacts. Changes to the way CGIAR
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p12pt1]
+All impact study submissions were reviewed for potential inclusion into the evidence base of the report. The two primary inclusion considerations were relevance and rigor (see Annex A. Selection of evidence). Studies were determined to be relevant if they considered the outcomes and impacts of CGIAR-supported interventions, regardless of the authorship of the study. Outcomes reported into the CGIAR PRMS are quality assessed for relevance (that is, CGIAR’s role in the outcome is validated); therefore, none of these reported outcomes were excluded on the basis of relevance. Studies with unclear or misleading methods were excluded on the basis of rigor. Studies meeting this threshold of clarity were then classed as “impact assessments” or “impact evaluations.” Impact evaluations were the primary study designs of interest. Impact evaluations are studies that use statistical methods (experimental or quasi-experimental) to quantify the causal change in a condition that was achieved by an intervention. Studies using other study designs were included under the umbrella term of impact assessments (including impact evaluations), if they provided information relevant to understanding impacts, such as cost- benefit analyses, reviews of CGIAR work, and measures of the adoption of CGIAR technology. These included the country studies supported by CGIAR’s SPIA. While impact evaluations are necessary to establish causal change linking intervention and impact, they can be limited in scope due to practical constraints, such as resources and measurement challenges. Other types of impact assessments can provide valuable insights into CGIAR’s contributions to real-world change in a wider spatial or temporal context; however , they do c This can be common for power calculations. Authors may have conducted power calculations but not r eported that they did so in-text. Assessment is based on what is reported in-text, not what may have been done but not reported. d See Annex A. Included studies and rigor of
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt2]
+Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt2]
+Reporting. We will progressively add curated datasets (such as Center-level databases) into the QA process to remove to the extent possible the need for double reporting. Existing experience gained through automated PRMS solutions (e.g. screening knowledge products against FAIR criteria) will be leveraged. 3. CGIAR Results Framework, MELIA, Indicator Toolkit and data collection protocols CGIAR Results Framework The CGIAR Results Framework will be used by Programs and Accelerators as the basis of their TOC design, MELIA and Technical Reporting. It will provide the basis for geographic portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt3]
+portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt3]
+portfolio-level outcome, and portfolio level contribution to Impact Area targets reporting. The foundations of the current Results Framework (2022-24) remain: • Impact Areas linked to Sustainable Development Goals • Impact, outcome, and output result levels • Result types/categories o Outcome: Innovation use, Policy change, Other. o Output: Innovation development, Capacity sharing, Knowledge products, Other • A small number of Standard Indicators The updated CGIAR Results Framework in Annex 1 will be finalized in Q1-2 2025. The m ain updates included in the 2025-30 Results Framework include: • Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p7pt2]
+2. Technical Report products Technical Report products will progressively integrate pooled and bilaterally and W3 -funded project and program information. Technical Report products will provide: 1. Assurance on delivery against portfolio-wide indicator targets and insight on specific topics driven by quality assured evidence, 2. Demand-driven support to decision making at different levels, 3. Curated content for use in communications, advocacy and resource mobilization. 4. Learnings and evidence for fact based adaptive management decisions at science program, accelerator, and center levels. 5. Line of sight between investment and results. The main changes that will be made to existing 22-24 Technical Products include: • Streamline reporting (less products, more integration, lower transaction costs). • Stronger impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets • Better linkage between annual Program
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p7pt2]
+2. Technical Report products Technical Report products will progressively integrate pooled and bilaterally and W3 -funded project and program information. Technical Report products will provide: 1. Assurance on delivery against portfolio-wide indicator targets and insight on specific topics driven by quality assured evidence, 2. Demand-driven support to decision making at different levels, 3. Curated content for use in communications, advocacy and resource mobilization. 4. Learnings and evidence for fact based adaptive management decisions at science program, accelerator, and center levels. 5. Line of sight between investment and results. The main changes that will be made to existing 22-24 Technical Products include: • Streamline reporting (less products, more integration, lower transaction costs). • Stronger impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets • Better linkage between annual Program
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p11pt3]
+the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. Figure 2.3. Number of RAFS results contributing to each Impact Area. Results are tagged as “principal” or “significant” to indicate their contribution to an Impact Area, with principal results shown in the orange and significant results in the yellow. Source: CGIAR Results Dashboard, accessed May 6, 2025. A total of 5,453 results were submitted over the three-year period, with annual
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p48pt4]
+against CGIAR’s Results Framework is that, apart from the SPIA country studies, other internal and external studies are designed in an uncoordinated bottom-up way. Because such studies are undertaken to meet specific information needs, opportunities to learn through synthesis or aggregation are missed due to the differences in indicators used and measurement approaches employed. For example, impact assessments are rarely connected with data on innovation use, preventing case study results from being used to extrapolate possible large-scale effects. Thus, moving forward, two areas for improvement are: (1) to collectively undertake strategic impact assessments that will answer high-priority impact assessment questions and (2) to develop and enforce the use of a core set of common indicators and measurement methodsq that should be used in impact assessment studies regardless of who initiates them. In addition, during the 2022 to 2024 period, Initiatives defined targets for outcomes and made commitments to measuring and reporting on those outcomes. They did not have a similar plan or commitment to measuring impacts. As CGIAR evolves to longer-term programs covering the whole of CGIAR, there should be commitments to the consistent measurement of impacts. However , this has been an ongoing challenge within the organization, with similar recommendations from a review of the 2017 to 2021 portfolio.176 Rigor of the evidence All impact evaluations identified were assessed for their rigor based on criteria established by Rao 2025.45 The most common score was a 4 of 9 key elements being present, suggesting moderate overall quality and room for improvement. A high number of impact evaluations used rigorous methods to infer causality between a CGIAR innovation and impacts (see Annex A. Included studies and rigor of evidence). However , many failed to consider heterogeneous treatment effects or report power calculations. Most of the impact evaluations used experimental or quasi-experimental designs with two or more measurement periods. However , a sizeable group of the studies were based on cross-sectional (single measurement) studies. While they are peer-reviewed and employ recommended methods of controlling for unobservable variables to enhance the likelihood of a causal inference, there remain limitations to such designs. In addition to rigor , this study paid attention to the relevance of the studies. Often, studies employing less rigorous, cross-sectional methodologies were able to provide evidence more relevant to policymaking and decision-making Tradititional rice variety in Ilagan, Isabela, the Philippines. Photo credit: Miguel Mamon/CIAT CGIAR Impacts in Agrifood Systems: | Learnings | Page 90 of 130 CGIAR CGIAR CGIAR Impacts in Agrifood Systems: | Learnings| Page 91 of 130
+---
+[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3]
+Impact assessment (IA) .............................................................................................................. 13 Program impact overview .................................................................................................................... 13 IA activities and collaboration plans ..................................................................................................... 14 IA studies ........................................................................................................................................... 15 5. Learning and adaptive management ........................................................................................... 16 Learning ............................................................................................................................................. 16 Annual review and adaptive planning ...................................................................................................
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3]
+Technical Reporting Arrangement 2025-30 Results
+---
+[ID: docx:Guidance on reporting outputs or outcomes.docx:u1-4]
+Guidance on reporting outputs or outcomes Output and outcome definitions Research results can be defined according to the nature of the change and the control over it. Output: Tangible products or services such as knowledge, technical or institutional advancement that result directly from CGIAR research, engagement and/or capacity development activities. They involve a change in knowledge or tools within the research process itself, produced under the control of the research team.
+---
+[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt4]
+Results Dashboard 2024 Technical Reports
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p11pt2]
+it was not possible in retrospect to piece together the relevant costs to link to reported outcomes and impacts. Thus, the report focuses primarily on achievements and benefits and not net benefits or returns to investments. Figure 4: The stages in CGIAR’s Theory of Change and the corresponding sources of evidence used in this report. Notes: This report focuses on outcomes and impacts. CGIAR’s annual reports focus on activities, outputs, and outcomes. Activities The daily work of CGIAR staff. Examples: research, partnership building, capacity and knowledge sharing, communication. Sources of evidence: Outputs Creation of tangible products. Examples: publications, innovations, policy advice. Outcomes Changes in behavior of partners and stakeholders. Examples: policy changes, investments, use of CGIAR innovations. Impacts Durable change in the condition of people and their environment. Examples: increased income for farmers, more nutritious diets for consumers. Annual technical reporting Adoption studies Impact assessment and casual evaluations The precise definition of the term “outcomes” used here is “change[s] in knowledge, skills, attitudes, and/ or relationships, manifested as a change in behavior , to which research outputs and related activities have contributed.”44 “Impact” is defined here as “durable change[s] in the condition of people and their environment brought about by a chain of events or change in how a system functions, to which research, innovations, and related activities have contributed.”44 Indicators in CGIAR’s Results Framework were consistently monitored at the outcome level and are presented in aggregate for the pooled-funded work. At the impact level, it was more common for indicators related, but not identical, to indicators in the Results Framework to be used. This causes challenges in aggregation; therefore, impact results are generally described individually. This is a key point of improvement in implementation of the portfolio 2025–2030 (see The 2022–2024 Results Framework and Annex B. Impact Indicators). Methods at a glance This report provides the evidence on CGIAR’s outcomes and impacts that was made available
+---
+[ID: pdf:Portfolio Narrative_2024.pdf:p58pt2]
+on critically relevant topics. 3,250 6,646 1,708 3,528 3,001 6,709 1,200 1,661 554 2,542 2,500 1,233 2022 results 3,415 2023 results 6,275 2024 results 8,237 Total results 16,605 2 = Principal: Contributing to one or more aspects of the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. 0 = Not targeted: The result has been screened against the Impact Area, but it has not been found to directly contribute to any aspect of the Impact Area as it is outlined in the CGIAR 2030 Research and Innovation strategy. Figure 5.9. Overview
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4]
+and Impact Area indicators. • Once priority Questions identified, engage SPIA &amp; CGIAR Impact Assessment specialists to refine &amp; design delivery approach, • Contribution from across all funding streams, • Adapt existing Program/Accelerator/w3 &amp; bilateral project data collection approach to strengthen linkage between MEL and IA, based on Impact Case study learnings. • Report Impact Case findings as they become available, and compile in Triennial Portfolio Outcome and Impact reports. Additionally, an Impact Compendium will provide stakeholders with ready access to relevant CGIAR impact-related studies and evidence dating back to 2017. Updated annually, users will be able to explore the impact data and syntheses from different perspectives including Impact Area, geography, type of impact study. The Impact compendium will be launched in Q2 2025.
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p17pt4]
+and Impact Area indicators. • Once priority Questions identified, engage SPIA &amp; CGIAR Impact Assessment specialists to refine &amp; design delivery approach, • Contribution from across all funding streams, • Adapt existing Program/Accelerator/w3 &amp; bilateral project data collection approach to strengthen linkage between MEL and IA, based on Impact Case study learnings. • Report Impact Case findings as they become available, and compile in Triennial Portfolio Outcome and Impact reports. Additionally, an Impact Compendium will provide stakeholders with ready access to relevant CGIAR impact-related studies and evidence dating back to 2017. Updated annually, users will be able to explore the impact data and syntheses from different perspectives including Impact Area, geography, type of impact study. The Impact compendium will be launched in Q2 2025.
+---
+[ID: docx:Guidance on reporting outputs or outcomes.docx:u19-22]
+What kind of change does this result represent? Is it a tangible product like a report, dataset, or publication (output)? Or is it a change in behavior, knowledge, attitudes, or skills of others (outcome)? Is the result immediate or downstream?
+---
+[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p46pt3]
+to ensure common terminology across the reporting units. At the impact level, there were 19 indicators across the five Impact Areas. The frequency of reporting against exact indicators is very low (18 percent of indicators assessed match those in the Results Framework; Annex B. Impact indicators). In addition, there is an imbalance across Impact Areas and indicators in the frequency with which 2022 to 2024 studies attempt to measure those indicators. There were many impact assessments that measured yields or income related to the poverty indicators, and relatively few that looked at environmental, climate, or gender indicators. This is consistent with what Templeton (2023)176 found in her review of evidence used to support the impact claims made by the CGIAR Research Programs between 2017 and 2021. Thus, there remains a huge challenge to define feasible indicators for
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p11pt4]
+• Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g. productivity), ambiguous terms (benefitting), and challenges in measurement (people assisted to exit poverty). A study was commissioned in 2023 to review the Result Framework indicators and started a process to collect inputs towards identifying and operationalizing impact level indicators. Revised impact level indicators are now included in the updated CGIAR Results Framework. • Science Group Outcomes converted into Portfolio Outcomes Given the change in organizational structure, current Science Group outcomes have been converted into Portfolio Outcomes. The Science Group Outcomes had emphas ized ‘next user’
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p11pt4]
+• Revised Impact Area indicators Shortcomings with the Impact Area indicators in the 2022-24 Results Framework have been identified, including absence of some important indicators for CGIAR (e.g. productivity), ambiguous terms (benefitting), and challenges in measurement (people assisted to exit poverty). A study was commissioned in 2023 to review the Result Framework indicators and started a process to collect inputs towards identifying and operationalizing impact level indicators. Revised impact level indicators are now included in the updated CGIAR Results Framework. • Science Group Outcomes converted into Portfolio Outcomes Given the change in organizational structure, current Science Group outcomes have been converted into Portfolio Outcomes. The Science Group Outcomes had emphas ized ‘next user’
+---
+[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p9pt2]
+on the success of the Initiative/Impact Area Platform Annual Technical Reports, the following content areas will be included: Section # Section Title Content overview 1 Fact Sheet Key Program/Accelerator parameters including budget, target geographies, Centers involved, details of aligned W3 &amp; bilateral projects, funding allocated to Partners. 2 Executive summary A summary o</t>
+  </si>
+  <si>
     <t>[{"role": "system", "content": "You are a RAG assistant. Use ONLY the provided context as your source, without copying full sentences verbatim from chunks (max 10 consecutive words). Write clearly and cohesively, interpreting the usage context to adapt the response. Do not invent or extrapolate beyond the context and preserve acronyms EXACTLY as written. ALWAYS answer in English, regardless of the user's language. If there is insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'Output instructions:\n- 3 to 5 sentences, neutral and direct style, no lists.\n- ALWAYS answer in English and adapt wording to the question's context.\n- End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'.\n- If insufficient evidence, return EXACTLY: 'I cannot find information in the provided chunks to answer this.'\n\n"}, {"role": "user", "content": "Question: According to the Annex pie chart, what was total 2024 revenue and the split by funding source?\n\nContext:\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p6]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 6\nContent: Research results can be defined according to the nature of the change and the control over it.\n\n---\n\n[ID: docx:Guidance on reporting outputs or outcomes.docx:p14]\nFile: Guidance on reporting outputs or outcomes.docx\nLocation: paragraph 14\nContent: Figure 1: Research results according to the kind of change and the control over it.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p23]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 23\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 23 Annex 2: ISDC feedback relating to pooled &amp; non-pooled alignment5 This section provides a direct extract from the ISDC Feedback on CGIAR Portfolio Narrative 2025- 2030. Comments relating to the alignment of pooled and non -pooled have been extracted from the broader set of comments. They have not been edited to e.g. update Program and Accelerator nomenclature. • Articulation of how the Portfolio, including bilateral and W1 funding, will be bundled into Megaprograms is still lacking. Bilateral funding is restricted and is provided for a specific purpose and with specific intended impacts. This needs to be honored a nd the lack of flexibility in shifting those funds into other areas should be clearly acknowledged. • Alignment of the entire Portfolio with the CGIAR 2030 Research and Innovation Strategy needs to be strong and explicit. How will management ensure that bilateral funding delivers against this Strategy? In addition: o What happens if a bilateral project is not strongly aligned with the Strategy and how will CGIAR ensure that opportunity costs are covered? o Will all bilateral projects across all Centers be mapped to support the Portfolio? • A challenge that should be acknowledged is incorporating bilateral funding into Megaprograms. Each Megaprogram and Accelerator will be large scale and staff will be consumed by the implementation of contracted work. Trying to build Megaprogram linkages in parallel with bilateral funding should be additional, allowing sufficient effort dedicated to ensuring the prevention of silos within the new Portfolio. • Including bilateral funding into the organizational structure will be challenging. Clearly articulating the KPIs for this task for 2025 would be helpful. • The efforts needed to transition to Megaprograms are considerable and may be underestimated given the funding integration foreseen. Integration of pooled and bilateral at the reporting stage, as indicated, might be too late. Avoiding the duplication and ensuring clear implementation will be key. How will duplication of outputs/outcomes be avoided with both pooled and bilateral funding towards shared results? 5 ISDC Feedback on CGIAR Portfolio Narrative 2025-2030\n\n---\n\n[ID: pdf:Type3_2024Report.pdf:p5]\nFile: Type3_2024Report.pdf\nLocation: page 5\nContent: Section 2: Portfolio Performance and Project Coordination Progress 2. As per the Charter of the CGIAR System Organization, Article 8.2, and CGIAR’s Technical Reporting Arrangement 2022-2024. 3. Science Group Projects (SGPs) are Center-specific awards looking to integrate holistic quality assurance and implementation processes that build on efficiencies and value-for-money approaches through One CGIAR Common Systems and Window 1 budgeting practices. They operate under an integrated structure by Science Group, following similar principles and processes to Initiatives, while recognizing the role and responsibility of Centers for project delivery, compliance and fiduciary oversight. 4. EiB II will report through two Genetic Innovation Initiatives: Accelerated Breeding and Breeding Resources. For each Initiative report, they will provide a concise, high-level summary (approximately one page) outlining the contributions of the Gates Foundation-funded work toward the outcomes described in the technical reports. 2.1. Technical Reporting Arrangement 2022-24 CGIAR Technical Reporting fulfils the System-level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each Funder and the System Organization.2 The 2024 Technical Report includes the following Initiatives, Impact Platforms and SGPs3: • All 32 Initiatives • Five Impact Platforms – Gender Equality, Youth and Social Inclusion – Environmental Health and Biodiversity – Nutrition, Health and Food Security – Climate Adaptation and Mitigation – Poverty Reduction, Livelihoods and Jobs • Six SGPs – Accelerated Varietal Improvement and Seed Delivery of Legumes and dryland Cereals in Africa (AVISA) – Roots Tubers and Banana (RTB) Breeding – Accelerating Genetic Gain and Varietal Replacement in Rice - Phase 2 (AGGRi 2) – Excellence in Breeding (EiB) II: Cross-Crop Support Services for Breeding Acceleration4 – Accelerating Crop Improvement Through Genome Editing 2023-2025 – Climate Adaptation Insight For 2024, CGIAR will produce and deliver a total of 46 Technical Reporting outputs: • March 2025: Results from 2024 published on the online CGIAR Results Dashboard (1). • May 2025: Publication of 42 Type 1 (32 x Initiative reports; 5 x Impact Platform reports; 5 x SGP reports) Reports and a Type 3 Report (1). • End of June 2025: Publication of the Portfolio Narrative (1). • End of June 2025: Publication of the Type 2 Report: CGIAR Contributions to Impact in Agrifood Systems (2022-24) (1). Each of these reports is released separately and will be available in PDF format. 2024 Technical Reporting covers USD 370 million (USD 322 million for Initiatives and Impact Platforms, and USD 49 million for W3 SGPs), representing nearly 40 percent of CGIAR’s total pooled and non-pooled funding for 2024. 2.1.1. Streamlining the process and adding value to stakeholders In 2022 CGIAR launched a new 2022-24 Technical Reporting Arrangement, co-developed with the System Council’s Strategic Impact Monitoring and Evaluation Committee (SIMEC). The 2022 rollout was regarded as a “first pancake” or trial phase, establishing minimum viable functionality and setting the foundation for annual improvements. Key achievements of 2022 Technical Reporting included the adoption of a common report template aligned with the Technical Reporting Arrangement for Initiatives and Impact Platforms; integration with CGIAR’s Results Framework; digital linking of results to theories of change (TOCs); and the introduction of quality assurance processes mediated by third parties. Additionally, a new interactive CGIAR Results Dashboard was launched, and the Performance and Results Management System (PRMS) – an online reporting system – was developed, alongside adaptive management processes and the rollout of Innovation Packages and Scaling Readiness plans. Building on this, 2023 Technical Reporting incorporated lessons from a 2022 Learning and Optimization process, documented in a 2022 Learning and Optimization report. Key advancements included transitioning to “Always on” reporting by opening the PRMS from September 2023, more than doubling the reporting window compared to 2022 and allowing greater flexibility for Initiatives, Impact Platforms, and SGPs. Quality assurance was optimized through four staggered batches across 2023 and 2024. Further enhancements included expanding per-result tagging to all five Impact Areas. A Risk Management Module was launched to support risk identification and reporting at the Initiative level. A large number of participants joined training sessions to support reporting, dashboard use, and onboarding, and the rapid uptake of adaptive management strengthened strategic agility, with positive feedback from across the Portfolio. The Research Plans of Results and Budgets section of the CGIAR website was updated to ensure easy open access to Initiative, SGP and Impact Platform Plans of Results and Budgets (PORBs). The 2024 reporting cycle continued this trajectory, integrating insights from the 2023 Learning and Optimization process and Action Plan to further refine CGIAR’s Technical Reporting processes and products. Key improvements in 2024 included: • Launching the PRMS Planning Module to support the replan process: The launch of an online Planning Module synchronized TOC and Planning data in the PRMS, improving the efficiency and quality of planning workflows. Enhanced replan guidelines were provided to help Initiatives, Impact Platforms, and SGPs implement 2023 Reflect recommendations and align budget forecasts with updated budget envelopes. To support continuous learning and adaptive management, a user experience survey on the Planning Module was conducted to assess effectiveness and inform user-centered enhancements for the 2025-30 Portfolio. • Further simplifying reporting processes and tools: A series of enhancements to PRMS functionalities were implemented to improve efficiency and usability. Improved filtering options, enhanced notification systems, and more clearly structured result PDFs now enable quicker access to relevant information. Innovation Packages and Scaling Readiness language and templates were simplified. Reporting was streamlined and modified to suit the final year of reporting for the Portfolio, with an Outcome Indicator Module co-developed with input from Initiatives, Impact Platforms and SGPs to provide them with the opportunity to assess their progress against targets for Work Package outcomes and end-of-Initiative outcomes; summative and yearly highlights were combined into a single report; and adaptive management processes removed. • Improving decision-making within the PRMS: Broader engagement from PRMS testers across reporting entities and Senior Program Managers was integrated into PRMS feature development, ensuring that system updates were aligned with user needs and supported consistent decision-making. • Enhancing product clarity: The Type 1 Annual Report template was reviewed to better accommodate end-of-Initiative outcome reporting for the final year of the Portfolio. Improvements to the Results Dashboard were made to enhance the accessibility of IPSR insights. • Strengthening quality assurance: Examples include updated and enhanced QA guidance, and updated guidance on Impact Area tagging. An AI tool was prototyped and tested on a series of data fields, with the intent to leverage lessons learned and develop an enhanced AI tool that can be applied to a broader set of reported data and integrated into the PRMS, supporting both the reporting and QA phases. • Developing the Semantic Natural Language Processing Aggregator Platform (SNAP): SNAP is an AI-powered tool enhancing access to and analysis of CGIAR’s reported outputs, outcomes, and impacts. It improves access to Portfolio information and results evidence through semantic searches, thematic clustering, and automated summaries, complementing the CGIAR Results Dashboard. SNAP-supported narratives were integrated into the CGIAR 2024 Portfolio Narrative, and ongoing refinements will further enhance its role in Portfolio reporting. • Further integrating SGPs and Impact Platforms: Between 2022 and 2024, CGIAR progressively aligned these entities with its Technical Reporting processes and common systems to enhance consistency and coherence. In 2023, three Impact Platforms – Nutrition, Health and Food Security; Climate Adaptation and Mitigation; and Environmental Health and Biodiversity – were onboarded alongside the Gender Equality, Youth and Social Inclusion Impact Platform (which reported in 2022), each receiving tailored support such as TOC and results framework development. The SGP pilot launched in 2023 further expanded CGIAR’s reporting ecosystem by integrating Center-specific Window 3 awards, with two SGPs submitting first-year results using the PRMS Reporting Tool and Type 1 Report template. In 2024, integration expanded to include the Poverty Reduction, Livelihoods and Jobs Impact Platform and four additional SGPs, further broadening the reporting ecosystem. • Enhancing risk management through the PRMS Risk Module: The Risk Management Module, launched in 2023 to support Initiative management and reporting of risks, was further enhanced in 2024, allowing Initiatives to capture transition-focused risks. It enabled Initiatives to review, update, or close risks, contributing to the design of the 2025-30 Portfolio. The updated Risk Management Module will be used by Programs and Accelerators from 2025 onward. Climate-Smart Village set-up under the Adaptation and Mitigation Initiative in Agriculture (AMIA) of the Department of Agriculture. Credit: Miguel Mamon/CIAT May 2025 54 CGIAR Portfolio Practice Change (Type 3) Report 2024\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p4]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 4\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 4 1. Technical Reporting Arrangement purpose, scope, value proposition, delivery and optimization, Purpose The purpose of th e Technical Reporting Arrangement 2025 -2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. The TRA 25-30: • Provides the parameters that e nable the Centers, the CGIAR System Partners and the System Organization to fulfil their technical reporting obligations under the funding agreements that apply to the use of Window 1 and Window 2 funds from the CGIAR Trust Fund (“Pooled Funding”). These parameters also allow the Integrated Partnership Board to fulfil its responsibility under the CGIAR System Charter to report on programmatic performance of CGIAR Research on an annual basis. • Provides, through the establishment of common technical reporting principles, enabling tools and mechanisms, progressive alignment and synergy between the technical reporting requirements that apply to components of the CGIAR Portfolio that are funded by Pooled Funding and those that apply to the components that are funded by other sources of funds (“Non-Pooled Funding”). • Sets transparency, performance tracking, and accountability expectations between CGIAR System Funders and CGIAR including Centres, • Informs decision making at different levels, underpins research management, operationalizes the Performance and Results Management Framework (PRMF), and guides portfolio -level MELIA and the design of the next Performance and Results management System (PRMS). The current Technical Reporting Arrangement that applies to the CGIAR Portfolio during the period 2022-24 (“TRA 22-24”) was co-developed by CGIAR and System Council/Strategic Impact Monitoring and Evaluation Committee (SIMEC) members in 2022. A new TRA is needed to match 2025-30 portfolio parameters, notably the alignment of pooled and non-pooled funding sources, and to apply lessons learnt from 2022-24. Scope The TRA 25-30 provides the operational and enabling basis to plan, monitor, learn and report on the 25-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled, bilaterally and W3-funded components of the 2025- 30 portfolio in an integrated and aligned way, without increasing reporting burdens of Centers and Scientists. Going forward, the CGIAR Integrated Partnership will work towards progressively greater alignment of W3/bilateral projects and programs with the 2030 outcomes and theories of change of the Programs and Accelerators. Centers will provide key agreed information on their W3/bilaterally funded projects and programs to enable Program/Accelerator leaderships to explore ways to achieve alignment based on, inter alia, complementarity of results as well as actual or potential thematic, geographic, and partnership overlaps. Reporting on and attribution\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p5]\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 5\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 5 of results across different sources of funding will be set out as part of this Technical Reporting Arrangement. The Programs and Accelerators aim to provide frameworks for greater complementarity and synergy across different sources and types of funding (CGIAR Trust Fund Windows 1 -2, Window 3 and bilateral funding), while enhancing transparency and accountability. A n updated results framework, underpinned by a new Technical Reporting Arrangement, will provide robust, continuous performance and results reporting across all funding sources, as well as adaptive management of the Portfolio. 1 Value Proposition The TRA 25-30: - Creates value by delivering an integrated approach that tracks the performance of each Program and Accelerator, - Brings together the inputs (including costs), outputs, outcomes and impacts of the total portfolio to allow for easier and more robust Return on Investment (ROI) calculations. - Avoids creating a significant additional and duplicative layer of complex reporting requirements for W3/ bilaterally funded work. - Informs decision making through providing ready access to demand-driven quality raw and curated data products. Delivery The TRA 25 -30 will be delivered in line with Management arrangements for CGIAR’s 2025 —30 science and innovation Portfolio. Specific roles and responsibilities will be defined in 2025. 1 CGIAR Portfolio Narrative, 1 November 2024\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:p7]\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboard. You most probably have seen that. Reading. It also informs and are the results. The practices results are included in the annual report, in the portfolio narrative, and then in the overall CGIR annual report. In terms of the the timeline, so we have this info session now to provide an overview on the technical reporting and there will be several other info session and deep dive scheduled. Throughout September and October of reporting 2025 results, we believe that it will be feasible to open the PRMS in November for program and accelerators to to report. The date is still to be confirmed. We're aiming to to, yeah, to meet to to to end November. Hopefully this will be this is feasible from the technical side quality assurance. It's planned for February 2026 reflect process as I was mentioning Q 1/20/26 and then annual technical reports are due in March, April 2026 as well. Where to find information pertaining to technical reporting and planning and media? There is a one stop shop for for um all this. It's called the Performance and Results Hub. I'm gonna stop sharing cause I wanna share. Um, I'm gonna stop sharing the deck. I wanna. We could resent the hub. I'm not going to go through each section, but at least. So that you can see for those who are new more specifically to see and we will also share the link obviously the performance and results hub as I was mentioning it has detail on reporting, planning, reflect, replan. So you come in here, you click on 2025 reporting and then you will have access to the latest information, to the timeline, latest update, upcoming events. So all the information, information. Session dates will be listed here. We'll also have a subsection here with. Recording from from meetings, so that will be posted. For example today after this session we'll post a recording and the deck here for you to access and there is a section on frequently asked question. We recycled a couple of questions from the previous portfolio and updated them so that they are applicable to the program and accelerator teams, so feel free to go here and and browse. As resources become available, we will place them here and we will notify you by e-mail. OK. Going back to my deck. Which? In terms of engagement plan, so in order to streamline communication and optimize support for program accelerators and centers with mapped window 3 bilateral projects, we will send bi-weekly emails to everyone in this. This goal with key updates on technical reporting, with reminders and also with the latest questions and answers available on the hub. There will be targeted emails focusing on specific categories within the program accelerators. We want to engage with some of you on technical reporting, revisions, developments. And the aim is to gather feedback from you. Program coordinators will be copied on these emails. Info session. So a specific topic and we'll plan info session on specific topics, for example the standard indicator, description shades, the guidance on technical reporting, quality assurance. Reporting on innovations, the PRMS, so deep dive on the PRMS, the updates, the tool and so on. And during the reporting phase and the QA we will have weekly drop-ins. So this drop-ins is there will be no presentation. Presentation during the during this drop-ins. The purpose is for us to provide live support, so to answer your questions on the spot and the primary focus will be as I was mentioning, reporting and the QA. For if you know for every question you have, we invite you to use this e-mail address performanceandresults@cgr.org. This is the. The e-mail address we use for all technical reporting questions. So you have the questions right to us at performanceandresult@cjr.org and you will receive a response. We are aiming to respond within the 24 hours. Just to give an example, you know going back here I've gotten the targeted targeted emails and feedback. So this is a good example on for example how we plan to engage and get get feedback from from you on the PRMS enhancements so. Usually we send there's an e-mail sent to invite you to provide feedback on a o</t>
   </si>
   <si>
@@ -2819,6 +3653,30 @@
   </si>
   <si>
     <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: Who is responsible for approving changes to reporting categories and for balancing the benefits of collecting detailed information against the reporting burden on P/A? \n\nContext:\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u7-10]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 8 to paragraph 11\nContent: Governance: Q: Who is responsible for approving changes to reporting categories and for balancing the benefits of collecting detailed information against the reporting burden on P/A? A: Ahead of each reporting cycle, CGIAR organizes focus group discussions, workshops, and individual meetings with donors and stakeholders (e.g., Initiative/Program leads/co-leads, MELIA experts, SO MEL, IPSR team, and Center representatives). Through these exchanges, feedback is collected on which reporting fields are valuable to keep, remove, or add, ensuring both alignment with CGIAR’s strategy and responsiveness to donor requirements. This input is then prioritized based on feasibility and strategic relevance, with decisions documented in the annual Learning &amp; Optimization (L&amp;O) report. In practice, adjustments to reporting categories are made through this iterative process of consultation, review, and refinement.\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 1 part 4\nContent: Reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 2\nContent: Reporting High\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p12pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 12 part 2\nContent: a new category. • 'Other' result categories to be better defined 2022-24 results reported in the ‘Other’ output and outcome categories are by definition a mixed bag, however do point to the need for a specific new category on partner engagement/ partnership building. Improved guidance on the use of the ‘Other’ categories has been available since mid-2024 and we will continue to improve guidance and support to results submitters. • Continuation and optimization of existing Genebank data integration Existing data flow from the Genebanks’ Online Reporting Tool (ORT), powering the CGIAR Results Dashboard Genebanks section will continue. Optimization of those data flows will form part of ongoing engagement with the Genebanks. • Streamline results reporting requirements The reporting burden will be minimized by a) critically assessing each data field against requirements, b)\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p12pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 12 part 2\nContent: a new category. • 'Other' result categories to be better defined 2022-24 results reported in the ‘Other’ output and outcome categories are by definition a mixed bag, however do point to the need for a specific new category on partner engagement/ partnership building. Improved guidance on the use of the ‘Other’ categories has been available since mid-2024 and we will continue to improve guidance and support to results submitters. • Continuation and optimization of existing Genebank data integration Existing data flow from the Genebanks’ Online Reporting Tool (ORT), powering the CGIAR Results Dashboard Genebanks section will continue. Optimization of those data flows will form part of ongoing engagement with the Genebanks. • Streamline results reporting requirements The reporting burden will be minimized by a) critically assessing each data field against requirements, b)\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u4-7]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 4 to paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:04 5 minutes and then we will move into. I will leave the floor for your questions if that's OK. OK. Presentation mode. This means I no longer see the chat, the questions in the chat, or if hands are raised. So please interrupt me if you have questions or if you you know you you don't see the deck or anything else. I would like to welcome everyone and thank you for joining today's session on the 2025 Technical Reporting. My name is Nicoletta Trifa. I'm part of the Portfolio Performance Unit, a support unit within the Office of the Chief Scientist. This session is the second of two plan, two session plans for today, planned for today. We had an another session this morning to accommodate colleagues in other time zones. Um. Coming straight to the agenda, here's an overview of of what I'm going to cover in the next couple of minutes. So I will provide an update on the technical reporting arrangements. We'll discuss priorities and changes for 2025 technical reporting. A brief introduction on the annual Technical reports and the enablers, so being the Performance and Reporting Management System and the quality assurance, Technical reporting timeline, available resources and support and also what's what's next and how to stay engaged. This session marks the start of the conversation around 2025 Technical reporting. We want to give you the early look at the key priorities and plans for the months ahead. The goal is to make sure that you all stay informed, prepared and supported. With a clear understanding of deliverables and timelines that it is clear for you who to reach out to in case you have questions or in case you need help along the way. Some of the people in this call are already familiar with the technical reporting arrangements. From the previous portfolio, while for others this might be entirely new. Our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, with this let me kick off. So the technical reporting arrangements for the new portfolio, the 2025 to 2030 portfolio has been approved by CJRGLD, so Global Leadership Team in June 2025. And provides the operational basis to plan, monitor, learn and report on the new portfolio. It is designed to progressively enable programs and accelerators and centres to report on the pooled and the Window 3 Bilateral projects. In an aligned and integrated way without increasing reporting burdens on centers or on the scientist. Main changes compared to previous technical reporting arrangement. So the focus will be on streamlined reporting, less products, more integration, lower transaction costs, stronger impact focus results to be clearly linked. To impact outcomes and their associated indicator targets and also better linkages between the annual program and accelerator theory of change, final results and budget, media and technical reporting. The primary audiences for technical reporting are funders and CGR staff at the Integrated Partnership, Portfolio and Program and Accelerator levels. A secondary audience is the partners. The Annual Technical Reporting covers the program and Accelerators Annual Technical Reports and the Portfolio Narrative report, which provides an overall view to thematic and geographic targets. Relevant components of the technical reporting products are also integrated into the CGR corporate reporting, so CGR annual report. 2025 priorities for technical reporting. So 2025 is a transition year. I believe everyone has a line on this being a transition year with the technical reporting arrangements, implementation focusing again as I mentioned on streamlined reporting. And also on strengthening linkages between the theory of change, the poor media and technical reporting. Many of you know are aware that. These components were not properly linked in the previous portfolio, so it was challenging to demonstrate progress against plans against theory of change. In terms of deliverables for 2025, these are the program and the accelerator technical reports which are due in. April 2026 A Portfolio Narrative report which is due in June 2026 Integration of top 80% window 3 bilateral projects by center and dollar value into technical reporting and planning. Application of the minimum data standards for window 3 and bilateral reporting and mapping refinement which will take place during reflect early Q12026. So as I was mentioning 2025 transition year toward KPI based planning and reporting. So efforts are underway to enable planning and reporting at the KPI level and this is aligned with the System Office objectives and key results for 2026 and 20. 2027 I've listed them here on the slide, but be mindful that these are to be confirmed, so not confirmed yet. So uh for 2026 OK Rs. 100 of Program Accelerator. PRBS and the Annual Technical Reporting starting with the 2026 will provide monitoring of performance and result against Smart KPIs by center, by year, by pooled fund invested. So for 2026, the aim is to have 80% of centers, window free and bilateral projects included in 2025 Technical reports, while for 2027 this will increase to 90% of center window free and bilateral projects included in 2026. Technical reports. Yep. Specifically for programs and accelerators deliverables, here the focus is on three key deliverables. So first one being reporting the 2025 results in the Performance and Reporting Management System, the PRMS. Programs and accelerators are strongly encouraged to report results that were planned and budgeted, so included in their PORB, since the technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of the reported reported results. The 2025 results will be quality assessed following a defined process and timeline. Once this is done, the quality assessed results will be available on the Results dashboard and it will also be available for you to inform, pause and reflect. And to fill into your technical reports and to your annual technical reports. A third deliverable is drafting and submission of the 2025 Annual Technical Report. So each program and accelerators is responsible for drafting and internally validating quality assessing their. Annual Technical Report before submitting it to to us to the PPU. To support this process, this year we will have an AI generated V0 draft of this report which will include pre-filled text, some narrative and analytics for each report section. And this will be available for you as a starting point to further refine and and finalize your annual technical report. On the three deliverables, I want to mention that we will plan in September, October specific info session. So there will be info session on PRMS. Like a deep dive on PRMS, there will be a deep dive on quality assurance and the process timeline, who does what and so on, and also a deep dive on the Annual Technical Report to further make you familiar with its content, the internal approval process. The external approval process, I mean by external, I mean outside of program and accelerator approval process, what will be available, where AI will help and so on. So more information on this will come. For the annual technical report, what are these? These reports provide assurance on the annual program and accelerator delivery against PORP and progress on theory of change. They are short, concise and targeted. They are based on the quality assess results. The requirement is to have this report submitted in April and then the aim is to publish them early May as I was mentioning template guidance and and. A I generated V0 report will be will be provided to You to the right on the right side of the screen You can see that the content areas of the annual Technical report. This is extracted from the Technical reporting arrangements document and IT has it's very similar to what we had for the initiatives and impact platforms in the previous portfolio. So You have a fact sheet, an executive summary, annual progress area for work details. A Results section, Partnerships, Portfolio Linkages, Adaptive Management and then Key Results story. For reference or especially for for People new to Technical reporting, which who want You to have a look at, You know how this this reports might look like in the end. I've I've pasted here the. Annual reports from initiatives, impact platforms and science Group projects from 2024, SO from this year and You also have a link to the Portfolio narrative report. And the Type 2 report, sorry, the Type 2 impact report, which is drafted every three years. The System where this will take Place with reporting will take place. It's called Performance and Results Management System, PRMS in short. We are currently validating the PRMS roles, SO we have reached out to Program Coordinators and asked them to. Give us the name and the role of the People in their teams which will be involved in Technical reporting. A reminder on this will be sent on Thursday to finalize the process and this will enable the Technical Team to. Create proper accesses in the System when the reporting period starts. Similar to previous information, SO we are working to to to draft the new users onboarding deck where You can find relevant information on PRMS and. We will keep You updated on what's new in the pyramids or on the enhancements that we're working on this year as we advance towards Technical reporting to the reporting period later in the year. Quality assurance process what IT is. So Results submitted by programs and accelerators in the PRMS are quality assessed by QA Team in February 2026. Your participation in this process is required. Guidance and resources will be provided and then also as I was mentioning, an info session will be scheduled for September, October. What is QA? It is a process that aims to improve the quality of reported data, to provide consistency across the system, to ensure reliability of reported results, inform learning, and overall improve CGR accountability and transparency. Quality assessed data, SO the Results quality assessed inform the reflect process. They Go into the Results dashboard. They are also featured in the annual reports in the Portfolio narrative and then further into the CJR corporate report. And oh, there's I I only noticed now the title says 2024. Apologies for this. It's 2025 Technical reporting timeline. This is a print screenshot of. Same information that can be seen on the PNR hub. So we have the first info session on Technical reporting now in July, August through November. We will engage Program accelerators and centers, media People in preparation of. Various guidance materials, testing, PRMS enhancement. We'll plan information sessions which will take Place in September, October to make sure that we everyone is properly prepared for the reporting period. Reporting 2025 results. Our intent is to open PRMS in November. Let's see how how well we advance with the changes to the System again 2025. Is a Transition year. There are many changes to be done since we moved from 1 Portfolio to another, many adjustments which need to take Place in the system, but hopefully in November we can open reporting on 2025 results. We will keep You updated on this though. Quality assurance will take Place as mentioned in February 2026. Reflect same thing will take Place in Q 1/20/26. And then the annual Technical reports are due in in April, in March, April for publication early May. The Performance and Results Hub is your one-stop shop for planning, Technical reporting and managing information. You'll find I want to stop sharing this deck for now and I want to. Take You to the PNR hub. Let me know if You see when I switch screens. Rose, Sabrina ( Alliance Bioversity-CIAT) 16:48 Yes, we can see. Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source.\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pause and reflect and will be included in the technical reports in the annual technical reports. A third deliverable for program and accelerators is drafting estimation of the 2025 Annual Technical Report. So each program and accelerator is responsible for drafting and internally validating quality assessing their 2025 Annual Technical Report. Before submitting it to the PPU, so to the perform portfolio performance unit. Again, guidance on this, the detailed process and validation process will be shared with you timely. Also to support this process, an AI generated V0 draft will be provided as a starting point. The annual technical reports. What are they? This the annual technical report. The the the aim is to make them short, so to 20 to 30 pages, concise and targeted. They provide assurance on annual program accelerator delivery against the boards, so plan of results and budget and progress on theory of change. They are based on quality assess results, the template guidance and as I mentioned and. AI V0 will be provided to all rogram and accelerator teams. Annual technical reports need to be submitted by each program and accelerator in March, April, so more details on this will follow and publication is intended to happen end of April, beginning of May. Here to the right side you have the. Content of the annual the proposed content for the annual technical report as per the technical reporting arrangements. Many of you will notice that there are not no big changes compared to previous portfolio, so the idea is to have a fact sheet and executive summary. The annual progress on theory of change, area of work details, a section on results, section on partnerships, portfolio linkages, adaptive management and then one key result story. But again, we will plan a detailed deep dive session on the annual technical report template and the guidance. So there will be time for you to ask questions in detail about about this and to receive support obviously. I've also included here for reference links to the 2024 Annual Technical Reports from the initiatives and impact platforms, and also a link to the 2024 Portfolio Narrative Report. In case you want to, you want to have a look to see, um, what it captures. PRMS. So this stands for Performance and Results Management System is the system the the the the environment where results need to be submitted. Again, the team is working on updating their resources. There will be. New users onboarding decks created with the links to different information and I I believe the PCU Alison together with the program coordinators. Are. The all the PRMS roles. So PCU is leading a work to define the PRMS roles and to get the information from program and accelerators regarding who from each program accelerator should have what role in PRMS. To enable us to to provide the right access to the platform when the time comes to report. Quality assurance process. So results submitted by program and accelerators in the PRMS will be quality assessed by a quality assessment team in February 2026. Your participation in this process is required. Guidance and resource resources will be provided and also an info session will be scheduled later this year. What is the QA? It is a process that aims to improve the quality of the reported data to provide consistency across the system, ensure reliability of reported results. Inform the learning process and improve the overall CGR accountability and transparency. Quality assess data informs the reflect process which takes place early Q12026, the results dashboard. So once the quality assessment of the results is finalized, the quality assess results will be pushed to results dashboa</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: What are the 2025 reporting timelines?\n\nContext:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 4\nContent: Reporting timeline\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 1 part 4\nContent: Reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 2\nContent: Reporting High\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 1\nContent: 2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 10 part 3\nContent: information. Technical Reporting resources HOW Latest updates Timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:General information on Technical Reporting .docx:u1-6]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General information on Technical Reporting .docx\nLocation: paragraph 1 to paragraph 7\nContent: General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 21 part 2\nContent: course correction, while an annual MELIA report (December) documents how learning drives adaptive decisions and improved program performance. 7. Reporting The SFP MELIA plan includes a reporting structure that adheres to the CGIAR Technical Reporting Arrangement and ensures accountability, learning, and adaptive management across the Program. Reporting will be structured around the results framework (which has been aligned with the CGIAR Results Framework and Theory of Change (ToC) which also aligns with the PRMS ToC Board structure, encompassing High-Level Outputs (HLOs), intermediate outcomes, and 2030 outcomes and contributions to Impact Areas and SDGs . The reporting process will be aligned with the CGIAR Technical Reporting Arrangement, adhering to the annual reporting timelines, templates and Performance Results Management System (PRMS) requirements, including results of W3/bilateral projects mapped to SFP . Evidence for reporting will be\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u4-7]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 4 to paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:04 5 minutes and then we will move into. I will leave the floor for your questions if that's OK. OK. Presentation mode. This means I no longer see the chat, the questions in the chat, or if hands are raised. So please interrupt me if you have questions or if you you know you you don't see the deck or anything else. I would like to welcome everyone and thank you for joining today's session on the 2025 Technical Reporting. My name is Nicoletta Trifa. I'm part of the Portfolio Performance Unit, a support unit within the Office of the Chief Scientist. This session is the second of two plan, two session plans for today, planned for today. We had an another session this morning to accommodate colleagues in other time zones. Um. Coming straight to the agenda, here's an overview of of what I'm going to cover in the next couple of minutes. So I will provide an update on the technical reporting arrangements. We'll discuss priorities and changes for 2025 technical reporting. A brief introduction on the annual Technical reports and the enablers, so being the Performance and Reporting Management System and the quality assurance, Technical reporting timeline, available resources and support and also what's what's next and how to stay engaged. This session marks the start of the conversation around 2025 Technical reporting. We want to give you the early look at the key priorities and plans for the months ahead. The goal is to make sure that you all stay informed, prepared and supported. With a clear understanding of deliverables and timelines that it is clear for you who to reach out to in case you have questions or in case you need help along the way. Some of the people in this call are already familiar with the technical reporting arrangements. From the previous portfolio, while for others this might be entirely new. Our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, with this let me kick off. So the technical reporting arrangements for the new portfolio, the 2025 to 2030 portfolio has been approved by CJRGLD, so Global Leadership Team in June 2025. And provides the operational basis to plan, monitor, learn and report on the new portfolio. It is designed to progressively enable programs and accelerators and centres to report on the pooled and the Window 3 Bilateral projects. In an aligned and integrated way without increasing reporting burdens on centers or on the scientist. Main changes compared to previous technical reporting arrangement. So the focus will be on streamlined reporting, less products, more integration, lower transaction costs, stronger impact focus results to be clearly linked. To impact outcomes and their associated indicator targets and also better linkages between the annual program and accelerator theory of change, final results and budget, media and technical reporting. The primary audiences for technical reporting are funders and CGR staff at the Integrated Partnership, Portfolio and Program and Accelerator levels. A secondary audience is the partners. The Annual Technical Reporting covers the program and Accelerators Annual Technical Reports and the Portfolio Narrative report, which provides an overall view to thematic and geographic targets. Relevant components of the technical reporting products are also integrated into the CGR corporate reporting, so CGR annual report. 2025 priorities for technical reporting. So 2025 is a transition year. I believe everyone has a line on this being a transition year with the technical reporting arrangements, implementation focusing again as I mentioned on streamlined reporting. And also on strengthening linkages between the theory of change, the poor media and technical reporting. Many of you know are aware that. These components were not properly linked in the previous portfolio, so it was challenging to demonstrate progress against plans against theory of change. In terms of deliverables for 2025, these are the program and the accelerator technical reports which are due in. April 2026 A Portfolio Narrative report which is due in June 2026 Integration of top 80% window 3 bilateral projects by center and dollar value into technical reporting and planning. Application of the minimum data standards for window 3 and bilateral reporting and mapping refinement which will take place during reflect early Q12026. So as I was mentioning 2025 transition year toward KPI based planning and reporting. So efforts are underway to enable planning and reporting at the KPI level and this is aligned with the System Office objectives and key results for 2026 and 20. 2027 I've listed them here on the slide, but be mindful that these are to be confirmed, so not confirmed yet. So uh for 2026 OK Rs. 100 of Program Accelerator. PRBS and the Annual Technical Reporting starting with the 2026 will provide monitoring of performance and result against Smart KPIs by center, by year, by pooled fund invested. So for 2026, the aim is to have 80% of centers, window free and bilateral projects included in 2025 Technical reports, while for 2027 this will increase to 90% of center window free and bilateral projects included in 2026. Technical reports. Yep. Specifically for programs and accelerators deliverables, here the focus is on three key deliverables. So first one being reporting the 2025 results in the Performance and Reporting Management System, the PRMS. Programs and accelerators are strongly encouraged to report results that were planned and budgeted, so included in their PORB, since the technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of the reported reported results. The 2025 results will be quality assessed following a defined process and timeline. Once this is done, the quality assessed results will be available on the Results dashboard and it will also be available for you to inform, pause and reflect. And to fill into your technical reports and to your annual technical reports. A third deliverable is drafting and submission of the 2025 Annual Technical Report. So each program and accelerators is responsible for drafting and internally validating quality assessing their. Annual Technical Report before submitting it to to us to the PPU. To support this process, this year we will have an AI generated V0 draft of this report which will include pre-filled text, some narrative and analytics for each report section. And this will be available for you as a starting point to further refine and and finalize your annual technical report. On the three deliverables, I want to mention that we will plan in September, October specific info session. So there will be info session on PRMS. Like a deep dive on PRMS, there will be a deep dive on quality assurance and the process timeline, who does what and so on, and also a deep dive on the Annual Technical Report to further make you familiar with its content, the internal approval process. The external approval process, I mean by external, I mean outside of program and accelerator approval process, what will be available, where AI will help and so on. So more information on this will come. For the annual technical report, what are these? These reports provide assurance on the annual program and accelerator delivery against PORP and progress on theory of change. They are short, concise and targeted. They are based on the quality assess results. The requirement is to have this report submitted in April and then the aim is to publish them early May as I was mentioning template guidance and and. A I generated V0 report will be will be provided to You to the right on the right side of the screen You can see that the content areas of the annual Technical report. This is extracted from the Technical reporting arrangements document and IT has it's very similar to what we had for the initiatives and impact platforms in the previous portfolio. So You have a fact sheet, an executive summary, annual progress area for work details. A Results section, Partnerships, Portfolio Linkages, Adaptive Management and then Key Results story. For reference or especially for for People new to Technical reporting, which who want You to have a look at, You know how this this reports might look like in the end. I've I've pasted here the. Annual reports from initiatives, impact platforms and science Group projects from 2024, SO from this year and You also have a link to the Portfolio narrative report. And the Type 2 report, sorry, the Type 2 impact report, which is drafted every three years. The System where this will take Place with reporting will take place. It's called Performance and Results Management System, PRMS in short. We are currently validating the PRMS roles, SO we have reached out to Program Coordinators and asked them to. Give us the name and the role of the People in their teams which will be involved in Technical reporting. A reminder on this will be sent on Thursday to finalize the process and this will enable the Technical Team to. Create proper accesses in the System when the reporting period starts. Similar to previous information, SO we are working to to to draft the new users onboarding deck where You can find relevant information on PRMS and. We will keep You updated on what's new in the pyramids or on the enhancements that we're working on this year as we advance towards Technical reporting to the reporting period later in the year. Quality assurance process what IT is. So Results submitted by programs and accelerators in the PRMS are quality assessed by QA Team in February 2026. Your participation in this process is required. Guidance and resources will be provided and then also as I was mentioning, an info session will be scheduled for September, October. What is QA? It is a process that aims to improve the quality of reported data, to provide consistency across the system, to ensure reliability of reported results, inform learning, and overall improve CGR accountability and transparency. Quality assessed data, SO the Results quality assessed inform the reflect process. They Go into the Results dashboard. They are also featured in the annual reports in the Portfolio narrative and then further into the CJR corporate report. And oh, there's I I only noticed now the title says 2024. Apologies for this. It's 2025 Technical reporting timeline. This is a print screenshot of. Same information that can be seen on the PNR hub. So we have the first info session on Technical reporting now in July, August through November. We will engage Program accelerators and centers, media People in preparation of. Various guidance materials, testing, PRMS enhancement. We'll plan information sessions which will take Place in September, October to make sure that we everyone is properly prepared for the reporting period. Reporting 2025 results. Our intent is to open PRMS in November. Let's see how how well we advance with the changes to the System again 2025. Is a Transition year. There are many changes to be done since we moved from 1 Portfolio to another, many adjustments which need to take Place in the system, but hopefully in November we can open reporting on 2025 results. We will keep You updated on this though. Quality assurance will take Place as mentioned in February 2026. Reflect same thing will take Place in Q 1/20/26. And then the annual Technical reports are due in in April, in March, April for publication early May. The Performance and Results Hub is your one-stop shop for planning, Technical reporting and managing information. You'll find I want to stop sharing this deck for now and I want to. Take You to the PNR hub. Let me know if You see when I switch screens. Rose, Sabrina ( Alliance Bioversity-CIAT) 16:48 Yes, we can see. Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 3\nContent: System (PRMS) Quality Assurance When Technical Reporting timeline How Resources Engagement\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 2\nContent: 2025 Technical Reporting Portfolio\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u13-16]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'A single location for all documents and resources' paragraph 25 to section 'A single location for all documents and resources' paragraph 31\nContent: The Performance and Results (P&amp;R) Hub will serve as the central repository for all materials related to Technical Reporting. This includes timelines, guidance documents, templates, updates, frequently asked questions (FAQs), and other relevant resources to support Programs and Accelerators throughout the reporting cycle. The Hub is structured around key phases of the reporting process, with dedicated pages for planning, reporting, and reflect/re-planning, making it easier for users to find what they need at each stage. The content and structure of the P&amp;R Hub have been reviewed and updated based on: Changes to the Technical Reporting process\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 1 to paragraph 4\nContent: Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u4-7]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 4 to paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:03 Will be available on the Performance and Results Hub later today and also will be shared by e-mail by the end of this week. Good. OK, so we can start. Welcome everyone. Thank you for joining today's session on the 2025 technical reporting. I'm going to share my screen. As I was mentioning, I have a couple of slides I want to share with you. She moved. I do not see the chat or hands raised or anything, so please let me know if you get if you can see my slide. Colomer, Julien (One CGIAR - France) 0:47 Yep. Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of re</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a helpful assistant that answers very detailedly to user questions"}, {"role": "user", "content": "Question: What are the 2025 reporting timelines?\n\nContext:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 4\nContent: Reporting timeline\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s1pt4]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 1 part 4\nContent: Reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 2\nContent: Reporting High\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 1\nContent: 2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 10 part 3\nContent: information. Technical Reporting resources HOW Latest updates Timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:General information on Technical Reporting .docx:u1-6]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General information on Technical Reporting .docx\nLocation: paragraph 1 to paragraph 7\nContent: General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 21 part 2\nContent: course correction, while an annual MELIA report (December) documents how learning drives adaptive decisions and improved program performance. 7. Reporting The SFP MELIA plan includes a reporting structure that adheres to the CGIAR Technical Reporting Arrangement and ensures accountability, learning, and adaptive management across the Program. Reporting will be structured around the results framework (which has been aligned with the CGIAR Results Framework and Theory of Change (ToC) which also aligns with the PRMS ToC Board structure, encompassing High-Level Outputs (HLOs), intermediate outcomes, and 2030 outcomes and contributions to Impact Areas and SDGs . The reporting process will be aligned with the CGIAR Technical Reporting Arrangement, adhering to the annual reporting timelines, templates and Performance Results Management System (PRMS) requirements, including results of W3/bilateral projects mapped to SFP . Evidence for reporting will be\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u4-7]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 4 to paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:04 5 minutes and then we will move into. I will leave the floor for your questions if that's OK. OK. Presentation mode. This means I no longer see the chat, the questions in the chat, or if hands are raised. So please interrupt me if you have questions or if you you know you you don't see the deck or anything else. I would like to welcome everyone and thank you for joining today's session on the 2025 Technical Reporting. My name is Nicoletta Trifa. I'm part of the Portfolio Performance Unit, a support unit within the Office of the Chief Scientist. This session is the second of two plan, two session plans for today, planned for today. We had an another session this morning to accommodate colleagues in other time zones. Um. Coming straight to the agenda, here's an overview of of what I'm going to cover in the next couple of minutes. So I will provide an update on the technical reporting arrangements. We'll discuss priorities and changes for 2025 technical reporting. A brief introduction on the annual Technical reports and the enablers, so being the Performance and Reporting Management System and the quality assurance, Technical reporting timeline, available resources and support and also what's what's next and how to stay engaged. This session marks the start of the conversation around 2025 Technical reporting. We want to give you the early look at the key priorities and plans for the months ahead. The goal is to make sure that you all stay informed, prepared and supported. With a clear understanding of deliverables and timelines that it is clear for you who to reach out to in case you have questions or in case you need help along the way. Some of the people in this call are already familiar with the technical reporting arrangements. From the previous portfolio, while for others this might be entirely new. Our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, with this let me kick off. So the technical reporting arrangements for the new portfolio, the 2025 to 2030 portfolio has been approved by CJRGLD, so Global Leadership Team in June 2025. And provides the operational basis to plan, monitor, learn and report on the new portfolio. It is designed to progressively enable programs and accelerators and centres to report on the pooled and the Window 3 Bilateral projects. In an aligned and integrated way without increasing reporting burdens on centers or on the scientist. Main changes compared to previous technical reporting arrangement. So the focus will be on streamlined reporting, less products, more integration, lower transaction costs, stronger impact focus results to be clearly linked. To impact outcomes and their associated indicator targets and also better linkages between the annual program and accelerator theory of change, final results and budget, media and technical reporting. The primary audiences for technical reporting are funders and CGR staff at the Integrated Partnership, Portfolio and Program and Accelerator levels. A secondary audience is the partners. The Annual Technical Reporting covers the program and Accelerators Annual Technical Reports and the Portfolio Narrative report, which provides an overall view to thematic and geographic targets. Relevant components of the technical reporting products are also integrated into the CGR corporate reporting, so CGR annual report. 2025 priorities for technical reporting. So 2025 is a transition year. I believe everyone has a line on this being a transition year with the technical reporting arrangements, implementation focusing again as I mentioned on streamlined reporting. And also on strengthening linkages between the theory of change, the poor media and technical reporting. Many of you know are aware that. These components were not properly linked in the previous portfolio, so it was challenging to demonstrate progress against plans against theory of change. In terms of deliverables for 2025, these are the program and the accelerator technical reports which are due in. April 2026 A Portfolio Narrative report which is due in June 2026 Integration of top 80% window 3 bilateral projects by center and dollar value into technical reporting and planning. Application of the minimum data standards for window 3 and bilateral reporting and mapping refinement which will take place during reflect early Q12026. So as I was mentioning 2025 transition year toward KPI based planning and reporting. So efforts are underway to enable planning and reporting at the KPI level and this is aligned with the System Office objectives and key results for 2026 and 20. 2027 I've listed them here on the slide, but be mindful that these are to be confirmed, so not confirmed yet. So uh for 2026 OK Rs. 100 of Program Accelerator. PRBS and the Annual Technical Reporting starting with the 2026 will provide monitoring of performance and result against Smart KPIs by center, by year, by pooled fund invested. So for 2026, the aim is to have 80% of centers, window free and bilateral projects included in 2025 Technical reports, while for 2027 this will increase to 90% of center window free and bilateral projects included in 2026. Technical reports. Yep. Specifically for programs and accelerators deliverables, here the focus is on three key deliverables. So first one being reporting the 2025 results in the Performance and Reporting Management System, the PRMS. Programs and accelerators are strongly encouraged to report results that were planned and budgeted, so included in their PORB, since the technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of the reported reported results. The 2025 results will be quality assessed following a defined process and timeline. Once this is done, the quality assessed results will be available on the Results dashboard and it will also be available for you to inform, pause and reflect. And to fill into your technical reports and to your annual technical reports. A third deliverable is drafting and submission of the 2025 Annual Technical Report. So each program and accelerators is responsible for drafting and internally validating quality assessing their. Annual Technical Report before submitting it to to us to the PPU. To support this process, this year we will have an AI generated V0 draft of this report which will include pre-filled text, some narrative and analytics for each report section. And this will be available for you as a starting point to further refine and and finalize your annual technical report. On the three deliverables, I want to mention that we will plan in September, October specific info session. So there will be info session on PRMS. Like a deep dive on PRMS, there will be a deep dive on quality assurance and the process timeline, who does what and so on, and also a deep dive on the Annual Technical Report to further make you familiar with its content, the internal approval process. The external approval process, I mean by external, I mean outside of program and accelerator approval process, what will be available, where AI will help and so on. So more information on this will come. For the annual technical report, what are these? These reports provide assurance on the annual program and accelerator delivery against PORP and progress on theory of change. They are short, concise and targeted. They are based on the quality assess results. The requirement is to have this report submitted in April and then the aim is to publish them early May as I was mentioning template guidance and and. A I generated V0 report will be will be provided to You to the right on the right side of the screen You can see that the content areas of the annual Technical report. This is extracted from the Technical reporting arrangements document and IT has it's very similar to what we had for the initiatives and impact platforms in the previous portfolio. So You have a fact sheet, an executive summary, annual progress area for work details. A Results section, Partnerships, Portfolio Linkages, Adaptive Management and then Key Results story. For reference or especially for for People new to Technical reporting, which who want You to have a look at, You know how this this reports might look like in the end. I've I've pasted here the. Annual reports from initiatives, impact platforms and science Group projects from 2024, SO from this year and You also have a link to the Portfolio narrative report. And the Type 2 report, sorry, the Type 2 impact report, which is drafted every three years. The System where this will take Place with reporting will take place. It's called Performance and Results Management System, PRMS in short. We are currently validating the PRMS roles, SO we have reached out to Program Coordinators and asked them to. Give us the name and the role of the People in their teams which will be involved in Technical reporting. A reminder on this will be sent on Thursday to finalize the process and this will enable the Technical Team to. Create proper accesses in the System when the reporting period starts. Similar to previous information, SO we are working to to to draft the new users onboarding deck where You can find relevant information on PRMS and. We will keep You updated on what's new in the pyramids or on the enhancements that we're working on this year as we advance towards Technical reporting to the reporting period later in the year. Quality assurance process what IT is. So Results submitted by programs and accelerators in the PRMS are quality assessed by QA Team in February 2026. Your participation in this process is required. Guidance and resources will be provided and then also as I was mentioning, an info session will be scheduled for September, October. What is QA? It is a process that aims to improve the quality of reported data, to provide consistency across the system, to ensure reliability of reported results, inform learning, and overall improve CGR accountability and transparency. Quality assessed data, SO the Results quality assessed inform the reflect process. They Go into the Results dashboard. They are also featured in the annual reports in the Portfolio narrative and then further into the CJR corporate report. And oh, there's I I only noticed now the title says 2024. Apologies for this. It's 2025 Technical reporting timeline. This is a print screenshot of. Same information that can be seen on the PNR hub. So we have the first info session on Technical reporting now in July, August through November. We will engage Program accelerators and centers, media People in preparation of. Various guidance materials, testing, PRMS enhancement. We'll plan information sessions which will take Place in September, October to make sure that we everyone is properly prepared for the reporting period. Reporting 2025 results. Our intent is to open PRMS in November. Let's see how how well we advance with the changes to the System again 2025. Is a Transition year. There are many changes to be done since we moved from 1 Portfolio to another, many adjustments which need to take Place in the system, but hopefully in November we can open reporting on 2025 results. We will keep You updated on this though. Quality assurance will take Place as mentioned in February 2026. Reflect same thing will take Place in Q 1/20/26. And then the annual Technical reports are due in in April, in March, April for publication early May. The Performance and Results Hub is your one-stop shop for planning, Technical reporting and managing information. You'll find I want to stop sharing this deck for now and I want to. Take You to the PNR hub. Let me know if You see when I switch screens. Rose, Sabrina ( Alliance Bioversity-CIAT) 16:48 Yes, we can see. Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 3\nContent: System (PRMS) Quality Assurance When Technical Reporting timeline How Resources Engagement\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 2\nContent: 2025 Technical Reporting Portfolio\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u13-16]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'A single location for all documents and resources' paragraph 25 to section 'A single location for all documents and resources' paragraph 31\nContent: The Performance and Results (P&amp;R) Hub will serve as the central repository for all materials related to Technical Reporting. This includes timelines, guidance documents, templates, updates, frequently asked questions (FAQs), and other relevant resources to support Programs and Accelerators throughout the reporting cycle. The Hub is structured around key phases of the reporting process, with dedicated pages for planning, reporting, and reflect/re-planning, making it easier for users to find what they need at each stage. The content and structure of the P&amp;R Hub have been reviewed and updated based on: Changes to the Technical Reporting process\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 1 to paragraph 4\nContent: Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u4-7]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 4 to paragraph 7\nContent: Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción Trifa, Nicoleta (CGIAR System Organization) 0:03 Will be available on the Performance and Results Hub later today and also will be shared by e-mail by the end of this week. Good. OK, so we can start. Welcome everyone. Thank you for joining today's session on the 2025 technical reporting. I'm going to share my screen. As I was mentioning, I have a couple of slides I want to share with you. She moved. I do not see the chat or hands raised or anything, so please let me know if you get if you can see my slide. Colomer, Julien (One CGIAR - France) 0:47 Yep. Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets and better linkages between the theory of change or so plan of results and budget and technical reporting. The primary audiences for technical reporting are funders and CGR staff at integrated partnership, portfolio and program and accelerator levels. A secondary audience is the partners. Annual technical reporting covers the individual annual technical reports for program and accelerators, as well as a portfolio view of aggregate contribution to thematic and geographic targets. And relevant content from this technical reports are integrated into the CJR corporate reporting. In terms of the 2025 technical reporting priorities, 2025 is a transition year with technical reporting arrangements, implementation again focusing on streamlined reporting and on strengthening the linkages between theory of change. Porb, media and technical reporting. As many of you know, in the previous portfolio these components were not properly linked, so it was a bit challenging to demonstrate progress against the theory of change or the plans, as you know. In terms of deliverables for 2025. These are the program and accelerator technical reports, which are due in April 2026, the portfolio narrative, which is due in 2026 in June. Integration of top 80% of window tree and bilateral projects by central dollar value into reporting and planning. Application of the minimum data standards for window tree and bilateral reporting. And mapping of refinement during the pause and reflect process which will take place early Q 1/20/26. So as I was mentioning, this year is seen more as a transition year towards KPI based planning and reporting and efforts are underway to enable planning and reporting at the KPI level, which is aligned with the system office objective and key results for 2026 and 20. These are to be confirmed, so they haven't been confirmed yet, but I've pasted them here so that you can see the 2026 objective and key results for the system office. So 100% program and accelerate the work plans and budget. An annual technical report. Which provide for software enabled monitoring of erformance and results against smart Ki by center, ear and ooled funds invested. So next year, 80% of centres, CGR, window three and bilateral funded work by value included in 2025 technical reports and then the following year in 2027, this will increase to 90% of centres. Window 3 and bilateral funded work included in 2026 technical reports. The following slides, what I have, what I have included in the following slides, it's a brief introduction into. What is expected in terms of deliverables from programs and accelerators together with an overview of the performance and results management system and the QA. I realized that some in this call some of you are already familiar with the reporting arrangements from the previous portfolio. While for others this might be entirely new. So our goal is to bring everyone to the same level of understanding so that we can move forward with clarity and shared expectations for the 2025 technical reporting. OK, so technical reporting for program and accelerator. We'll focus on three key deliverables. So first is reporting results, the 2025 results in the Performance and Reporting Management system, PRMS. Each program accelerator and mapped window 3 project will report 2025 results in the system and we strongly encourage to report results that were planned and budgeted. So results which have been included in the reports. As the outdated technical reporting system will allow for tracking results against plans. Secondly is the quality assurance of reporting results. As you know, the results submitted go through the quality assessment process and we will share more details on this process in the timeline in an info session scheduled for later. Which we will schedule later in in September, October and the quality assess results will be available on the results dashboard. Inform the pa</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a RAG assistant for deeper research. Preserve acronyms EXACTLY as written. Exactly phrase: 'I cannot find information in the provided chunks to answer this.' Output instructions: - 3 to 5 sentences, neutral and direct style, no lists. - ALWAYS answer in English and adapt wording to the question's context. - End with the literal 'Sources:' and then, as a list, each line as 'File — Location — Cited IDs'."}, {"role": "user", "content": "Question: What are the technical reporting timelines for 2025?\n\nContext:\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p1pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 1 part 2\nContent: 2024 Technical Reporting 2024\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: docx:General information on Technical Reporting .docx:u1-6]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General information on Technical Reporting .docx\nLocation: paragraph 1 to paragraph 7\nContent: General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 1\nContent: 2024 Technical\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 10 part 3\nContent: information. Technical Reporting resources HOW Latest updates Timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 2\nContent: 2025 Technical Reporting Portfolio\n\n---\n\n[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 3\nContent: defined in the 2024 Technical Reporting Guidance are listed below. An\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 15 part 3\nContent: Technical Reporting Arrangement 2025-30 Results\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 4 part 1\nContent: 2025 Technical reporting priorities (transition year) The TRA will be implemented through a phased approach, with the first phase focusing on streamlined reporting and stronger linkages across Program/Accelerator ToCs, PoRBs, MELIA and technical reporting. Key deliverables in this initial phase include: Delivery of 2025 Program and Accelerator Technical Reports by April 2026. Delivery of the 2025 Portfolio Narrative by June 2026. Integration of the top 80% of W3 and bilateral projects (by Center portfolio value) into Program/Accelerator ToC, MELIA, PoRBs, and Technical Reporting. Application of the\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 1\nContent: Information Session on 2025\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 1 to paragraph 4\nContent: Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 4\nContent: Reporting timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 1\nContent: 2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 6 part 2\nContent: report is available here The 2024 Initiatives, Impact Platforms and Science Group Projects annual technical (Type 1) reports are available here WHAT Annual Technical Reports provide assurance on annual Program/Accelerator delivery against PORBs and\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u52-55]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Fortnightly update emails' paragraph 87 to section 'Monthly drop-ins' paragraph 93\nContent: Additional emails will be sent out from this email address with any time-sensitive information. Info-sessions A limited number of targeted info-sessions will be held to provide focused guidance on key aspects of the 2025 Technical Reporting process, and will be timed to align with critical points in the reporting timeline. Each session will include a short presentation followed by time for questions and discussion. Invitations and materials will be circulated in advance, and recordings will be made available for those unable to attend live. Monthly drop-ins\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 11 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 3 part 1\nContent: Technical Reporting Arrangement (TRA) 2025-30 Approved by the CGIAR Global Leadership Team on 5 June 2025, provides the operational basis to plan, monitor, learn, and report on the 2025-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled and W3/bilateral projects of the 2025-30 portfolio in\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u4-7]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Background' paragraph 8 to section 'Objective' paragraph 14\nContent: Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process. Lessons from previous reporting cycles have highlighted the importance of timely, clear, and responsive support to reporting teams. Building on the progress made in recent years, this document outlines a plan to further streamline and optimize communication and engagement mechanisms for the 2025 reporting cycle. Objective\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 2\nContent: results that were planned and budgeted, as the updated technical reporting system will allow for tracking results against plans. QA of reported results 2025 Results will be quality assessed following a defined process and timeline. QA’ed results will be available on the CGIAR Results\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u1-4]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: paragraph 1 to section 'Background' paragraph 8\nContent: Engagement Plan: Technical Reporting 2025 Background Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process.\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 31 to paragraph 34\nContent: Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source. Colomer, Julien (One CGIAR - France) 23:53 Nicoletta, maybe I can just say a few words about this one. Thanks. Thanks so much, Nicoletta, for the presentation so far. So the dashboard here is just a a working version. Obviously we can develop a much more polished version. However, at this stage it's going to be sort of a portfolio Explorer. Trifa, Nicoleta (CGIAR System Organization) 23:54 Go ahead. Yes, yes. Mm. Colomer, Julien (One CGIAR - France) 24:11 So really internally facing and the idea is to consolidate all relevant types of information that we can, you know, make available about the portfolios, the program and accelerator result frameworks, Melia studies, I think we'll try and get the proposal inception reports. You know, whatever else we can get on there, that's really to allow you to coordinate with other programs and accelerators. So we'll keep building this out. And yeah, as mentioned, so this is an internally facing dashboard. And we'll keep improving it over time and eventually we'll put it on the Performance and Results Hub. But for the moment, if you wouldn't mind having a poke through and making sure everything looks as good as it should, the two geographic tabs there map and removed and inception just to give we were asked to have a look. At proposal versus inception geographic footprint. So we've done that. Again, those both the proposal and the inception didn't have a, let's say a very strong geographic component. So that that one is probably the diciest I would say in terms of the data quality and completeness, but please do have. Have a look and let us know if you spot anything. Thanks very much.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and center</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a helpful assistant"}, {"role": "user", "content": "Question: What are the technical reporting timelines for 2025?\n\nContext:\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p1pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 1 part 2\nContent: 2024 Technical Reporting 2024\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: docx:General information on Technical Reporting .docx:u1-6]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General information on Technical Reporting .docx\nLocation: paragraph 1 to paragraph 7\nContent: General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 1\nContent: 2024 Technical\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 10 part 3\nContent: information. Technical Reporting resources HOW Latest updates Timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 2\nContent: 2025 Technical Reporting Portfolio\n\n---\n\n[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 3\nContent: defined in the 2024 Technical Reporting Guidance are listed below. An\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 15 part 3\nContent: Technical Reporting Arrangement 2025-30 Results\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 4 part 1\nContent: 2025 Technical reporting priorities (transition year) The TRA will be implemented through a phased approach, with the first phase focusing on streamlined reporting and stronger linkages across Program/Accelerator ToCs, PoRBs, MELIA and technical reporting. Key deliverables in this initial phase include: Delivery of 2025 Program and Accelerator Technical Reports by April 2026. Delivery of the 2025 Portfolio Narrative by June 2026. Integration of the top 80% of W3 and bilateral projects (by Center portfolio value) into Program/Accelerator ToC, MELIA, PoRBs, and Technical Reporting. Application of the\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 1\nContent: Information Session on 2025\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 1 to paragraph 4\nContent: Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 4\nContent: Reporting timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 1\nContent: 2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 6 part 2\nContent: report is available here The 2024 Initiatives, Impact Platforms and Science Group Projects annual technical (Type 1) reports are available here WHAT Annual Technical Reports provide assurance on annual Program/Accelerator delivery against PORBs and\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u52-55]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Fortnightly update emails' paragraph 87 to section 'Monthly drop-ins' paragraph 93\nContent: Additional emails will be sent out from this email address with any time-sensitive information. Info-sessions A limited number of targeted info-sessions will be held to provide focused guidance on key aspects of the 2025 Technical Reporting process, and will be timed to align with critical points in the reporting timeline. Each session will include a short presentation followed by time for questions and discussion. Invitations and materials will be circulated in advance, and recordings will be made available for those unable to attend live. Monthly drop-ins\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 11 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 3 part 1\nContent: Technical Reporting Arrangement (TRA) 2025-30 Approved by the CGIAR Global Leadership Team on 5 June 2025, provides the operational basis to plan, monitor, learn, and report on the 2025-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled and W3/bilateral projects of the 2025-30 portfolio in\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u4-7]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Background' paragraph 8 to section 'Objective' paragraph 14\nContent: Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process. Lessons from previous reporting cycles have highlighted the importance of timely, clear, and responsive support to reporting teams. Building on the progress made in recent years, this document outlines a plan to further streamline and optimize communication and engagement mechanisms for the 2025 reporting cycle. Objective\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 2\nContent: results that were planned and budgeted, as the updated technical reporting system will allow for tracking results against plans. QA of reported results 2025 Results will be quality assessed following a defined process and timeline. QA’ed results will be available on the CGIAR Results\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u1-4]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: paragraph 1 to section 'Background' paragraph 8\nContent: Engagement Plan: Technical Reporting 2025 Background Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process.\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 31 to paragraph 34\nContent: Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source. Colomer, Julien (One CGIAR - France) 23:53 Nicoletta, maybe I can just say a few words about this one. Thanks. Thanks so much, Nicoletta, for the presentation so far. So the dashboard here is just a a working version. Obviously we can develop a much more polished version. However, at this stage it's going to be sort of a portfolio Explorer. Trifa, Nicoleta (CGIAR System Organization) 23:54 Go ahead. Yes, yes. Mm. Colomer, Julien (One CGIAR - France) 24:11 So really internally facing and the idea is to consolidate all relevant types of information that we can, you know, make available about the portfolios, the program and accelerator result frameworks, Melia studies, I think we'll try and get the proposal inception reports. You know, whatever else we can get on there, that's really to allow you to coordinate with other programs and accelerators. So we'll keep building this out. And yeah, as mentioned, so this is an internally facing dashboard. And we'll keep improving it over time and eventually we'll put it on the Performance and Results Hub. But for the moment, if you wouldn't mind having a poke through and making sure everything looks as good as it should, the two geographic tabs there map and removed and inception just to give we were asked to have a look. At proposal versus inception geographic footprint. So we've done that. Again, those both the proposal and the inception didn't have a, let's say a very strong geographic component. So that that one is probably the diciest I would say in terms of the data quality and completeness, but please do have. Have a look and let us know if you spot anything. Thanks very much.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower transaction costs, stronger impact, focus results. To be clearly lin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"role": "system", "content": "You are a helpful assistant that answer user questions in a very detailed and comprehensive way"}, {"role": "user", "content": "Question: What are the technical reporting timelines for 2025?\n\nContext:\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p1pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 1 part 2\nContent: 2024 Technical Reporting 2024\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Agenda Technical Reporting Arrangement 2025-30 Technical reporting priorities for 2025 What\n\n---\n\n[ID: docx:General information on Technical Reporting .docx:u1-6]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: General information on Technical Reporting .docx\nLocation: paragraph 1 to paragraph 7\nContent: General information on Technical Reporting Where can I find the key dates for Technical Reporting for 2025? An overall Technical Reporting timeline can be found on this page of the P&amp;R Hub. Upcoming key reporting dates and deadlines are also presented on this page. Any updates or changes to the reporting timeline will be communicated via performanceandresults@cgiar.org. Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Is there a CGIAR Style Guide to follow for preparing the narrative components of the Technical Reporting? Yes, the CGIAR Style Guide can be used as a reference.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 1\nContent: 2024 Technical\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s10pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 10 part 3\nContent: information. Technical Reporting resources HOW Latest updates Timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 2\nContent: 2025 Technical Reporting Portfolio\n\n---\n\n[ID: pdf:Digital Transformation_MELIA Plan 30-06-2025 (1).pdf:p21pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation%2FDigital%20Transformation%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP12%20%2D%20Digital%20Transformation&amp;p=true&amp;ga=1\nFile: Digital Transformation_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 3\nContent: defined in the 2024 Technical Reporting Guidance are listed below. An\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s15pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 15 part 3\nContent: Technical Reporting Arrangement 2025-30 Results\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s4pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 4 part 1\nContent: 2025 Technical reporting priorities (transition year) The TRA will be implemented through a phased approach, with the first phase focusing on streamlined reporting and stronger linkages across Program/Accelerator ToCs, PoRBs, MELIA and technical reporting. Key deliverables in this initial phase include: Delivery of 2025 Program and Accelerator Technical Reports by April 2026. Delivery of the 2025 Portfolio Narrative by June 2026. Integration of the top 80% of W3 and bilateral projects (by Center portfolio value) into Program/Accelerator ToC, MELIA, PoRBs, and Technical Reporting. Application of the\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s1pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 1 part 1\nContent: Information Session on 2025\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u1-4]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 1 to paragraph 4\nContent: Answers to questions received during the Tech reporting info sessions on Reporting on Outputs Timeline for reporting: Q: Does the results submission deadline end in January or in February 2026? A: The deadline depends on the type of results being reported:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s9pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 9 part 4\nContent: Reporting timeline\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 1\nContent: 2025 Technical Reporting WHAT Program/Accelerator deliverables Reporting results in the Performance and Reporting Management System (PRMS) Each Program, Accelerator and mapped W3 project will report 2025 results. Programs/Accelerator are strongly encouraged to report results that were planned and budgeted, as the updated technical reporting\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s6pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 6 part 2\nContent: report is available here The 2024 Initiatives, Impact Platforms and Science Group Projects annual technical (Type 1) reports are available here WHAT Annual Technical Reports provide assurance on annual Program/Accelerator delivery against PORBs and\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u52-55]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Fortnightly update emails' paragraph 87 to section 'Monthly drop-ins' paragraph 93\nContent: Additional emails will be sent out from this email address with any time-sensitive information. Info-sessions A limited number of targeted info-sessions will be held to provide focused guidance on key aspects of the 2025 Technical Reporting process, and will be timed to align with critical points in the reporting timeline. Each session will include a short presentation followed by time for questions and discussion. Invitations and materials will be circulated in advance, and recordings will be made available for those unable to attend live. Monthly drop-ins\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt3]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt3]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 3\nContent: to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are being delivered in Q2 2025 under the existing 22-24 Technical Reporting Arrangement. The CGIAR Technical Reporting Arrangement fulfills the System -level programmatic reporting requirements set out in the Standard Provisions annexed to the Funding Agreement or Arrangement signed between each\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 1)-20250729_100141-Meeting Recording 29 de julio de 2025, 8:01a.m. 53 min 5 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 11 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 1 CGIAR Technical Reporting Arrangement 2025-30 Approved by the CGIAR Global Leadership Team 5 June 2025 Purpose The purpose of the Technical Reporting Arrangement 2025-2030 (“TRA 25-30”) is to set out the technical reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u1-4]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 1 to paragraph 4\nContent: 2025 Technical Reporting Information (Session 2)-20250729_150218-Meeting Recording 29 de julio de 2025, 1:02p.m. 47 min 36 s Trifa, Nicoleta (CGIAR System Organization) ha iniciado la transcripción\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 3 part 1\nContent: Technical Reporting Arrangement (TRA) 2025-30 Approved by the CGIAR Global Leadership Team on 5 June 2025, provides the operational basis to plan, monitor, learn, and report on the 2025-30 Portfolio. It is designed to progressively enable Programs and Accelerators, Centers and their research teams to report on the pooled and W3/bilateral projects of the 2025-30 portfolio in\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u4-7]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Background' paragraph 8 to section 'Objective' paragraph 14\nContent: Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process. Lessons from previous reporting cycles have highlighted the importance of timely, clear, and responsive support to reporting teams. Building on the progress made in recent years, this document outlines a plan to further streamline and optimize communication and engagement mechanisms for the 2025 reporting cycle. Objective\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s5pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 5 part 2\nContent: results that were planned and budgeted, as the updated technical reporting system will allow for tracking results against plans. QA of reported results 2025 Results will be quality assessed following a defined process and timeline. QA’ed results will be available on the CGIAR Results\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u1-4]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: paragraph 1 to section 'Background' paragraph 8\nContent: Engagement Plan: Technical Reporting 2025 Background Effective communication and engagement with CGIAR's Programs and Accelerators (P/As) and Centers (on W3/bilateral projects mapped to P/As) is essential for ensuring a smooth and efficient 2025 Technical Reporting process.\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u31-34]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 31 to paragraph 34\nContent: Nirmal, Rajalakshmi (IFPRI) 36:04 But. Colomer, Julien (One CGIAR - France) 36:06 Yeah, yeah. Basically anything that's not finished or nailed down, I get to answer for. So and then I SO look, 2025 is a Transition year and. We everybody recognizes like the amount of pressure that everyone's under. So that final step of transferring over the, let's say, key Performance indicator or target output and target outcome values from the window three and bilaterals into the theory of change. And into the planning module, et cetera, will not be done for the 2025 Technical report. So for the 2025 Technical report, IT being a Transition year, we want programs to report against the targets that they've already got in there obviously. And for the Window 3 bilats that have been mapped, we will really ask them to contribute the Results that they can contribute to in this first year. We have an objective and key result there for the System organization, which says that 80% of Window 3 bilats are included. In the Technical reports, exactly what is included is not defined. So we kind of have a bit of a Long leash there or You know, wide goal posts, but that's a discussion to have with centers and we'll be working with centers and with the Program and accelerators to better define like what can be reported, what is the lowest cost. Path to report, et cetera for 2025. Now for 2026, however, Nicoletta put up that objective which said something like 100% of Program and accelerator plans and Results and budget and Technical reports, You know, allow for that sort of, You know, what did You plan, what did you? Deliver. And in that context, the 2026 plan of Results and budget and 2026 Technical reports, we will be asking the mapping of Window 3 bilateral targets down to the specific, You know, KPI within the high level outputs or at the intermediate outcome level. And then asking centres to then report against what they what they had planned. So that's gonna be for 2026 plan of Results and budget and the 2026 Technical report. 2025 is a Transition year. So that final step of transferring over the target information is not being done. Is that clear? Nirmal, Rajalakshmi (IFPRI) 38:32 Yeah. So for 2025, we are not reporting against bilateral projects in the RMS, right? Colomer, Julien (One CGIAR - France) 38:38 We will be, we will be. It's just that we will not be entering in target values. Yeah. So, SO I mean, unless that is useful in some way, like it's either if it's more useful to enter them in.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p16pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p16pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 16 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June 2025 16 In doing so the line of sight will primarily focus on the outputs produced with pooled resources (sphere of control) while the outcomes are co -produced and do not require differentiation by source of funding. The rate of change Because Technical Report products will progressively integrate bilateral and W3 information, we expect that they will contain differing levels and types of W3 and bilateral project technical content (e.g. results data and narrative) and that this will evolve over time. There are likely to be different levels of bilateral and W3 technical information:\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 16:49 Yes. OK, good. So this is the revised PNR Hub adapted, updated with the new CGR logo and branding colors. You'll have the homepage reporting, planning, reflect and replan and then archive if you. If You Go to archive, You will find previous information on Technical reporting from previous years. What's of interest for this presentation as well As for Technical reporting, You will Go to 2025 reporting and this is where You will find pertinent information to Technical reporting this year. So again, it's the timeline here. Latest update. This section will post and keep this section updated as information comes becomes available. Upcoming events, so. We've only listed today's info session, but the other info session will follow once we have defined a date for them. Event event recording, SO meeting recording and link to the decks will also be available here. And under the frequently asked questions, we were able to recycle to say SO a couple of key questions from previous Portfolio which still apply to to this Portfolio to the Program and accelerator team. So I invite You to Go there. And and browse a bit the the questions and answers under various section. Be mindful that this is this Hub is live a live Hub SO as information becomes available we want to make IT available to the end users here so. Any feedback on how to improve, what You improve and SO on is is welcome. So feel free to reach out to us if You have any suggestions or would like to see some things more preeminently maybe. Features here. Good. Back to this. I only have 1-2 slides and then I will will open for questions. In terms of engaging with Program accelerators and centers on Technical reporting this year, the we have a couple of channels to engage with you. So first is through the bi-weekly emails. Every two weeks You will receive an e-mail with technical. Supporting updates that will include reminders, summaries, latest questions and answers we want to share with everyone and SO on. There will be targeted emails and this emails will engage specific categories within the program. Accelerators and the centers center many Focal Points based on Technical reporting, revisions, developments and that the purpose is to gather targeted feedback on nonspecific things. Um. Info session planned for on specific topics, for example QA, PRMS, innovation, reporting on outputs, reporting on on outputs and SO on. So those info session will be planned for September, October and we will keep You appraised on the exact. Select dates and themes topics ahead of time and then the drop ins. We've seen that it was specifically valuable to initiatives when these drop ins were planned during reporting and during QA. So during this drop-ins will not come with presentations, but you will have several people from our team be available to respond to your questions live and the primary focus as I was mentioning will be reporting and the QA. Um. This is the process that we used with initiatives and it worked pretty well to to test PRMS enhancements and receive feedback from initiatives and the same process will be used this year to engage programs and accelerators and center media focal point. So usually when a new enhancement is proposed, we will send the targeted e-mail. We'll invite specific roles within the PMUs to test, provide feedback, then the feedback. Becomes an update in the PRMS and once it's live, we will notify you so that everyone has access to that enhancements, to those enhancements in the PRMS with an explanation of why the enhancement, who asked for it. You know, oh, and so on. In terms of upcoming activities, as I was mentioning the bi-weekly technical reporting updates, the first e-mail will get out this Thursday with the link to this deck and to the recording for people who were not able to join today. There are the targeted engagement goals for PRMS testing, info session on specific topics and there is also an engagement on window 3 bilateral. Jules Colomer is leading on this together with alignment working group. I believe this is it. I only have a link here to a theory of change dashboard. I will take advantage of Jules being in this call. So to briefly introduce this, but what I understand this. The Theory of Change dashboard, I hope you can see it on my screen now, has been developed based on all theory of change of programs and accelerators as per the inception reports. So you have an overview of. Of the Results framework of the 2030 outcome, outcomes, media studies and also on map which you can filter. So you have V1 and V2 here and the request to you. We will share the link to this dashboard. It's an internal dashboard. We will share the link with you. You and the request is to have a look at your program and accelerator and the data in this dashboard and if you notice error, please let us know right e-mail us at Performance and Results at cgr.org. So that we can fix the error either in the dashboard or you know, whatever needs to be fixed in the original data source. Colomer, Julien (One CGIAR - France) 23:53 Nicoletta, maybe I can just say a few words about this one. Thanks. Thanks so much, Nicoletta, for the presentation so far. So the dashboard here is just a a working version. Obviously we can develop a much more polished version. However, at this stage it's going to be sort of a portfolio Explorer. Trifa, Nicoleta (CGIAR System Organization) 23:54 Go ahead. Yes, yes. Mm. Colomer, Julien (One CGIAR - France) 24:11 So really internally facing and the idea is to consolidate all relevant types of information that we can, you know, make available about the portfolios, the program and accelerator result frameworks, Melia studies, I think we'll try and get the proposal inception reports. You know, whatever else we can get on there, that's really to allow you to coordinate with other programs and accelerators. So we'll keep building this out. And yeah, as mentioned, so this is an internally facing dashboard. And we'll keep improving it over time and eventually we'll put it on the Performance and Results Hub. But for the moment, if you wouldn't mind having a poke through and making sure everything looks as good as it should, the two geographic tabs there map and removed and inception just to give we were asked to have a look. At proposal versus inception geographic footprint. So we've done that. Again, those both the proposal and the inception didn't have a, let's say a very strong geographic component. So that that one is probably the diciest I would say in terms of the data quality and completeness, but please do have. Have a look and let us know if you spot anything. Thanks very much.\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p1pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p1pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 1 part 2\nContent: reporting requirements that apply to the CGIAR Portfolio during the period 2025-2030. Prepared by; Content developed by the Portfolio Performance Unit in collaboration with a x- CGIAR working group and System Council Strategic Impact Monitoring and Evaluation Committee members. Note to readers: 2024 Annual Technical Reports including the 2022-24 Type 2 Report are\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt1]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt1]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 1\nContent: CGIAR Technical Reporting Arrangement 2025-30 June\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u7-10]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 7 to paragraph 10\nContent: Trifa, Nicoleta (CGIAR System Organization) 0:48 Yep. OK, good. So thank you. This session is the first of two session plans for today, planned for today, with the second being scheduled later at 3:00 PM CET to accommodate colleagues in other time zones. Technical reporting. My name is Nicoletta Trifa. By the way, I'm part of the Portfolio Performance Unit, the support unit within the Office of the Chief Scientist. Here is an overview of what we'll cover in the next minutes. I believe my presentation will take 2025 minutes and then we'll leave room for questions at the end, if that's OK. So what we'll cover an update of the technical reporting arrangements 2025 to 2030, priorities and changes for 2025, a brief introduction on the annual technical report and the neighbors. So this mean the performance and results. Management system and the quality assurance, the technical reporting timeline, available resources and support and what's next and how to stay engaged. I want to mention that this session marks the start of the conversation around 2025 technical reporting. We want to give you the early look at the key priorities and plans for the months ahead, and the goal is to make sure that you stay informed, prepared and supported with a clear understanding of upcoming deliverables and timelines. And also clarity on who to reach out to if you have questions or if you need help along the way. Good. Technical reporting arrangements for the new portfolio. The 2025 to 2030 portfolio has been approved by the CGR Global Leadership team on in June 2025 and provides the operational basis to plan, monitor, learn and report. On the new portfolio. It is designed to progressively enable programs, accelerators and centers to report on the pooled and window 3 bilateral projects of the new portfolio in an integrated and aligned way without increasing the burden on centers and the scientists. Main changes compared to the previous technical reporting arrangements, streamline reported reporting. So less products, more integration, lower </t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a helpful assistant that answer user questions in a very detailed and comprehensive way"}, {"role": "user", "content": "Question: When does PRMS opens?\n\nContext:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s12pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 12 part 1\nContent: PRMS\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s3pt1]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 3 part 1\nContent: PRMS\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u40-42]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 48 to paragraph 50\nContent: PRMS access Q: When will our role in PRMS change? When I log in, it shows my role in the Initiative? A: You will be able to see your new role assigned to the specific Program/Accelerator once the 2025 reporting phase opens in PRMS.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s8pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 8 part 3\nContent: in the PRMS will be quality assessed (QA) by a QA team in February 2026. Your participation in this process is required. Guidance and resources will be provided.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s13pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 13 part 2\nContent: on 31 July. Targeted engagement calls for PRMS testing. Info sessions on specific topics (e.g. QA,\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 7 part 1\nContent: PRMS Reporting Tool PRMS\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 7 part 2\nContent: PRMS REPORTING TOOL PRMS\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s7pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 7 part 3\nContent: PRMS roles PRMS resources:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt2]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 2\nContent: 2025 What Annual Technical Reports Performance and Reporting Management System (PRMS)\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u55-58]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Monthly drop-ins' paragraph 93 to section 'PRMS enhancements and feedback process' paragraph 99\nContent: Monthly drop-ins To provide ongoing, accessible support throughout the reporting period, monthly drop-in sessions will be held via Microsoft Teams. These informal sessions will offer Programs and Accelerators the opportunity to raise questions, seek clarification, and engage directly with PPU/PCU. No formal presentations will be given; instead, the focus will be on open dialogue and timely support. Invitations and calendar holds will be shared in advance, with reminders included in the regular update emails. PRMS enhancements and feedback process The PRMS Reporting Tool is continuously improved in response to user needs and feedback. The update process follows these steps:\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt4]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 4\nContent: Resources Engagement plan Process for PRMS enhancements What next Upcoming activities\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u49-52]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 49 to paragraph 52\nContent: Trifa, Nicoleta (CGIAR System Organization) 43:52 Other questions, comments. No, good. Again, we will paste the link to the deck and to the meeting recording and share with you by e-mail. Be available. This will be available on the PNR Hub as well. So if there are no other questions or comments, I want to thank you all for your participation to this session. Yeah, don't hesitate to reach out to us. OK, I see a question there. When does the PRMS open for reporting? This is to be confirmed, Raja. Again, we're aiming for November. It's, you know, we will inform you the closer we get to the date about the the final official. Opening date for PRMS. Thanks everyone. Have a wonderful day. Colomer, Julien (One CGIAR - France) 44:46 Thank you, Nicoleta. Thanks everybody. Ciao. Bye, bye. Trifa, Nicoleta (CGIAR System Organization) 44:47 Bye. Aryal, Bishal (IFPRI) 44:47 Thank you. Thank you.\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt1]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 2 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Engagement plan – Technical Reporting 2025 Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s11pt1]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 11 part 1\nContent: Technical Reporting questions: performanceandresults@cgiar.org PRMS support: prmstechsupport@cgiar.org Technical Reporting engagement plan Support period: July 2025 – June 2026 Purpose: Streamline communication and optimize support for Programs,\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u58-61]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'PRMS enhancements and feedback process' paragraph 99 to section 'PRMS enhancements and feedback process' paragraph 104\nContent: The PRMS Reporting Tool is continuously improved in response to user needs and feedback. The update process follows these steps: The Sounding Board will consist of representatives from: PRMS Team PCU Team\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u10-13]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 10 to paragraph 13\nContent: Marshall, Karen (ILRI) 25:21 Yeah. Hi, everybody. And thank you for that great update. Just a question, whilst PRMS is being sort of, I think you said streamlined or updated August to November, can we also put results into the system during that time because? You know, a start date from late November, December will will be too late for us. Trifa, Nicoleta (CGIAR System Organization) 25:43 So have them in editing mode. You mean like not submit them just. Marshall, Karen (ILRI) 25:45 Yes, yes. Because I was really hoping that by August we could start putting things into PRMS because you, you know, it would be, we don't want to have like a long period of upgrading PRMS and then very short time for us to to actually put things in there. Yeah. So if we could actually be putting them in where we're tweaking it, that would be very useful or. Trifa, Nicoleta (CGIAR System Organization) 25:48 Yeah.\n\n---\n\n[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p16pt3]\nLink: N/A\nFile: CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf\nLocation: page 16 part 3\nContent: Target users of the PRMS include CGIAR staff for day-to-day Initiative management and reporting, portfolio management and resource mobilization , and Funders and partners to access evidence of CGIAR thematic and geographic presence and progress against stated objectives such as the SDGs. Security, hosting, maintenance and support The PRMS will incorporate:\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 14 part 3\nContent: critical process for both internal and external communication, ensuring accountability, transparency, and progress tracking. It facilitates decision -making, supports adaptive management, and communicates Program/Accelerator achievements to stakeholders. Relevant information from Program Results Frameworks will be integrated into the PRMS Reporting tool from the PRMS ToC Board to facilitate the\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p23pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 23 part 4\nContent: program learning as well as the refinement of the Theory of Change during the annual “Pause and Reflect” sessions. These sessions will also contribute to the overall annual reporting procedures. To facilitate results reporting within the PRMS framework, each Area of Work (AoW) will appoint designated focal persons who will collaborate with the Monitoring, Evaluation, and Learning (MEL) team to upload pertinent r esults and supporting evidence. A comprehensive checklist, in alignment with PRMS metadata requirements, will be employed to guide and standardize the reporting process.\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p6pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 6 part 3\nContent: has been developed in the PRMS TOC Board and updated to\n\n---\n\n[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt3]\nLink: N/A\nFile: CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf\nLocation: page 15 part 3\nContent: and accessible Performance &amp; Results Management System (PRMS) that encompasses planning, monitoring, and reporting will provide robust information upon which to take informed decisions. It will provide: • Practical services aligned to meet learning, accountability and resource mobilization objectives, • Dashboards open to Funders and partners, with access to the full set of underlying quality-checked data , including communications-focused products capturing collated evidence of CGIAR contribution to change (e.g. outcome/impact case reports). • Alignment with international standards such as IATI (International Aid Transparency Initiative). Key PRMS features The CGIAR PRMS will feature: • A common system housing plan of work and budget, theory of change management, stage-gate decision points, and annual reporting processes. It will allow real- time\n\n---\n\n[ID: pdf:Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf:p21pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition%2FBetter%20Diets%20and%20Nutrition%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP05%20%2D%20Better%20Diets%20and%20Nutrition&amp;p=true&amp;ga=1\nFile: Better Diets and Nutrition_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 3\nContent: to guide consistent and credible reporting into the PRMS system. Key elements include: • Use of standardized data collection tools • Training and calibration of enumerators or field staff • Spot-checks and validation missions by MELIA or AoW focal points • Automated consistency checks in digital entry platforms (if used during the program implementation) • Clear metadata documentation for each indicator • Peer review or AoW lead/Director sign-off before data submission (especially at outcome level) 5. Contingency Plan for Data Collection Risks To address potential disruptions, the program will maintain a risk mitigation table that is regularly updated. Initial measures include: Risk Potential Impact Mitigation Strategy Budget constraints Incomplete\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u34-37]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Technical Reporting questions' paragraph 61 to section 'Fortnightly update emails' paragraph 67\nContent: All questions and comments on Technical Reporting should be sent via email to performanceandresults@cgiar.org. For technical questions related to using the PRMS Reporting Tool, emails should be sent to prmstechsupport@cgiar.org. PPU/PCU will endeavor to reply to queries as soon as possible; please note that delays are usually due to ensuring that responses have been reviewed and align with the latest updates and guidance. Responses will also be posted in real time on the P&amp;R Hub for wider reference. Fortnightly update emails To ensure transparent and regular communication throughout the reporting cycle, a centralized update mechanism will be used.\n\n---\n\n[ID: docx:Using the PRMS Reporting Tool.docx:u7-9]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Using the PRMS Reporting Tool.docx\nLocation: section 'Using the PRMS Reporting Tool' paragraph 10 to section 'Using the PRMS Reporting Tool' paragraph 13\nContent: Yes. The PDF function is always available. The system will generate the PDF with the information that you have entered when you press the button, even if the result entry is not fully complete at the time. What should I do if I encounter a bug in the PRMS Reporting Tool? Please ensure you create technical tickets for the bugs you encounter by sending an email to prmstechsupport@cgiar.org. This will help the PRMS team to track requests and prioritize them.\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p14pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 14 part 4\nContent: the PRMS Reporting tool from the PRMS ToC Board to facilitate the reporting and evidencing of achievement of both output and outcome indicator targets, as well as links to MELIA studies as sources of evidence. Further details on Technical Reporting processes, products and support will be shared in 2025.\n\n---\n\n[ID: docx:Engagement Plan 2025 Technical Reporting.docx:u49-52]\nLink: https://docs.google.com/document/d/1bxyVhlOayJqgreqiv4xhOu9xQ3Vz3Ymg/edit\nFile: Engagement Plan 2025 Technical Reporting.docx\nLocation: section 'Fortnightly update emails' paragraph 83 to section 'Fortnightly update emails' paragraph 87\nContent: PRMS Team PCU Team PPU Team Additional emails will be sent out from this email address with any time-sensitive information.\n\n---\n\n[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p11pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_MELIA Plan 30-06-2025.pdf\nLocation: page 11 part 3\nContent: outlines the types of reports required at diƯerent time intervals. It also aligns with the CGIAR Technical Reporting Arrangement (TRA) 2025–30 (in draft), which standardizes reporting processes and ensures coherence across funding streams. An updated PRMS Outcome Indicator Module will be used to report\n\n---\n\n[ID: pdf:CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf:p15pt2]\nLink: N/A\nFile: CGIAR-Performance-and-Results-Management-Framework-2022-30.pdf\nLocation: page 15 part 2\nContent: criteria: Based on past results plus projected costs and development impact (considerations could include ToC, QoR4D, Scaling Readiness , risk assessment, portfolio risk/reward profile review, Gender in research &amp; Gender, Diversity and Inclusion). Stage-gate delivery and use A Performance and Results Management System (PRMS) will be used to collect relevant data and make it available for use in CGIAR, Action Area, Initiative and component management, including stage-gate decisions. 7. Performance and results management system Building on investments made in the current phase of CGIAR research programming, a comprehensive, mature and accessible Performance &amp; Results Management System (PRMS) that encompasses planning, monitoring, and reporting will provide robust information upon which to take informed decisions. It will provide: • Practical\n\n---\n\n[ID: docx:Submitting evidence.docx:u16-19]\nLink: https://sites.google.com/cgxchange.org/cgiarprhub/2025-reporting?authuser=0\nFile: Submitting evidence.docx\nLocation: section 'Submitting evidence' paragraph 20 to section 'Submitting evidence' paragraph 23\nContent: You confirm that all intellectual property rights related to the file have been observed. This includes any rights relevant to the document owner’s Center affiliation and any specific rights tied to content within the document, such as images. You agree to the file link being displayed on the CGIAR Results Dashboard. If you indicate that the file being uploaded to the PRMS is NOT public: You confirm that the file should not be publicly accessible.\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s2pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 2 part 3\nContent: System (PRMS) Quality Assurance When Technical Reporting timeline How Resources Engagement\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p57pt4]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 57 part 4\nContent: Tomorrow.indd 57 08/08/2025 16:0208/08/2025\n\n---\n\n[ID: pdf:CGIAR_PORB_Breeding_Tomorrow.pdf:p86pt4]\nLink: https://cgspace.cgiar.org/items/e5edf9cd-51b3-4b13-80dd-3bb21975fdcf\nFile: CGIAR_PORB_Breeding_Tomorrow.pdf\nLocation: page 86 part 4\nContent: Tomorrow.indd 86 08/08/2025 16:0208/08/2025 16:02\n\n---\n\n[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p21pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 21 part 2\nContent: not only results, but also key decisions, implementation challenges, and signals of change as they emerge. Data submission will occur on a rolling basis, supported by automated quality checks and centralized review from the MELIA and Program management teams. Quarterly validation and entry into the PRMS system will help maintain momentum and avoid year-end data backlogs, while also enabling continuous insight generation. In line with CGIAR’s Open and FAIR Data Assets Policy, databases generated by research teams will be managed by those teams\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 1).docx:u22-25]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%201%29%2D20250729%5F100141%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E76da6c8e%2D6234%2D41ff%2Dba2c%2Dc2068392ed82\nFile: 2025 Technical Reporting Information (Session 1).docx\nLocation: paragraph 22 to paragraph 25\nContent: Trifa, Nicoleta (CGIAR System Organization) 30:25 Mhm. And safe, this is exactly what we're aiming to do this year. So in August in two weeks to three weeks, the the intent is to share with you the PRMS data fields by indicator categories of innovation, policies, capacity sharing and so on. So you know exactly what data fields. Will be capturing PRMS when reporting will open, so you could use those documents to to inform you when gathering information on on your results. And secondly, and Nico also mentioned in the chat here. The intent is to apply the same logic we apply to the out communicator module from the get go, so from the reporting. So we if last year we had that special module at the end of reporting to link results to targets. This will happen now from the get go, so when you enter results you will be asked to link your result to your plans. To your targets. So I hope this answer your question safe, Karen. Marshall, Karen (ILRI) 31:47 Yeah, I I just want to come back to what Enrique said. And Enrique, I really understand that there's quite a lot of, you know, effort and and time put into updating PRMS and it's really getting better every year. But I mean the the problem that happens is that things take long and then we as a scientist are set with a fixed date and we get squeezed to get everything in because. That. It can't be moved because the reports are dependent on it, you know, an ISDC date. So I mean, maybe one way to say is we need so much time for reporting. Yeah, let's say we open it in mid-october or September if we could. Wherever PRMS is there is where it is, yeah, because it cannot be always the people doing the reporting who are the ones who ultimately get squeezed. So I think, you know, really in the initiatives there was, you know, I really had a sense that everything was done from one side and I took the time and then we were just stuck with whatever time was left. It should be the other way around really the people reporting, you know, so let's maybe consider making a deadline saying this is when the reporting has to open, where Pyramus is, is, is where it is. Yeah. Bonaiuti, Enrico (CIP-ICARDA) 32:49 Yeah, yeah, I mean maybe 11 aspect Karen and my reflection the fact of flipping a bit the PRMS using the experience of the outcome module. So you you see first your targets should in theory let programs focus first on. Trifa, Nicoleta (CGIAR System Organization) 32:50 Thanks, Karen.\n\n---\n\n[ID: pptx:Engagement Plan 2025 Technical Reporting.pptx:s2pt3]\nLink: https://docs.google.com/presentation/d/1WbVFx3MD32HUZXlnY_sMF2APNxr6JgGG/edit?slide=id.p1#slide=id.p1\nFile: Engagement Plan 2025 Technical Reporting.pptx\nLocation: slide 2 part 3\nContent: activated only during scheduled meetings and closed immediately after. performanceandresults@cgiar.org is the official communication channel. Full engagement plan available via the P&amp;R Hub and here: Full\n\n---\n\n[ID: docx:Questions and Answers from Tech reporting info sessions.docx:u4-7]\nLink: N/A\nFile: Questions and Answers from Tech reporting info sessions.docx\nLocation: paragraph 4 to paragraph 8\nContent: A: The deadline depends on the type of results being reported: Pooled results (reported by P/A under W1/W2 funding): must be submitted by end of January 2026. These results undergo a quality assurance (QA) process in February 2026. W3/bilateral results: since these do not go through QA, they can be reported in PRMS until late February 2026. Governance:\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p10pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 10 part 2\nContent: also needs to be verified to maintain quality control and reference relevant documentation for evidence. The PRMS system will be used currently to store and maintain the data collected. Reported HLOs and Intermediate Outcomes from AoWs will be quality checked through the internal review process within AoWs before reporting to the PRMS system. Data repositories will be created and maintained at the AoW level to ensure evidence preservation. Data and reporting on HLOs from bilaterals will be checked by Center delegates for the Program for quality assurance. Data will be cross -checked and validated at the Program level during reporting period. The Program MELIA lead will work closely\n\n---\n\n[ID: docx:2025 Technical Reporting Information (Session 2).docx:u46-49]\nLink: https://cgiar.sharepoint.com/sites/InitiativeDesignTeams/_layouts/15/stream.aspx?id=%2Fsites%2FInitiativeDesignTeams%2FShared%20Documents%2FGeneral%2FC%2E%20Meeting%20Recordings%5FFeb%202022%20and%20beyond%2F2025%20Technical%20Reporting%20Information%20%28Session%202%29%2D20250729%5F150218%2DMeeting%20Recording%2Emp4&amp;referrer=StreamWebApp%2EWeb&amp;referrerScenario=AddressBarCopied%2Eview%2E57e21346%2Dc6ca%2D4c63%2D8839%2D3e2a327c5116\nFile: 2025 Technical Reporting Information (Session 2).docx\nLocation: paragraph 46 to paragraph 49\nContent: Colomer, Julien (One CGIAR - France) 42:25 So that they also understand, you know how how things work. Now there's 1000 plus active grants, 500 new ones already since November. So that's a lot of onboarding sessions. Perhaps what we need is a set of materials that can be shared and accessed easily like a recording and and stuff like that. So I think we'll look. For the most scalable low cost solution that helps people you know understand what we do and perhaps for the for the program and accelerator directors once they come on board then we have the in person you know live one and then for the new projects they get the recorded one, something like that. But it's a it's a good idea. Yeah. Thanks. Trifa, Nicoleta (CGIAR System Organization) 43:04 Good idea. We, as I was mentioning, we are making a drafting a PRMS new user deck if you want. So it's two or three slides with relevant information on PRMS like the access, the roles, guidance on how to report, who needs to report when and so on. So that will be available soon on the PNR Hub. And we will notify you once that's available. So feel free to disseminate that to, you know, colleagues from Windows 3 bathroom projects which have a role in providing information, technical reporting, if not, you know, actually reporting in the system. Nirmal, Rajalakshmi (IFPRI) 43:44 Thanks. Trifa, Nicoleta (CGIAR System Organization) 43:52 Other questions, comments. No, good. Again, we will paste the link to the deck and to the meeting recording and share with you by e-mail. Be available. This will be available on the PNR Hub as well. So if there are no other questions or comments, I want to thank you all for your participation to this session. Yeah, don't hesitate to reach out to us. OK, I see a question there. When does the PRMS open for reporting? This is to be confirmed, Raja. Again, we're aiming for November. It's, you know, we will inform you the closer we get to the date about the the final official</t>
+  </si>
+  <si>
+    <t>[{"role": "system", "content": "You are a helpful assistant that answer user questions in a very detailed and comprehensive way"}, {"role": "user", "content": "Question: What is impact?\n\nContext:\n\n---\n\n[ID: pdf:Sustainable Farming_MELIA Plan 30-06-2025.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming%2FSustainable%20Farming%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP02%20%2D%20Sustainable%20Farming&amp;p=true&amp;ga=1\nFile: Sustainable Farming_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing%2FCapacity%20Sharing%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP11%20%2D%20Capacity%20Sharing&amp;p=true&amp;ga=1\nFile: Capacity Sharing_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Policy Innovations - MELIA Plan 30-06-2025-.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations%2FPolicy%20Innovations%20%2D%20MELIA%20Plan%2030%2D06%2D2025%2D%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP07%20%2D%20Policy%20Innovations&amp;p=true&amp;ga=1\nFile: Policy Innovations - MELIA Plan 30-06-2025-.pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 2\nContent: Learning and Impact Assessment\n\n---\n\n[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p8pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_MELIA Plan 30-06-2025.pdf\nLocation: page 8 part 4\nContent: exercise. 4. Impact assessment Impact assessment (IA) is assessment that estimates the causal effects of research outputs and related activities and assesses the magnitude of impact achieved. Impact assessments are conducted after an intervention has been completed and are used to substantiate claims of sustained results. They seek to measure impact at scale, i.e., benefits to a large number of people/large areas of land. It employs both quantitative and qualitative methods, often combined for deeper insights. IA goes beyond monitoring indicators to evidenced attribution of observed changes to CGIAR interventions. IA will help to ensure that Programs/Accelerators contribute meaningfully to CGIAR’s Results Framework and the 2025–30 Portfolio objectives.\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p10pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 10 part 3\nContent: Impact Indicate the result short title from the Results Framework Indicate the indicator title from the Results Framewo rk Provid e the assu mptio n(s) state ment from the Resul ts Fram ework Indicate the location( s) where the study will be conducte d Indicate the methods and design approache s that will be used for the study List the Progr am(s) and Accel erato\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p70pt4]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 70 part 4\nContent: Impact program to enhance farm productivity and mitigate environmental pressure, making agriculture more efficient, affordable, and sustainable. Credit: Abdul Momin, CIMMYT CGI21-508007-PORB-Scaling for Impact.indd 70CGI21-508007-PORB-Scaling for Impact.indd 70\n\n---\n\n[ID: pdf:Climate Action_MELIA Plan 30-06-2025 (1).pdf:p2pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action%2FClimate%20Action%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP06%20%2D%20Climate%20Action&amp;p=true&amp;ga=1\nFile: Climate Action_MELIA Plan 30-06-2025 (1).pdf\nLocation: page 2 part 3\nContent: Impact assessment (IA) .............................................................................................................. 13 Program impact overview .................................................................................................................... 13 IA activities and collaboration plans ..................................................................................................... 14 IA studies ........................................................................................................................................... 15 5. Learning and adaptive management ........................................................................................... 16 Learning ............................................................................................................................................. 16 Annual review and adaptive planning ...................................................................................................\n\n---\n\n[ID: pdf:Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf:p1pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion%2FGender%20Equality%20and%20Inclusion%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP10%20%2D%20Gender%20Equality%20and%20Inclusion&amp;p=true&amp;ga=1\nFile: Gender Equality and Inclusion_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 2\nContent: and Impact Assessment (MELIA)\n\n---\n\n[ID: pdf:Genebanks_MELIA Plan 30-06-2025.pdf:p1pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks%2FGenebanks%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP13%20%2D%20Genebanks&amp;p=true&amp;ga=1\nFile: Genebanks_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 3\nContent: and Impact Assessment (MELIA)\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p58pt2]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 58 part 2\nContent: on critically relevant topics. 3,250 6,646 1,708 3,528 3,001 6,709 1,200 1,661 554 2,542 2,500 1,233 2022 results 3,415 2023 results 6,275 2024 results 8,237 Total results 16,605 2 = Principal: Contributing to one or more aspects of the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. 0 = Not targeted: The result has been screened against the Impact Area, but it has not been found to directly contribute to any aspect of the Impact Area as it is outlined in the CGIAR 2030 Research and Innovation strategy. Figure 5.9. Overview\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p47pt1]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 47 part 1\nContent: Impact Area indicator quantification Given these limitations and opportunities, the Portfolio Performance Unit (PPU) commissioned subject matter experts for each Impact Area to review the Impact Area indicators and the aligned outcomes and impacts reported, with a view to assessing the feasibility of aggregating the reported results to inform on total progress toward the Impact Area indicators during the 2022 to 2024 period. This was very challenging, and partial quantification was attempted in three of the Impact Areas but was not feasible in the remaining two. Several common observations and recommendations emerged from across the different studies: • The Impact Area indicators used in CGIAR’s Results Framework were generally not sufficiently specific, measurable, achievable, relevant, or timebound (SMART).177 They used ambiguous terms such as “benefiting” and “improved management.” Functional units and methods of measurement were often not prescribed, and time or geographic bounds were often not applied. • Potential solution: Revise the Impact Area indicators to ensure full SMART compliance, define methods and tools to be used in data collection, and roll these out through the CGIAR Programs and Accelerators. • The stage along the impact pathway assessed by each Impact Area indicator is highly variable, and different measurements apply at different stages along the impact pathway. For example, in the Poverty Impact Area, an indicator of the ultimate goal is the number of people assisted to exit poverty, but the most common means through which CGIAR affects poverty is by enhancing agricultural productivity, which could be defined as a more proximate goal. • Potential solution: Define proximate and ultimate Impact Area indicators, which relate to stages in the impact pathways and include more studies that attempt to demonstrate the relationships between the two. Defining common impact pathways used in CGIAR programming would also be beneficial. • There is fragmentation in the indicators measured in impact evaluations and the Impact Area indicators required in the Results Framework. There is also a disconnect between studies that\n\n---\n\n[ID: pdf:Scaling for Impact_Inception Report 30-06-2025.pdf:p17pt3]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FInception%20Report%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_Inception Report 30-06-2025.pdf\nLocation: page 17 part 3\nContent: private sector impact investments. These efforts will be designed to be consistent with and complement the objectives, priorities, and activities of the CGIAR Standing Panel on Impact Assessment (SPIA). Impact assessment studies are implemented across AoWs and coordinated by S4I’s MELIA unit, with scientific input from AoW 5’s Cluster 5.2 on Dynamic Learning and Impact Assessment. This cluster\n\n---\n\n[ID: pdf:Portfolio Narrative_2024.pdf:p11pt3]\nLink: https://cgspace.cgiar.org/items/04bd63a9-1b58-4eb5-84f2-b54c8bde226e\nFile: Portfolio Narrative_2024.pdf\nLocation: page 11 part 3\nContent: the Impact Area is the principal objective of the result. The Impact Area is fundamental to the design of the activity leading to the result; the activity would not have been undertaken without this objective. 1 = Significant: The result directly contributes to one or more aspects of the Impact Area. However, contributing to the Impact Area is not the principal objective of the result. Figure 2.3. Number of RAFS results contributing to each Impact Area. Results are tagged as “principal” or “significant” to indicate their contribution to an Impact Area, with principal results shown in the orange and significant results in the yellow. Source: CGIAR Results Dashboard, accessed May 6, 2025. A total of 5,453 results were submitted over the three-year period, with annual\n\n---\n\n[ID: pdf:Scaling for Impact_MELIA Plan 30-06-2025.pdf:p1pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact%2FScaling%20for%20Impact%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP09%20%2D%20Scaling%20for%20Impact&amp;p=true&amp;ga=1\nFile: Scaling for Impact_MELIA Plan 30-06-2025.pdf\nLocation: page 1 part 4\nContent: Scaling for Impact Program\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p30pt2]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 30 part 2\nContent: of the studies that will allow us to answer impact assessment questions (outcomes\n\n---\n\n[ID: pdf:Food Frontiers and Security_MELIA Plan 30-06-2025.pdf:p8pt1]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security%2FFood%20Frontiers%20and%20Security%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP08%20%2D%20Food%20Frontiers%20and%20Security&amp;p=true&amp;ga=1\nFile: Food Frontiers and Security_MELIA Plan 30-06-2025.pdf\nLocation: page 8 part 1\nContent: Version 1.0 8 evidence is relevant for wider adoption and systemic change. While the exact number of studies is not speciﬁed, the focus on “selected interventions” implies a targeted approach to eƯectively deploy robust methods for evaluating short- and medium-term impacts contributing to the ﬁve CGIAR Impact Areas, prioritizing those with the greatest potential for learning and scaling. CollaboraƟon with other Programs/Accelerators, W3/bilateral projects, and/or partners to deliver the impact assessment work. While speciﬁc details regarding the Frontiers Program’s collaborative impact assessment work are still being formalized, its approach aligns with a broader CGIAR emphasis on synergistic eƯorts. The program is committed to working with other Programs (Policy Innovations and Scaling for Impact SPs), Accelerators,\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p13pt2]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 13 part 2\nContent: additional studies from SPIA (see Impact assessments). Most impacts stemmed from earlier work but were published during this period. Some studies were based on one- or two-years’ worth of data, and other studies were based on data spanning up to four decades (Figure 6). Many of these longer-term studies consider the aggregate effects and net returns of large and longstanding CGIAR work streams. Like the outcomes, measured impacts span all the five Impact Areas, though some Impact Areas are more represented than others. Figure 6. Global evidence base of the impacts and outcomes. Top panel: 18 impact assessment studies did not specify the dates covered by their data and so are not represented. Where studies used datasets with different time periods for different indicators, each time period is represented by a horizontal bar . Middle panel: The middle-center panel expresses the methods used by non-causal impact\n\n---\n\n[ID: pdf:Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf:p26pt4]\nLink: https://cgiar.sharepoint.com/sites/PCUInterim/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes%2FMultifunctional%20Landscapes%5FMELIA%20Plan%2030%2D06%2D2025%2Epdf&amp;parent=%2Fsites%2FPCUInterim%2FShared%20Documents%2F04%2E%20Technical%20Reporting%20%28Allison%29%2F7%2E%20P25%20Inception%2F000%2E%20Inception%20Report%20%2D%20Final%20Attachments%20%2826%20June%29%2FSP04%20%2D%20Multifunctional%20Landscapes&amp;p=true&amp;ga=1\nFile: Multifunctional Landscapes_MELIA Plan 30-06-2025.pdf\nLocation: page 26 part 4\nContent: (from farmer to national level) and to assess different assumptions on how impacts are generated through Multifunctional Landscapes approaches based on co-design and systemic thinking. The specific methodologies used include quantitative counterfactual analysis for adoption and impact measurement (where feasible, as well as evaluation methods that allow to capture multidimensional, unintended and unexpected consequences. Given the complexity and breath of the impacts that the Program aims to influence, impact studies will be targeted to the key areas of success of the Program and will therefore be defined by: • Availability of baselines from the three Initiatives • The results of monitoring and evaluation that will provide guidance on the key Outcomes achieved • The collaboration with other Programs/Accelerators • The studies developed in bilaterals mapped to specific outcomes of\n\n---\n\n[ID: pptx:Information Session on 2025 Technical Reporting.pptx:s3pt3]\nLink: https://docs.google.com/presentation/d/1iH7kEQrUqQywkG9wVkCCBq_tRp-d1Ws0/edit?slide=id.p1#slide=id.p1\nFile: Information Session on 2025 Technical Reporting.pptx\nLocation: slide 3 part 3\nContent: impact-focus: results to be clearly linked and packaged under impacts, outcomes and associated agreed indicator targets. Better linkage between annual Program/Accelerator Theory of Change, Plan of Results and Budget, and Technical Reporting. The primary audiences for Technical Reporting are Funders and CGIAR staff at Integrated Partnership, Portfolio, and Program/Accelerator Levels. The secondary audience is Partners. Annual Technical\n\n---\n\n[ID: pdf:CGIAR_PORB_Scaling_4Impact.pdf:p63pt4]\nLink: https://cgspace.cgiar.org/items/a5c4b258-81b8-42ba-84d5-dad9f42e91dc\nFile: CGIAR_PORB_Scaling_4Impact.pdf\nLocation: page 63 part 4\nContent: program to take these good ideas to scale, reaching more people and places. Credit: Abdul Momin, CIMMYT CGI21-508007-PORB-Scaling for Impact.indd 63CGI21-508007-PORB-Scaling for Impact.indd 63 07/08/2025 13:2407/08/2025\n\n---\n\n[ID: pdf:CGIAR_ImpactReport_2022-24.pdf:p16pt1]\nLink: https://cgspace.cgiar.org/items/ee7728da-7575-4e37-9b7e-c2a7cd23b1c9\nFile: CGIAR_ImpactReport_2022-24.pdf\nLocation: page 16 part 1\nContent: Impacts and outcomes by Impact Area In the following sections, we present evidence of the real- world impacts of CGIAR-supported interventions for each CGIAR Impact Area. Each section starts with an overview of current challenges and CGIAR’s work in that Impact Area. We then summarize the evidence identified pertaining to the Impact Area. Each Impact Area section focuses on the evidence of impact or outcomes on three to four types of work that CGIAR conducts\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p22pt2]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 22 part 2\nContent: June 2025 22 Impact level –\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf:p22pt2]\nLink: N/A\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30 (1).pdf\nLocation: page 22 part 2\nContent: June 2025 22 Impact level –\n\n---\n\n[ID: pdf:CGIAR-Technical-Reporting-Arrangement-2025-30.pdf:p17pt4]\nLink: https://storage.googleapis.com/cgiarorg/2025/06/CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nFile: CGIAR-Technical-Reporting-Arrangement-2025-30.pdf\nLocation: page 17 part 4\nContent: and Impact Area indicators. • Once priority Questions identified, engage SPIA &amp; CGIAR Impact Assessment specialists to refine &amp; design delivery approach, • Contribution from across all funding streams, • Adapt existing Program/Accelerator/w3 &amp; bilateral project data collection approach to strengthen linkage between MEL and IA, based on Impact Case study learnings. • Report Impact Case findings as they become available, and compile in Tri